<commit_message>
auto: anime list update (PC) 2026-09-14
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -1788,7 +1788,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026年10月10日（土）〜 TOKYO MXにて</t>
+          <t>2026年10月10日（土）～ TOKYO MX・BS日テレほか</t>
         </is>
       </c>
       <c r="H27" t="inlineStr"/>
@@ -1874,14 +1874,30 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026年10月～ 読売テレビ・日本テレビ系全国ネットにて</t>
+          <t>2026年10月10日（土）～ 読売テレビ・日本テレビ系全国ネットにて</t>
         </is>
       </c>
       <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Firestarter</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>MAN WITH A MISSION</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>声</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>yutori</t>
+        </is>
+      </c>
       <c r="M29" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=26362</t>
@@ -7114,7 +7130,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O96"/>
+  <dimension ref="A1:O98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8491,7 +8507,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>獣王武神ダンデヴァイン</t>
+          <t>朱色の仮面</t>
         </is>
       </c>
       <c r="D28" t="b">
@@ -8507,12 +8523,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>曲名未発表</t>
+          <t>Firestarter</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>西川貴教</t>
+          <t>MAN WITH A MISSION</t>
         </is>
       </c>
       <c r="I28" t="inlineStr"/>
@@ -8534,7 +8550,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>獣王武神ダンデヴァイン</t>
+          <t>朱色の仮面</t>
         </is>
       </c>
       <c r="D29" t="b">
@@ -8550,12 +8566,12 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>ミカンセイオーディナリー</t>
+          <t>声</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>DayRe:</t>
+          <t>yutori</t>
         </is>
       </c>
       <c r="I29" t="inlineStr"/>
@@ -8577,7 +8593,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>信者ゼロの女神サマと始める異世界攻略</t>
+          <t>獣王武神ダンデヴァイン</t>
         </is>
       </c>
       <c r="D30" t="b">
@@ -8585,7 +8601,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F30" t="n">
@@ -8593,12 +8609,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Fall in Dream</t>
+          <t>曲名未発表</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Suupeas</t>
+          <t>西川貴教</t>
         </is>
       </c>
       <c r="I30" t="inlineStr"/>
@@ -8620,7 +8636,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
+          <t>獣王武神ダンデヴァイン</t>
         </is>
       </c>
       <c r="D31" t="b">
@@ -8628,7 +8644,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F31" t="n">
@@ -8636,12 +8652,12 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Walls And Bridges</t>
+          <t>ミカンセイオーディナリー</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>青酢（越前リョーマ、⼿塚国光、⼤⽯秀⼀郎、不⼆周助）</t>
+          <t>DayRe:</t>
         </is>
       </c>
       <c r="I31" t="inlineStr"/>
@@ -8663,7 +8679,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
+          <t>信者ゼロの女神サマと始める異世界攻略</t>
         </is>
       </c>
       <c r="D32" t="b">
@@ -8679,35 +8695,21 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>金環蝕 phenomenal</t>
+          <t>Fall in Dream</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>跡部景吾＆忍足侑士</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=LLCVfhquaAU</t>
-        </is>
-      </c>
-      <c r="J32" t="n">
-        <v>196660</v>
-      </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>アニメ 新テニスの王子様 オフィシャルチャンネル</t>
-        </is>
-      </c>
+          <t>Suupeas</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t>2026-09-09T09:02:38</t>
-        </is>
-      </c>
+      <c r="O32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -8720,7 +8722,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>生徒会にも穴はある！</t>
+          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
         </is>
       </c>
       <c r="D33" t="b">
@@ -8736,12 +8738,12 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>風の中は走るっきゃないっ！</t>
+          <t>Walls And Bridges</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>三月のパンタシア</t>
+          <t>青酢（越前リョーマ、⼿塚国光、⼤⽯秀⼀郎、不⼆周助）</t>
         </is>
       </c>
       <c r="I33" t="inlineStr"/>
@@ -8763,7 +8765,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>世界最強の魔女、始めました</t>
+          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
         </is>
       </c>
       <c r="D34" t="b">
@@ -8771,7 +8773,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F34" t="n">
@@ -8779,21 +8781,35 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>影響力∞アイドル</t>
+          <t>金環蝕 phenomenal</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>HoneyWorks feat.ハコニワリリィ</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
+          <t>跡部景吾＆忍足侑士</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=LLCVfhquaAU</t>
+        </is>
+      </c>
+      <c r="J34" t="n">
+        <v>196660</v>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>アニメ 新テニスの王子様 オフィシャルチャンネル</t>
+        </is>
+      </c>
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
       <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>2026-09-09T09:02:38</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -8806,7 +8822,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>世界最強の魔女、始めました</t>
+          <t>生徒会にも穴はある！</t>
         </is>
       </c>
       <c r="D35" t="b">
@@ -8814,7 +8830,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F35" t="n">
@@ -8822,12 +8838,12 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>星を巡る</t>
+          <t>風の中は走るっきゃないっ！</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>ロクデナシ</t>
+          <t>三月のパンタシア</t>
         </is>
       </c>
       <c r="I35" t="inlineStr"/>
@@ -8849,7 +8865,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>DARK MACHINE THE ANIMATION</t>
+          <t>世界最強の魔女、始めました</t>
         </is>
       </c>
       <c r="D36" t="b">
@@ -8865,12 +8881,12 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>存在理由 改</t>
+          <t>影響力∞アイドル</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>BUCK∞TICK</t>
+          <t>HoneyWorks feat.ハコニワリリィ</t>
         </is>
       </c>
       <c r="I36" t="inlineStr"/>
@@ -8892,7 +8908,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
+          <t>世界最強の魔女、始めました</t>
         </is>
       </c>
       <c r="D37" t="b">
@@ -8900,7 +8916,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -8908,12 +8924,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Let's Go Crazy</t>
+          <t>星を巡る</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Baby Canta</t>
+          <t>ロクデナシ</t>
         </is>
       </c>
       <c r="I37" t="inlineStr"/>
@@ -8935,7 +8951,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
+          <t>DARK MACHINE THE ANIMATION</t>
         </is>
       </c>
       <c r="D38" t="b">
@@ -8943,7 +8959,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -8951,12 +8967,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>NUMBER</t>
+          <t>存在理由 改</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>SUPER★DRAGON</t>
+          <t>BUCK∞TICK</t>
         </is>
       </c>
       <c r="I38" t="inlineStr"/>
@@ -8978,7 +8994,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>TANK CHAIR-戦車椅子-</t>
+          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
         </is>
       </c>
       <c r="D39" t="b">
@@ -8994,12 +9010,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>DALALA</t>
+          <t>Let's Go Crazy</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>SiM</t>
+          <t>Baby Canta</t>
         </is>
       </c>
       <c r="I39" t="inlineStr"/>
@@ -9021,7 +9037,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>TANK CHAIR-戦車椅子-</t>
+          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
         </is>
       </c>
       <c r="D40" t="b">
@@ -9037,12 +9053,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>SYNC</t>
+          <t>NUMBER</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Daoko</t>
+          <t>SUPER★DRAGON</t>
         </is>
       </c>
       <c r="I40" t="inlineStr"/>
@@ -9064,7 +9080,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>探偵はもう、死んでいる。Season2</t>
+          <t>TANK CHAIR-戦車椅子-</t>
         </is>
       </c>
       <c r="D41" t="b">
@@ -9080,21 +9096,45 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>この心臓に花束を</t>
+          <t>DALALA</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>心梅</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr"/>
-      <c r="O41" t="inlineStr"/>
+          <t>SiM</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=7lbUMzWGK4g</t>
+        </is>
+      </c>
+      <c r="J41" t="n">
+        <v>7569</v>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=7lbUMzWGK4g</t>
+        </is>
+      </c>
+      <c r="M41" t="n">
+        <v>7569</v>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>2026-09-14T09:02:42</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -9107,7 +9147,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>探偵はもう、死んでいる。Season2</t>
+          <t>TANK CHAIR-戦車椅子-</t>
         </is>
       </c>
       <c r="D42" t="b">
@@ -9123,35 +9163,21 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>白昼夢</t>
+          <t>SYNC</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>カグラナナ</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=WAjXT8Q109U</t>
-        </is>
-      </c>
-      <c r="J42" t="n">
-        <v>2568317</v>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>カグラナナchannel／ななかぐら</t>
-        </is>
-      </c>
+          <t>Daoko</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr"/>
       <c r="N42" t="inlineStr"/>
-      <c r="O42" t="inlineStr">
-        <is>
-          <t>2026-09-11T09:03:02</t>
-        </is>
-      </c>
+      <c r="O42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -9164,7 +9190,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>千歳くんはラムネ瓶のなか 第2クール</t>
+          <t>探偵はもう、死んでいる。Season2</t>
         </is>
       </c>
       <c r="D43" t="b">
@@ -9180,45 +9206,21 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>ライアー</t>
+          <t>この心臓に花束を</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Kucci</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
-        </is>
-      </c>
-      <c r="J43" t="n">
-        <v>732591</v>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
-        </is>
-      </c>
-      <c r="M43" t="n">
-        <v>732591</v>
-      </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="O43" t="inlineStr">
-        <is>
-          <t>2026-09-09T09:03:29</t>
-        </is>
-      </c>
+          <t>心梅</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -9231,7 +9233,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>千歳くんはラムネ瓶のなか 第2クール</t>
+          <t>探偵はもう、死んでいる。Season2</t>
         </is>
       </c>
       <c r="D44" t="b">
@@ -9247,43 +9249,33 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>陽炎</t>
+          <t>白昼夢</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>サイダーガール</t>
+          <t>カグラナナ</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
+          <t>https://www.youtube.com/watch?v=WAjXT8Q109U</t>
         </is>
       </c>
       <c r="J44" t="n">
-        <v>411641</v>
+        <v>2568317</v>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
-        </is>
-      </c>
-      <c r="M44" t="n">
-        <v>411641</v>
-      </c>
-      <c r="N44" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
+          <t>カグラナナchannel／ななかぐら</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" t="inlineStr"/>
       <c r="O44" t="inlineStr">
         <is>
-          <t>2026-09-09T09:03:38</t>
+          <t>2026-09-11T09:03:02</t>
         </is>
       </c>
     </row>
@@ -9298,7 +9290,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>追放されたチート付与魔術師は気ままなセカンドライフを謳歌する。</t>
+          <t>千歳くんはラムネ瓶のなか 第2クール</t>
         </is>
       </c>
       <c r="D45" t="b">
@@ -9314,21 +9306,45 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>エンバートーチ</t>
+          <t>ライアー</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>sumika</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
-      <c r="O45" t="inlineStr"/>
+          <t>Kucci</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
+        </is>
+      </c>
+      <c r="J45" t="n">
+        <v>732591</v>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
+        </is>
+      </c>
+      <c r="M45" t="n">
+        <v>732591</v>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>2026-09-09T09:03:29</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -9341,7 +9357,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>てつりょー！meet with 鉄道むすめ</t>
+          <t>千歳くんはラムネ瓶のなか 第2クール</t>
         </is>
       </c>
       <c r="D46" t="b">
@@ -9357,21 +9373,45 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>わたし未来線</t>
+          <t>陽炎</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>てつりょー会（橘めい・庄子真央・福嶋晴菜・月城日花）</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
-      <c r="N46" t="inlineStr"/>
-      <c r="O46" t="inlineStr"/>
+          <t>サイダーガール</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
+        </is>
+      </c>
+      <c r="J46" t="n">
+        <v>411641</v>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
+        </is>
+      </c>
+      <c r="M46" t="n">
+        <v>411641</v>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>2026-09-09T09:03:38</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -9384,7 +9424,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>テムパル～アイテムの力～</t>
+          <t>追放されたチート付与魔術師は気ままなセカンドライフを謳歌する。</t>
         </is>
       </c>
       <c r="D47" t="b">
@@ -9400,12 +9440,12 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>SATISFY</t>
+          <t>エンバートーチ</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Re:name</t>
+          <t>sumika</t>
         </is>
       </c>
       <c r="I47" t="inlineStr"/>
@@ -9427,7 +9467,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>テムパル～アイテムの力～</t>
+          <t>てつりょー！meet with 鉄道むすめ</t>
         </is>
       </c>
       <c r="D48" t="b">
@@ -9443,12 +9483,12 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Ray of Emotion</t>
+          <t>わたし未来線</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>導凰</t>
+          <t>てつりょー会（橘めい・庄子真央・福嶋晴菜・月城日花）</t>
         </is>
       </c>
       <c r="I48" t="inlineStr"/>
@@ -9470,7 +9510,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>デモンズ・クレスト</t>
+          <t>テムパル～アイテムの力～</t>
         </is>
       </c>
       <c r="D49" t="b">
@@ -9486,12 +9526,12 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>シンカ</t>
+          <t>SATISFY</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Ado</t>
+          <t>Re:name</t>
         </is>
       </c>
       <c r="I49" t="inlineStr"/>
@@ -9513,7 +9553,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Duel Masters LOST ～断罪の少年～</t>
+          <t>テムパル～アイテムの力～</t>
         </is>
       </c>
       <c r="D50" t="b">
@@ -9521,7 +9561,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F50" t="n">
@@ -9529,35 +9569,21 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>あやかしあやし</t>
+          <t>Ray of Emotion</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>伊東歌詞太郎</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=dYHTC2QyGTs</t>
-        </is>
-      </c>
-      <c r="J50" t="n">
-        <v>49742</v>
-      </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>デュエチューブ-DM公式-</t>
-        </is>
-      </c>
+          <t>導凰</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr"/>
       <c r="M50" t="inlineStr"/>
       <c r="N50" t="inlineStr"/>
-      <c r="O50" t="inlineStr">
-        <is>
-          <t>2026-09-09T09:04:16</t>
-        </is>
-      </c>
+      <c r="O50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -9570,7 +9596,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Duel Masters LOST ～断罪の少年～</t>
+          <t>デモンズ・クレスト</t>
         </is>
       </c>
       <c r="D51" t="b">
@@ -9578,7 +9604,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F51" t="n">
@@ -9586,45 +9612,21 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>朔日 feat. 吉乃</t>
+          <t>シンカ</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>月詠み</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=L3JeU4bIHNk</t>
-        </is>
-      </c>
-      <c r="J51" t="n">
-        <v>48571</v>
-      </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>デュエチューブ-DM公式-</t>
-        </is>
-      </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=L3JeU4bIHNk</t>
-        </is>
-      </c>
-      <c r="M51" t="n">
-        <v>48571</v>
-      </c>
-      <c r="N51" t="inlineStr">
-        <is>
-          <t>デュエチューブ-DM公式-</t>
-        </is>
-      </c>
-      <c r="O51" t="inlineStr">
-        <is>
-          <t>2026-09-09T09:04:22</t>
-        </is>
-      </c>
+          <t>Ado</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="inlineStr"/>
+      <c r="O51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -9637,7 +9639,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>転生貴族、鑑定スキルで成り上がる 第3期</t>
+          <t>Duel Masters LOST ～断罪の少年～</t>
         </is>
       </c>
       <c r="D52" t="b">
@@ -9653,21 +9655,35 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Still Water</t>
+          <t>あやかしあやし</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>佐々木李子</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
+          <t>伊東歌詞太郎</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=dYHTC2QyGTs</t>
+        </is>
+      </c>
+      <c r="J52" t="n">
+        <v>49742</v>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>デュエチューブ-DM公式-</t>
+        </is>
+      </c>
       <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr"/>
       <c r="N52" t="inlineStr"/>
-      <c r="O52" t="inlineStr"/>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>2026-09-09T09:04:16</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -9680,7 +9696,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>転生貴族、鑑定スキルで成り上がる 第3期</t>
+          <t>Duel Masters LOST ～断罪の少年～</t>
         </is>
       </c>
       <c r="D53" t="b">
@@ -9696,21 +9712,45 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>日々を越えて</t>
+          <t>朔日 feat. 吉乃</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>明くる夜の羊</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr"/>
-      <c r="M53" t="inlineStr"/>
-      <c r="N53" t="inlineStr"/>
-      <c r="O53" t="inlineStr"/>
+          <t>月詠み</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=L3JeU4bIHNk</t>
+        </is>
+      </c>
+      <c r="J53" t="n">
+        <v>48571</v>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>デュエチューブ-DM公式-</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=L3JeU4bIHNk</t>
+        </is>
+      </c>
+      <c r="M53" t="n">
+        <v>48571</v>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>デュエチューブ-DM公式-</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>2026-09-09T09:04:22</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -9723,7 +9763,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>転生ゴブリンだけど質問ある？</t>
+          <t>転生貴族、鑑定スキルで成り上がる 第3期</t>
         </is>
       </c>
       <c r="D54" t="b">
@@ -9739,12 +9779,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>ハロー</t>
+          <t>Still Water</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Sou</t>
+          <t>佐々木李子</t>
         </is>
       </c>
       <c r="I54" t="inlineStr"/>
@@ -9766,7 +9806,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>転生ゴブリンだけど質問ある？</t>
+          <t>転生貴族、鑑定スキルで成り上がる 第3期</t>
         </is>
       </c>
       <c r="D55" t="b">
@@ -9782,12 +9822,12 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>小さな僕ら</t>
+          <t>日々を越えて</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>エイハブ</t>
+          <t>明くる夜の羊</t>
         </is>
       </c>
       <c r="I55" t="inlineStr"/>
@@ -9809,7 +9849,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>転生ゴブリンだけど質問ある？</t>
         </is>
       </c>
       <c r="D56" t="b">
@@ -9825,12 +9865,12 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Flare of Soul</t>
+          <t>ハロー</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>花耶</t>
+          <t>Sou</t>
         </is>
       </c>
       <c r="I56" t="inlineStr"/>
@@ -9852,7 +9892,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>転生ゴブリンだけど質問ある？</t>
         </is>
       </c>
       <c r="D57" t="b">
@@ -9868,12 +9908,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>STELLAR</t>
+          <t>小さな僕ら</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>ウタヒメドリーム オールスターズ</t>
+          <t>エイハブ</t>
         </is>
       </c>
       <c r="I57" t="inlineStr"/>
@@ -9895,7 +9935,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>転生したら剣でしたII</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="D58" t="b">
@@ -9911,12 +9951,12 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>DREAM OF BUTTERFLY</t>
+          <t>Flare of Soul</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>FZMZ</t>
+          <t>花耶</t>
         </is>
       </c>
       <c r="I58" t="inlineStr"/>
@@ -9938,7 +9978,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>転生したら剣でしたII</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="D59" t="b">
@@ -9954,12 +9994,12 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>バリバリBuddy</t>
+          <t>STELLAR</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>花冷え。</t>
+          <t>ウタヒメドリーム オールスターズ</t>
         </is>
       </c>
       <c r="I59" t="inlineStr"/>
@@ -9981,7 +10021,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>とある暗部の少女共棲</t>
+          <t>転生したら剣でしたII</t>
         </is>
       </c>
       <c r="D60" t="b">
@@ -9997,12 +10037,12 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Ghost Sequence</t>
+          <t>DREAM OF BUTTERFLY</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>East Of Eden</t>
+          <t>FZMZ</t>
         </is>
       </c>
       <c r="I60" t="inlineStr"/>
@@ -10024,7 +10064,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>とある暗部の少女共棲</t>
+          <t>転生したら剣でしたII</t>
         </is>
       </c>
       <c r="D61" t="b">
@@ -10040,12 +10080,12 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>原子崩し(メルトダウナー)</t>
+          <t>バリバリBuddy</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>岸田教団&amp;THE明星ロケッツ</t>
+          <t>花冷え。</t>
         </is>
       </c>
       <c r="I61" t="inlineStr"/>
@@ -10067,7 +10107,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>東京リベンジャーズ 三天戦争編</t>
+          <t>とある暗部の少女共棲</t>
         </is>
       </c>
       <c r="D62" t="b">
@@ -10083,35 +10123,21 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>IGNITE</t>
+          <t>Ghost Sequence</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>JO1</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=u0uxN_2wZ_w</t>
-        </is>
-      </c>
-      <c r="J62" t="n">
-        <v>139300</v>
-      </c>
-      <c r="K62" t="inlineStr">
-        <is>
-          <t>JO1</t>
-        </is>
-      </c>
+          <t>East Of Eden</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr"/>
       <c r="M62" t="inlineStr"/>
       <c r="N62" t="inlineStr"/>
-      <c r="O62" t="inlineStr">
-        <is>
-          <t>2026-09-07T09:04:27</t>
-        </is>
-      </c>
+      <c r="O62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -10124,7 +10150,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>東京リベンジャーズ 三天戦争編</t>
+          <t>とある暗部の少女共棲</t>
         </is>
       </c>
       <c r="D63" t="b">
@@ -10140,43 +10166,33 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>トリックスター</t>
+          <t>原子崩し(メルトダウナー)</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>go!go!vanillas</t>
+          <t>岸田教団&amp;THE明星ロケッツ</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=qcmjeeCS380</t>
+          <t>https://www.youtube.com/watch?v=JH927fq9qaM</t>
         </is>
       </c>
       <c r="J63" t="n">
-        <v>151085</v>
+        <v>3888</v>
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>go!go!vanillas</t>
-        </is>
-      </c>
-      <c r="L63" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=PX-RhjDLVDQ</t>
-        </is>
-      </c>
-      <c r="M63" t="n">
-        <v>3846269</v>
-      </c>
-      <c r="N63" t="inlineStr">
-        <is>
-          <t>TV anime "Tokyo Revengers"</t>
-        </is>
-      </c>
+          <t>Kisidakyoudan &amp; the Akebosi rockets official</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr"/>
+      <c r="N63" t="inlineStr"/>
       <c r="O63" t="inlineStr">
         <is>
-          <t>2026-09-07T09:04:39</t>
+          <t>2026-09-14T09:04:34</t>
         </is>
       </c>
     </row>
@@ -10191,7 +10207,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>ドラゴンボール超 ビルス</t>
+          <t>東京リベンジャーズ 三天戦争編</t>
         </is>
       </c>
       <c r="D64" t="b">
@@ -10207,43 +10223,43 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>オノガミ</t>
+          <t>IGNITE</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>メガテラ・ゼロ</t>
+          <t>JO1</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=iyKK-RTzf1o</t>
+          <t>https://www.youtube.com/watch?v=3rTOBRwAi24</t>
         </is>
       </c>
       <c r="J64" t="n">
-        <v>28231</v>
+        <v>262450</v>
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>hyou - Anime on Piano</t>
+          <t>JO1</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=iyKK-RTzf1o</t>
+          <t>https://www.youtube.com/watch?v=tYuPxILnixw</t>
         </is>
       </c>
       <c r="M64" t="n">
-        <v>28231</v>
+        <v>7195703</v>
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t>hyou - Anime on Piano</t>
+          <t>TV anime "Tokyo Revengers"</t>
         </is>
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>2026-09-11T09:04:43</t>
+          <t>2026-09-14T09:04:48</t>
         </is>
       </c>
     </row>
@@ -10258,7 +10274,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>ドラゴンボール超 ビルス</t>
+          <t>東京リベンジャーズ 三天戦争編</t>
         </is>
       </c>
       <c r="D65" t="b">
@@ -10274,21 +10290,45 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>完璧のペキ</t>
+          <t>トリックスター</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>ビッケブランカ</t>
-        </is>
-      </c>
-      <c r="I65" t="inlineStr"/>
-      <c r="J65" t="inlineStr"/>
-      <c r="K65" t="inlineStr"/>
-      <c r="L65" t="inlineStr"/>
-      <c r="M65" t="inlineStr"/>
-      <c r="N65" t="inlineStr"/>
-      <c r="O65" t="inlineStr"/>
+          <t>go!go!vanillas</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=qcmjeeCS380</t>
+        </is>
+      </c>
+      <c r="J65" t="n">
+        <v>180739</v>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>go!go!vanillas</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=PX-RhjDLVDQ</t>
+        </is>
+      </c>
+      <c r="M65" t="n">
+        <v>3867868</v>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>TV anime "Tokyo Revengers"</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>2026-09-14T09:05:01</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -10301,7 +10341,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>ねずみくんのチョッキ 2期</t>
+          <t>ドラゴンボール超 ビルス</t>
         </is>
       </c>
       <c r="D66" t="b">
@@ -10309,7 +10349,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F66" t="n">
@@ -10317,21 +10357,45 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>グッドラック！マイフレンド feat.ムロツヨシ &amp; さかなクン</t>
+          <t>オノガミ</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>東京スカパラダイスオーケストラ</t>
-        </is>
-      </c>
-      <c r="I66" t="inlineStr"/>
-      <c r="J66" t="inlineStr"/>
-      <c r="K66" t="inlineStr"/>
-      <c r="L66" t="inlineStr"/>
-      <c r="M66" t="inlineStr"/>
-      <c r="N66" t="inlineStr"/>
-      <c r="O66" t="inlineStr"/>
+          <t>メガテラ・ゼロ</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=iyKK-RTzf1o</t>
+        </is>
+      </c>
+      <c r="J66" t="n">
+        <v>28231</v>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>hyou - Anime on Piano</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=iyKK-RTzf1o</t>
+        </is>
+      </c>
+      <c r="M66" t="n">
+        <v>28231</v>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>hyou - Anime on Piano</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>2026-09-11T09:04:43</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -10344,7 +10408,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>パンどろぼう</t>
+          <t>ドラゴンボール超 ビルス</t>
         </is>
       </c>
       <c r="D67" t="b">
@@ -10352,7 +10416,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F67" t="n">
@@ -10360,12 +10424,12 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>パンどろぼうのうた</t>
+          <t>完璧のペキ</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>パンどろぼうとパンやのおじさん（CV：朝井彩加とCV：諏訪部順一）</t>
+          <t>ビッケブランカ</t>
         </is>
       </c>
       <c r="I67" t="inlineStr"/>
@@ -10387,7 +10451,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>冰剣の魔術師が世界を統べるⅡ</t>
+          <t>ねずみくんのチョッキ 2期</t>
         </is>
       </c>
       <c r="D68" t="b">
@@ -10395,7 +10459,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F68" t="n">
@@ -10403,35 +10467,21 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Diamond Dust</t>
+          <t>グッドラック！マイフレンド feat.ムロツヨシ &amp; さかなクン</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>Sizuk</t>
-        </is>
-      </c>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=GuMiQyzuJSs</t>
-        </is>
-      </c>
-      <c r="J68" t="n">
-        <v>6308</v>
-      </c>
-      <c r="K68" t="inlineStr">
-        <is>
-          <t>Sizuk / Shunryu</t>
-        </is>
-      </c>
+          <t>東京スカパラダイスオーケストラ</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr"/>
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr"/>
       <c r="M68" t="inlineStr"/>
       <c r="N68" t="inlineStr"/>
-      <c r="O68" t="inlineStr">
-        <is>
-          <t>2026-09-11T09:05:34</t>
-        </is>
-      </c>
+      <c r="O68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -10444,7 +10494,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>冰剣の魔術師が世界を統べるⅡ</t>
+          <t>パンどろぼう</t>
         </is>
       </c>
       <c r="D69" t="b">
@@ -10452,7 +10502,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F69" t="n">
@@ -10460,35 +10510,21 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>COMPRESSION :[</t>
+          <t>パンどろぼうのうた</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>内田真礼</t>
-        </is>
-      </c>
-      <c r="I69" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=MFiWYth0mpg</t>
-        </is>
-      </c>
-      <c r="J69" t="n">
-        <v>11608</v>
-      </c>
-      <c r="K69" t="inlineStr">
-        <is>
-          <t>内田真礼（UCHIDA MAAYA）Official Channel</t>
-        </is>
-      </c>
+          <t>パンどろぼうとパンやのおじさん（CV：朝井彩加とCV：諏訪部順一）</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr"/>
       <c r="M69" t="inlineStr"/>
       <c r="N69" t="inlineStr"/>
-      <c r="O69" t="inlineStr">
-        <is>
-          <t>2026-09-09T09:06:00</t>
-        </is>
-      </c>
+      <c r="O69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -10501,7 +10537,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>ブラッククローバー 2nd Season</t>
+          <t>冰剣の魔術師が世界を統べるⅡ</t>
         </is>
       </c>
       <c r="D70" t="b">
@@ -10517,43 +10553,33 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>消えない理由</t>
+          <t>Diamond Dust</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>WANIMA</t>
+          <t>Sizuk</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
+          <t>https://www.youtube.com/watch?v=GuMiQyzuJSs</t>
         </is>
       </c>
       <c r="J70" t="n">
-        <v>5969</v>
+        <v>6308</v>
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>Anime Trailer アニメ</t>
-        </is>
-      </c>
-      <c r="L70" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
-        </is>
-      </c>
-      <c r="M70" t="n">
-        <v>5969</v>
-      </c>
-      <c r="N70" t="inlineStr">
-        <is>
-          <t>Anime Trailer アニメ</t>
-        </is>
-      </c>
+          <t>Sizuk / Shunryu</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr"/>
+      <c r="M70" t="inlineStr"/>
+      <c r="N70" t="inlineStr"/>
       <c r="O70" t="inlineStr">
         <is>
-          <t>2026-09-09T09:06:07</t>
+          <t>2026-09-11T09:05:34</t>
         </is>
       </c>
     </row>
@@ -10568,7 +10594,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>ブラッククローバー 2nd Season</t>
+          <t>冰剣の魔術師が世界を統べるⅡ</t>
         </is>
       </c>
       <c r="D71" t="b">
@@ -10584,21 +10610,35 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Yellow Brick Road</t>
+          <t>COMPRESSION :[</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>ONE OR EIGHT</t>
-        </is>
-      </c>
-      <c r="I71" t="inlineStr"/>
-      <c r="J71" t="inlineStr"/>
-      <c r="K71" t="inlineStr"/>
+          <t>内田真礼</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=MFiWYth0mpg</t>
+        </is>
+      </c>
+      <c r="J71" t="n">
+        <v>11608</v>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>内田真礼（UCHIDA MAAYA）Official Channel</t>
+        </is>
+      </c>
       <c r="L71" t="inlineStr"/>
       <c r="M71" t="inlineStr"/>
       <c r="N71" t="inlineStr"/>
-      <c r="O71" t="inlineStr"/>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>2026-09-09T09:06:00</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -10611,7 +10651,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>ホタルの嫁入り</t>
+          <t>ブラッククローバー 2nd Season</t>
         </is>
       </c>
       <c r="D72" t="b">
@@ -10619,7 +10659,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F72" t="n">
@@ -10627,33 +10667,43 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>夢心地</t>
+          <t>消えない理由</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>TOOBOE</t>
+          <t>WANIMA</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=TE3McAbD7DA</t>
+          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
         </is>
       </c>
       <c r="J72" t="n">
-        <v>786238</v>
+        <v>5969</v>
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>john / TOOBOE</t>
-        </is>
-      </c>
-      <c r="L72" t="inlineStr"/>
-      <c r="M72" t="inlineStr"/>
-      <c r="N72" t="inlineStr"/>
+          <t>Anime Trailer アニメ</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
+        </is>
+      </c>
+      <c r="M72" t="n">
+        <v>5969</v>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>Anime Trailer アニメ</t>
+        </is>
+      </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>2026-09-09T09:06:32</t>
+          <t>2026-09-09T09:06:07</t>
         </is>
       </c>
     </row>
@@ -10668,7 +10718,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>マウスカーソルで現実を操作できるようになったので、女の子をいっぱいクリックしまーす</t>
+          <t>ブラッククローバー 2nd Season</t>
         </is>
       </c>
       <c r="D73" t="b">
@@ -10676,7 +10726,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F73" t="n">
@@ -10684,12 +10734,12 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>MOUSE DRIVE</t>
+          <t>Yellow Brick Road</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>Maware Isogavva</t>
+          <t>ONE OR EIGHT</t>
         </is>
       </c>
       <c r="I73" t="inlineStr"/>
@@ -10711,7 +10761,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>マジカル★エクスプローラー</t>
+          <t>ホタルの嫁入り</t>
         </is>
       </c>
       <c r="D74" t="b">
@@ -10719,7 +10769,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F74" t="n">
@@ -10727,21 +10777,35 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Remedy</t>
+          <t>夢心地</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>ASCA</t>
-        </is>
-      </c>
-      <c r="I74" t="inlineStr"/>
-      <c r="J74" t="inlineStr"/>
-      <c r="K74" t="inlineStr"/>
+          <t>TOOBOE</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=TE3McAbD7DA</t>
+        </is>
+      </c>
+      <c r="J74" t="n">
+        <v>786238</v>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>john / TOOBOE</t>
+        </is>
+      </c>
       <c r="L74" t="inlineStr"/>
       <c r="M74" t="inlineStr"/>
       <c r="N74" t="inlineStr"/>
-      <c r="O74" t="inlineStr"/>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>2026-09-09T09:06:32</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -10754,7 +10818,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>マジカル★エクスプローラー</t>
+          <t>マウスカーソルで現実を操作できるようになったので、女の子をいっぱいクリックしまーす</t>
         </is>
       </c>
       <c r="D75" t="b">
@@ -10762,7 +10826,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F75" t="n">
@@ -10770,12 +10834,12 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Double Wings</t>
+          <t>MOUSE DRIVE</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>ASCA</t>
+          <t>Maware Isogavva</t>
         </is>
       </c>
       <c r="I75" t="inlineStr"/>
@@ -10797,7 +10861,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>マジカル★エクスプローラー</t>
         </is>
       </c>
       <c r="D76" t="b">
@@ -10813,35 +10877,21 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>No tears here</t>
+          <t>Remedy</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>茅原実里</t>
-        </is>
-      </c>
-      <c r="I76" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=-PX7FqZ55tE</t>
-        </is>
-      </c>
-      <c r="J76" t="n">
-        <v>109555</v>
-      </c>
-      <c r="K76" t="inlineStr">
-        <is>
-          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
-        </is>
-      </c>
+          <t>ASCA</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr"/>
+      <c r="J76" t="inlineStr"/>
+      <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr"/>
       <c r="M76" t="inlineStr"/>
       <c r="N76" t="inlineStr"/>
-      <c r="O76" t="inlineStr">
-        <is>
-          <t>2026-09-09T09:07:02</t>
-        </is>
-      </c>
+      <c r="O76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -10854,7 +10904,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>マジカル★エクスプローラー</t>
         </is>
       </c>
       <c r="D77" t="b">
@@ -10870,35 +10920,21 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>ReMind</t>
+          <t>Double Wings</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>Daisy×Daisy</t>
-        </is>
-      </c>
-      <c r="I77" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=iD1hmEvGQmM</t>
-        </is>
-      </c>
-      <c r="J77" t="n">
-        <v>85746</v>
-      </c>
-      <c r="K77" t="inlineStr">
-        <is>
-          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
-        </is>
-      </c>
+          <t>ASCA</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr"/>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr"/>
       <c r="M77" t="inlineStr"/>
       <c r="N77" t="inlineStr"/>
-      <c r="O77" t="inlineStr">
-        <is>
-          <t>2026-09-11T09:06:07</t>
-        </is>
-      </c>
+      <c r="O77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -10911,7 +10947,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+          <t>魔法少女育成計画restart</t>
         </is>
       </c>
       <c r="D78" t="b">
@@ -10927,43 +10963,33 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Bubee</t>
+          <t>No tears here</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>ILLIT</t>
+          <t>茅原実里</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+          <t>https://www.youtube.com/watch?v=-PX7FqZ55tE</t>
         </is>
       </c>
       <c r="J78" t="n">
-        <v>314538</v>
+        <v>109555</v>
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
-      <c r="L78" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
-        </is>
-      </c>
-      <c r="M78" t="n">
-        <v>314538</v>
-      </c>
-      <c r="N78" t="inlineStr">
-        <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
+          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr"/>
+      <c r="M78" t="inlineStr"/>
+      <c r="N78" t="inlineStr"/>
       <c r="O78" t="inlineStr">
         <is>
-          <t>2026-09-07T09:05:41</t>
+          <t>2026-09-09T09:07:02</t>
         </is>
       </c>
     </row>
@@ -10978,7 +11004,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+          <t>魔法少女育成計画restart</t>
         </is>
       </c>
       <c r="D79" t="b">
@@ -10986,29 +11012,43 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Swingin' Magic</t>
+          <t>ReMind</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>ILLIT</t>
-        </is>
-      </c>
-      <c r="I79" t="inlineStr"/>
-      <c r="J79" t="inlineStr"/>
-      <c r="K79" t="inlineStr"/>
+          <t>Daisy×Daisy</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=iD1hmEvGQmM</t>
+        </is>
+      </c>
+      <c r="J79" t="n">
+        <v>85746</v>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
+        </is>
+      </c>
       <c r="L79" t="inlineStr"/>
       <c r="M79" t="inlineStr"/>
       <c r="N79" t="inlineStr"/>
-      <c r="O79" t="inlineStr"/>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>2026-09-11T09:06:07</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -11029,7 +11069,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F80" t="n">
@@ -11037,12 +11077,12 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Calling</t>
+          <t>Bubee</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
+          <t>ILLIT</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -11051,7 +11091,7 @@
         </is>
       </c>
       <c r="J80" t="n">
-        <v>314538</v>
+        <v>317795</v>
       </c>
       <c r="K80" t="inlineStr">
         <is>
@@ -11064,7 +11104,7 @@
         </is>
       </c>
       <c r="M80" t="n">
-        <v>314538</v>
+        <v>317795</v>
       </c>
       <c r="N80" t="inlineStr">
         <is>
@@ -11073,7 +11113,7 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>2026-09-07T09:05:54</t>
+          <t>2026-09-14T09:06:07</t>
         </is>
       </c>
     </row>
@@ -11096,7 +11136,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F81" t="n">
@@ -11104,12 +11144,12 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>どりぃむアラモード</t>
+          <t>Swingin' Magic</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
+          <t>ILLIT</t>
         </is>
       </c>
       <c r="I81" t="inlineStr"/>
@@ -11131,7 +11171,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>マロニエ王国の七人の騎士</t>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
         </is>
       </c>
       <c r="D82" t="b">
@@ -11139,7 +11179,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F82" t="n">
@@ -11147,21 +11187,45 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>さよならは言わない</t>
+          <t>Calling</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>yama</t>
-        </is>
-      </c>
-      <c r="I82" t="inlineStr"/>
-      <c r="J82" t="inlineStr"/>
-      <c r="K82" t="inlineStr"/>
-      <c r="L82" t="inlineStr"/>
-      <c r="M82" t="inlineStr"/>
-      <c r="N82" t="inlineStr"/>
-      <c r="O82" t="inlineStr"/>
+          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="J82" t="n">
+        <v>317802</v>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="M82" t="n">
+        <v>317802</v>
+      </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>2026-09-14T09:06:21</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -11174,7 +11238,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
         </is>
       </c>
       <c r="D83" t="b">
@@ -11182,20 +11246,20 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F83" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>UNSTOPPABLE</t>
+          <t>どりぃむアラモード</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>FLOW</t>
+          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
         </is>
       </c>
       <c r="I83" t="inlineStr"/>
@@ -11217,7 +11281,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>マロニエ王国の七人の騎士</t>
         </is>
       </c>
       <c r="D84" t="b">
@@ -11225,7 +11289,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F84" t="n">
@@ -11233,12 +11297,12 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>MY WAY</t>
+          <t>さよならは言わない</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>ASTERISM</t>
+          <t>yama</t>
         </is>
       </c>
       <c r="I84" t="inlineStr"/>
@@ -11260,11 +11324,11 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>メダリスト</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="D85" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -11276,12 +11340,12 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>BOW AND ARROW</t>
+          <t>UNSTOPPABLE</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>米津玄師</t>
+          <t>FLOW</t>
         </is>
       </c>
       <c r="I85" t="inlineStr"/>
@@ -11303,11 +11367,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>メダリスト</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="D86" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -11319,12 +11383,12 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>アタシのドレス</t>
+          <t>MY WAY</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>ねぐせ。</t>
+          <t>ASTERISM</t>
         </is>
       </c>
       <c r="I86" t="inlineStr"/>
@@ -11346,11 +11410,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>野生のラスボスが現れた！ 第2期</t>
+          <t>メダリスト</t>
         </is>
       </c>
       <c r="D87" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -11362,12 +11426,12 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Melodic Impact</t>
+          <t>BOW AND ARROW</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>Suspended 4th</t>
+          <t>米津玄師</t>
         </is>
       </c>
       <c r="I87" t="inlineStr"/>
@@ -11389,15 +11453,15 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>メダリスト</t>
         </is>
       </c>
       <c r="D88" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F88" t="n">
@@ -11405,45 +11469,21 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>What's "KAZOKU"</t>
+          <t>アタシのドレス</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>櫻坂46</t>
-        </is>
-      </c>
-      <c r="I88" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=4SdeuouXcWI</t>
-        </is>
-      </c>
-      <c r="J88" t="n">
-        <v>1079508</v>
-      </c>
-      <c r="K88" t="inlineStr">
-        <is>
-          <t>櫻坂46 OFFICIAL YouTube CHANNEL</t>
-        </is>
-      </c>
-      <c r="L88" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=AIspds2UVts</t>
-        </is>
-      </c>
-      <c r="M88" t="n">
-        <v>421795</v>
-      </c>
-      <c r="N88" t="inlineStr">
-        <is>
-          <t>NBCUniversal Anime/Music</t>
-        </is>
-      </c>
-      <c r="O88" t="inlineStr">
-        <is>
-          <t>2026-09-09T09:07:37</t>
-        </is>
-      </c>
+          <t>ねぐせ。</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr"/>
+      <c r="J88" t="inlineStr"/>
+      <c r="K88" t="inlineStr"/>
+      <c r="L88" t="inlineStr"/>
+      <c r="M88" t="inlineStr"/>
+      <c r="N88" t="inlineStr"/>
+      <c r="O88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -11456,7 +11496,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>野生のラスボスが現れた！ 第2期</t>
         </is>
       </c>
       <c r="D89" t="b">
@@ -11468,16 +11508,16 @@
         </is>
       </c>
       <c r="F89" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>フォーエバーソング</t>
+          <t>Melodic Impact</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>ハンブレッダーズ</t>
+          <t>Suspended 4th</t>
         </is>
       </c>
       <c r="I89" t="inlineStr"/>
@@ -11507,7 +11547,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F90" t="n">
@@ -11515,34 +11555,34 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Shalala</t>
+          <t>What's "KAZOKU"</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>ピラフ星人</t>
+          <t>櫻坂46</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=Y3NFoDTvt6I</t>
+          <t>https://www.youtube.com/watch?v=4SdeuouXcWI</t>
         </is>
       </c>
       <c r="J90" t="n">
-        <v>474339</v>
+        <v>1079508</v>
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>ピラフ星人</t>
+          <t>櫻坂46 OFFICIAL YouTube CHANNEL</t>
         </is>
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=X6fNe1uPs9E</t>
+          <t>https://www.youtube.com/watch?v=AIspds2UVts</t>
         </is>
       </c>
       <c r="M90" t="n">
-        <v>424665</v>
+        <v>421795</v>
       </c>
       <c r="N90" t="inlineStr">
         <is>
@@ -11551,7 +11591,7 @@
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>2026-09-09T09:07:52</t>
+          <t>2026-09-09T09:07:37</t>
         </is>
       </c>
     </row>
@@ -11574,7 +11614,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F91" t="n">
@@ -11582,12 +11622,12 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>I’m still breathing</t>
+          <t>フォーエバーソング</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>KID PHENOMENON</t>
+          <t>ハンブレッダーズ</t>
         </is>
       </c>
       <c r="I91" t="inlineStr"/>
@@ -11609,7 +11649,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>弱気MAX令嬢なのに、辣腕婚約者様の賭けに乗ってしまった</t>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
         </is>
       </c>
       <c r="D92" t="b">
@@ -11617,7 +11657,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F92" t="n">
@@ -11625,21 +11665,45 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>強気MAX宣言</t>
+          <t>Shalala</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>鈴木このみ</t>
-        </is>
-      </c>
-      <c r="I92" t="inlineStr"/>
-      <c r="J92" t="inlineStr"/>
-      <c r="K92" t="inlineStr"/>
-      <c r="L92" t="inlineStr"/>
-      <c r="M92" t="inlineStr"/>
-      <c r="N92" t="inlineStr"/>
-      <c r="O92" t="inlineStr"/>
+          <t>ピラフ星人</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Y3NFoDTvt6I</t>
+        </is>
+      </c>
+      <c r="J92" t="n">
+        <v>474339</v>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>ピラフ星人</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=X6fNe1uPs9E</t>
+        </is>
+      </c>
+      <c r="M92" t="n">
+        <v>424665</v>
+      </c>
+      <c r="N92" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>2026-09-09T09:07:52</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -11652,7 +11716,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>弱気MAX令嬢なのに、辣腕婚約者様の賭けに乗ってしまった</t>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
         </is>
       </c>
       <c r="D93" t="b">
@@ -11664,49 +11728,25 @@
         </is>
       </c>
       <c r="F93" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>夜明けまでに</t>
+          <t>I’m still breathing</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>伊藤美来</t>
-        </is>
-      </c>
-      <c r="I93" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=Pxi9I9R-td8</t>
-        </is>
-      </c>
-      <c r="J93" t="n">
-        <v>279370</v>
-      </c>
-      <c r="K93" t="inlineStr">
-        <is>
-          <t>KADOKAWA Official Channel</t>
-        </is>
-      </c>
-      <c r="L93" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=Pxi9I9R-td8</t>
-        </is>
-      </c>
-      <c r="M93" t="n">
-        <v>279370</v>
-      </c>
-      <c r="N93" t="inlineStr">
-        <is>
-          <t>KADOKAWA Official Channel</t>
-        </is>
-      </c>
-      <c r="O93" t="inlineStr">
-        <is>
-          <t>2026-09-09T09:08:07</t>
-        </is>
-      </c>
+          <t>KID PHENOMENON</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr"/>
+      <c r="J93" t="inlineStr"/>
+      <c r="K93" t="inlineStr"/>
+      <c r="L93" t="inlineStr"/>
+      <c r="M93" t="inlineStr"/>
+      <c r="N93" t="inlineStr"/>
+      <c r="O93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -11719,7 +11759,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>わたしの幸せな結婚 特別篇</t>
+          <t>弱気MAX令嬢なのに、辣腕婚約者様の賭けに乗ってしまった</t>
         </is>
       </c>
       <c r="D94" t="b">
@@ -11727,7 +11767,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F94" t="n">
@@ -11735,12 +11775,12 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>プレリュードの手前に ～for me&amp;you～</t>
+          <t>強気MAX宣言</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>伊東歌詞太郎</t>
+          <t>鈴木このみ</t>
         </is>
       </c>
       <c r="I94" t="inlineStr"/>
@@ -11753,16 +11793,16 @@
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>6212</v>
+        <v>5947</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2027冬アニメ</t>
+          <t>2026秋アニメ</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>気になってる人が男じゃなかった</t>
+          <t>弱気MAX令嬢なのに、辣腕婚約者様の賭けに乗ってしまった</t>
         </is>
       </c>
       <c r="D95" t="b">
@@ -11770,7 +11810,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F95" t="n">
@@ -11778,48 +11818,58 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>Breed</t>
+          <t>夜明けまでに</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>Nirvana</t>
+          <t>伊藤美来</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=J6EDW5WFb2M</t>
+          <t>https://www.youtube.com/watch?v=Pxi9I9R-td8</t>
         </is>
       </c>
       <c r="J95" t="n">
-        <v>8866513</v>
+        <v>279370</v>
       </c>
       <c r="K95" t="inlineStr">
         <is>
-          <t>Nirvana</t>
-        </is>
-      </c>
-      <c r="L95" t="inlineStr"/>
-      <c r="M95" t="inlineStr"/>
-      <c r="N95" t="inlineStr"/>
+          <t>KADOKAWA Official Channel</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Pxi9I9R-td8</t>
+        </is>
+      </c>
+      <c r="M95" t="n">
+        <v>279370</v>
+      </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>KADOKAWA Official Channel</t>
+        </is>
+      </c>
       <c r="O95" t="inlineStr">
         <is>
-          <t>2026-09-09T09:08:40</t>
+          <t>2026-09-09T09:08:07</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>6212</v>
+        <v>5947</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2027冬アニメ</t>
+          <t>2026秋アニメ</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>茉莉花官吏伝</t>
+          <t>わたしの幸せな結婚 特別篇</t>
         </is>
       </c>
       <c r="D96" t="b">
@@ -11827,7 +11877,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F96" t="n">
@@ -11835,41 +11885,141 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
+          <t>プレリュードの手前に ～for me&amp;you～</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>伊東歌詞太郎</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr"/>
+      <c r="J96" t="inlineStr"/>
+      <c r="K96" t="inlineStr"/>
+      <c r="L96" t="inlineStr"/>
+      <c r="M96" t="inlineStr"/>
+      <c r="N96" t="inlineStr"/>
+      <c r="O96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>6212</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>2027冬アニメ</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>気になってる人が男じゃなかった</t>
+        </is>
+      </c>
+      <c r="D97" t="b">
+        <v>0</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F97" t="n">
+        <v>1</v>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Breed</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Nirvana</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=J6EDW5WFb2M</t>
+        </is>
+      </c>
+      <c r="J97" t="n">
+        <v>8866513</v>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>Nirvana</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr"/>
+      <c r="M97" t="inlineStr"/>
+      <c r="N97" t="inlineStr"/>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>2026-09-09T09:08:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>6212</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>2027冬アニメ</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>茉莉花官吏伝</t>
+        </is>
+      </c>
+      <c r="D98" t="b">
+        <v>0</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F98" t="n">
+        <v>1</v>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
           <t>花噺</t>
         </is>
       </c>
-      <c r="H96" t="inlineStr">
+      <c r="H98" t="inlineStr">
         <is>
           <t>KANA-BOON</t>
         </is>
       </c>
-      <c r="I96" t="inlineStr">
+      <c r="I98" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=7ja8PqzctBg</t>
         </is>
       </c>
-      <c r="J96" t="n">
+      <c r="J98" t="n">
         <v>109034</v>
       </c>
-      <c r="K96" t="inlineStr">
+      <c r="K98" t="inlineStr">
         <is>
           <t>KADOKAWAanime</t>
         </is>
       </c>
-      <c r="L96" t="inlineStr">
+      <c r="L98" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=7ja8PqzctBg</t>
         </is>
       </c>
-      <c r="M96" t="n">
+      <c r="M98" t="n">
         <v>109034</v>
       </c>
-      <c r="N96" t="inlineStr">
+      <c r="N98" t="inlineStr">
         <is>
           <t>KADOKAWAanime</t>
         </is>
       </c>
-      <c r="O96" t="inlineStr">
+      <c r="O98" t="inlineStr">
         <is>
           <t>2026-09-09T09:08:45</t>
         </is>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-09-20
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -9116,13 +9116,27 @@
           <t>ano（あの）</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=y0URm3qCTpc</t>
+        </is>
+      </c>
+      <c r="J26" t="n">
+        <v>1658609</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>ano official channel</t>
+        </is>
+      </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>2026-09-20T09:08:36</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -14236,13 +14250,37 @@
           <t>『ユイカ』</t>
         </is>
       </c>
-      <c r="I128" t="inlineStr"/>
-      <c r="J128" t="inlineStr"/>
-      <c r="K128" t="inlineStr"/>
-      <c r="L128" t="inlineStr"/>
-      <c r="M128" t="inlineStr"/>
-      <c r="N128" t="inlineStr"/>
-      <c r="O128" t="inlineStr"/>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ic9XKLWMbCw</t>
+        </is>
+      </c>
+      <c r="J128" t="n">
+        <v>839607</v>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>『ユイカ』</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=X-SOSlnkXAc</t>
+        </is>
+      </c>
+      <c r="M128" t="n">
+        <v>827382</v>
+      </c>
+      <c r="N128" t="inlineStr">
+        <is>
+          <t>MAPPA CHANNEL</t>
+        </is>
+      </c>
+      <c r="O128" t="inlineStr">
+        <is>
+          <t>2026-09-20T09:17:24</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="n">

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-09-21
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -10473,7 +10473,7 @@
         </is>
       </c>
       <c r="J55" t="n">
-        <v>7569</v>
+        <v>8335</v>
       </c>
       <c r="K55" t="inlineStr">
         <is>
@@ -10486,7 +10486,7 @@
         </is>
       </c>
       <c r="M55" t="n">
-        <v>7569</v>
+        <v>8335</v>
       </c>
       <c r="N55" t="inlineStr">
         <is>
@@ -10495,7 +10495,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>2026-09-14T09:02:42</t>
+          <t>2026-09-21T09:03:32</t>
         </is>
       </c>
     </row>
@@ -11671,27 +11671,13 @@
           <t>岸田教団&amp;THE明星ロケッツ</t>
         </is>
       </c>
-      <c r="I79" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=JH927fq9qaM</t>
-        </is>
-      </c>
-      <c r="J79" t="n">
-        <v>3888</v>
-      </c>
-      <c r="K79" t="inlineStr">
-        <is>
-          <t>Kisidakyoudan &amp; the Akebosi rockets official</t>
-        </is>
-      </c>
+      <c r="I79" t="inlineStr"/>
+      <c r="J79" t="inlineStr"/>
+      <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr"/>
       <c r="M79" t="inlineStr"/>
       <c r="N79" t="inlineStr"/>
-      <c r="O79" t="inlineStr">
-        <is>
-          <t>2026-09-14T09:04:34</t>
-        </is>
-      </c>
+      <c r="O79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -11734,7 +11720,7 @@
         </is>
       </c>
       <c r="J80" t="n">
-        <v>262450</v>
+        <v>537135</v>
       </c>
       <c r="K80" t="inlineStr">
         <is>
@@ -11743,11 +11729,11 @@
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=tYuPxILnixw</t>
+          <t>https://www.youtube.com/watch?v=keFRueltLIU</t>
         </is>
       </c>
       <c r="M80" t="n">
-        <v>7195703</v>
+        <v>15819102</v>
       </c>
       <c r="N80" t="inlineStr">
         <is>
@@ -11756,7 +11742,7 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>2026-09-14T09:04:48</t>
+          <t>2026-09-21T09:05:37</t>
         </is>
       </c>
     </row>
@@ -11801,7 +11787,7 @@
         </is>
       </c>
       <c r="J81" t="n">
-        <v>180739</v>
+        <v>211070</v>
       </c>
       <c r="K81" t="inlineStr">
         <is>
@@ -11814,7 +11800,7 @@
         </is>
       </c>
       <c r="M81" t="n">
-        <v>3867868</v>
+        <v>3888617</v>
       </c>
       <c r="N81" t="inlineStr">
         <is>
@@ -11823,7 +11809,7 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>2026-09-14T09:05:01</t>
+          <t>2026-09-21T09:05:50</t>
         </is>
       </c>
     </row>
@@ -13204,7 +13190,7 @@
         </is>
       </c>
       <c r="J108" t="n">
-        <v>317795</v>
+        <v>320908</v>
       </c>
       <c r="K108" t="inlineStr">
         <is>
@@ -13217,7 +13203,7 @@
         </is>
       </c>
       <c r="M108" t="n">
-        <v>317795</v>
+        <v>320908</v>
       </c>
       <c r="N108" t="inlineStr">
         <is>
@@ -13226,7 +13212,7 @@
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t>2026-09-14T09:06:07</t>
+          <t>2026-09-21T09:07:04</t>
         </is>
       </c>
     </row>
@@ -13314,7 +13300,7 @@
         </is>
       </c>
       <c r="J110" t="n">
-        <v>317802</v>
+        <v>320908</v>
       </c>
       <c r="K110" t="inlineStr">
         <is>
@@ -13327,7 +13313,7 @@
         </is>
       </c>
       <c r="M110" t="n">
-        <v>317802</v>
+        <v>320908</v>
       </c>
       <c r="N110" t="inlineStr">
         <is>
@@ -13336,7 +13322,7 @@
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>2026-09-14T09:06:21</t>
+          <t>2026-09-21T09:07:21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-09-22
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -8228,7 +8228,7 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>10200755</v>
+        <v>10244577</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -8241,7 +8241,7 @@
         </is>
       </c>
       <c r="M8" t="n">
-        <v>10200755</v>
+        <v>10244577</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
@@ -8250,7 +8250,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>2026-09-15T08:33:42</t>
+          <t>2026-09-22T09:00:43</t>
         </is>
       </c>
     </row>
@@ -8859,7 +8859,7 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>1063833</v>
+        <v>1453643</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -8872,7 +8872,7 @@
         </is>
       </c>
       <c r="M21" t="n">
-        <v>1063833</v>
+        <v>1453643</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
@@ -8881,7 +8881,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>2026-09-15T08:34:35</t>
+          <t>2026-09-22T09:01:45</t>
         </is>
       </c>
     </row>
@@ -9289,7 +9289,7 @@
         </is>
       </c>
       <c r="J29" t="n">
-        <v>24179</v>
+        <v>27235</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
@@ -9302,7 +9302,7 @@
         </is>
       </c>
       <c r="M29" t="n">
-        <v>24179</v>
+        <v>27235</v>
       </c>
       <c r="N29" t="inlineStr">
         <is>
@@ -9311,7 +9311,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>2026-09-15T08:35:09</t>
+          <t>2026-09-22T09:02:25</t>
         </is>
       </c>
     </row>
@@ -10774,7 +10774,7 @@
         </is>
       </c>
       <c r="J60" t="n">
-        <v>740443</v>
+        <v>750960</v>
       </c>
       <c r="K60" t="inlineStr">
         <is>
@@ -10787,7 +10787,7 @@
         </is>
       </c>
       <c r="M60" t="n">
-        <v>740443</v>
+        <v>750960</v>
       </c>
       <c r="N60" t="inlineStr">
         <is>
@@ -10796,7 +10796,7 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>2026-09-15T08:38:33</t>
+          <t>2026-09-22T09:04:19</t>
         </is>
       </c>
     </row>
@@ -14309,7 +14309,7 @@
         </is>
       </c>
       <c r="J129" t="n">
-        <v>117602</v>
+        <v>239272</v>
       </c>
       <c r="K129" t="inlineStr">
         <is>
@@ -14321,7 +14321,7 @@
       <c r="N129" t="inlineStr"/>
       <c r="O129" t="inlineStr">
         <is>
-          <t>2026-09-15T08:42:34</t>
+          <t>2026-09-22T09:08:29</t>
         </is>
       </c>
     </row>
@@ -14366,7 +14366,7 @@
         </is>
       </c>
       <c r="J130" t="n">
-        <v>117602</v>
+        <v>239272</v>
       </c>
       <c r="K130" t="inlineStr">
         <is>
@@ -14378,7 +14378,7 @@
       <c r="N130" t="inlineStr"/>
       <c r="O130" t="inlineStr">
         <is>
-          <t>2026-09-15T08:42:43</t>
+          <t>2026-09-22T09:08:37</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: anime list update 2026-09-23
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -18,16 +18,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +35,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,21 +43,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -426,71 +414,71 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M147"/>
+  <dimension ref="A1:M171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>season_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>season_label</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>order</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>is_rerun</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>broadcast_format</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>broadcast_start</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>animation_studio</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>op_title</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>op_artist</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>ed_title</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>ed_artist</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>detail_url</t>
         </is>
@@ -7835,6 +7823,1086 @@
       <c r="M147" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=26354</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>-208829</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>2026夏アニメ</t>
+        </is>
+      </c>
+      <c r="C148" t="n">
+        <v>0</v>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>クレヨンしんちゃん 奇々怪々! オラの妖怪バケ~ション</t>
+        </is>
+      </c>
+      <c r="E148" t="b">
+        <v>0</v>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>2026年7月31日</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>Shin-Ei Animation</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr"/>
+      <c r="J148" t="inlineStr"/>
+      <c r="K148" t="inlineStr"/>
+      <c r="L148" t="inlineStr"/>
+      <c r="M148" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/208829</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>-213908</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>2026夏アニメ</t>
+        </is>
+      </c>
+      <c r="C149" t="n">
+        <v>0</v>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>るすばん</t>
+        </is>
+      </c>
+      <c r="E149" t="b">
+        <v>0</v>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>2026年8月1日</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>ROCK'N ROLL MOUNTAIN</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr"/>
+      <c r="J149" t="inlineStr"/>
+      <c r="K149" t="inlineStr"/>
+      <c r="L149" t="inlineStr"/>
+      <c r="M149" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/213908</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>-211308</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>2026夏アニメ</t>
+        </is>
+      </c>
+      <c r="C150" t="n">
+        <v>0</v>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>THE RIBBON HERO</t>
+        </is>
+      </c>
+      <c r="E150" t="b">
+        <v>0</v>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>2026年8月8日</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>OUTLINE</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr"/>
+      <c r="J150" t="inlineStr"/>
+      <c r="K150" t="inlineStr"/>
+      <c r="L150" t="inlineStr"/>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/211308</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>-176373</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>2026夏アニメ</t>
+        </is>
+      </c>
+      <c r="C151" t="n">
+        <v>0</v>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>しらぬひ</t>
+        </is>
+      </c>
+      <c r="E151" t="b">
+        <v>0</v>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>2026年8月21日</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>CoMix Wave</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr"/>
+      <c r="J151" t="inlineStr"/>
+      <c r="K151" t="inlineStr"/>
+      <c r="L151" t="inlineStr"/>
+      <c r="M151" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/176373</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>-133007</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>2026夏アニメ</t>
+        </is>
+      </c>
+      <c r="C152" t="n">
+        <v>0</v>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>劇場版 魔法少女まどか☆マギカ〈ワルプルギスの廻天〉</t>
+        </is>
+      </c>
+      <c r="E152" t="b">
+        <v>0</v>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>2026年8月28日</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>Shaft</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr"/>
+      <c r="J152" t="inlineStr"/>
+      <c r="K152" t="inlineStr"/>
+      <c r="L152" t="inlineStr"/>
+      <c r="M152" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/133007</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="n">
+        <v>-194116</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>2026夏アニメ</t>
+        </is>
+      </c>
+      <c r="C153" t="n">
+        <v>0</v>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>最終楽章 響け！ユーフォニアム後編</t>
+        </is>
+      </c>
+      <c r="E153" t="b">
+        <v>0</v>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>2026年9月11日</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>Kyoto Animation</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr"/>
+      <c r="J153" t="inlineStr"/>
+      <c r="K153" t="inlineStr"/>
+      <c r="L153" t="inlineStr"/>
+      <c r="M153" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/194116</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="n">
+        <v>-198654</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>2026夏アニメ</t>
+        </is>
+      </c>
+      <c r="C154" t="n">
+        <v>0</v>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>名探偵プリキュア！不思議な庭と2人の秘密</t>
+        </is>
+      </c>
+      <c r="E154" t="b">
+        <v>0</v>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>2026年9月18日</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>Toei Animation</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr"/>
+      <c r="J154" t="inlineStr"/>
+      <c r="K154" t="inlineStr"/>
+      <c r="L154" t="inlineStr"/>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/198654</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="n">
+        <v>-202429</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>2026夏アニメ</t>
+        </is>
+      </c>
+      <c r="C155" t="n">
+        <v>0</v>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>我々は宇宙人</t>
+        </is>
+      </c>
+      <c r="E155" t="b">
+        <v>0</v>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>2026年9月25日</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>NOTHING NEW, Miyu Productions</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr"/>
+      <c r="J155" t="inlineStr"/>
+      <c r="K155" t="inlineStr"/>
+      <c r="L155" t="inlineStr"/>
+      <c r="M155" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/202429</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>-202390</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C156" t="n">
+        <v>0</v>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>ガールズ＆パンツァー 最終章 第5話</t>
+        </is>
+      </c>
+      <c r="E156" t="b">
+        <v>0</v>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>2026年10月9日</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>Actas</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr"/>
+      <c r="J156" t="inlineStr"/>
+      <c r="K156" t="inlineStr"/>
+      <c r="L156" t="inlineStr"/>
+      <c r="M156" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/202390</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="n">
+        <v>-207327</v>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C157" t="n">
+        <v>0</v>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>どこよりも遠い場所にいる君へ</t>
+        </is>
+      </c>
+      <c r="E157" t="b">
+        <v>0</v>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>2026年10月9日</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>TMS Entertainment</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr"/>
+      <c r="J157" t="inlineStr"/>
+      <c r="K157" t="inlineStr"/>
+      <c r="L157" t="inlineStr"/>
+      <c r="M157" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/207327</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="n">
+        <v>-197543</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C158" t="n">
+        <v>0</v>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>BanG Dream! Ave Mujica prima aurora</t>
+        </is>
+      </c>
+      <c r="E158" t="b">
+        <v>0</v>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>NICHICALINE</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr"/>
+      <c r="J158" t="inlineStr"/>
+      <c r="K158" t="inlineStr"/>
+      <c r="L158" t="inlineStr"/>
+      <c r="M158" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/197543</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="n">
+        <v>-199340</v>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C159" t="n">
+        <v>0</v>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>青春ブタ野郎はディアフレンドの夢を見ない</t>
+        </is>
+      </c>
+      <c r="E159" t="b">
+        <v>0</v>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>2026年10月16日</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>CloverWorks</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr"/>
+      <c r="J159" t="inlineStr"/>
+      <c r="K159" t="inlineStr"/>
+      <c r="L159" t="inlineStr"/>
+      <c r="M159" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/199340</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="n">
+        <v>-160275</v>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C160" t="n">
+        <v>0</v>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>メイドインアビス 目覚める神秘</t>
+        </is>
+      </c>
+      <c r="E160" t="b">
+        <v>0</v>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>Kinema Citrus</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr"/>
+      <c r="J160" t="inlineStr"/>
+      <c r="K160" t="inlineStr"/>
+      <c r="L160" t="inlineStr"/>
+      <c r="M160" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/160275</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="n">
+        <v>-209642</v>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C161" t="n">
+        <v>0</v>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>劇場版 前橋ウィッチーズ ～魔女見習いのエモエモリーズ～</t>
+        </is>
+      </c>
+      <c r="E161" t="b">
+        <v>0</v>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>2026年10月23日</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>Sunrise</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr"/>
+      <c r="J161" t="inlineStr"/>
+      <c r="K161" t="inlineStr"/>
+      <c r="L161" t="inlineStr"/>
+      <c r="M161" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/209642</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="n">
+        <v>-178972</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C162" t="n">
+        <v>0</v>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>GROTESQQQUE -グロテスク-</t>
+        </is>
+      </c>
+      <c r="E162" t="b">
+        <v>0</v>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>2026年11月6日</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>CloverWorks</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr"/>
+      <c r="J162" t="inlineStr"/>
+      <c r="K162" t="inlineStr"/>
+      <c r="L162" t="inlineStr"/>
+      <c r="M162" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/178972</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="n">
+        <v>-157330</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C163" t="n">
+        <v>0</v>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>楽園追放 心のレゾナンス</t>
+        </is>
+      </c>
+      <c r="E163" t="b">
+        <v>0</v>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>2026年11月13日</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>Toei Animation</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr"/>
+      <c r="J163" t="inlineStr"/>
+      <c r="K163" t="inlineStr"/>
+      <c r="L163" t="inlineStr"/>
+      <c r="M163" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/157330</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="n">
+        <v>-143103</v>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C164" t="n">
+        <v>0</v>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>魔法使いの夜</t>
+        </is>
+      </c>
+      <c r="E164" t="b">
+        <v>0</v>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>2026年11月20日</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>ufotable</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr"/>
+      <c r="J164" t="inlineStr"/>
+      <c r="K164" t="inlineStr"/>
+      <c r="L164" t="inlineStr"/>
+      <c r="M164" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/143103</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="n">
+        <v>-206163</v>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C165" t="n">
+        <v>0</v>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>装甲騎兵ボトムズ 灰色の魔女</t>
+        </is>
+      </c>
+      <c r="E165" t="b">
+        <v>0</v>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>2026年11月20日</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>Production I.G, Sunrise</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr"/>
+      <c r="J165" t="inlineStr"/>
+      <c r="K165" t="inlineStr"/>
+      <c r="L165" t="inlineStr"/>
+      <c r="M165" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/206163</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="n">
+        <v>-212539</v>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C166" t="n">
+        <v>0</v>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>タコピーの原罪 -ありがとう、また明日-</t>
+        </is>
+      </c>
+      <c r="E166" t="b">
+        <v>0</v>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>2026年11月27日</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>ENISHIYA</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr"/>
+      <c r="J166" t="inlineStr"/>
+      <c r="K166" t="inlineStr"/>
+      <c r="L166" t="inlineStr"/>
+      <c r="M166" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/212539</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="n">
+        <v>-205289</v>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C167" t="n">
+        <v>0</v>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>ノーマン・ザ・スノーマン ~こどもたちのひとつ星~</t>
+        </is>
+      </c>
+      <c r="E167" t="b">
+        <v>0</v>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>2026年12月</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>TECARAT</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr"/>
+      <c r="J167" t="inlineStr"/>
+      <c r="K167" t="inlineStr"/>
+      <c r="L167" t="inlineStr"/>
+      <c r="M167" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/205289</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="n">
+        <v>-200929</v>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C168" t="n">
+        <v>0</v>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>薬屋のひとりごと 亡妃の秘宝</t>
+        </is>
+      </c>
+      <c r="E168" t="b">
+        <v>0</v>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>2026年12月11日</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>TOHO animation STUDIO</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr"/>
+      <c r="J168" t="inlineStr"/>
+      <c r="K168" t="inlineStr"/>
+      <c r="L168" t="inlineStr"/>
+      <c r="M168" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/200929</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="n">
+        <v>-194213</v>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>2027冬アニメ</t>
+        </is>
+      </c>
+      <c r="C169" t="n">
+        <v>0</v>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>ghost／夜の果て</t>
+        </is>
+      </c>
+      <c r="E169" t="b">
+        <v>0</v>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>2027年2月11日</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>MADHOUSE</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr"/>
+      <c r="J169" t="inlineStr"/>
+      <c r="K169" t="inlineStr"/>
+      <c r="L169" t="inlineStr"/>
+      <c r="M169" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/194213</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="n">
+        <v>-206298</v>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>2027冬アニメ</t>
+        </is>
+      </c>
+      <c r="C170" t="n">
+        <v>0</v>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>劇場版 メダリスト</t>
+        </is>
+      </c>
+      <c r="E170" t="b">
+        <v>0</v>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>2027年2月19日</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>ENGI</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr"/>
+      <c r="J170" t="inlineStr"/>
+      <c r="K170" t="inlineStr"/>
+      <c r="L170" t="inlineStr"/>
+      <c r="M170" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/206298</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="n">
+        <v>-216623</v>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>2027冬アニメ</t>
+        </is>
+      </c>
+      <c r="C171" t="n">
+        <v>0</v>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>ドラえもん のび太の蒸気時間車</t>
+        </is>
+      </c>
+      <c r="E171" t="b">
+        <v>0</v>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>2027年3月5日</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>Shin-Ei Animation</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr"/>
+      <c r="J171" t="inlineStr"/>
+      <c r="K171" t="inlineStr"/>
+      <c r="L171" t="inlineStr"/>
+      <c r="M171" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/216623</t>
         </is>
       </c>
     </row>
@@ -7853,77 +8921,77 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>season_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>season_label</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>anime_title</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>is_rerun</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>kind</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>index</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>song_title</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>artist</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>youtube_url</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>youtube_views</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>youtube_channel</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>anime_youtube_url</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>anime_youtube_views</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>anime_youtube_channel</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>last_searched_at</t>
         </is>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-09-27
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M266"/>
+  <dimension ref="A1:M276"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13310,6 +13310,456 @@
       <c r="M266" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=12846</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="n">
+        <v>-208829</v>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>2026夏アニメ</t>
+        </is>
+      </c>
+      <c r="C267" t="n">
+        <v>0</v>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>クレヨンしんちゃん 奇々怪々! オラの妖怪バケ~ション</t>
+        </is>
+      </c>
+      <c r="E267" t="b">
+        <v>0</v>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>2026年7月31日</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>Shin-Ei Animation</t>
+        </is>
+      </c>
+      <c r="I267" t="inlineStr"/>
+      <c r="J267" t="inlineStr"/>
+      <c r="K267" t="inlineStr"/>
+      <c r="L267" t="inlineStr"/>
+      <c r="M267" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/208829</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="n">
+        <v>-211308</v>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>2026夏アニメ</t>
+        </is>
+      </c>
+      <c r="C268" t="n">
+        <v>0</v>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>THE RIBBON HERO</t>
+        </is>
+      </c>
+      <c r="E268" t="b">
+        <v>0</v>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>2026年8月8日</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>OUTLINE</t>
+        </is>
+      </c>
+      <c r="I268" t="inlineStr"/>
+      <c r="J268" t="inlineStr"/>
+      <c r="K268" t="inlineStr"/>
+      <c r="L268" t="inlineStr"/>
+      <c r="M268" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/211308</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="n">
+        <v>-194116</v>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>2026夏アニメ</t>
+        </is>
+      </c>
+      <c r="C269" t="n">
+        <v>0</v>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>最終楽章 響け！ユーフォニアム後編</t>
+        </is>
+      </c>
+      <c r="E269" t="b">
+        <v>0</v>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>2026年9月11日</t>
+        </is>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>Kyoto Animation</t>
+        </is>
+      </c>
+      <c r="I269" t="inlineStr"/>
+      <c r="J269" t="inlineStr"/>
+      <c r="K269" t="inlineStr"/>
+      <c r="L269" t="inlineStr"/>
+      <c r="M269" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/194116</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="n">
+        <v>-198654</v>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>2026夏アニメ</t>
+        </is>
+      </c>
+      <c r="C270" t="n">
+        <v>0</v>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>名探偵プリキュア！不思議な庭と2人の秘密</t>
+        </is>
+      </c>
+      <c r="E270" t="b">
+        <v>0</v>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>2026年9月18日</t>
+        </is>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>Toei Animation</t>
+        </is>
+      </c>
+      <c r="I270" t="inlineStr"/>
+      <c r="J270" t="inlineStr"/>
+      <c r="K270" t="inlineStr"/>
+      <c r="L270" t="inlineStr"/>
+      <c r="M270" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/198654</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="n">
+        <v>-206163</v>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C271" t="n">
+        <v>0</v>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>装甲騎兵ボトムズ 灰色の魔女</t>
+        </is>
+      </c>
+      <c r="E271" t="b">
+        <v>0</v>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>2026年11月20日</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>Production I.G, Sunrise</t>
+        </is>
+      </c>
+      <c r="I271" t="inlineStr"/>
+      <c r="J271" t="inlineStr"/>
+      <c r="K271" t="inlineStr"/>
+      <c r="L271" t="inlineStr"/>
+      <c r="M271" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/206163</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="n">
+        <v>-212539</v>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C272" t="n">
+        <v>0</v>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>タコピーの原罪 -ありがとう、また明日-</t>
+        </is>
+      </c>
+      <c r="E272" t="b">
+        <v>0</v>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>2026年11月27日</t>
+        </is>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>ENISHIYA</t>
+        </is>
+      </c>
+      <c r="I272" t="inlineStr"/>
+      <c r="J272" t="inlineStr"/>
+      <c r="K272" t="inlineStr"/>
+      <c r="L272" t="inlineStr"/>
+      <c r="M272" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/212539</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="n">
+        <v>-205289</v>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C273" t="n">
+        <v>0</v>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>ノーマン・ザ・スノーマン ~こどもたちのひとつ星~</t>
+        </is>
+      </c>
+      <c r="E273" t="b">
+        <v>0</v>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>2026年12月</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>TECARAT</t>
+        </is>
+      </c>
+      <c r="I273" t="inlineStr"/>
+      <c r="J273" t="inlineStr"/>
+      <c r="K273" t="inlineStr"/>
+      <c r="L273" t="inlineStr"/>
+      <c r="M273" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/205289</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="n">
+        <v>-200929</v>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C274" t="n">
+        <v>0</v>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>薬屋のひとりごと 亡妃の秘宝</t>
+        </is>
+      </c>
+      <c r="E274" t="b">
+        <v>0</v>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>2026年12月11日</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>TOHO animation STUDIO</t>
+        </is>
+      </c>
+      <c r="I274" t="inlineStr"/>
+      <c r="J274" t="inlineStr"/>
+      <c r="K274" t="inlineStr"/>
+      <c r="L274" t="inlineStr"/>
+      <c r="M274" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/200929</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="n">
+        <v>-206298</v>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>2027冬アニメ</t>
+        </is>
+      </c>
+      <c r="C275" t="n">
+        <v>0</v>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>劇場版 メダリスト</t>
+        </is>
+      </c>
+      <c r="E275" t="b">
+        <v>0</v>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>2027年2月19日</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>ENGI</t>
+        </is>
+      </c>
+      <c r="I275" t="inlineStr"/>
+      <c r="J275" t="inlineStr"/>
+      <c r="K275" t="inlineStr"/>
+      <c r="L275" t="inlineStr"/>
+      <c r="M275" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/206298</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="n">
+        <v>-216623</v>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>2027冬アニメ</t>
+        </is>
+      </c>
+      <c r="C276" t="n">
+        <v>0</v>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>ドラえもん のび太の蒸気時間車</t>
+        </is>
+      </c>
+      <c r="E276" t="b">
+        <v>0</v>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>2027年3月5日</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>Shin-Ei Animation</t>
+        </is>
+      </c>
+      <c r="I276" t="inlineStr"/>
+      <c r="J276" t="inlineStr"/>
+      <c r="K276" t="inlineStr"/>
+      <c r="L276" t="inlineStr"/>
+      <c r="M276" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/216623</t>
         </is>
       </c>
     </row>
@@ -18154,13 +18604,37 @@
           <t>パンどろぼうとパンやのおじさん（CV：朝井彩加とCV：諏訪部順一）</t>
         </is>
       </c>
-      <c r="I99" t="inlineStr"/>
-      <c r="J99" t="inlineStr"/>
-      <c r="K99" t="inlineStr"/>
-      <c r="L99" t="inlineStr"/>
-      <c r="M99" t="inlineStr"/>
-      <c r="N99" t="inlineStr"/>
-      <c r="O99" t="inlineStr"/>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=YMLnoxAdeIk</t>
+        </is>
+      </c>
+      <c r="J99" t="n">
+        <v>243377</v>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>パンどろぼう / PANDOROBO【公式】</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=YMLnoxAdeIk</t>
+        </is>
+      </c>
+      <c r="M99" t="n">
+        <v>243377</v>
+      </c>
+      <c r="N99" t="inlineStr">
+        <is>
+          <t>パンどろぼう / PANDOROBO【公式】</t>
+        </is>
+      </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>2026-09-27T09:07:12</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -18197,13 +18671,27 @@
           <t>きゃりーぱみゅぱみゅ</t>
         </is>
       </c>
-      <c r="I100" t="inlineStr"/>
-      <c r="J100" t="inlineStr"/>
-      <c r="K100" t="inlineStr"/>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=YMLnoxAdeIk</t>
+        </is>
+      </c>
+      <c r="J100" t="n">
+        <v>243377</v>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>パンどろぼう / PANDOROBO【公式】</t>
+        </is>
+      </c>
       <c r="L100" t="inlineStr"/>
       <c r="M100" t="inlineStr"/>
       <c r="N100" t="inlineStr"/>
-      <c r="O100" t="inlineStr"/>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>2026-09-27T09:07:27</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="n">

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-10-04
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -15179,13 +15179,37 @@
           <t>BUDDiiS</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=R5veWbUAM-I</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>5114</v>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>tv asahi  animation YouTubeチャンネル</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=R5veWbUAM-I</t>
+        </is>
+      </c>
+      <c r="M18" t="n">
+        <v>5114</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>tv asahi  animation YouTubeチャンネル</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>2026-10-04T09:01:22</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -15222,13 +15246,37 @@
           <t>こたに</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=gYZJcSSnAVY</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>3019</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>tv asahi  animation YouTubeチャンネル</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=gYZJcSSnAVY</t>
+        </is>
+      </c>
+      <c r="M19" t="n">
+        <v>3019</v>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>tv asahi  animation YouTubeチャンネル</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>2026-10-04T09:01:31</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -15590,13 +15638,37 @@
           <t>Juice=Juice</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=y8dxEBdlISk</t>
+        </is>
+      </c>
+      <c r="J27" t="n">
+        <v>93031</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Juice=Juice</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=y8dxEBdlISk</t>
+        </is>
+      </c>
+      <c r="M27" t="n">
+        <v>93031</v>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>Juice=Juice</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>2026-10-04T09:02:21</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -17185,13 +17257,37 @@
           <t>すりぃ</t>
         </is>
       </c>
-      <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr"/>
-      <c r="M60" t="inlineStr"/>
-      <c r="N60" t="inlineStr"/>
-      <c r="O60" t="inlineStr"/>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zhK-ugQnTgA</t>
+        </is>
+      </c>
+      <c r="J60" t="n">
+        <v>18568</v>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zhK-ugQnTgA</t>
+        </is>
+      </c>
+      <c r="M60" t="n">
+        <v>18568</v>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>2026-10-04T09:04:24</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -18499,13 +18595,37 @@
           <t>佐々木李子</t>
         </is>
       </c>
-      <c r="I86" t="inlineStr"/>
-      <c r="J86" t="inlineStr"/>
-      <c r="K86" t="inlineStr"/>
-      <c r="L86" t="inlineStr"/>
-      <c r="M86" t="inlineStr"/>
-      <c r="N86" t="inlineStr"/>
-      <c r="O86" t="inlineStr"/>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-LQfgkvHY8k</t>
+        </is>
+      </c>
+      <c r="J86" t="n">
+        <v>48794</v>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>isekai channel @バンダイナムコフィルムワークス</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-LQfgkvHY8k</t>
+        </is>
+      </c>
+      <c r="M86" t="n">
+        <v>48794</v>
+      </c>
+      <c r="N86" t="inlineStr">
+        <is>
+          <t>isekai channel @バンダイナムコフィルムワークス</t>
+        </is>
+      </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>2026-10-04T09:06:02</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -18695,13 +18815,37 @@
           <t>花耶</t>
         </is>
       </c>
-      <c r="I90" t="inlineStr"/>
-      <c r="J90" t="inlineStr"/>
-      <c r="K90" t="inlineStr"/>
-      <c r="L90" t="inlineStr"/>
-      <c r="M90" t="inlineStr"/>
-      <c r="N90" t="inlineStr"/>
-      <c r="O90" t="inlineStr"/>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Zh22JniyJy4</t>
+        </is>
+      </c>
+      <c r="J90" t="n">
+        <v>4393</v>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kaya Official YouTube Channel </t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=lP8RbpwGUO8</t>
+        </is>
+      </c>
+      <c r="M90" t="n">
+        <v>8293</v>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>博報堂DY ミュージック&amp;ピクチャーズ【Showgate】ch</t>
+        </is>
+      </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>2026-10-04T09:06:24</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -19776,11 +19920,11 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=YMLnoxAdeIk</t>
+          <t>https://www.youtube.com/watch?v=Z2fmYtMNi-o</t>
         </is>
       </c>
       <c r="J111" t="n">
-        <v>243377</v>
+        <v>281584</v>
       </c>
       <c r="K111" t="inlineStr">
         <is>
@@ -19789,11 +19933,11 @@
       </c>
       <c r="L111" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=YMLnoxAdeIk</t>
+          <t>https://www.youtube.com/watch?v=jz7Jqz6SYzk</t>
         </is>
       </c>
       <c r="M111" t="n">
-        <v>243377</v>
+        <v>44037</v>
       </c>
       <c r="N111" t="inlineStr">
         <is>
@@ -19802,7 +19946,7 @@
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>2026-09-27T09:07:12</t>
+          <t>2026-10-04T09:07:44</t>
         </is>
       </c>
     </row>
@@ -19843,23 +19987,33 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=YMLnoxAdeIk</t>
+          <t>https://www.youtube.com/watch?v=Z2fmYtMNi-o</t>
         </is>
       </c>
       <c r="J112" t="n">
-        <v>243377</v>
+        <v>281584</v>
       </c>
       <c r="K112" t="inlineStr">
         <is>
           <t>パンどろぼう / PANDOROBO【公式】</t>
         </is>
       </c>
-      <c r="L112" t="inlineStr"/>
-      <c r="M112" t="inlineStr"/>
-      <c r="N112" t="inlineStr"/>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=oUDFr8Ktaxs</t>
+        </is>
+      </c>
+      <c r="M112" t="n">
+        <v>135608</v>
+      </c>
+      <c r="N112" t="inlineStr">
+        <is>
+          <t>パンどろぼう / PANDOROBO【公式】</t>
+        </is>
+      </c>
       <c r="O112" t="inlineStr">
         <is>
-          <t>2026-09-27T09:07:27</t>
+          <t>2026-10-04T09:07:53</t>
         </is>
       </c>
     </row>
@@ -20122,13 +20276,37 @@
           <t>ONE OR EIGHT</t>
         </is>
       </c>
-      <c r="I117" t="inlineStr"/>
-      <c r="J117" t="inlineStr"/>
-      <c r="K117" t="inlineStr"/>
-      <c r="L117" t="inlineStr"/>
-      <c r="M117" t="inlineStr"/>
-      <c r="N117" t="inlineStr"/>
-      <c r="O117" t="inlineStr"/>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=umzOm3846cA</t>
+        </is>
+      </c>
+      <c r="J117" t="n">
+        <v>113007</v>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>テレ東アニメ</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=umzOm3846cA</t>
+        </is>
+      </c>
+      <c r="M117" t="n">
+        <v>113007</v>
+      </c>
+      <c r="N117" t="inlineStr">
+        <is>
+          <t>テレ東アニメ</t>
+        </is>
+      </c>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>2026-10-04T09:08:06</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -20385,13 +20563,27 @@
           <t>TOOBOE</t>
         </is>
       </c>
-      <c r="I122" t="inlineStr"/>
-      <c r="J122" t="inlineStr"/>
-      <c r="K122" t="inlineStr"/>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=TE3McAbD7DA</t>
+        </is>
+      </c>
+      <c r="J122" t="n">
+        <v>827599</v>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>john / TOOBOE</t>
+        </is>
+      </c>
       <c r="L122" t="inlineStr"/>
       <c r="M122" t="inlineStr"/>
       <c r="N122" t="inlineStr"/>
-      <c r="O122" t="inlineStr"/>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>2026-10-04T09:08:29</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -21087,13 +21279,37 @@
           <t>yama</t>
         </is>
       </c>
-      <c r="I136" t="inlineStr"/>
-      <c r="J136" t="inlineStr"/>
-      <c r="K136" t="inlineStr"/>
-      <c r="L136" t="inlineStr"/>
-      <c r="M136" t="inlineStr"/>
-      <c r="N136" t="inlineStr"/>
-      <c r="O136" t="inlineStr"/>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=HYm0nNqk9Aw</t>
+        </is>
+      </c>
+      <c r="J136" t="n">
+        <v>9616</v>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>NHK ENTERPRISES Animation</t>
+        </is>
+      </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=HYm0nNqk9Aw</t>
+        </is>
+      </c>
+      <c r="M136" t="n">
+        <v>9616</v>
+      </c>
+      <c r="N136" t="inlineStr">
+        <is>
+          <t>NHK ENTERPRISES Animation</t>
+        </is>
+      </c>
+      <c r="O136" t="inlineStr">
+        <is>
+          <t>2026-10-04T09:09:22</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -21852,13 +22068,37 @@
           <t>ふみの</t>
         </is>
       </c>
-      <c r="I151" t="inlineStr"/>
-      <c r="J151" t="inlineStr"/>
-      <c r="K151" t="inlineStr"/>
-      <c r="L151" t="inlineStr"/>
-      <c r="M151" t="inlineStr"/>
-      <c r="N151" t="inlineStr"/>
-      <c r="O151" t="inlineStr"/>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=hNiixLqIi64</t>
+        </is>
+      </c>
+      <c r="J151" t="n">
+        <v>70474</v>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>MAPPA CHANNEL</t>
+        </is>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=hNiixLqIi64</t>
+        </is>
+      </c>
+      <c r="M151" t="n">
+        <v>70474</v>
+      </c>
+      <c r="N151" t="inlineStr">
+        <is>
+          <t>MAPPA CHANNEL</t>
+        </is>
+      </c>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>2026-10-04T09:10:15</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="n">

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-10-05
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -14830,13 +14830,37 @@
           <t>エルスウェア紀行</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=8B3d4x0m7n4</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>56736</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>TMSアニメ公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=8B3d4x0m7n4</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
+        <v>56736</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>TMSアニメ公式チャンネル</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>2026-10-05T09:00:56</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -14983,13 +15007,37 @@
           <t>福賀くるみ（CV：鈴木愛奈）</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=OiQo6YyJ_pM</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>754993</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=OiQo6YyJ_pM</t>
+        </is>
+      </c>
+      <c r="M14" t="n">
+        <v>754993</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>2026-10-05T09:01:05</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -15442,13 +15490,37 @@
           <t>Ceui</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=By3eIjul98c</t>
+        </is>
+      </c>
+      <c r="J23" t="n">
+        <v>2655</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>デレギュラ【新アニメレーベル】</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=By3eIjul98c</t>
+        </is>
+      </c>
+      <c r="M23" t="n">
+        <v>2655</v>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>デレギュラ【新アニメレーベル】</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>2026-10-05T09:01:43</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -16221,13 +16293,37 @@
           <t>Koji Nakamura</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr"/>
-      <c r="O38" t="inlineStr"/>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=2mkPF8PO4GY</t>
+        </is>
+      </c>
+      <c r="J38" t="n">
+        <v>12269</v>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=2mkPF8PO4GY</t>
+        </is>
+      </c>
+      <c r="M38" t="n">
+        <v>12269</v>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>2026-10-05T09:02:41</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -16431,13 +16527,37 @@
           <t>CLAN QUEEN</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr"/>
-      <c r="O42" t="inlineStr"/>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Uitds6Ysj08</t>
+        </is>
+      </c>
+      <c r="J42" t="n">
+        <v>1</v>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Zuax anime and music</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Uitds6Ysj08</t>
+        </is>
+      </c>
+      <c r="M42" t="n">
+        <v>1</v>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>Zuax anime and music</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>2026-10-05T09:02:58</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -20477,13 +20597,37 @@
           <t>宮﨑歩・谷本貴義</t>
         </is>
       </c>
-      <c r="I120" t="inlineStr"/>
-      <c r="J120" t="inlineStr"/>
-      <c r="K120" t="inlineStr"/>
-      <c r="L120" t="inlineStr"/>
-      <c r="M120" t="inlineStr"/>
-      <c r="N120" t="inlineStr"/>
-      <c r="O120" t="inlineStr"/>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=uqIOdbe7rtI</t>
+        </is>
+      </c>
+      <c r="J120" t="n">
+        <v>284752</v>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>Digimon Official Channel</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=uqIOdbe7rtI</t>
+        </is>
+      </c>
+      <c r="M120" t="n">
+        <v>284752</v>
+      </c>
+      <c r="N120" t="inlineStr">
+        <is>
+          <t>Digimon Official Channel</t>
+        </is>
+      </c>
+      <c r="O120" t="inlineStr">
+        <is>
+          <t>2026-10-05T09:07:06</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -20520,13 +20664,37 @@
           <t>宮﨑歩・谷本貴義</t>
         </is>
       </c>
-      <c r="I121" t="inlineStr"/>
-      <c r="J121" t="inlineStr"/>
-      <c r="K121" t="inlineStr"/>
-      <c r="L121" t="inlineStr"/>
-      <c r="M121" t="inlineStr"/>
-      <c r="N121" t="inlineStr"/>
-      <c r="O121" t="inlineStr"/>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=irjWjYsfVk0</t>
+        </is>
+      </c>
+      <c r="J121" t="n">
+        <v>79492</v>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>Digimon Official Channel</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=irjWjYsfVk0</t>
+        </is>
+      </c>
+      <c r="M121" t="n">
+        <v>79492</v>
+      </c>
+      <c r="N121" t="inlineStr">
+        <is>
+          <t>Digimon Official Channel</t>
+        </is>
+      </c>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>2026-10-05T09:07:09</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -20620,13 +20788,37 @@
           <t>GAN（岩田剛典）</t>
         </is>
       </c>
-      <c r="I123" t="inlineStr"/>
-      <c r="J123" t="inlineStr"/>
-      <c r="K123" t="inlineStr"/>
-      <c r="L123" t="inlineStr"/>
-      <c r="M123" t="inlineStr"/>
-      <c r="N123" t="inlineStr"/>
-      <c r="O123" t="inlineStr"/>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=3MFyyGVajvA</t>
+        </is>
+      </c>
+      <c r="J123" t="n">
+        <v>4136</v>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>テレ東アニメ</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=3MFyyGVajvA</t>
+        </is>
+      </c>
+      <c r="M123" t="n">
+        <v>4136</v>
+      </c>
+      <c r="N123" t="inlineStr">
+        <is>
+          <t>テレ東アニメ</t>
+        </is>
+      </c>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t>2026-10-05T09:07:16</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -20663,13 +20855,37 @@
           <t>ファントムシータ</t>
         </is>
       </c>
-      <c r="I124" t="inlineStr"/>
-      <c r="J124" t="inlineStr"/>
-      <c r="K124" t="inlineStr"/>
-      <c r="L124" t="inlineStr"/>
-      <c r="M124" t="inlineStr"/>
-      <c r="N124" t="inlineStr"/>
-      <c r="O124" t="inlineStr"/>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=BUxVzKyGrsw</t>
+        </is>
+      </c>
+      <c r="J124" t="n">
+        <v>5833</v>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>テレ東アニメ</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=BUxVzKyGrsw</t>
+        </is>
+      </c>
+      <c r="M124" t="n">
+        <v>5833</v>
+      </c>
+      <c r="N124" t="inlineStr">
+        <is>
+          <t>テレ東アニメ</t>
+        </is>
+      </c>
+      <c r="O124" t="inlineStr">
+        <is>
+          <t>2026-10-05T09:07:25</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -21346,13 +21562,37 @@
           <t>FLOW</t>
         </is>
       </c>
-      <c r="I137" t="inlineStr"/>
-      <c r="J137" t="inlineStr"/>
-      <c r="K137" t="inlineStr"/>
-      <c r="L137" t="inlineStr"/>
-      <c r="M137" t="inlineStr"/>
-      <c r="N137" t="inlineStr"/>
-      <c r="O137" t="inlineStr"/>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=VzCsxgQ_4_M</t>
+        </is>
+      </c>
+      <c r="J137" t="n">
+        <v>37838</v>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>アニプレックス チャンネル</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=VzCsxgQ_4_M</t>
+        </is>
+      </c>
+      <c r="M137" t="n">
+        <v>37838</v>
+      </c>
+      <c r="N137" t="inlineStr">
+        <is>
+          <t>アニプレックス チャンネル</t>
+        </is>
+      </c>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>2026-10-05T09:08:06</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -21389,13 +21629,37 @@
           <t>ASTERISM</t>
         </is>
       </c>
-      <c r="I138" t="inlineStr"/>
-      <c r="J138" t="inlineStr"/>
-      <c r="K138" t="inlineStr"/>
-      <c r="L138" t="inlineStr"/>
-      <c r="M138" t="inlineStr"/>
-      <c r="N138" t="inlineStr"/>
-      <c r="O138" t="inlineStr"/>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=6GDMDhzPctA</t>
+        </is>
+      </c>
+      <c r="J138" t="n">
+        <v>20481</v>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>アニプレックス チャンネル</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=6GDMDhzPctA</t>
+        </is>
+      </c>
+      <c r="M138" t="n">
+        <v>20481</v>
+      </c>
+      <c r="N138" t="inlineStr">
+        <is>
+          <t>アニプレックス チャンネル</t>
+        </is>
+      </c>
+      <c r="O138" t="inlineStr">
+        <is>
+          <t>2026-10-05T09:08:16</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="n">

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-10-08
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -10244,7 +10244,7 @@
         </is>
       </c>
       <c r="C196" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D196" t="inlineStr">
         <is>
@@ -10289,7 +10289,7 @@
         </is>
       </c>
       <c r="C197" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D197" t="inlineStr">
         <is>
@@ -10330,7 +10330,7 @@
         </is>
       </c>
       <c r="C198" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D198" t="inlineStr">
         <is>
@@ -10371,7 +10371,7 @@
         </is>
       </c>
       <c r="C199" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D199" t="inlineStr">
         <is>
@@ -10412,7 +10412,7 @@
         </is>
       </c>
       <c r="C200" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D200" t="inlineStr">
         <is>
@@ -10465,7 +10465,7 @@
         </is>
       </c>
       <c r="C201" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D201" t="inlineStr">
         <is>
@@ -10506,7 +10506,7 @@
         </is>
       </c>
       <c r="C202" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D202" t="inlineStr">
         <is>
@@ -10547,7 +10547,7 @@
         </is>
       </c>
       <c r="C203" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D203" t="inlineStr">
         <is>
@@ -10608,7 +10608,7 @@
         </is>
       </c>
       <c r="C204" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D204" t="inlineStr">
         <is>
@@ -10649,7 +10649,7 @@
         </is>
       </c>
       <c r="C205" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D205" t="inlineStr">
         <is>
@@ -10690,7 +10690,7 @@
         </is>
       </c>
       <c r="C206" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D206" t="inlineStr">
         <is>
@@ -10747,7 +10747,7 @@
         </is>
       </c>
       <c r="C207" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D207" t="inlineStr">
         <is>
@@ -10792,7 +10792,7 @@
         </is>
       </c>
       <c r="C208" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D208" t="inlineStr">
         <is>
@@ -10833,7 +10833,7 @@
         </is>
       </c>
       <c r="C209" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D209" t="inlineStr">
         <is>
@@ -10886,7 +10886,7 @@
         </is>
       </c>
       <c r="C210" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D210" t="inlineStr">
         <is>
@@ -10927,7 +10927,7 @@
         </is>
       </c>
       <c r="C211" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D211" t="inlineStr">
         <is>
@@ -10972,7 +10972,7 @@
         </is>
       </c>
       <c r="C212" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D212" t="inlineStr">
         <is>
@@ -11025,7 +11025,7 @@
         </is>
       </c>
       <c r="C213" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D213" t="inlineStr">
         <is>
@@ -11066,7 +11066,7 @@
         </is>
       </c>
       <c r="C214" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D214" t="inlineStr">
         <is>
@@ -11111,7 +11111,7 @@
         </is>
       </c>
       <c r="C215" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D215" t="inlineStr">
         <is>
@@ -11168,7 +11168,7 @@
         </is>
       </c>
       <c r="C216" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D216" t="inlineStr">
         <is>
@@ -11213,7 +11213,7 @@
         </is>
       </c>
       <c r="C217" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D217" t="inlineStr">
         <is>
@@ -11254,7 +11254,7 @@
         </is>
       </c>
       <c r="C218" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D218" t="inlineStr">
         <is>
@@ -11295,7 +11295,7 @@
         </is>
       </c>
       <c r="C219" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D219" t="inlineStr">
         <is>
@@ -11336,7 +11336,7 @@
         </is>
       </c>
       <c r="C220" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D220" t="inlineStr">
         <is>
@@ -11381,7 +11381,7 @@
         </is>
       </c>
       <c r="C221" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D221" t="inlineStr">
         <is>
@@ -11426,7 +11426,7 @@
         </is>
       </c>
       <c r="C222" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D222" t="inlineStr">
         <is>
@@ -11467,7 +11467,7 @@
         </is>
       </c>
       <c r="C223" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D223" t="inlineStr">
         <is>
@@ -11508,7 +11508,7 @@
         </is>
       </c>
       <c r="C224" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D224" t="inlineStr">
         <is>
@@ -11557,7 +11557,7 @@
         </is>
       </c>
       <c r="C225" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D225" t="inlineStr">
         <is>
@@ -11602,7 +11602,7 @@
         </is>
       </c>
       <c r="C226" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D226" t="inlineStr">
         <is>
@@ -11643,7 +11643,7 @@
         </is>
       </c>
       <c r="C227" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D227" t="inlineStr">
         <is>
@@ -11704,7 +11704,7 @@
         </is>
       </c>
       <c r="C228" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D228" t="inlineStr">
         <is>
@@ -11749,7 +11749,7 @@
         </is>
       </c>
       <c r="C229" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D229" t="inlineStr">
         <is>
@@ -11790,7 +11790,7 @@
         </is>
       </c>
       <c r="C230" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D230" t="inlineStr">
         <is>
@@ -11851,7 +11851,7 @@
         </is>
       </c>
       <c r="C231" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D231" t="inlineStr">
         <is>
@@ -11892,7 +11892,7 @@
         </is>
       </c>
       <c r="C232" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D232" t="inlineStr">
         <is>
@@ -11937,7 +11937,7 @@
         </is>
       </c>
       <c r="C233" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D233" t="inlineStr">
         <is>
@@ -11982,7 +11982,7 @@
         </is>
       </c>
       <c r="C234" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D234" t="inlineStr">
         <is>
@@ -12023,7 +12023,7 @@
         </is>
       </c>
       <c r="C235" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D235" t="inlineStr">
         <is>
@@ -12064,7 +12064,7 @@
         </is>
       </c>
       <c r="C236" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D236" t="inlineStr">
         <is>
@@ -12109,7 +12109,7 @@
         </is>
       </c>
       <c r="C237" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D237" t="inlineStr">
         <is>
@@ -12154,7 +12154,7 @@
         </is>
       </c>
       <c r="C238" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D238" t="inlineStr">
         <is>
@@ -12199,7 +12199,7 @@
         </is>
       </c>
       <c r="C239" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D239" t="inlineStr">
         <is>
@@ -12244,7 +12244,7 @@
         </is>
       </c>
       <c r="C240" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D240" t="inlineStr">
         <is>
@@ -12305,7 +12305,7 @@
         </is>
       </c>
       <c r="C241" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D241" t="inlineStr">
         <is>
@@ -12346,7 +12346,7 @@
         </is>
       </c>
       <c r="C242" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D242" t="inlineStr">
         <is>
@@ -12391,7 +12391,7 @@
         </is>
       </c>
       <c r="C243" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D243" t="inlineStr">
         <is>
@@ -12432,7 +12432,7 @@
         </is>
       </c>
       <c r="C244" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D244" t="inlineStr">
         <is>
@@ -12489,7 +12489,7 @@
         </is>
       </c>
       <c r="C245" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D245" t="inlineStr">
         <is>
@@ -12530,7 +12530,7 @@
         </is>
       </c>
       <c r="C246" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D246" t="inlineStr">
         <is>
@@ -12575,7 +12575,7 @@
         </is>
       </c>
       <c r="C247" t="n">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D247" t="inlineStr">
         <is>
@@ -12620,7 +12620,7 @@
         </is>
       </c>
       <c r="C248" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D248" t="inlineStr">
         <is>
@@ -12661,7 +12661,7 @@
         </is>
       </c>
       <c r="C249" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D249" t="inlineStr">
         <is>
@@ -12702,7 +12702,7 @@
         </is>
       </c>
       <c r="C250" t="n">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D250" t="inlineStr">
         <is>
@@ -12743,7 +12743,7 @@
         </is>
       </c>
       <c r="C251" t="n">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D251" t="inlineStr">
         <is>
@@ -12784,7 +12784,7 @@
         </is>
       </c>
       <c r="C252" t="n">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D252" t="inlineStr">
         <is>
@@ -12825,7 +12825,7 @@
         </is>
       </c>
       <c r="C253" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D253" t="inlineStr">
         <is>
@@ -12866,7 +12866,7 @@
         </is>
       </c>
       <c r="C254" t="n">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D254" t="inlineStr">
         <is>
@@ -12907,7 +12907,7 @@
         </is>
       </c>
       <c r="C255" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D255" t="inlineStr">
         <is>
@@ -12952,7 +12952,7 @@
         </is>
       </c>
       <c r="C256" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D256" t="inlineStr">
         <is>
@@ -13001,7 +13001,7 @@
         </is>
       </c>
       <c r="C257" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D257" t="inlineStr">
         <is>
@@ -13042,7 +13042,7 @@
         </is>
       </c>
       <c r="C258" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D258" t="inlineStr">
         <is>
@@ -13087,7 +13087,7 @@
         </is>
       </c>
       <c r="C259" t="n">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D259" t="inlineStr">
         <is>
@@ -13132,7 +13132,7 @@
         </is>
       </c>
       <c r="C260" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D260" t="inlineStr">
         <is>
@@ -13177,7 +13177,7 @@
         </is>
       </c>
       <c r="C261" t="n">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D261" t="inlineStr">
         <is>
@@ -13222,7 +13222,7 @@
         </is>
       </c>
       <c r="C262" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D262" t="inlineStr">
         <is>
@@ -13263,7 +13263,7 @@
         </is>
       </c>
       <c r="C263" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D263" t="inlineStr">
         <is>
@@ -13324,7 +13324,7 @@
         </is>
       </c>
       <c r="C264" t="n">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D264" t="inlineStr">
         <is>
@@ -13365,7 +13365,7 @@
         </is>
       </c>
       <c r="C265" t="n">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D265" t="inlineStr">
         <is>
@@ -13406,7 +13406,7 @@
         </is>
       </c>
       <c r="C266" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D266" t="inlineStr">
         <is>
@@ -13451,7 +13451,7 @@
         </is>
       </c>
       <c r="C267" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D267" t="inlineStr">
         <is>
@@ -13492,7 +13492,7 @@
         </is>
       </c>
       <c r="C268" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D268" t="inlineStr">
         <is>
@@ -13537,7 +13537,7 @@
         </is>
       </c>
       <c r="C269" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D269" t="inlineStr">
         <is>
@@ -13578,7 +13578,7 @@
         </is>
       </c>
       <c r="C270" t="n">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D270" t="inlineStr">
         <is>
@@ -13639,7 +13639,7 @@
         </is>
       </c>
       <c r="C271" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D271" t="inlineStr">
         <is>
@@ -13684,7 +13684,7 @@
         </is>
       </c>
       <c r="C272" t="n">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D272" t="inlineStr">
         <is>
@@ -13729,7 +13729,7 @@
         </is>
       </c>
       <c r="C273" t="n">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D273" t="inlineStr">
         <is>
@@ -13774,7 +13774,7 @@
         </is>
       </c>
       <c r="C274" t="n">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D274" t="inlineStr">
         <is>
@@ -13815,7 +13815,7 @@
         </is>
       </c>
       <c r="C275" t="n">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D275" t="inlineStr">
         <is>
@@ -13856,7 +13856,7 @@
         </is>
       </c>
       <c r="C276" t="n">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D276" t="inlineStr">
         <is>
@@ -13897,7 +13897,7 @@
         </is>
       </c>
       <c r="C277" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D277" t="inlineStr">
         <is>
@@ -13938,7 +13938,7 @@
         </is>
       </c>
       <c r="C278" t="n">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D278" t="inlineStr">
         <is>
@@ -13983,7 +13983,7 @@
         </is>
       </c>
       <c r="C279" t="n">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D279" t="inlineStr">
         <is>
@@ -14032,7 +14032,7 @@
         </is>
       </c>
       <c r="C280" t="n">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D280" t="inlineStr">
         <is>
@@ -14073,7 +14073,7 @@
         </is>
       </c>
       <c r="C281" t="n">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D281" t="inlineStr">
         <is>
@@ -15122,7 +15122,7 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>219632</v>
+        <v>312734</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -15135,7 +15135,7 @@
         </is>
       </c>
       <c r="M12" t="n">
-        <v>219632</v>
+        <v>312734</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
@@ -15144,7 +15144,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>2026-09-30T09:00:58</t>
+          <t>2026-10-08T09:00:34</t>
         </is>
       </c>
     </row>
@@ -15604,13 +15604,27 @@
           <t>原因は自分にある。</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=TKY-lAGnP50</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>85318</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>原因は自分にある。Official</t>
+        </is>
+      </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>2026-10-08T09:01:13</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -17640,13 +17654,37 @@
           <t>HoneyWorks feat.ハコニワリリィ</t>
         </is>
       </c>
-      <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
-      <c r="L58" t="inlineStr"/>
-      <c r="M58" t="inlineStr"/>
-      <c r="N58" t="inlineStr"/>
-      <c r="O58" t="inlineStr"/>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=kX0ZBPvZc-4</t>
+        </is>
+      </c>
+      <c r="J58" t="n">
+        <v>20033</v>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>ぽにきゃん-Anime PONY CANYON</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=kX0ZBPvZc-4</t>
+        </is>
+      </c>
+      <c r="M58" t="n">
+        <v>20033</v>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>ぽにきゃん-Anime PONY CANYON</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>2026-10-08T09:02:54</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -18328,13 +18366,37 @@
           <t>心梅</t>
         </is>
       </c>
-      <c r="I72" t="inlineStr"/>
-      <c r="J72" t="inlineStr"/>
-      <c r="K72" t="inlineStr"/>
-      <c r="L72" t="inlineStr"/>
-      <c r="M72" t="inlineStr"/>
-      <c r="N72" t="inlineStr"/>
-      <c r="O72" t="inlineStr"/>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=0C9t6lrFM_o</t>
+        </is>
+      </c>
+      <c r="J72" t="n">
+        <v>51040</v>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=0C9t6lrFM_o</t>
+        </is>
+      </c>
+      <c r="M72" t="n">
+        <v>51040</v>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>2026-10-08T09:03:43</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -19475,13 +19537,37 @@
           <t>FZMZ</t>
         </is>
       </c>
-      <c r="I93" t="inlineStr"/>
-      <c r="J93" t="inlineStr"/>
-      <c r="K93" t="inlineStr"/>
-      <c r="L93" t="inlineStr"/>
-      <c r="M93" t="inlineStr"/>
-      <c r="N93" t="inlineStr"/>
-      <c r="O93" t="inlineStr"/>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=4FCUWOqNwCc</t>
+        </is>
+      </c>
+      <c r="J93" t="n">
+        <v>18627</v>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=4FCUWOqNwCc</t>
+        </is>
+      </c>
+      <c r="M93" t="n">
+        <v>18627</v>
+      </c>
+      <c r="N93" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>2026-10-08T09:05:01</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -19518,13 +19604,37 @@
           <t>花冷え。</t>
         </is>
       </c>
-      <c r="I94" t="inlineStr"/>
-      <c r="J94" t="inlineStr"/>
-      <c r="K94" t="inlineStr"/>
-      <c r="L94" t="inlineStr"/>
-      <c r="M94" t="inlineStr"/>
-      <c r="N94" t="inlineStr"/>
-      <c r="O94" t="inlineStr"/>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=SYbP5PxHZvM</t>
+        </is>
+      </c>
+      <c r="J94" t="n">
+        <v>11012</v>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=SYbP5PxHZvM</t>
+        </is>
+      </c>
+      <c r="M94" t="n">
+        <v>11012</v>
+      </c>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>2026-10-08T09:05:10</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -22865,24 +22975,24 @@
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=ic9XKLWMbCw</t>
+          <t>https://www.youtube.com/watch?v=uUVjCC6So30</t>
         </is>
       </c>
       <c r="J153" t="n">
-        <v>856429</v>
+        <v>159571</v>
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>『ユイカ』</t>
+          <t>MAPPA CHANNEL</t>
         </is>
       </c>
       <c r="L153" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=X-SOSlnkXAc</t>
+          <t>https://www.youtube.com/watch?v=uUVjCC6So30</t>
         </is>
       </c>
       <c r="M153" t="n">
-        <v>841862</v>
+        <v>159571</v>
       </c>
       <c r="N153" t="inlineStr">
         <is>
@@ -22891,7 +23001,7 @@
       </c>
       <c r="O153" t="inlineStr">
         <is>
-          <t>2026-09-30T09:09:21</t>
+          <t>2026-10-08T09:07:04</t>
         </is>
       </c>
     </row>
@@ -22932,23 +23042,33 @@
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=PxXPcoo8uGM</t>
+          <t>https://www.youtube.com/watch?v=k8G3_ZYNC-I</t>
         </is>
       </c>
       <c r="J154" t="n">
-        <v>607462</v>
+        <v>1025615</v>
       </c>
       <c r="K154" t="inlineStr">
         <is>
           <t>TVアニメ「ロメリア戦記」Official Channel</t>
         </is>
       </c>
-      <c r="L154" t="inlineStr"/>
-      <c r="M154" t="inlineStr"/>
-      <c r="N154" t="inlineStr"/>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=_PIj78IgPmA</t>
+        </is>
+      </c>
+      <c r="M154" t="n">
+        <v>30703</v>
+      </c>
+      <c r="N154" t="inlineStr">
+        <is>
+          <t>TVアニメ「ロメリア戦記」Official Channel</t>
+        </is>
+      </c>
       <c r="O154" t="inlineStr">
         <is>
-          <t>2026-09-30T09:09:36</t>
+          <t>2026-10-08T09:07:12</t>
         </is>
       </c>
     </row>
@@ -22993,7 +23113,7 @@
         </is>
       </c>
       <c r="J155" t="n">
-        <v>607462</v>
+        <v>1032680</v>
       </c>
       <c r="K155" t="inlineStr">
         <is>
@@ -23005,7 +23125,7 @@
       <c r="N155" t="inlineStr"/>
       <c r="O155" t="inlineStr">
         <is>
-          <t>2026-09-30T09:09:44</t>
+          <t>2026-10-08T09:07:27</t>
         </is>
       </c>
     </row>
@@ -26391,37 +26511,13 @@
           <t>LiSA</t>
         </is>
       </c>
-      <c r="I221" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=S23MKJP0lCw</t>
-        </is>
-      </c>
-      <c r="J221" t="n">
-        <v>9660</v>
-      </c>
-      <c r="K221" t="inlineStr">
-        <is>
-          <t>LiSA Official YouTube</t>
-        </is>
-      </c>
-      <c r="L221" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=GFW7P55j0-g</t>
-        </is>
-      </c>
-      <c r="M221" t="n">
-        <v>2416342</v>
-      </c>
-      <c r="N221" t="inlineStr">
-        <is>
-          <t>アニプレックス チャンネル</t>
-        </is>
-      </c>
-      <c r="O221" t="inlineStr">
-        <is>
-          <t>2026-09-30T09:12:34</t>
-        </is>
-      </c>
+      <c r="I221" t="inlineStr"/>
+      <c r="J221" t="inlineStr"/>
+      <c r="K221" t="inlineStr"/>
+      <c r="L221" t="inlineStr"/>
+      <c r="M221" t="inlineStr"/>
+      <c r="N221" t="inlineStr"/>
+      <c r="O221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="n">

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-10-09
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M289"/>
+  <dimension ref="A1:M290"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7705,7 +7705,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>Acca effe×フロンティアエンジン</t>
+          <t>Acca effe</t>
         </is>
       </c>
       <c r="I139" t="inlineStr"/>
@@ -8527,7 +8527,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>Qzil.la studio keel</t>
+          <t>Qzil.la</t>
         </is>
       </c>
       <c r="I157" t="inlineStr"/>
@@ -14376,7 +14376,7 @@
     </row>
     <row r="288">
       <c r="A288" t="n">
-        <v>-206298</v>
+        <v>-183692</v>
       </c>
       <c r="B288" t="inlineStr">
         <is>
@@ -14388,7 +14388,7 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>劇場版 メダリスト</t>
+          <t>機動戦士ガンダムSEED FREEDOM ZERO</t>
         </is>
       </c>
       <c r="E288" t="b">
@@ -14401,12 +14401,12 @@
       </c>
       <c r="G288" t="inlineStr">
         <is>
-          <t>2027年2月19日</t>
+          <t>2027年1月15日</t>
         </is>
       </c>
       <c r="H288" t="inlineStr">
         <is>
-          <t>ENGI</t>
+          <t>Sunrise</t>
         </is>
       </c>
       <c r="I288" t="inlineStr"/>
@@ -14415,13 +14415,13 @@
       <c r="L288" t="inlineStr"/>
       <c r="M288" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/206298</t>
+          <t>https://anilist.co/anime/183692</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="n">
-        <v>-216623</v>
+        <v>-206298</v>
       </c>
       <c r="B289" t="inlineStr">
         <is>
@@ -14433,7 +14433,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>ドラえもん のび太の蒸気時間車</t>
+          <t>劇場版 メダリスト</t>
         </is>
       </c>
       <c r="E289" t="b">
@@ -14446,12 +14446,12 @@
       </c>
       <c r="G289" t="inlineStr">
         <is>
-          <t>2027年3月5日</t>
+          <t>2027年2月19日</t>
         </is>
       </c>
       <c r="H289" t="inlineStr">
         <is>
-          <t>Shin-Ei Animation</t>
+          <t>ENGI</t>
         </is>
       </c>
       <c r="I289" t="inlineStr"/>
@@ -14459,6 +14459,51 @@
       <c r="K289" t="inlineStr"/>
       <c r="L289" t="inlineStr"/>
       <c r="M289" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/206298</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="n">
+        <v>-216623</v>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>2027冬アニメ</t>
+        </is>
+      </c>
+      <c r="C290" t="n">
+        <v>0</v>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>ドラえもん のび太の蒸気時間車</t>
+        </is>
+      </c>
+      <c r="E290" t="b">
+        <v>0</v>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>2027年3月5日</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>Shin-Ei Animation</t>
+        </is>
+      </c>
+      <c r="I290" t="inlineStr"/>
+      <c r="J290" t="inlineStr"/>
+      <c r="K290" t="inlineStr"/>
+      <c r="L290" t="inlineStr"/>
+      <c r="M290" t="inlineStr">
         <is>
           <t>https://anilist.co/anime/216623</t>
         </is>
@@ -16742,13 +16787,37 @@
           <t>THE BEAT GARDEN</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
-      <c r="O40" t="inlineStr"/>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=nMp5XQo-_Zg</t>
+        </is>
+      </c>
+      <c r="J40" t="n">
+        <v>41279</v>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>TBSアニメ</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=nMp5XQo-_Zg</t>
+        </is>
+      </c>
+      <c r="M40" t="n">
+        <v>41279</v>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>TBSアニメ</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>2026-10-09T09:01:41</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -16787,23 +16856,33 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=NPUnblFfI2w</t>
+          <t>https://www.youtube.com/watch?v=m6IBZor25nM</t>
         </is>
       </c>
       <c r="J41" t="n">
-        <v>17071</v>
+        <v>194530</v>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>Superfly</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr"/>
+          <t>TBSアニメ</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=m6IBZor25nM</t>
+        </is>
+      </c>
+      <c r="M41" t="n">
+        <v>194530</v>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>TBSアニメ</t>
+        </is>
+      </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>2026-10-01T09:03:13</t>
+          <t>2026-10-09T09:01:51</t>
         </is>
       </c>
     </row>
@@ -16976,13 +17055,37 @@
           <t>MADKID</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=rPaWkpG1wAs</t>
+        </is>
+      </c>
+      <c r="J44" t="n">
+        <v>55629</v>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=rPaWkpG1wAs</t>
+        </is>
+      </c>
+      <c r="M44" t="n">
+        <v>55629</v>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>2026-10-09T09:02:00</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -17286,13 +17389,37 @@
           <t>西川貴教</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr"/>
-      <c r="N50" t="inlineStr"/>
-      <c r="O50" t="inlineStr"/>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=a8fgR7YAUj4</t>
+        </is>
+      </c>
+      <c r="J50" t="n">
+        <v>310019</v>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>GOOD SMILE CHANNEL</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=a8fgR7YAUj4</t>
+        </is>
+      </c>
+      <c r="M50" t="n">
+        <v>310019</v>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>GOOD SMILE CHANNEL</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>2026-10-09T09:02:25</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -17415,13 +17542,27 @@
           <t>Suupeas</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=O_vYVXH9m3E</t>
+        </is>
+      </c>
+      <c r="J53" t="n">
+        <v>471</v>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Suupeas</t>
+        </is>
+      </c>
       <c r="L53" t="inlineStr"/>
       <c r="M53" t="inlineStr"/>
       <c r="N53" t="inlineStr"/>
-      <c r="O53" t="inlineStr"/>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>2026-10-09T09:02:55</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -18777,13 +18918,37 @@
           <t>亜咲花</t>
         </is>
       </c>
-      <c r="I79" t="inlineStr"/>
-      <c r="J79" t="inlineStr"/>
-      <c r="K79" t="inlineStr"/>
-      <c r="L79" t="inlineStr"/>
-      <c r="M79" t="inlineStr"/>
-      <c r="N79" t="inlineStr"/>
-      <c r="O79" t="inlineStr"/>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=YOZAtTfugI8</t>
+        </is>
+      </c>
+      <c r="J79" t="n">
+        <v>10838</v>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>ぽにきゃん-Anime PONY CANYON</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=YOZAtTfugI8</t>
+        </is>
+      </c>
+      <c r="M79" t="n">
+        <v>10838</v>
+      </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>ぽにきゃん-Anime PONY CANYON</t>
+        </is>
+      </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>2026-10-09T09:04:18</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -20504,7 +20669,7 @@
         </is>
       </c>
       <c r="J110" t="n">
-        <v>83733</v>
+        <v>105107</v>
       </c>
       <c r="K110" t="inlineStr">
         <is>
@@ -20516,7 +20681,7 @@
       <c r="N110" t="inlineStr"/>
       <c r="O110" t="inlineStr">
         <is>
-          <t>2026-10-01T09:07:46</t>
+          <t>2026-10-09T09:06:05</t>
         </is>
       </c>
     </row>
@@ -20561,7 +20726,7 @@
         </is>
       </c>
       <c r="J111" t="n">
-        <v>83733</v>
+        <v>105107</v>
       </c>
       <c r="K111" t="inlineStr">
         <is>
@@ -20573,7 +20738,7 @@
       <c r="N111" t="inlineStr"/>
       <c r="O111" t="inlineStr">
         <is>
-          <t>2026-10-01T09:08:00</t>
+          <t>2026-10-09T09:06:20</t>
         </is>
       </c>
     </row>
@@ -22533,13 +22698,37 @@
           <t>SHY</t>
         </is>
       </c>
-      <c r="I145" t="inlineStr"/>
-      <c r="J145" t="inlineStr"/>
-      <c r="K145" t="inlineStr"/>
-      <c r="L145" t="inlineStr"/>
-      <c r="M145" t="inlineStr"/>
-      <c r="N145" t="inlineStr"/>
-      <c r="O145" t="inlineStr"/>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=mOm7K-klguU</t>
+        </is>
+      </c>
+      <c r="J145" t="n">
+        <v>593</v>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>テレ東アニメKids</t>
+        </is>
+      </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=mOm7K-klguU</t>
+        </is>
+      </c>
+      <c r="M145" t="n">
+        <v>593</v>
+      </c>
+      <c r="N145" t="inlineStr">
+        <is>
+          <t>テレ東アニメKids</t>
+        </is>
+      </c>
+      <c r="O145" t="inlineStr">
+        <is>
+          <t>2026-10-09T09:07:10</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -28340,27 +28529,13 @@
           <t>adieu（上白石萌歌）</t>
         </is>
       </c>
-      <c r="I258" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=fBfs6ZE1L-M</t>
-        </is>
-      </c>
-      <c r="J258" t="n">
-        <v>56411</v>
-      </c>
-      <c r="K258" t="inlineStr">
-        <is>
-          <t>adieu [ 上白石萌歌 ] official YouTube channel</t>
-        </is>
-      </c>
+      <c r="I258" t="inlineStr"/>
+      <c r="J258" t="inlineStr"/>
+      <c r="K258" t="inlineStr"/>
       <c r="L258" t="inlineStr"/>
       <c r="M258" t="inlineStr"/>
       <c r="N258" t="inlineStr"/>
-      <c r="O258" t="inlineStr">
-        <is>
-          <t>2026-10-01T09:14:47</t>
-        </is>
-      </c>
+      <c r="O258" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-10-11
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -15434,7 +15434,7 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>1214557</v>
+        <v>5760056</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -15447,16 +15447,16 @@
         </is>
       </c>
       <c r="M17" t="n">
-        <v>632993</v>
+        <v>635124</v>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>ヴァンガードチャンネル【アニメ「Divinez 幻真星戦編」配信中!!】</t>
+          <t>ヴァンガードチャンネル【アニメ「Divinez 運命星戦編」劇場先行上映公開中!】</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2026-10-03T09:01:29</t>
+          <t>2026-10-11T09:01:10</t>
         </is>
       </c>
     </row>
@@ -16107,13 +16107,37 @@
           <t>月追う彼方</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=HwJXu_CirFQ</t>
+        </is>
+      </c>
+      <c r="J28" t="n">
+        <v>497</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AnimationID </t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=HwJXu_CirFQ</t>
+        </is>
+      </c>
+      <c r="M28" t="n">
+        <v>497</v>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AnimationID </t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>2026-10-11T09:01:25</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -16266,7 +16290,7 @@
         </is>
       </c>
       <c r="J31" t="n">
-        <v>2605197</v>
+        <v>2689336</v>
       </c>
       <c r="K31" t="inlineStr">
         <is>
@@ -16279,7 +16303,7 @@
         </is>
       </c>
       <c r="M31" t="n">
-        <v>825411</v>
+        <v>2667984</v>
       </c>
       <c r="N31" t="inlineStr">
         <is>
@@ -16288,7 +16312,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>2026-10-03T09:02:58</t>
+          <t>2026-10-11T09:01:39</t>
         </is>
       </c>
     </row>
@@ -16592,33 +16616,33 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=ZpClwSAbjgA</t>
+          <t>https://www.youtube.com/watch?v=UgJ6bYkIKYY</t>
         </is>
       </c>
       <c r="J37" t="n">
-        <v>835367</v>
+        <v>137475</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>amazarashi Official YouTube Channel</t>
+          <t>NBCUniversal Anime/Music</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=gupmw0_6Bu4</t>
+          <t>https://www.youtube.com/watch?v=UgJ6bYkIKYY</t>
         </is>
       </c>
       <c r="M37" t="n">
-        <v>191716</v>
+        <v>137475</v>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>KONAMI公式</t>
+          <t>NBCUniversal Anime/Music</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>2026-10-03T09:03:17</t>
+          <t>2026-10-11T09:02:00</t>
         </is>
       </c>
     </row>
@@ -17132,19 +17156,29 @@
         </is>
       </c>
       <c r="J45" t="n">
-        <v>2105920</v>
+        <v>2293064</v>
       </c>
       <c r="K45" t="inlineStr">
         <is>
           <t>のんふぃく！【Non¬Fiction】</t>
         </is>
       </c>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=29Vi0JilpVQ</t>
+        </is>
+      </c>
+      <c r="M45" t="n">
+        <v>26313</v>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>2026-10-03T09:03:53</t>
+          <t>2026-10-11T09:02:11</t>
         </is>
       </c>
     </row>
@@ -17293,13 +17327,37 @@
           <t>MAN WITH A MISSION</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
-      <c r="N48" t="inlineStr"/>
-      <c r="O48" t="inlineStr"/>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=w9Y4BqDs_DU</t>
+        </is>
+      </c>
+      <c r="J48" t="n">
+        <v>26763</v>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>【ytv animation】読売テレビ アニメ公式</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=w9Y4BqDs_DU</t>
+        </is>
+      </c>
+      <c r="M48" t="n">
+        <v>26763</v>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>【ytv animation】読売テレビ アニメ公式</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>2026-10-11T09:02:23</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -17336,13 +17394,37 @@
           <t>yutori</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
-      <c r="N49" t="inlineStr"/>
-      <c r="O49" t="inlineStr"/>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-cv3r0fV3F8</t>
+        </is>
+      </c>
+      <c r="J49" t="n">
+        <v>7768</v>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>【ytv animation】読売テレビ アニメ公式</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-cv3r0fV3F8</t>
+        </is>
+      </c>
+      <c r="M49" t="n">
+        <v>7768</v>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>【ytv animation】読売テレビ アニメ公式</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>2026-10-11T09:02:32</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -17638,7 +17720,7 @@
         </is>
       </c>
       <c r="J55" t="n">
-        <v>829180</v>
+        <v>831170</v>
       </c>
       <c r="K55" t="inlineStr">
         <is>
@@ -17651,7 +17733,7 @@
         </is>
       </c>
       <c r="M55" t="n">
-        <v>75541</v>
+        <v>105329</v>
       </c>
       <c r="N55" t="inlineStr">
         <is>
@@ -17660,7 +17742,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>2026-10-03T09:04:45</t>
+          <t>2026-10-11T09:02:58</t>
         </is>
       </c>
     </row>
@@ -17962,13 +18044,37 @@
           <t>cadode</t>
         </is>
       </c>
-      <c r="I61" t="inlineStr"/>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
-      <c r="L61" t="inlineStr"/>
-      <c r="M61" t="inlineStr"/>
-      <c r="N61" t="inlineStr"/>
-      <c r="O61" t="inlineStr"/>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=h6Vsivg4jyM</t>
+        </is>
+      </c>
+      <c r="J61" t="n">
+        <v>11261</v>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=h6Vsivg4jyM</t>
+        </is>
+      </c>
+      <c r="M61" t="n">
+        <v>11261</v>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>2026-10-11T09:03:22</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -18306,27 +18412,13 @@
           <t>OxT</t>
         </is>
       </c>
-      <c r="I69" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=6G3ftpd4itQ</t>
-        </is>
-      </c>
-      <c r="J69" t="n">
-        <v>25634</v>
-      </c>
-      <c r="K69" t="inlineStr">
-        <is>
-          <t>OxT - Topic</t>
-        </is>
-      </c>
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr"/>
       <c r="M69" t="inlineStr"/>
       <c r="N69" t="inlineStr"/>
-      <c r="O69" t="inlineStr">
-        <is>
-          <t>2026-10-03T09:06:02</t>
-        </is>
-      </c>
+      <c r="O69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -18432,11 +18524,11 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=IrHhljLwzXw</t>
+          <t>https://www.youtube.com/watch?v=AQ8euxxP7JQ</t>
         </is>
       </c>
       <c r="J71" t="n">
-        <v>9359</v>
+        <v>28989</v>
       </c>
       <c r="K71" t="inlineStr">
         <is>
@@ -18445,11 +18537,11 @@
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=IrHhljLwzXw</t>
+          <t>https://www.youtube.com/watch?v=AQ8euxxP7JQ</t>
         </is>
       </c>
       <c r="M71" t="n">
-        <v>9359</v>
+        <v>28989</v>
       </c>
       <c r="N71" t="inlineStr">
         <is>
@@ -18458,7 +18550,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>2026-10-03T09:06:08</t>
+          <t>2026-10-11T09:04:00</t>
         </is>
       </c>
     </row>
@@ -18570,7 +18662,7 @@
         </is>
       </c>
       <c r="J73" t="n">
-        <v>2588507</v>
+        <v>2597390</v>
       </c>
       <c r="K73" t="inlineStr">
         <is>
@@ -18582,7 +18674,7 @@
       <c r="N73" t="inlineStr"/>
       <c r="O73" t="inlineStr">
         <is>
-          <t>2026-10-03T09:06:36</t>
+          <t>2026-10-11T09:04:20</t>
         </is>
       </c>
     </row>
@@ -18627,7 +18719,7 @@
         </is>
       </c>
       <c r="J74" t="n">
-        <v>767715</v>
+        <v>779768</v>
       </c>
       <c r="K74" t="inlineStr">
         <is>
@@ -18640,7 +18732,7 @@
         </is>
       </c>
       <c r="M74" t="n">
-        <v>767715</v>
+        <v>779768</v>
       </c>
       <c r="N74" t="inlineStr">
         <is>
@@ -18649,7 +18741,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>2026-10-03T09:06:46</t>
+          <t>2026-10-11T09:04:30</t>
         </is>
       </c>
     </row>
@@ -18761,7 +18853,7 @@
         </is>
       </c>
       <c r="J76" t="n">
-        <v>431264</v>
+        <v>437643</v>
       </c>
       <c r="K76" t="inlineStr">
         <is>
@@ -18774,7 +18866,7 @@
         </is>
       </c>
       <c r="M76" t="n">
-        <v>431264</v>
+        <v>437643</v>
       </c>
       <c r="N76" t="inlineStr">
         <is>
@@ -18783,7 +18875,7 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>2026-10-03T09:06:55</t>
+          <t>2026-10-11T09:04:39</t>
         </is>
       </c>
     </row>
@@ -19268,7 +19360,7 @@
         </is>
       </c>
       <c r="J85" t="n">
-        <v>51786</v>
+        <v>52535</v>
       </c>
       <c r="K85" t="inlineStr">
         <is>
@@ -19281,7 +19373,7 @@
         </is>
       </c>
       <c r="M85" t="n">
-        <v>50074</v>
+        <v>51420</v>
       </c>
       <c r="N85" t="inlineStr">
         <is>
@@ -19290,7 +19382,7 @@
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>2026-10-03T09:07:54</t>
+          <t>2026-10-11T09:05:15</t>
         </is>
       </c>
     </row>
@@ -19335,7 +19427,7 @@
         </is>
       </c>
       <c r="J86" t="n">
-        <v>219044</v>
+        <v>221811</v>
       </c>
       <c r="K86" t="inlineStr">
         <is>
@@ -19348,7 +19440,7 @@
         </is>
       </c>
       <c r="M86" t="n">
-        <v>219044</v>
+        <v>221811</v>
       </c>
       <c r="N86" t="inlineStr">
         <is>
@@ -19357,7 +19449,7 @@
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>2026-10-03T09:08:02</t>
+          <t>2026-10-11T09:05:25</t>
         </is>
       </c>
     </row>
@@ -19884,13 +19976,27 @@
           <t>East Of Eden</t>
         </is>
       </c>
-      <c r="I95" t="inlineStr"/>
-      <c r="J95" t="inlineStr"/>
-      <c r="K95" t="inlineStr"/>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=5ChLZwJZn9s</t>
+        </is>
+      </c>
+      <c r="J95" t="n">
+        <v>11682</v>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>East Of Eden</t>
+        </is>
+      </c>
       <c r="L95" t="inlineStr"/>
       <c r="M95" t="inlineStr"/>
       <c r="N95" t="inlineStr"/>
-      <c r="O95" t="inlineStr"/>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>2026-10-11T09:05:51</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -20106,33 +20212,33 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=ZmCOHpUBXo0</t>
+          <t>https://www.youtube.com/watch?v=QWY9TDnIJg8</t>
         </is>
       </c>
       <c r="J99" t="n">
-        <v>476878</v>
+        <v>1003754</v>
       </c>
       <c r="K99" t="inlineStr">
         <is>
+          <t>Hiromitsu Kitayama</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=CBC9M-UH58c</t>
+        </is>
+      </c>
+      <c r="M99" t="n">
+        <v>297654</v>
+      </c>
+      <c r="N99" t="inlineStr">
+        <is>
           <t>『桃源暗鬼』プロジェクト公式チャンネル</t>
         </is>
       </c>
-      <c r="L99" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=yI3PSYmU8ig</t>
-        </is>
-      </c>
-      <c r="M99" t="n">
-        <v>1289695</v>
-      </c>
-      <c r="N99" t="inlineStr">
-        <is>
-          <t>『桃源暗鬼』プロジェクト公式チャンネル</t>
-        </is>
-      </c>
       <c r="O99" t="inlineStr">
         <is>
-          <t>2026-10-03T09:09:10</t>
+          <t>2026-10-11T09:06:04</t>
         </is>
       </c>
     </row>
@@ -20177,19 +20283,29 @@
         </is>
       </c>
       <c r="J100" t="n">
-        <v>476878</v>
+        <v>512255</v>
       </c>
       <c r="K100" t="inlineStr">
         <is>
           <t>『桃源暗鬼』プロジェクト公式チャンネル</t>
         </is>
       </c>
-      <c r="L100" t="inlineStr"/>
-      <c r="M100" t="inlineStr"/>
-      <c r="N100" t="inlineStr"/>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=J8h3zQN4JRA</t>
+        </is>
+      </c>
+      <c r="M100" t="n">
+        <v>48804</v>
+      </c>
+      <c r="N100" t="inlineStr">
+        <is>
+          <t>『桃源暗鬼』プロジェクト公式チャンネル</t>
+        </is>
+      </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>2026-10-03T09:09:27</t>
+          <t>2026-10-11T09:06:13</t>
         </is>
       </c>
     </row>
@@ -20368,7 +20484,7 @@
         </is>
       </c>
       <c r="J103" t="n">
-        <v>31767</v>
+        <v>33417</v>
       </c>
       <c r="K103" t="inlineStr">
         <is>
@@ -20381,7 +20497,7 @@
         </is>
       </c>
       <c r="M103" t="n">
-        <v>31767</v>
+        <v>33417</v>
       </c>
       <c r="N103" t="inlineStr">
         <is>
@@ -20390,7 +20506,7 @@
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>2026-10-03T09:09:48</t>
+          <t>2026-10-11T09:06:22</t>
         </is>
       </c>
     </row>
@@ -20607,7 +20723,7 @@
         </is>
       </c>
       <c r="J108" t="n">
-        <v>304405</v>
+        <v>329548</v>
       </c>
       <c r="K108" t="inlineStr">
         <is>
@@ -20620,7 +20736,7 @@
         </is>
       </c>
       <c r="M108" t="n">
-        <v>304405</v>
+        <v>329548</v>
       </c>
       <c r="N108" t="inlineStr">
         <is>
@@ -20629,7 +20745,7 @@
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t>2026-10-03T09:10:24</t>
+          <t>2026-10-11T09:06:57</t>
         </is>
       </c>
     </row>
@@ -20668,13 +20784,37 @@
           <t>はしメロ</t>
         </is>
       </c>
-      <c r="I109" t="inlineStr"/>
-      <c r="J109" t="inlineStr"/>
-      <c r="K109" t="inlineStr"/>
-      <c r="L109" t="inlineStr"/>
-      <c r="M109" t="inlineStr"/>
-      <c r="N109" t="inlineStr"/>
-      <c r="O109" t="inlineStr"/>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=oJESb0W2J3A</t>
+        </is>
+      </c>
+      <c r="J109" t="n">
+        <v>27424</v>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>アニプレックス チャンネル</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=oJESb0W2J3A</t>
+        </is>
+      </c>
+      <c r="M109" t="n">
+        <v>27424</v>
+      </c>
+      <c r="N109" t="inlineStr">
+        <is>
+          <t>アニプレックス チャンネル</t>
+        </is>
+      </c>
+      <c r="O109" t="inlineStr">
+        <is>
+          <t>2026-10-11T09:07:06</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -21008,19 +21148,29 @@
         </is>
       </c>
       <c r="J115" t="n">
-        <v>5278875</v>
+        <v>5292069</v>
       </c>
       <c r="K115" t="inlineStr">
         <is>
           <t>Sizuk / Shunryu</t>
         </is>
       </c>
-      <c r="L115" t="inlineStr"/>
-      <c r="M115" t="inlineStr"/>
-      <c r="N115" t="inlineStr"/>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=P0Mk5q_Vjbo</t>
+        </is>
+      </c>
+      <c r="M115" t="n">
+        <v>28441</v>
+      </c>
+      <c r="N115" t="inlineStr">
+        <is>
+          <t>TBSアニメ</t>
+        </is>
+      </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>2026-10-03T09:10:49</t>
+          <t>2026-10-11T09:07:18</t>
         </is>
       </c>
     </row>
@@ -21065,19 +21215,29 @@
         </is>
       </c>
       <c r="J116" t="n">
-        <v>999112</v>
+        <v>1001704</v>
       </c>
       <c r="K116" t="inlineStr">
         <is>
           <t>内田真礼（UCHIDA MAAYA）Official Channel</t>
         </is>
       </c>
-      <c r="L116" t="inlineStr"/>
-      <c r="M116" t="inlineStr"/>
-      <c r="N116" t="inlineStr"/>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=V73Kz89G1HA</t>
+        </is>
+      </c>
+      <c r="M116" t="n">
+        <v>19991</v>
+      </c>
+      <c r="N116" t="inlineStr">
+        <is>
+          <t>TBSアニメ</t>
+        </is>
+      </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>2026-10-03T09:11:04</t>
+          <t>2026-10-11T09:07:28</t>
         </is>
       </c>
     </row>
@@ -21118,33 +21278,33 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
+          <t>https://www.youtube.com/watch?v=PtBmc0oFIx4</t>
         </is>
       </c>
       <c r="J117" t="n">
-        <v>11081</v>
+        <v>1949671</v>
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>Anime Trailer アニメ</t>
+          <t>テレ東アニメ</t>
         </is>
       </c>
       <c r="L117" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
+          <t>https://www.youtube.com/watch?v=PtBmc0oFIx4</t>
         </is>
       </c>
       <c r="M117" t="n">
-        <v>11081</v>
+        <v>1949671</v>
       </c>
       <c r="N117" t="inlineStr">
         <is>
-          <t>Anime Trailer アニメ</t>
+          <t>テレ東アニメ</t>
         </is>
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>2026-10-03T09:11:13</t>
+          <t>2026-10-11T09:07:39</t>
         </is>
       </c>
     </row>
@@ -21252,11 +21412,11 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=HvcYTLw9HiE</t>
+          <t>https://www.youtube.com/watch?v=6bPTWRJibJU</t>
         </is>
       </c>
       <c r="J119" t="n">
-        <v>56915</v>
+        <v>127896</v>
       </c>
       <c r="K119" t="inlineStr">
         <is>
@@ -21265,11 +21425,11 @@
       </c>
       <c r="L119" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=HvcYTLw9HiE</t>
+          <t>https://www.youtube.com/watch?v=6bPTWRJibJU</t>
         </is>
       </c>
       <c r="M119" t="n">
-        <v>56915</v>
+        <v>127896</v>
       </c>
       <c r="N119" t="inlineStr">
         <is>
@@ -21278,7 +21438,7 @@
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>2026-10-03T09:11:29</t>
+          <t>2026-10-11T09:07:49</t>
         </is>
       </c>
     </row>
@@ -21319,11 +21479,11 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=HvcYTLw9HiE</t>
+          <t>https://www.youtube.com/watch?v=6bPTWRJibJU</t>
         </is>
       </c>
       <c r="J120" t="n">
-        <v>56907</v>
+        <v>127896</v>
       </c>
       <c r="K120" t="inlineStr">
         <is>
@@ -21332,11 +21492,11 @@
       </c>
       <c r="L120" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=OOsNusJNFlM</t>
+          <t>https://www.youtube.com/watch?v=fxKLvhf3qto</t>
         </is>
       </c>
       <c r="M120" t="n">
-        <v>18057</v>
+        <v>57396</v>
       </c>
       <c r="N120" t="inlineStr">
         <is>
@@ -21345,7 +21505,7 @@
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>2026-10-03T09:11:38</t>
+          <t>2026-10-11T09:07:58</t>
         </is>
       </c>
     </row>
@@ -21866,13 +22026,37 @@
           <t>十明</t>
         </is>
       </c>
-      <c r="I129" t="inlineStr"/>
-      <c r="J129" t="inlineStr"/>
-      <c r="K129" t="inlineStr"/>
-      <c r="L129" t="inlineStr"/>
-      <c r="M129" t="inlineStr"/>
-      <c r="N129" t="inlineStr"/>
-      <c r="O129" t="inlineStr"/>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=eyps2lFMx18</t>
+        </is>
+      </c>
+      <c r="J129" t="n">
+        <v>337772</v>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>TMSアニメ公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=eyps2lFMx18</t>
+        </is>
+      </c>
+      <c r="M129" t="n">
+        <v>337772</v>
+      </c>
+      <c r="N129" t="inlineStr">
+        <is>
+          <t>TMSアニメ公式チャンネル</t>
+        </is>
+      </c>
+      <c r="O129" t="inlineStr">
+        <is>
+          <t>2026-10-11T09:08:12</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -21954,11 +22138,11 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=-PX7FqZ55tE</t>
+          <t>https://www.youtube.com/watch?v=iD1hmEvGQmM</t>
         </is>
       </c>
       <c r="J131" t="n">
-        <v>115737</v>
+        <v>133038</v>
       </c>
       <c r="K131" t="inlineStr">
         <is>
@@ -21970,7 +22154,7 @@
       <c r="N131" t="inlineStr"/>
       <c r="O131" t="inlineStr">
         <is>
-          <t>2026-10-03T09:12:50</t>
+          <t>2026-10-11T09:08:32</t>
         </is>
       </c>
     </row>
@@ -22015,7 +22199,7 @@
         </is>
       </c>
       <c r="J132" t="n">
-        <v>112781</v>
+        <v>133038</v>
       </c>
       <c r="K132" t="inlineStr">
         <is>
@@ -22027,7 +22211,7 @@
       <c r="N132" t="inlineStr"/>
       <c r="O132" t="inlineStr">
         <is>
-          <t>2026-10-03T09:13:05</t>
+          <t>2026-10-11T09:08:49</t>
         </is>
       </c>
     </row>
@@ -22139,7 +22323,7 @@
         </is>
       </c>
       <c r="J134" t="n">
-        <v>333264</v>
+        <v>341950</v>
       </c>
       <c r="K134" t="inlineStr">
         <is>
@@ -22152,7 +22336,7 @@
         </is>
       </c>
       <c r="M134" t="n">
-        <v>333264</v>
+        <v>341950</v>
       </c>
       <c r="N134" t="inlineStr">
         <is>
@@ -22161,7 +22345,7 @@
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>2026-10-03T09:13:14</t>
+          <t>2026-10-11T09:08:59</t>
         </is>
       </c>
     </row>
@@ -22666,11 +22850,11 @@
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=clLABf_c_wI</t>
+          <t>https://www.youtube.com/watch?v=i7XLEFdGMYU</t>
         </is>
       </c>
       <c r="J143" t="n">
-        <v>4207</v>
+        <v>87762</v>
       </c>
       <c r="K143" t="inlineStr">
         <is>
@@ -22679,11 +22863,11 @@
       </c>
       <c r="L143" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=clLABf_c_wI</t>
+          <t>https://www.youtube.com/watch?v=i7XLEFdGMYU</t>
         </is>
       </c>
       <c r="M143" t="n">
-        <v>4207</v>
+        <v>87762</v>
       </c>
       <c r="N143" t="inlineStr">
         <is>
@@ -22692,7 +22876,7 @@
       </c>
       <c r="O143" t="inlineStr">
         <is>
-          <t>2026-10-03T09:13:50</t>
+          <t>2026-10-11T09:09:12</t>
         </is>
       </c>
     </row>
@@ -22737,7 +22921,7 @@
         </is>
       </c>
       <c r="J144" t="n">
-        <v>3945</v>
+        <v>4088</v>
       </c>
       <c r="K144" t="inlineStr">
         <is>
@@ -22750,7 +22934,7 @@
         </is>
       </c>
       <c r="M144" t="n">
-        <v>3945</v>
+        <v>4088</v>
       </c>
       <c r="N144" t="inlineStr">
         <is>
@@ -22759,7 +22943,7 @@
       </c>
       <c r="O144" t="inlineStr">
         <is>
-          <t>2026-10-03T09:13:59</t>
+          <t>2026-10-11T09:09:27</t>
         </is>
       </c>
     </row>
@@ -22914,7 +23098,7 @@
         </is>
       </c>
       <c r="J147" t="n">
-        <v>1221145</v>
+        <v>1254010</v>
       </c>
       <c r="K147" t="inlineStr">
         <is>
@@ -22927,7 +23111,7 @@
         </is>
       </c>
       <c r="M147" t="n">
-        <v>451055</v>
+        <v>459312</v>
       </c>
       <c r="N147" t="inlineStr">
         <is>
@@ -22936,7 +23120,7 @@
       </c>
       <c r="O147" t="inlineStr">
         <is>
-          <t>2026-10-03T09:14:17</t>
+          <t>2026-10-11T09:09:44</t>
         </is>
       </c>
     </row>
@@ -23024,7 +23208,7 @@
         </is>
       </c>
       <c r="J149" t="n">
-        <v>523453</v>
+        <v>536152</v>
       </c>
       <c r="K149" t="inlineStr">
         <is>
@@ -23037,7 +23221,7 @@
         </is>
       </c>
       <c r="M149" t="n">
-        <v>446544</v>
+        <v>453607</v>
       </c>
       <c r="N149" t="inlineStr">
         <is>
@@ -23046,7 +23230,7 @@
       </c>
       <c r="O149" t="inlineStr">
         <is>
-          <t>2026-10-03T09:14:34</t>
+          <t>2026-10-11T09:10:02</t>
         </is>
       </c>
     </row>
@@ -23201,7 +23385,7 @@
         </is>
       </c>
       <c r="J152" t="n">
-        <v>280662</v>
+        <v>282585</v>
       </c>
       <c r="K152" t="inlineStr">
         <is>
@@ -23214,7 +23398,7 @@
         </is>
       </c>
       <c r="M152" t="n">
-        <v>280662</v>
+        <v>282585</v>
       </c>
       <c r="N152" t="inlineStr">
         <is>
@@ -23223,7 +23407,7 @@
       </c>
       <c r="O152" t="inlineStr">
         <is>
-          <t>2026-10-03T09:14:59</t>
+          <t>2026-10-11T09:10:18</t>
         </is>
       </c>
     </row>
@@ -23268,7 +23452,7 @@
         </is>
       </c>
       <c r="J153" t="n">
-        <v>70474</v>
+        <v>284414</v>
       </c>
       <c r="K153" t="inlineStr">
         <is>
@@ -23281,7 +23465,7 @@
         </is>
       </c>
       <c r="M153" t="n">
-        <v>70474</v>
+        <v>284414</v>
       </c>
       <c r="N153" t="inlineStr">
         <is>
@@ -23290,7 +23474,7 @@
       </c>
       <c r="O153" t="inlineStr">
         <is>
-          <t>2026-10-04T09:10:15</t>
+          <t>2026-10-11T09:10:29</t>
         </is>
       </c>
     </row>
@@ -23626,7 +23810,7 @@
         </is>
       </c>
       <c r="J159" t="n">
-        <v>232215</v>
+        <v>237134</v>
       </c>
       <c r="K159" t="inlineStr">
         <is>
@@ -23639,7 +23823,7 @@
         </is>
       </c>
       <c r="M159" t="n">
-        <v>232215</v>
+        <v>237134</v>
       </c>
       <c r="N159" t="inlineStr">
         <is>
@@ -23648,7 +23832,7 @@
       </c>
       <c r="O159" t="inlineStr">
         <is>
-          <t>2026-10-03T09:15:19</t>
+          <t>2026-10-11T09:10:40</t>
         </is>
       </c>
     </row>
@@ -23736,7 +23920,7 @@
         </is>
       </c>
       <c r="J161" t="n">
-        <v>9067279</v>
+        <v>9145226</v>
       </c>
       <c r="K161" t="inlineStr">
         <is>
@@ -23748,7 +23932,7 @@
       <c r="N161" t="inlineStr"/>
       <c r="O161" t="inlineStr">
         <is>
-          <t>2026-10-03T09:15:54</t>
+          <t>2026-10-11T09:11:13</t>
         </is>
       </c>
     </row>
@@ -23965,7 +24149,7 @@
         </is>
       </c>
       <c r="J166" t="n">
-        <v>196635</v>
+        <v>210673</v>
       </c>
       <c r="K166" t="inlineStr">
         <is>
@@ -23978,7 +24162,7 @@
         </is>
       </c>
       <c r="M166" t="n">
-        <v>196635</v>
+        <v>210673</v>
       </c>
       <c r="N166" t="inlineStr">
         <is>
@@ -23987,7 +24171,7 @@
       </c>
       <c r="O166" t="inlineStr">
         <is>
-          <t>2026-10-03T09:16:17</t>
+          <t>2026-10-11T09:11:43</t>
         </is>
       </c>
     </row>
@@ -24032,7 +24216,7 @@
         </is>
       </c>
       <c r="J167" t="n">
-        <v>278269</v>
+        <v>290598</v>
       </c>
       <c r="K167" t="inlineStr">
         <is>
@@ -24044,7 +24228,7 @@
       <c r="N167" t="inlineStr"/>
       <c r="O167" t="inlineStr">
         <is>
-          <t>2026-10-03T09:16:42</t>
+          <t>2026-10-11T09:12:08</t>
         </is>
       </c>
     </row>
@@ -24085,7 +24269,7 @@
         </is>
       </c>
       <c r="J168" t="n">
-        <v>424334</v>
+        <v>466516</v>
       </c>
       <c r="K168" t="inlineStr">
         <is>
@@ -24097,7 +24281,7 @@
       <c r="N168" t="inlineStr"/>
       <c r="O168" t="inlineStr">
         <is>
-          <t>2026-10-03T09:17:07</t>
+          <t>2026-10-11T09:12:34</t>
         </is>
       </c>
     </row>
@@ -24228,7 +24412,7 @@
         </is>
       </c>
       <c r="J171" t="n">
-        <v>75923</v>
+        <v>77893</v>
       </c>
       <c r="K171" t="inlineStr">
         <is>
@@ -24241,7 +24425,7 @@
         </is>
       </c>
       <c r="M171" t="n">
-        <v>75923</v>
+        <v>77893</v>
       </c>
       <c r="N171" t="inlineStr">
         <is>
@@ -24250,7 +24434,7 @@
       </c>
       <c r="O171" t="inlineStr">
         <is>
-          <t>2026-10-03T09:17:21</t>
+          <t>2026-10-11T09:12:52</t>
         </is>
       </c>
     </row>
@@ -24424,7 +24608,7 @@
         </is>
       </c>
       <c r="J175" t="n">
-        <v>232219</v>
+        <v>237134</v>
       </c>
       <c r="K175" t="inlineStr">
         <is>
@@ -24437,7 +24621,7 @@
         </is>
       </c>
       <c r="M175" t="n">
-        <v>232219</v>
+        <v>237134</v>
       </c>
       <c r="N175" t="inlineStr">
         <is>
@@ -24446,7 +24630,7 @@
       </c>
       <c r="O175" t="inlineStr">
         <is>
-          <t>2026-10-03T09:17:31</t>
+          <t>2026-10-11T09:13:05</t>
         </is>
       </c>
     </row>
@@ -24816,7 +25000,7 @@
         </is>
       </c>
       <c r="J183" t="n">
-        <v>228874</v>
+        <v>229750</v>
       </c>
       <c r="K183" t="inlineStr">
         <is>
@@ -24828,7 +25012,7 @@
       <c r="N183" t="inlineStr"/>
       <c r="O183" t="inlineStr">
         <is>
-          <t>2026-10-03T09:18:01</t>
+          <t>2026-10-11T09:13:35</t>
         </is>
       </c>
     </row>
@@ -24916,7 +25100,7 @@
         </is>
       </c>
       <c r="J185" t="n">
-        <v>649870</v>
+        <v>655104</v>
       </c>
       <c r="K185" t="inlineStr">
         <is>
@@ -24928,7 +25112,7 @@
       <c r="N185" t="inlineStr"/>
       <c r="O185" t="inlineStr">
         <is>
-          <t>2026-10-03T09:18:33</t>
+          <t>2026-10-11T09:14:09</t>
         </is>
       </c>
     </row>
@@ -24973,7 +25157,7 @@
         </is>
       </c>
       <c r="J186" t="n">
-        <v>1053582</v>
+        <v>1056625</v>
       </c>
       <c r="K186" t="inlineStr">
         <is>
@@ -24985,7 +25169,7 @@
       <c r="N186" t="inlineStr"/>
       <c r="O186" t="inlineStr">
         <is>
-          <t>2026-10-03T09:19:02</t>
+          <t>2026-10-11T09:14:38</t>
         </is>
       </c>
     </row>
@@ -25159,7 +25343,7 @@
         </is>
       </c>
       <c r="J190" t="n">
-        <v>80028</v>
+        <v>83045</v>
       </c>
       <c r="K190" t="inlineStr">
         <is>
@@ -25172,7 +25356,7 @@
         </is>
       </c>
       <c r="M190" t="n">
-        <v>80028</v>
+        <v>83045</v>
       </c>
       <c r="N190" t="inlineStr">
         <is>
@@ -25181,7 +25365,7 @@
       </c>
       <c r="O190" t="inlineStr">
         <is>
-          <t>2026-10-03T09:19:20</t>
+          <t>2026-10-11T09:14:57</t>
         </is>
       </c>
     </row>
@@ -25226,7 +25410,7 @@
         </is>
       </c>
       <c r="J191" t="n">
-        <v>74388</v>
+        <v>76414</v>
       </c>
       <c r="K191" t="inlineStr">
         <is>
@@ -25239,7 +25423,7 @@
         </is>
       </c>
       <c r="M191" t="n">
-        <v>74388</v>
+        <v>76414</v>
       </c>
       <c r="N191" t="inlineStr">
         <is>
@@ -25248,7 +25432,7 @@
       </c>
       <c r="O191" t="inlineStr">
         <is>
-          <t>2026-10-03T09:19:28</t>
+          <t>2026-10-11T09:15:05</t>
         </is>
       </c>
     </row>
@@ -25289,11 +25473,11 @@
       </c>
       <c r="I192" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=jaKESlyUmWI</t>
+          <t>https://www.youtube.com/watch?v=L9_KqJJwniE</t>
         </is>
       </c>
       <c r="J192" t="n">
-        <v>3338879</v>
+        <v>2229998</v>
       </c>
       <c r="K192" t="inlineStr">
         <is>
@@ -25306,7 +25490,7 @@
         </is>
       </c>
       <c r="M192" t="n">
-        <v>129295</v>
+        <v>131192</v>
       </c>
       <c r="N192" t="inlineStr">
         <is>
@@ -25315,7 +25499,7 @@
       </c>
       <c r="O192" t="inlineStr">
         <is>
-          <t>2026-10-03T09:19:38</t>
+          <t>2026-10-11T09:15:15</t>
         </is>
       </c>
     </row>
@@ -25360,7 +25544,7 @@
         </is>
       </c>
       <c r="J193" t="n">
-        <v>362012689</v>
+        <v>363421063</v>
       </c>
       <c r="K193" t="inlineStr">
         <is>
@@ -25372,7 +25556,7 @@
       <c r="N193" t="inlineStr"/>
       <c r="O193" t="inlineStr">
         <is>
-          <t>2026-10-03T09:19:57</t>
+          <t>2026-10-11T09:15:35</t>
         </is>
       </c>
     </row>
@@ -25460,7 +25644,7 @@
         </is>
       </c>
       <c r="J195" t="n">
-        <v>108567</v>
+        <v>108573</v>
       </c>
       <c r="K195" t="inlineStr">
         <is>
@@ -25473,7 +25657,7 @@
         </is>
       </c>
       <c r="M195" t="n">
-        <v>108567</v>
+        <v>108573</v>
       </c>
       <c r="N195" t="inlineStr">
         <is>
@@ -25482,7 +25666,7 @@
       </c>
       <c r="O195" t="inlineStr">
         <is>
-          <t>2026-10-03T09:20:17</t>
+          <t>2026-10-11T09:15:53</t>
         </is>
       </c>
     </row>
@@ -25652,11 +25836,11 @@
       </c>
       <c r="I199" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=VD_ztcqWBAY</t>
+          <t>https://www.youtube.com/watch?v=bqigIHMComE</t>
         </is>
       </c>
       <c r="J199" t="n">
-        <v>4332258</v>
+        <v>28642451</v>
       </c>
       <c r="K199" t="inlineStr">
         <is>
@@ -25669,7 +25853,7 @@
         </is>
       </c>
       <c r="M199" t="n">
-        <v>12561447</v>
+        <v>12609575</v>
       </c>
       <c r="N199" t="inlineStr">
         <is>
@@ -25678,7 +25862,7 @@
       </c>
       <c r="O199" t="inlineStr">
         <is>
-          <t>2026-10-03T09:20:47</t>
+          <t>2026-10-11T09:16:22</t>
         </is>
       </c>
     </row>
@@ -25723,7 +25907,7 @@
         </is>
       </c>
       <c r="J200" t="n">
-        <v>5151990</v>
+        <v>5165659</v>
       </c>
       <c r="K200" t="inlineStr">
         <is>
@@ -25735,7 +25919,7 @@
       <c r="N200" t="inlineStr"/>
       <c r="O200" t="inlineStr">
         <is>
-          <t>2026-10-03T09:21:16</t>
+          <t>2026-10-11T09:16:50</t>
         </is>
       </c>
     </row>
@@ -25780,7 +25964,7 @@
         </is>
       </c>
       <c r="J201" t="n">
-        <v>44592</v>
+        <v>45009</v>
       </c>
       <c r="K201" t="inlineStr">
         <is>
@@ -25793,7 +25977,7 @@
         </is>
       </c>
       <c r="M201" t="n">
-        <v>44592</v>
+        <v>45009</v>
       </c>
       <c r="N201" t="inlineStr">
         <is>
@@ -25802,7 +25986,7 @@
       </c>
       <c r="O201" t="inlineStr">
         <is>
-          <t>2026-10-03T09:21:20</t>
+          <t>2026-10-11T09:16:54</t>
         </is>
       </c>
     </row>
@@ -25847,7 +26031,7 @@
         </is>
       </c>
       <c r="J202" t="n">
-        <v>6030017</v>
+        <v>6188918</v>
       </c>
       <c r="K202" t="inlineStr">
         <is>
@@ -25859,7 +26043,7 @@
       <c r="N202" t="inlineStr"/>
       <c r="O202" t="inlineStr">
         <is>
-          <t>2026-10-03T09:21:51</t>
+          <t>2026-10-11T09:17:23</t>
         </is>
       </c>
     </row>
@@ -25904,7 +26088,7 @@
         </is>
       </c>
       <c r="J203" t="n">
-        <v>273700</v>
+        <v>279008</v>
       </c>
       <c r="K203" t="inlineStr">
         <is>
@@ -25916,7 +26100,7 @@
       <c r="N203" t="inlineStr"/>
       <c r="O203" t="inlineStr">
         <is>
-          <t>2026-10-03T09:22:14</t>
+          <t>2026-10-11T09:17:47</t>
         </is>
       </c>
     </row>
@@ -26047,7 +26231,7 @@
         </is>
       </c>
       <c r="J206" t="n">
-        <v>222587</v>
+        <v>229372</v>
       </c>
       <c r="K206" t="inlineStr">
         <is>
@@ -26059,7 +26243,7 @@
       <c r="N206" t="inlineStr"/>
       <c r="O206" t="inlineStr">
         <is>
-          <t>2026-10-03T09:22:40</t>
+          <t>2026-10-11T09:18:12</t>
         </is>
       </c>
     </row>
@@ -26104,7 +26288,7 @@
         </is>
       </c>
       <c r="J207" t="n">
-        <v>3755900</v>
+        <v>3767636</v>
       </c>
       <c r="K207" t="inlineStr">
         <is>
@@ -26117,7 +26301,7 @@
         </is>
       </c>
       <c r="M207" t="n">
-        <v>523479</v>
+        <v>523954</v>
       </c>
       <c r="N207" t="inlineStr">
         <is>
@@ -26126,7 +26310,7 @@
       </c>
       <c r="O207" t="inlineStr">
         <is>
-          <t>2026-10-03T09:22:49</t>
+          <t>2026-10-11T09:18:21</t>
         </is>
       </c>
     </row>
@@ -26171,7 +26355,7 @@
         </is>
       </c>
       <c r="J208" t="n">
-        <v>223548</v>
+        <v>225124</v>
       </c>
       <c r="K208" t="inlineStr">
         <is>
@@ -26183,7 +26367,7 @@
       <c r="N208" t="inlineStr"/>
       <c r="O208" t="inlineStr">
         <is>
-          <t>2026-10-03T09:23:04</t>
+          <t>2026-10-11T09:18:37</t>
         </is>
       </c>
     </row>
@@ -26271,7 +26455,7 @@
         </is>
       </c>
       <c r="J210" t="n">
-        <v>1268092</v>
+        <v>1275975</v>
       </c>
       <c r="K210" t="inlineStr">
         <is>
@@ -26284,7 +26468,7 @@
         </is>
       </c>
       <c r="M210" t="n">
-        <v>793640</v>
+        <v>805775</v>
       </c>
       <c r="N210" t="inlineStr">
         <is>
@@ -26293,7 +26477,7 @@
       </c>
       <c r="O210" t="inlineStr">
         <is>
-          <t>2026-10-03T09:23:13</t>
+          <t>2026-10-11T09:18:46</t>
         </is>
       </c>
     </row>
@@ -26682,7 +26866,7 @@
         </is>
       </c>
       <c r="J219" t="n">
-        <v>334807</v>
+        <v>335958</v>
       </c>
       <c r="K219" t="inlineStr">
         <is>
@@ -26694,7 +26878,7 @@
       <c r="N219" t="inlineStr"/>
       <c r="O219" t="inlineStr">
         <is>
-          <t>2026-10-03T09:24:05</t>
+          <t>2026-10-11T09:19:40</t>
         </is>
       </c>
     </row>
@@ -26739,7 +26923,7 @@
         </is>
       </c>
       <c r="J220" t="n">
-        <v>7410759</v>
+        <v>7497421</v>
       </c>
       <c r="K220" t="inlineStr">
         <is>
@@ -26752,7 +26936,7 @@
         </is>
       </c>
       <c r="M220" t="n">
-        <v>522850</v>
+        <v>533270</v>
       </c>
       <c r="N220" t="inlineStr">
         <is>
@@ -26761,7 +26945,7 @@
       </c>
       <c r="O220" t="inlineStr">
         <is>
-          <t>2026-10-03T09:24:26</t>
+          <t>2026-10-11T09:19:59</t>
         </is>
       </c>
     </row>
@@ -26806,7 +26990,7 @@
         </is>
       </c>
       <c r="J221" t="n">
-        <v>419886</v>
+        <v>428469</v>
       </c>
       <c r="K221" t="inlineStr">
         <is>
@@ -26819,7 +27003,7 @@
         </is>
       </c>
       <c r="M221" t="n">
-        <v>1540046</v>
+        <v>1553317</v>
       </c>
       <c r="N221" t="inlineStr">
         <is>
@@ -26828,7 +27012,7 @@
       </c>
       <c r="O221" t="inlineStr">
         <is>
-          <t>2026-10-03T09:24:40</t>
+          <t>2026-10-11T09:20:15</t>
         </is>
       </c>
     </row>
@@ -26959,7 +27143,7 @@
         </is>
       </c>
       <c r="J224" t="n">
-        <v>228874</v>
+        <v>229750</v>
       </c>
       <c r="K224" t="inlineStr">
         <is>
@@ -26971,7 +27155,7 @@
       <c r="N224" t="inlineStr"/>
       <c r="O224" t="inlineStr">
         <is>
-          <t>2026-10-03T09:24:55</t>
+          <t>2026-10-11T09:20:39</t>
         </is>
       </c>
     </row>
@@ -27571,7 +27755,7 @@
         </is>
       </c>
       <c r="J238" t="n">
-        <v>1688947</v>
+        <v>1717541</v>
       </c>
       <c r="K238" t="inlineStr">
         <is>
@@ -27584,7 +27768,7 @@
         </is>
       </c>
       <c r="M238" t="n">
-        <v>804810</v>
+        <v>840753</v>
       </c>
       <c r="N238" t="inlineStr">
         <is>
@@ -27593,7 +27777,7 @@
       </c>
       <c r="O238" t="inlineStr">
         <is>
-          <t>2026-10-03T09:26:30</t>
+          <t>2026-10-11T09:22:15</t>
         </is>
       </c>
     </row>
@@ -27638,7 +27822,7 @@
         </is>
       </c>
       <c r="J239" t="n">
-        <v>1688947</v>
+        <v>1717541</v>
       </c>
       <c r="K239" t="inlineStr">
         <is>
@@ -27651,7 +27835,7 @@
         </is>
       </c>
       <c r="M239" t="n">
-        <v>804810</v>
+        <v>840753</v>
       </c>
       <c r="N239" t="inlineStr">
         <is>
@@ -27660,7 +27844,7 @@
       </c>
       <c r="O239" t="inlineStr">
         <is>
-          <t>2026-10-03T09:26:40</t>
+          <t>2026-10-11T09:22:25</t>
         </is>
       </c>
     </row>
@@ -27744,33 +27928,33 @@
       </c>
       <c r="I241" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/watch?v=j-6s1L3MIbI</t>
+        </is>
+      </c>
+      <c r="J241" t="n">
+        <v>1381759</v>
+      </c>
+      <c r="K241" t="inlineStr">
+        <is>
+          <t>timelesz</t>
+        </is>
+      </c>
+      <c r="L241" t="inlineStr">
+        <is>
           <t>https://www.youtube.com/watch?v=TY8BNUB43Y8</t>
         </is>
       </c>
-      <c r="J241" t="n">
-        <v>400165</v>
-      </c>
-      <c r="K241" t="inlineStr">
+      <c r="M241" t="n">
+        <v>431609</v>
+      </c>
+      <c r="N241" t="inlineStr">
         <is>
           <t>SHOCHIKU anime Channel</t>
         </is>
       </c>
-      <c r="L241" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=TY8BNUB43Y8</t>
-        </is>
-      </c>
-      <c r="M241" t="n">
-        <v>400165</v>
-      </c>
-      <c r="N241" t="inlineStr">
-        <is>
-          <t>SHOCHIKU anime Channel</t>
-        </is>
-      </c>
       <c r="O241" t="inlineStr">
         <is>
-          <t>2026-10-03T09:26:49</t>
+          <t>2026-10-11T09:22:36</t>
         </is>
       </c>
     </row>
@@ -27858,7 +28042,7 @@
         </is>
       </c>
       <c r="J243" t="n">
-        <v>3052428</v>
+        <v>3256375</v>
       </c>
       <c r="K243" t="inlineStr">
         <is>
@@ -27871,7 +28055,7 @@
         </is>
       </c>
       <c r="M243" t="n">
-        <v>3052428</v>
+        <v>3256375</v>
       </c>
       <c r="N243" t="inlineStr">
         <is>
@@ -27880,7 +28064,7 @@
       </c>
       <c r="O243" t="inlineStr">
         <is>
-          <t>2026-10-03T09:27:08</t>
+          <t>2026-10-11T09:22:57</t>
         </is>
       </c>
     </row>
@@ -27968,7 +28152,7 @@
         </is>
       </c>
       <c r="J245" t="n">
-        <v>1815678</v>
+        <v>1902936</v>
       </c>
       <c r="K245" t="inlineStr">
         <is>
@@ -27980,7 +28164,7 @@
       <c r="N245" t="inlineStr"/>
       <c r="O245" t="inlineStr">
         <is>
-          <t>2026-10-03T09:27:33</t>
+          <t>2026-10-11T09:23:33</t>
         </is>
       </c>
     </row>
@@ -28111,7 +28295,7 @@
         </is>
       </c>
       <c r="J248" t="n">
-        <v>1072033</v>
+        <v>1086918</v>
       </c>
       <c r="K248" t="inlineStr">
         <is>
@@ -28123,7 +28307,7 @@
       <c r="N248" t="inlineStr"/>
       <c r="O248" t="inlineStr">
         <is>
-          <t>2026-10-03T09:27:55</t>
+          <t>2026-10-11T09:23:56</t>
         </is>
       </c>
     </row>
@@ -28168,7 +28352,7 @@
         </is>
       </c>
       <c r="J249" t="n">
-        <v>228874</v>
+        <v>229750</v>
       </c>
       <c r="K249" t="inlineStr">
         <is>
@@ -28180,7 +28364,7 @@
       <c r="N249" t="inlineStr"/>
       <c r="O249" t="inlineStr">
         <is>
-          <t>2026-10-03T09:28:09</t>
+          <t>2026-10-11T09:24:11</t>
         </is>
       </c>
     </row>
@@ -28521,7 +28705,7 @@
         </is>
       </c>
       <c r="J256" t="n">
-        <v>419886</v>
+        <v>428469</v>
       </c>
       <c r="K256" t="inlineStr">
         <is>
@@ -28534,7 +28718,7 @@
         </is>
       </c>
       <c r="M256" t="n">
-        <v>1540046</v>
+        <v>1553390</v>
       </c>
       <c r="N256" t="inlineStr">
         <is>
@@ -28543,7 +28727,7 @@
       </c>
       <c r="O256" t="inlineStr">
         <is>
-          <t>2026-10-03T09:28:52</t>
+          <t>2026-10-11T09:24:46</t>
         </is>
       </c>
     </row>
@@ -28631,7 +28815,7 @@
         </is>
       </c>
       <c r="J258" t="n">
-        <v>4393</v>
+        <v>6409</v>
       </c>
       <c r="K258" t="inlineStr">
         <is>
@@ -28643,7 +28827,7 @@
       <c r="N258" t="inlineStr"/>
       <c r="O258" t="inlineStr">
         <is>
-          <t>2026-10-03T09:29:24</t>
+          <t>2026-10-11T09:25:24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-10-12
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M290"/>
+  <dimension ref="A1:M291"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14510,6 +14510,51 @@
       <c r="M290" t="inlineStr">
         <is>
           <t>https://anilist.co/anime/216623</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="n">
+        <v>-190244</v>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>2027冬アニメ</t>
+        </is>
+      </c>
+      <c r="C291" t="n">
+        <v>0</v>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>デート・ア・ライブF Last Date</t>
+        </is>
+      </c>
+      <c r="E291" t="b">
+        <v>0</v>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>2027年3月26日</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>Fugaku</t>
+        </is>
+      </c>
+      <c r="I291" t="inlineStr"/>
+      <c r="J291" t="inlineStr"/>
+      <c r="K291" t="inlineStr"/>
+      <c r="L291" t="inlineStr"/>
+      <c r="M291" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/190244</t>
         </is>
       </c>
     </row>
@@ -15074,37 +15119,13 @@
           <t>エルスウェア紀行</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=8B3d4x0m7n4</t>
-        </is>
-      </c>
-      <c r="J11" t="n">
-        <v>56736</v>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>TMSアニメ公式チャンネル</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=8B3d4x0m7n4</t>
-        </is>
-      </c>
-      <c r="M11" t="n">
-        <v>56736</v>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>TMSアニメ公式チャンネル</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>2026-10-05T09:00:56</t>
-        </is>
-      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -15275,37 +15296,13 @@
           <t>福賀くるみ（CV：鈴木愛奈）</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=OiQo6YyJ_pM</t>
-        </is>
-      </c>
-      <c r="J14" t="n">
-        <v>754993</v>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=OiQo6YyJ_pM</t>
-        </is>
-      </c>
-      <c r="M14" t="n">
-        <v>754993</v>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>2026-10-05T09:01:05</t>
-        </is>
-      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -15495,37 +15492,13 @@
           <t>BUDDiiS</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=R5veWbUAM-I</t>
-        </is>
-      </c>
-      <c r="J18" t="n">
-        <v>5114</v>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>tv asahi  animation YouTubeチャンネル</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=R5veWbUAM-I</t>
-        </is>
-      </c>
-      <c r="M18" t="n">
-        <v>5114</v>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>tv asahi  animation YouTubeチャンネル</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>2026-10-04T09:01:22</t>
-        </is>
-      </c>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -15562,37 +15535,13 @@
           <t>こたに</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=gYZJcSSnAVY</t>
-        </is>
-      </c>
-      <c r="J19" t="n">
-        <v>3019</v>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>tv asahi  animation YouTubeチャンネル</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=gYZJcSSnAVY</t>
-        </is>
-      </c>
-      <c r="M19" t="n">
-        <v>3019</v>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>tv asahi  animation YouTubeチャンネル</t>
-        </is>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>2026-10-04T09:01:31</t>
-        </is>
-      </c>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -15796,37 +15745,13 @@
           <t>Ceui</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=By3eIjul98c</t>
-        </is>
-      </c>
-      <c r="J23" t="n">
-        <v>2655</v>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>デレギュラ【新アニメレーベル】</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=By3eIjul98c</t>
-        </is>
-      </c>
-      <c r="M23" t="n">
-        <v>2655</v>
-      </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>デレギュラ【新アニメレーベル】</t>
-        </is>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>2026-10-05T09:01:43</t>
-        </is>
-      </c>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -16040,37 +15965,13 @@
           <t>Juice=Juice</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=y8dxEBdlISk</t>
-        </is>
-      </c>
-      <c r="J27" t="n">
-        <v>93031</v>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>Juice=Juice</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=y8dxEBdlISk</t>
-        </is>
-      </c>
-      <c r="M27" t="n">
-        <v>93031</v>
-      </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>Juice=Juice</t>
-        </is>
-      </c>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t>2026-10-04T09:02:21</t>
-        </is>
-      </c>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -16681,37 +16582,13 @@
           <t>Koji Nakamura</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=2mkPF8PO4GY</t>
-        </is>
-      </c>
-      <c r="J38" t="n">
-        <v>12269</v>
-      </c>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>NBCUniversal Anime/Music</t>
-        </is>
-      </c>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=2mkPF8PO4GY</t>
-        </is>
-      </c>
-      <c r="M38" t="n">
-        <v>12269</v>
-      </c>
-      <c r="N38" t="inlineStr">
-        <is>
-          <t>NBCUniversal Anime/Music</t>
-        </is>
-      </c>
-      <c r="O38" t="inlineStr">
-        <is>
-          <t>2026-10-05T09:02:41</t>
-        </is>
-      </c>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -16949,37 +16826,13 @@
           <t>CLAN QUEEN</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=Uitds6Ysj08</t>
-        </is>
-      </c>
-      <c r="J42" t="n">
-        <v>1</v>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>Zuax anime and music</t>
-        </is>
-      </c>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=Uitds6Ysj08</t>
-        </is>
-      </c>
-      <c r="M42" t="n">
-        <v>1</v>
-      </c>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>Zuax anime and music</t>
-        </is>
-      </c>
-      <c r="O42" t="inlineStr">
-        <is>
-          <t>2026-10-05T09:02:58</t>
-        </is>
-      </c>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -17977,37 +17830,13 @@
           <t>すりぃ</t>
         </is>
       </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=zhK-ugQnTgA</t>
-        </is>
-      </c>
-      <c r="J60" t="n">
-        <v>18568</v>
-      </c>
-      <c r="K60" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="L60" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=zhK-ugQnTgA</t>
-        </is>
-      </c>
-      <c r="M60" t="n">
-        <v>18568</v>
-      </c>
-      <c r="N60" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="O60" t="inlineStr">
-        <is>
-          <t>2026-10-04T09:04:24</t>
-        </is>
-      </c>
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr"/>
+      <c r="N60" t="inlineStr"/>
+      <c r="O60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -19488,37 +19317,13 @@
           <t>佐々木李子</t>
         </is>
       </c>
-      <c r="I87" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=-LQfgkvHY8k</t>
-        </is>
-      </c>
-      <c r="J87" t="n">
-        <v>48794</v>
-      </c>
-      <c r="K87" t="inlineStr">
-        <is>
-          <t>isekai channel @バンダイナムコフィルムワークス</t>
-        </is>
-      </c>
-      <c r="L87" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=-LQfgkvHY8k</t>
-        </is>
-      </c>
-      <c r="M87" t="n">
-        <v>48794</v>
-      </c>
-      <c r="N87" t="inlineStr">
-        <is>
-          <t>isekai channel @バンダイナムコフィルムワークス</t>
-        </is>
-      </c>
-      <c r="O87" t="inlineStr">
-        <is>
-          <t>2026-10-04T09:06:02</t>
-        </is>
-      </c>
+      <c r="I87" t="inlineStr"/>
+      <c r="J87" t="inlineStr"/>
+      <c r="K87" t="inlineStr"/>
+      <c r="L87" t="inlineStr"/>
+      <c r="M87" t="inlineStr"/>
+      <c r="N87" t="inlineStr"/>
+      <c r="O87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -19708,37 +19513,13 @@
           <t>花耶</t>
         </is>
       </c>
-      <c r="I91" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=Zh22JniyJy4</t>
-        </is>
-      </c>
-      <c r="J91" t="n">
-        <v>4393</v>
-      </c>
-      <c r="K91" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Kaya Official YouTube Channel </t>
-        </is>
-      </c>
-      <c r="L91" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=lP8RbpwGUO8</t>
-        </is>
-      </c>
-      <c r="M91" t="n">
-        <v>8293</v>
-      </c>
-      <c r="N91" t="inlineStr">
-        <is>
-          <t>博報堂DY ミュージック&amp;ピクチャーズ【Showgate】ch</t>
-        </is>
-      </c>
-      <c r="O91" t="inlineStr">
-        <is>
-          <t>2026-10-04T09:06:24</t>
-        </is>
-      </c>
+      <c r="I91" t="inlineStr"/>
+      <c r="J91" t="inlineStr"/>
+      <c r="K91" t="inlineStr"/>
+      <c r="L91" t="inlineStr"/>
+      <c r="M91" t="inlineStr"/>
+      <c r="N91" t="inlineStr"/>
+      <c r="O91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -20965,37 +20746,13 @@
           <t>パンどろぼうとパンやのおじさん（CV：朝井彩加とCV：諏訪部順一）</t>
         </is>
       </c>
-      <c r="I112" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=Z2fmYtMNi-o</t>
-        </is>
-      </c>
-      <c r="J112" t="n">
-        <v>281584</v>
-      </c>
-      <c r="K112" t="inlineStr">
-        <is>
-          <t>パンどろぼう / PANDOROBO【公式】</t>
-        </is>
-      </c>
-      <c r="L112" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=jz7Jqz6SYzk</t>
-        </is>
-      </c>
-      <c r="M112" t="n">
-        <v>44037</v>
-      </c>
-      <c r="N112" t="inlineStr">
-        <is>
-          <t>パンどろぼう / PANDOROBO【公式】</t>
-        </is>
-      </c>
-      <c r="O112" t="inlineStr">
-        <is>
-          <t>2026-10-04T09:07:44</t>
-        </is>
-      </c>
+      <c r="I112" t="inlineStr"/>
+      <c r="J112" t="inlineStr"/>
+      <c r="K112" t="inlineStr"/>
+      <c r="L112" t="inlineStr"/>
+      <c r="M112" t="inlineStr"/>
+      <c r="N112" t="inlineStr"/>
+      <c r="O112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -21032,37 +20789,13 @@
           <t>きゃりーぱみゅぱみゅ</t>
         </is>
       </c>
-      <c r="I113" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=Z2fmYtMNi-o</t>
-        </is>
-      </c>
-      <c r="J113" t="n">
-        <v>281584</v>
-      </c>
-      <c r="K113" t="inlineStr">
-        <is>
-          <t>パンどろぼう / PANDOROBO【公式】</t>
-        </is>
-      </c>
-      <c r="L113" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=oUDFr8Ktaxs</t>
-        </is>
-      </c>
-      <c r="M113" t="n">
-        <v>135608</v>
-      </c>
-      <c r="N113" t="inlineStr">
-        <is>
-          <t>パンどろぼう / PANDOROBO【公式】</t>
-        </is>
-      </c>
-      <c r="O113" t="inlineStr">
-        <is>
-          <t>2026-10-04T09:07:53</t>
-        </is>
-      </c>
+      <c r="I113" t="inlineStr"/>
+      <c r="J113" t="inlineStr"/>
+      <c r="K113" t="inlineStr"/>
+      <c r="L113" t="inlineStr"/>
+      <c r="M113" t="inlineStr"/>
+      <c r="N113" t="inlineStr"/>
+      <c r="O113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -21343,37 +21076,13 @@
           <t>ONE OR EIGHT</t>
         </is>
       </c>
-      <c r="I118" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=umzOm3846cA</t>
-        </is>
-      </c>
-      <c r="J118" t="n">
-        <v>113007</v>
-      </c>
-      <c r="K118" t="inlineStr">
-        <is>
-          <t>テレ東アニメ</t>
-        </is>
-      </c>
-      <c r="L118" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=umzOm3846cA</t>
-        </is>
-      </c>
-      <c r="M118" t="n">
-        <v>113007</v>
-      </c>
-      <c r="N118" t="inlineStr">
-        <is>
-          <t>テレ東アニメ</t>
-        </is>
-      </c>
-      <c r="O118" t="inlineStr">
-        <is>
-          <t>2026-10-04T09:08:06</t>
-        </is>
-      </c>
+      <c r="I118" t="inlineStr"/>
+      <c r="J118" t="inlineStr"/>
+      <c r="K118" t="inlineStr"/>
+      <c r="L118" t="inlineStr"/>
+      <c r="M118" t="inlineStr"/>
+      <c r="N118" t="inlineStr"/>
+      <c r="O118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -21544,37 +21253,13 @@
           <t>宮﨑歩・谷本貴義</t>
         </is>
       </c>
-      <c r="I121" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=uqIOdbe7rtI</t>
-        </is>
-      </c>
-      <c r="J121" t="n">
-        <v>284752</v>
-      </c>
-      <c r="K121" t="inlineStr">
-        <is>
-          <t>Digimon Official Channel</t>
-        </is>
-      </c>
-      <c r="L121" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=uqIOdbe7rtI</t>
-        </is>
-      </c>
-      <c r="M121" t="n">
-        <v>284752</v>
-      </c>
-      <c r="N121" t="inlineStr">
-        <is>
-          <t>Digimon Official Channel</t>
-        </is>
-      </c>
-      <c r="O121" t="inlineStr">
-        <is>
-          <t>2026-10-05T09:07:06</t>
-        </is>
-      </c>
+      <c r="I121" t="inlineStr"/>
+      <c r="J121" t="inlineStr"/>
+      <c r="K121" t="inlineStr"/>
+      <c r="L121" t="inlineStr"/>
+      <c r="M121" t="inlineStr"/>
+      <c r="N121" t="inlineStr"/>
+      <c r="O121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -21611,37 +21296,13 @@
           <t>宮﨑歩・谷本貴義</t>
         </is>
       </c>
-      <c r="I122" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=irjWjYsfVk0</t>
-        </is>
-      </c>
-      <c r="J122" t="n">
-        <v>79492</v>
-      </c>
-      <c r="K122" t="inlineStr">
-        <is>
-          <t>Digimon Official Channel</t>
-        </is>
-      </c>
-      <c r="L122" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=irjWjYsfVk0</t>
-        </is>
-      </c>
-      <c r="M122" t="n">
-        <v>79492</v>
-      </c>
-      <c r="N122" t="inlineStr">
-        <is>
-          <t>Digimon Official Channel</t>
-        </is>
-      </c>
-      <c r="O122" t="inlineStr">
-        <is>
-          <t>2026-10-05T09:07:09</t>
-        </is>
-      </c>
+      <c r="I122" t="inlineStr"/>
+      <c r="J122" t="inlineStr"/>
+      <c r="K122" t="inlineStr"/>
+      <c r="L122" t="inlineStr"/>
+      <c r="M122" t="inlineStr"/>
+      <c r="N122" t="inlineStr"/>
+      <c r="O122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -21678,27 +21339,13 @@
           <t>TOOBOE</t>
         </is>
       </c>
-      <c r="I123" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=TE3McAbD7DA</t>
-        </is>
-      </c>
-      <c r="J123" t="n">
-        <v>827599</v>
-      </c>
-      <c r="K123" t="inlineStr">
-        <is>
-          <t>john / TOOBOE</t>
-        </is>
-      </c>
+      <c r="I123" t="inlineStr"/>
+      <c r="J123" t="inlineStr"/>
+      <c r="K123" t="inlineStr"/>
       <c r="L123" t="inlineStr"/>
       <c r="M123" t="inlineStr"/>
       <c r="N123" t="inlineStr"/>
-      <c r="O123" t="inlineStr">
-        <is>
-          <t>2026-10-04T09:08:29</t>
-        </is>
-      </c>
+      <c r="O123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -21735,37 +21382,13 @@
           <t>GAN（岩田剛典）</t>
         </is>
       </c>
-      <c r="I124" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=3MFyyGVajvA</t>
-        </is>
-      </c>
-      <c r="J124" t="n">
-        <v>4136</v>
-      </c>
-      <c r="K124" t="inlineStr">
-        <is>
-          <t>テレ東アニメ</t>
-        </is>
-      </c>
-      <c r="L124" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=3MFyyGVajvA</t>
-        </is>
-      </c>
-      <c r="M124" t="n">
-        <v>4136</v>
-      </c>
-      <c r="N124" t="inlineStr">
-        <is>
-          <t>テレ東アニメ</t>
-        </is>
-      </c>
-      <c r="O124" t="inlineStr">
-        <is>
-          <t>2026-10-05T09:07:16</t>
-        </is>
-      </c>
+      <c r="I124" t="inlineStr"/>
+      <c r="J124" t="inlineStr"/>
+      <c r="K124" t="inlineStr"/>
+      <c r="L124" t="inlineStr"/>
+      <c r="M124" t="inlineStr"/>
+      <c r="N124" t="inlineStr"/>
+      <c r="O124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -21802,37 +21425,13 @@
           <t>ファントムシータ</t>
         </is>
       </c>
-      <c r="I125" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=BUxVzKyGrsw</t>
-        </is>
-      </c>
-      <c r="J125" t="n">
-        <v>5833</v>
-      </c>
-      <c r="K125" t="inlineStr">
-        <is>
-          <t>テレ東アニメ</t>
-        </is>
-      </c>
-      <c r="L125" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=BUxVzKyGrsw</t>
-        </is>
-      </c>
-      <c r="M125" t="n">
-        <v>5833</v>
-      </c>
-      <c r="N125" t="inlineStr">
-        <is>
-          <t>テレ東アニメ</t>
-        </is>
-      </c>
-      <c r="O125" t="inlineStr">
-        <is>
-          <t>2026-10-05T09:07:25</t>
-        </is>
-      </c>
+      <c r="I125" t="inlineStr"/>
+      <c r="J125" t="inlineStr"/>
+      <c r="K125" t="inlineStr"/>
+      <c r="L125" t="inlineStr"/>
+      <c r="M125" t="inlineStr"/>
+      <c r="N125" t="inlineStr"/>
+      <c r="O125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -22494,37 +22093,13 @@
           <t>yama</t>
         </is>
       </c>
-      <c r="I137" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=HYm0nNqk9Aw</t>
-        </is>
-      </c>
-      <c r="J137" t="n">
-        <v>9616</v>
-      </c>
-      <c r="K137" t="inlineStr">
-        <is>
-          <t>NHK ENTERPRISES Animation</t>
-        </is>
-      </c>
-      <c r="L137" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=HYm0nNqk9Aw</t>
-        </is>
-      </c>
-      <c r="M137" t="n">
-        <v>9616</v>
-      </c>
-      <c r="N137" t="inlineStr">
-        <is>
-          <t>NHK ENTERPRISES Animation</t>
-        </is>
-      </c>
-      <c r="O137" t="inlineStr">
-        <is>
-          <t>2026-10-04T09:09:22</t>
-        </is>
-      </c>
+      <c r="I137" t="inlineStr"/>
+      <c r="J137" t="inlineStr"/>
+      <c r="K137" t="inlineStr"/>
+      <c r="L137" t="inlineStr"/>
+      <c r="M137" t="inlineStr"/>
+      <c r="N137" t="inlineStr"/>
+      <c r="O137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -22628,37 +22203,13 @@
           <t>FLOW</t>
         </is>
       </c>
-      <c r="I139" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=VzCsxgQ_4_M</t>
-        </is>
-      </c>
-      <c r="J139" t="n">
-        <v>37838</v>
-      </c>
-      <c r="K139" t="inlineStr">
-        <is>
-          <t>アニプレックス チャンネル</t>
-        </is>
-      </c>
-      <c r="L139" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=VzCsxgQ_4_M</t>
-        </is>
-      </c>
-      <c r="M139" t="n">
-        <v>37838</v>
-      </c>
-      <c r="N139" t="inlineStr">
-        <is>
-          <t>アニプレックス チャンネル</t>
-        </is>
-      </c>
-      <c r="O139" t="inlineStr">
-        <is>
-          <t>2026-10-05T09:08:06</t>
-        </is>
-      </c>
+      <c r="I139" t="inlineStr"/>
+      <c r="J139" t="inlineStr"/>
+      <c r="K139" t="inlineStr"/>
+      <c r="L139" t="inlineStr"/>
+      <c r="M139" t="inlineStr"/>
+      <c r="N139" t="inlineStr"/>
+      <c r="O139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -22695,37 +22246,13 @@
           <t>ASTERISM</t>
         </is>
       </c>
-      <c r="I140" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=6GDMDhzPctA</t>
-        </is>
-      </c>
-      <c r="J140" t="n">
-        <v>20481</v>
-      </c>
-      <c r="K140" t="inlineStr">
-        <is>
-          <t>アニプレックス チャンネル</t>
-        </is>
-      </c>
-      <c r="L140" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=6GDMDhzPctA</t>
-        </is>
-      </c>
-      <c r="M140" t="n">
-        <v>20481</v>
-      </c>
-      <c r="N140" t="inlineStr">
-        <is>
-          <t>アニプレックス チャンネル</t>
-        </is>
-      </c>
-      <c r="O140" t="inlineStr">
-        <is>
-          <t>2026-10-05T09:08:16</t>
-        </is>
-      </c>
+      <c r="I140" t="inlineStr"/>
+      <c r="J140" t="inlineStr"/>
+      <c r="K140" t="inlineStr"/>
+      <c r="L140" t="inlineStr"/>
+      <c r="M140" t="inlineStr"/>
+      <c r="N140" t="inlineStr"/>
+      <c r="O140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="n">

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-10-13
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -15119,13 +15119,37 @@
           <t>エルスウェア紀行</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=8B3d4x0m7n4</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>147264</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>TMSアニメ公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=8B3d4x0m7n4</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
+        <v>147264</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>TMSアニメ公式チャンネル</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>2026-10-13T09:00:43</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -15296,13 +15320,37 @@
           <t>福賀くるみ（CV：鈴木愛奈）</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=OiQo6YyJ_pM</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>1085780</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=OiQo6YyJ_pM</t>
+        </is>
+      </c>
+      <c r="M14" t="n">
+        <v>1085780</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>2026-10-13T09:00:53</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -15339,13 +15387,37 @@
           <t>八木勇征</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Rtw__04Gzbw</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>8766</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>メテオ・ポラリス公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Rtw__04Gzbw</t>
+        </is>
+      </c>
+      <c r="M15" t="n">
+        <v>8766</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>メテオ・ポラリス公式チャンネル</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>2026-10-13T09:01:03</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -15492,13 +15564,37 @@
           <t>BUDDiiS</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=R5veWbUAM-I</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>42301</v>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>tv asahi  animation YouTubeチャンネル</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=R5veWbUAM-I</t>
+        </is>
+      </c>
+      <c r="M18" t="n">
+        <v>42301</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>tv asahi  animation YouTubeチャンネル</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>2026-10-13T09:01:18</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -15535,13 +15631,37 @@
           <t>こたに</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=gYZJcSSnAVY</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>18642</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>tv asahi  animation YouTubeチャンネル</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=gYZJcSSnAVY</t>
+        </is>
+      </c>
+      <c r="M19" t="n">
+        <v>18642</v>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>tv asahi  animation YouTubeチャンネル</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>2026-10-13T09:01:30</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -15641,7 +15761,7 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>19315</v>
+        <v>96551</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -15654,7 +15774,7 @@
         </is>
       </c>
       <c r="M21" t="n">
-        <v>19315</v>
+        <v>96551</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
@@ -15663,7 +15783,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>2026-10-06T09:01:19</t>
+          <t>2026-10-13T09:01:40</t>
         </is>
       </c>
     </row>
@@ -15745,13 +15865,37 @@
           <t>Ceui</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=By3eIjul98c</t>
+        </is>
+      </c>
+      <c r="J23" t="n">
+        <v>14710</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>デレギュラ【新アニメレーベル】</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=By3eIjul98c</t>
+        </is>
+      </c>
+      <c r="M23" t="n">
+        <v>14710</v>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>デレギュラ【新アニメレーベル】</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>2026-10-13T09:01:48</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -15965,13 +16109,37 @@
           <t>Juice=Juice</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=y8dxEBdlISk</t>
+        </is>
+      </c>
+      <c r="J27" t="n">
+        <v>195870</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Juice=Juice</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=y8dxEBdlISk</t>
+        </is>
+      </c>
+      <c r="M27" t="n">
+        <v>195870</v>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>Juice=Juice</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>2026-10-13T09:02:05</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -16472,13 +16640,37 @@
           <t>PURPLE BUBBLE</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=A8b6GHtgpWI</t>
+        </is>
+      </c>
+      <c r="J36" t="n">
+        <v>75212</v>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>【公式】ケロロチャンネル</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=A8b6GHtgpWI</t>
+        </is>
+      </c>
+      <c r="M36" t="n">
+        <v>75212</v>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>【公式】ケロロチャンネル</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>2026-10-13T09:02:24</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -16582,13 +16774,37 @@
           <t>Koji Nakamura</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr"/>
-      <c r="O38" t="inlineStr"/>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=2mkPF8PO4GY</t>
+        </is>
+      </c>
+      <c r="J38" t="n">
+        <v>34069</v>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=2mkPF8PO4GY</t>
+        </is>
+      </c>
+      <c r="M38" t="n">
+        <v>34069</v>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>2026-10-13T09:02:33</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -16826,13 +17042,37 @@
           <t>CLAN QUEEN</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr"/>
-      <c r="O42" t="inlineStr"/>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=gk3f0vgTkFw</t>
+        </is>
+      </c>
+      <c r="J42" t="n">
+        <v>230</v>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Anime Melodies</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=gk3f0vgTkFw</t>
+        </is>
+      </c>
+      <c r="M42" t="n">
+        <v>230</v>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>Anime Melodies</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>2026-10-13T09:02:40</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -17830,13 +18070,37 @@
           <t>すりぃ</t>
         </is>
       </c>
-      <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr"/>
-      <c r="M60" t="inlineStr"/>
-      <c r="N60" t="inlineStr"/>
-      <c r="O60" t="inlineStr"/>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zhK-ugQnTgA</t>
+        </is>
+      </c>
+      <c r="J60" t="n">
+        <v>44960</v>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zhK-ugQnTgA</t>
+        </is>
+      </c>
+      <c r="M60" t="n">
+        <v>44960</v>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>2026-10-13T09:03:23</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -19317,13 +19581,37 @@
           <t>佐々木李子</t>
         </is>
       </c>
-      <c r="I87" t="inlineStr"/>
-      <c r="J87" t="inlineStr"/>
-      <c r="K87" t="inlineStr"/>
-      <c r="L87" t="inlineStr"/>
-      <c r="M87" t="inlineStr"/>
-      <c r="N87" t="inlineStr"/>
-      <c r="O87" t="inlineStr"/>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-LQfgkvHY8k</t>
+        </is>
+      </c>
+      <c r="J87" t="n">
+        <v>192870</v>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>isekai channel @バンダイナムコフィルムワークス</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-LQfgkvHY8k</t>
+        </is>
+      </c>
+      <c r="M87" t="n">
+        <v>192870</v>
+      </c>
+      <c r="N87" t="inlineStr">
+        <is>
+          <t>isekai channel @バンダイナムコフィルムワークス</t>
+        </is>
+      </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>2026-10-13T09:04:25</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -19513,13 +19801,37 @@
           <t>花耶</t>
         </is>
       </c>
-      <c r="I91" t="inlineStr"/>
-      <c r="J91" t="inlineStr"/>
-      <c r="K91" t="inlineStr"/>
-      <c r="L91" t="inlineStr"/>
-      <c r="M91" t="inlineStr"/>
-      <c r="N91" t="inlineStr"/>
-      <c r="O91" t="inlineStr"/>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Zh22JniyJy4</t>
+        </is>
+      </c>
+      <c r="J91" t="n">
+        <v>32250</v>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kaya Official YouTube Channel </t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=lP8RbpwGUO8</t>
+        </is>
+      </c>
+      <c r="M91" t="n">
+        <v>44714</v>
+      </c>
+      <c r="N91" t="inlineStr">
+        <is>
+          <t>博報堂DY ミュージック&amp;ピクチャーズ【Showgate】ch</t>
+        </is>
+      </c>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>2026-10-13T09:04:48</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -20746,13 +21058,37 @@
           <t>パンどろぼうとパンやのおじさん（CV：朝井彩加とCV：諏訪部順一）</t>
         </is>
       </c>
-      <c r="I112" t="inlineStr"/>
-      <c r="J112" t="inlineStr"/>
-      <c r="K112" t="inlineStr"/>
-      <c r="L112" t="inlineStr"/>
-      <c r="M112" t="inlineStr"/>
-      <c r="N112" t="inlineStr"/>
-      <c r="O112" t="inlineStr"/>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=oUDFr8Ktaxs</t>
+        </is>
+      </c>
+      <c r="J112" t="n">
+        <v>405409</v>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>パンどろぼう / PANDOROBO【公式】</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=jz7Jqz6SYzk</t>
+        </is>
+      </c>
+      <c r="M112" t="n">
+        <v>226750</v>
+      </c>
+      <c r="N112" t="inlineStr">
+        <is>
+          <t>パンどろぼう / PANDOROBO【公式】</t>
+        </is>
+      </c>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>2026-10-13T09:05:25</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -20789,13 +21125,37 @@
           <t>きゃりーぱみゅぱみゅ</t>
         </is>
       </c>
-      <c r="I113" t="inlineStr"/>
-      <c r="J113" t="inlineStr"/>
-      <c r="K113" t="inlineStr"/>
-      <c r="L113" t="inlineStr"/>
-      <c r="M113" t="inlineStr"/>
-      <c r="N113" t="inlineStr"/>
-      <c r="O113" t="inlineStr"/>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=oUDFr8Ktaxs</t>
+        </is>
+      </c>
+      <c r="J113" t="n">
+        <v>405409</v>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>パンどろぼう / PANDOROBO【公式】</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=oUDFr8Ktaxs</t>
+        </is>
+      </c>
+      <c r="M113" t="n">
+        <v>405409</v>
+      </c>
+      <c r="N113" t="inlineStr">
+        <is>
+          <t>パンどろぼう / PANDOROBO【公式】</t>
+        </is>
+      </c>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>2026-10-13T09:05:34</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -21076,13 +21436,37 @@
           <t>ONE OR EIGHT</t>
         </is>
       </c>
-      <c r="I118" t="inlineStr"/>
-      <c r="J118" t="inlineStr"/>
-      <c r="K118" t="inlineStr"/>
-      <c r="L118" t="inlineStr"/>
-      <c r="M118" t="inlineStr"/>
-      <c r="N118" t="inlineStr"/>
-      <c r="O118" t="inlineStr"/>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=umzOm3846cA</t>
+        </is>
+      </c>
+      <c r="J118" t="n">
+        <v>464787</v>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>テレ東アニメ</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=umzOm3846cA</t>
+        </is>
+      </c>
+      <c r="M118" t="n">
+        <v>464787</v>
+      </c>
+      <c r="N118" t="inlineStr">
+        <is>
+          <t>テレ東アニメ</t>
+        </is>
+      </c>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t>2026-10-13T09:05:48</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -21253,13 +21637,37 @@
           <t>宮﨑歩・谷本貴義</t>
         </is>
       </c>
-      <c r="I121" t="inlineStr"/>
-      <c r="J121" t="inlineStr"/>
-      <c r="K121" t="inlineStr"/>
-      <c r="L121" t="inlineStr"/>
-      <c r="M121" t="inlineStr"/>
-      <c r="N121" t="inlineStr"/>
-      <c r="O121" t="inlineStr"/>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=uqIOdbe7rtI</t>
+        </is>
+      </c>
+      <c r="J121" t="n">
+        <v>518845</v>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>Digimon Official Channel</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=uqIOdbe7rtI</t>
+        </is>
+      </c>
+      <c r="M121" t="n">
+        <v>518845</v>
+      </c>
+      <c r="N121" t="inlineStr">
+        <is>
+          <t>Digimon Official Channel</t>
+        </is>
+      </c>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>2026-10-13T09:05:54</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -21296,13 +21704,37 @@
           <t>宮﨑歩・谷本貴義</t>
         </is>
       </c>
-      <c r="I122" t="inlineStr"/>
-      <c r="J122" t="inlineStr"/>
-      <c r="K122" t="inlineStr"/>
-      <c r="L122" t="inlineStr"/>
-      <c r="M122" t="inlineStr"/>
-      <c r="N122" t="inlineStr"/>
-      <c r="O122" t="inlineStr"/>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=uqIOdbe7rtI</t>
+        </is>
+      </c>
+      <c r="J122" t="n">
+        <v>518845</v>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>Digimon Official Channel</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=uqIOdbe7rtI</t>
+        </is>
+      </c>
+      <c r="M122" t="n">
+        <v>518845</v>
+      </c>
+      <c r="N122" t="inlineStr">
+        <is>
+          <t>Digimon Official Channel</t>
+        </is>
+      </c>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>2026-10-13T09:06:00</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -21339,13 +21771,37 @@
           <t>TOOBOE</t>
         </is>
       </c>
-      <c r="I123" t="inlineStr"/>
-      <c r="J123" t="inlineStr"/>
-      <c r="K123" t="inlineStr"/>
-      <c r="L123" t="inlineStr"/>
-      <c r="M123" t="inlineStr"/>
-      <c r="N123" t="inlineStr"/>
-      <c r="O123" t="inlineStr"/>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=IqJEHa3PLCQ</t>
+        </is>
+      </c>
+      <c r="J123" t="n">
+        <v>112501</v>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>【フジテレビ】アニメ公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=IqJEHa3PLCQ</t>
+        </is>
+      </c>
+      <c r="M123" t="n">
+        <v>112501</v>
+      </c>
+      <c r="N123" t="inlineStr">
+        <is>
+          <t>【フジテレビ】アニメ公式チャンネル</t>
+        </is>
+      </c>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t>2026-10-13T09:06:09</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -21382,13 +21838,37 @@
           <t>GAN（岩田剛典）</t>
         </is>
       </c>
-      <c r="I124" t="inlineStr"/>
-      <c r="J124" t="inlineStr"/>
-      <c r="K124" t="inlineStr"/>
-      <c r="L124" t="inlineStr"/>
-      <c r="M124" t="inlineStr"/>
-      <c r="N124" t="inlineStr"/>
-      <c r="O124" t="inlineStr"/>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=3MFyyGVajvA</t>
+        </is>
+      </c>
+      <c r="J124" t="n">
+        <v>15528</v>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>テレ東アニメ</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=3MFyyGVajvA</t>
+        </is>
+      </c>
+      <c r="M124" t="n">
+        <v>15528</v>
+      </c>
+      <c r="N124" t="inlineStr">
+        <is>
+          <t>テレ東アニメ</t>
+        </is>
+      </c>
+      <c r="O124" t="inlineStr">
+        <is>
+          <t>2026-10-13T09:06:17</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -21425,13 +21905,37 @@
           <t>ファントムシータ</t>
         </is>
       </c>
-      <c r="I125" t="inlineStr"/>
-      <c r="J125" t="inlineStr"/>
-      <c r="K125" t="inlineStr"/>
-      <c r="L125" t="inlineStr"/>
-      <c r="M125" t="inlineStr"/>
-      <c r="N125" t="inlineStr"/>
-      <c r="O125" t="inlineStr"/>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=BUxVzKyGrsw</t>
+        </is>
+      </c>
+      <c r="J125" t="n">
+        <v>35662</v>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>テレ東アニメ</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=BUxVzKyGrsw</t>
+        </is>
+      </c>
+      <c r="M125" t="n">
+        <v>35662</v>
+      </c>
+      <c r="N125" t="inlineStr">
+        <is>
+          <t>テレ東アニメ</t>
+        </is>
+      </c>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>2026-10-13T09:06:26</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -22093,13 +22597,37 @@
           <t>yama</t>
         </is>
       </c>
-      <c r="I137" t="inlineStr"/>
-      <c r="J137" t="inlineStr"/>
-      <c r="K137" t="inlineStr"/>
-      <c r="L137" t="inlineStr"/>
-      <c r="M137" t="inlineStr"/>
-      <c r="N137" t="inlineStr"/>
-      <c r="O137" t="inlineStr"/>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=0Ldh_MWIIFk</t>
+        </is>
+      </c>
+      <c r="J137" t="n">
+        <v>58362</v>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>yama</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=HYm0nNqk9Aw</t>
+        </is>
+      </c>
+      <c r="M137" t="n">
+        <v>46749</v>
+      </c>
+      <c r="N137" t="inlineStr">
+        <is>
+          <t>NHK ENTERPRISES Animation</t>
+        </is>
+      </c>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>2026-10-13T09:06:43</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -22203,13 +22731,37 @@
           <t>FLOW</t>
         </is>
       </c>
-      <c r="I139" t="inlineStr"/>
-      <c r="J139" t="inlineStr"/>
-      <c r="K139" t="inlineStr"/>
-      <c r="L139" t="inlineStr"/>
-      <c r="M139" t="inlineStr"/>
-      <c r="N139" t="inlineStr"/>
-      <c r="O139" t="inlineStr"/>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=VzCsxgQ_4_M</t>
+        </is>
+      </c>
+      <c r="J139" t="n">
+        <v>111910</v>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>アニプレックス チャンネル</t>
+        </is>
+      </c>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=VzCsxgQ_4_M</t>
+        </is>
+      </c>
+      <c r="M139" t="n">
+        <v>111910</v>
+      </c>
+      <c r="N139" t="inlineStr">
+        <is>
+          <t>アニプレックス チャンネル</t>
+        </is>
+      </c>
+      <c r="O139" t="inlineStr">
+        <is>
+          <t>2026-10-13T09:06:53</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -22246,13 +22798,37 @@
           <t>ASTERISM</t>
         </is>
       </c>
-      <c r="I140" t="inlineStr"/>
-      <c r="J140" t="inlineStr"/>
-      <c r="K140" t="inlineStr"/>
-      <c r="L140" t="inlineStr"/>
-      <c r="M140" t="inlineStr"/>
-      <c r="N140" t="inlineStr"/>
-      <c r="O140" t="inlineStr"/>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=6GDMDhzPctA</t>
+        </is>
+      </c>
+      <c r="J140" t="n">
+        <v>40974</v>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>アニプレックス チャンネル</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=6GDMDhzPctA</t>
+        </is>
+      </c>
+      <c r="M140" t="n">
+        <v>40974</v>
+      </c>
+      <c r="N140" t="inlineStr">
+        <is>
+          <t>アニプレックス チャンネル</t>
+        </is>
+      </c>
+      <c r="O140" t="inlineStr">
+        <is>
+          <t>2026-10-13T09:07:02</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -22686,13 +23262,37 @@
           <t>ハンブレッダーズ</t>
         </is>
       </c>
-      <c r="I148" t="inlineStr"/>
-      <c r="J148" t="inlineStr"/>
-      <c r="K148" t="inlineStr"/>
-      <c r="L148" t="inlineStr"/>
-      <c r="M148" t="inlineStr"/>
-      <c r="N148" t="inlineStr"/>
-      <c r="O148" t="inlineStr"/>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=f7QJtQL-LFU</t>
+        </is>
+      </c>
+      <c r="J148" t="n">
+        <v>1964349</v>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=f7QJtQL-LFU</t>
+        </is>
+      </c>
+      <c r="M148" t="n">
+        <v>1964349</v>
+      </c>
+      <c r="N148" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>2026-10-13T09:07:18</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -23584,13 +24184,27 @@
           <t>milet</t>
         </is>
       </c>
-      <c r="I164" t="inlineStr"/>
-      <c r="J164" t="inlineStr"/>
-      <c r="K164" t="inlineStr"/>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=nR_vqhD2rGM</t>
+        </is>
+      </c>
+      <c r="J164" t="n">
+        <v>814119</v>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>TOHO animation</t>
+        </is>
+      </c>
       <c r="L164" t="inlineStr"/>
       <c r="M164" t="inlineStr"/>
       <c r="N164" t="inlineStr"/>
-      <c r="O164" t="inlineStr"/>
+      <c r="O164" t="inlineStr">
+        <is>
+          <t>2026-10-13T09:08:06</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="n">

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-10-18
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M297"/>
+  <dimension ref="A1:M299"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14743,7 +14743,7 @@
     </row>
     <row r="295">
       <c r="A295" t="n">
-        <v>-206298</v>
+        <v>-213814</v>
       </c>
       <c r="B295" t="inlineStr">
         <is>
@@ -14755,7 +14755,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>劇場版 メダリスト</t>
+          <t>アイカツスターズ！ ～星々のProgress～</t>
         </is>
       </c>
       <c r="E295" t="b">
@@ -14768,12 +14768,12 @@
       </c>
       <c r="G295" t="inlineStr">
         <is>
-          <t>2027年2月19日</t>
+          <t>2027年1月22日</t>
         </is>
       </c>
       <c r="H295" t="inlineStr">
         <is>
-          <t>ENGI</t>
+          <t>Bandai Namco Pictures</t>
         </is>
       </c>
       <c r="I295" t="inlineStr"/>
@@ -14782,13 +14782,13 @@
       <c r="L295" t="inlineStr"/>
       <c r="M295" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/206298</t>
+          <t>https://anilist.co/anime/213814</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="n">
-        <v>-216623</v>
+        <v>-186603</v>
       </c>
       <c r="B296" t="inlineStr">
         <is>
@@ -14800,7 +14800,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>ドラえもん のび太の蒸気時間車</t>
+          <t>ラブライブ！虹ヶ咲学園スクールアイドル同好会 完結編 最終章</t>
         </is>
       </c>
       <c r="E296" t="b">
@@ -14813,12 +14813,12 @@
       </c>
       <c r="G296" t="inlineStr">
         <is>
-          <t>2027年3月5日</t>
+          <t>2027年2月5日</t>
         </is>
       </c>
       <c r="H296" t="inlineStr">
         <is>
-          <t>Shin-Ei Animation</t>
+          <t>Sunrise</t>
         </is>
       </c>
       <c r="I296" t="inlineStr"/>
@@ -14827,13 +14827,13 @@
       <c r="L296" t="inlineStr"/>
       <c r="M296" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/216623</t>
+          <t>https://anilist.co/anime/186603</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="n">
-        <v>-190244</v>
+        <v>-206298</v>
       </c>
       <c r="B297" t="inlineStr">
         <is>
@@ -14845,7 +14845,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>デート・ア・ライブF Last Date</t>
+          <t>劇場版 メダリスト</t>
         </is>
       </c>
       <c r="E297" t="b">
@@ -14858,12 +14858,12 @@
       </c>
       <c r="G297" t="inlineStr">
         <is>
-          <t>2027年3月26日</t>
+          <t>2027年2月19日</t>
         </is>
       </c>
       <c r="H297" t="inlineStr">
         <is>
-          <t>Fugaku</t>
+          <t>ENGI</t>
         </is>
       </c>
       <c r="I297" t="inlineStr"/>
@@ -14871,6 +14871,96 @@
       <c r="K297" t="inlineStr"/>
       <c r="L297" t="inlineStr"/>
       <c r="M297" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/206298</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="n">
+        <v>-216623</v>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>2027冬アニメ</t>
+        </is>
+      </c>
+      <c r="C298" t="n">
+        <v>0</v>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>ドラえもん のび太の蒸気時間車</t>
+        </is>
+      </c>
+      <c r="E298" t="b">
+        <v>0</v>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>2027年3月5日</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>Shin-Ei Animation</t>
+        </is>
+      </c>
+      <c r="I298" t="inlineStr"/>
+      <c r="J298" t="inlineStr"/>
+      <c r="K298" t="inlineStr"/>
+      <c r="L298" t="inlineStr"/>
+      <c r="M298" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/216623</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="n">
+        <v>-190244</v>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>2027冬アニメ</t>
+        </is>
+      </c>
+      <c r="C299" t="n">
+        <v>0</v>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>デート・ア・ライブF Last Date</t>
+        </is>
+      </c>
+      <c r="E299" t="b">
+        <v>0</v>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>2027年3月26日</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>Fugaku</t>
+        </is>
+      </c>
+      <c r="I299" t="inlineStr"/>
+      <c r="J299" t="inlineStr"/>
+      <c r="K299" t="inlineStr"/>
+      <c r="L299" t="inlineStr"/>
+      <c r="M299" t="inlineStr">
         <is>
           <t>https://anilist.co/anime/190244</t>
         </is>
@@ -16709,13 +16799,37 @@
           <t>スガシカオ</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=tG7X7oUnbZc</t>
+        </is>
+      </c>
+      <c r="J29" t="n">
+        <v>7690</v>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>NHK ENTERPRISES Animation</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=tG7X7oUnbZc</t>
+        </is>
+      </c>
+      <c r="M29" t="n">
+        <v>7690</v>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>NHK ENTERPRISES Animation</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>2026-10-18T09:00:33</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -18780,13 +18894,37 @@
           <t>BUCK∞TICK</t>
         </is>
       </c>
-      <c r="I64" t="inlineStr"/>
-      <c r="J64" t="inlineStr"/>
-      <c r="K64" t="inlineStr"/>
-      <c r="L64" t="inlineStr"/>
-      <c r="M64" t="inlineStr"/>
-      <c r="N64" t="inlineStr"/>
-      <c r="O64" t="inlineStr"/>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=flcjEA7l9jM</t>
+        </is>
+      </c>
+      <c r="J64" t="n">
+        <v>135144</v>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>【フジテレビ】アニメ公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=flcjEA7l9jM</t>
+        </is>
+      </c>
+      <c r="M64" t="n">
+        <v>135144</v>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>【フジテレビ】アニメ公式チャンネル</t>
+        </is>
+      </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>2026-10-18T09:01:19</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-10-24
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -10228,7 +10228,7 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>1107241</v>
+        <v>1130097</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -10241,7 +10241,7 @@
         </is>
       </c>
       <c r="M2" t="n">
-        <v>861955</v>
+        <v>880592</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
@@ -10250,7 +10250,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>2026-10-16T09:00:24</t>
+          <t>2026-10-24T09:00:26</t>
         </is>
       </c>
     </row>
@@ -10295,7 +10295,7 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>1107241</v>
+        <v>1130097</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -10307,7 +10307,7 @@
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2026-10-16T09:00:49</t>
+          <t>2026-10-24T09:00:51</t>
         </is>
       </c>
     </row>
@@ -10352,7 +10352,7 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>1107241</v>
+        <v>1130097</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -10365,7 +10365,7 @@
         </is>
       </c>
       <c r="M4" t="n">
-        <v>1107241</v>
+        <v>1130097</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
@@ -10374,7 +10374,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-10-16T09:00:54</t>
+          <t>2026-10-24T09:00:57</t>
         </is>
       </c>
     </row>
@@ -10419,29 +10419,19 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>389629</v>
+        <v>395590</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
           <t>アイカツ!チャンネル【公式】</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=1EerxsyYXpw</t>
-        </is>
-      </c>
-      <c r="M5" t="n">
-        <v>269572</v>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>アイカツ!チャンネル【公式】</t>
-        </is>
-      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr">
         <is>
-          <t>2026-10-16T09:01:07</t>
+          <t>2026-10-24T09:01:15</t>
         </is>
       </c>
     </row>
@@ -10620,7 +10610,7 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>5959</v>
+        <v>7890</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -10632,7 +10622,7 @@
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr">
         <is>
-          <t>2026-10-16T09:01:17</t>
+          <t>2026-10-24T09:01:26</t>
         </is>
       </c>
     </row>
@@ -10677,7 +10667,7 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>5959</v>
+        <v>7890</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -10689,7 +10679,7 @@
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr">
         <is>
-          <t>2026-10-16T09:01:27</t>
+          <t>2026-10-24T09:01:36</t>
         </is>
       </c>
     </row>
@@ -10844,7 +10834,7 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>353625</v>
+        <v>377568</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -10857,7 +10847,7 @@
         </is>
       </c>
       <c r="M12" t="n">
-        <v>353625</v>
+        <v>377568</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
@@ -10866,7 +10856,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>2026-10-16T09:01:37</t>
+          <t>2026-10-24T09:01:48</t>
         </is>
       </c>
     </row>
@@ -11356,7 +11346,7 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>3035520</v>
+        <v>3068591</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -11369,7 +11359,7 @@
         </is>
       </c>
       <c r="M20" t="n">
-        <v>111516</v>
+        <v>152531</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
@@ -11378,7 +11368,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026-10-16T09:01:53</t>
+          <t>2026-10-24T09:02:01</t>
         </is>
       </c>
     </row>
@@ -11600,7 +11590,7 @@
         </is>
       </c>
       <c r="J24" t="n">
-        <v>2401569</v>
+        <v>2689290</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
@@ -11613,7 +11603,7 @@
         </is>
       </c>
       <c r="M24" t="n">
-        <v>2401569</v>
+        <v>2689290</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
@@ -11622,7 +11612,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>2026-10-16T09:02:06</t>
+          <t>2026-10-24T09:02:15</t>
         </is>
       </c>
     </row>
@@ -11734,7 +11724,7 @@
         </is>
       </c>
       <c r="J26" t="n">
-        <v>36537</v>
+        <v>55910</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
@@ -11747,7 +11737,7 @@
         </is>
       </c>
       <c r="M26" t="n">
-        <v>36537</v>
+        <v>55910</v>
       </c>
       <c r="N26" t="inlineStr">
         <is>
@@ -11756,7 +11746,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>2026-10-16T09:02:15</t>
+          <t>2026-10-24T09:02:25</t>
         </is>
       </c>
     </row>
@@ -12069,7 +12059,7 @@
         </is>
       </c>
       <c r="J31" t="n">
-        <v>947392</v>
+        <v>1235169</v>
       </c>
       <c r="K31" t="inlineStr">
         <is>
@@ -12082,7 +12072,7 @@
         </is>
       </c>
       <c r="M31" t="n">
-        <v>947392</v>
+        <v>1235169</v>
       </c>
       <c r="N31" t="inlineStr">
         <is>
@@ -12091,7 +12081,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>2026-10-16T09:02:31</t>
+          <t>2026-10-24T09:02:36</t>
         </is>
       </c>
     </row>
@@ -12270,7 +12260,7 @@
         </is>
       </c>
       <c r="J34" t="n">
-        <v>4504690</v>
+        <v>5705635</v>
       </c>
       <c r="K34" t="inlineStr">
         <is>
@@ -12283,7 +12273,7 @@
         </is>
       </c>
       <c r="M34" t="n">
-        <v>1268358</v>
+        <v>1380776</v>
       </c>
       <c r="N34" t="inlineStr">
         <is>
@@ -12292,7 +12282,7 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>2026-10-16T09:02:40</t>
+          <t>2026-10-24T09:02:47</t>
         </is>
       </c>
     </row>
@@ -12423,7 +12413,7 @@
         </is>
       </c>
       <c r="J37" t="n">
-        <v>1729878</v>
+        <v>1745762</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
@@ -12436,7 +12426,7 @@
         </is>
       </c>
       <c r="M37" t="n">
-        <v>407220</v>
+        <v>443884</v>
       </c>
       <c r="N37" t="inlineStr">
         <is>
@@ -12445,7 +12435,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>2026-10-16T09:02:55</t>
+          <t>2026-10-24T09:03:04</t>
         </is>
       </c>
     </row>
@@ -12691,7 +12681,7 @@
         </is>
       </c>
       <c r="J41" t="n">
-        <v>32526</v>
+        <v>33877</v>
       </c>
       <c r="K41" t="inlineStr">
         <is>
@@ -12704,7 +12694,7 @@
         </is>
       </c>
       <c r="M41" t="n">
-        <v>32526</v>
+        <v>33877</v>
       </c>
       <c r="N41" t="inlineStr">
         <is>
@@ -12713,7 +12703,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>2026-10-16T09:03:04</t>
+          <t>2026-10-24T09:03:13</t>
         </is>
       </c>
     </row>
@@ -12758,7 +12748,7 @@
         </is>
       </c>
       <c r="J42" t="n">
-        <v>409843</v>
+        <v>521563</v>
       </c>
       <c r="K42" t="inlineStr">
         <is>
@@ -12771,7 +12761,7 @@
         </is>
       </c>
       <c r="M42" t="n">
-        <v>409843</v>
+        <v>521563</v>
       </c>
       <c r="N42" t="inlineStr">
         <is>
@@ -12780,7 +12770,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>2026-10-16T09:03:14</t>
+          <t>2026-10-24T09:03:23</t>
         </is>
       </c>
     </row>
@@ -12825,7 +12815,7 @@
         </is>
       </c>
       <c r="J43" t="n">
-        <v>240644</v>
+        <v>279346</v>
       </c>
       <c r="K43" t="inlineStr">
         <is>
@@ -12838,7 +12828,7 @@
         </is>
       </c>
       <c r="M43" t="n">
-        <v>240644</v>
+        <v>279346</v>
       </c>
       <c r="N43" t="inlineStr">
         <is>
@@ -12847,7 +12837,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>2026-10-16T09:03:22</t>
+          <t>2026-10-24T09:03:33</t>
         </is>
       </c>
     </row>
@@ -12959,7 +12949,7 @@
         </is>
       </c>
       <c r="J45" t="n">
-        <v>266</v>
+        <v>612</v>
       </c>
       <c r="K45" t="inlineStr">
         <is>
@@ -12972,7 +12962,7 @@
         </is>
       </c>
       <c r="M45" t="n">
-        <v>266</v>
+        <v>612</v>
       </c>
       <c r="N45" t="inlineStr">
         <is>
@@ -12981,7 +12971,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>2026-10-16T09:03:29</t>
+          <t>2026-10-24T09:03:40</t>
         </is>
       </c>
     </row>
@@ -13026,7 +13016,7 @@
         </is>
       </c>
       <c r="J46" t="n">
-        <v>1074325</v>
+        <v>1080444</v>
       </c>
       <c r="K46" t="inlineStr">
         <is>
@@ -13039,7 +13029,7 @@
         </is>
       </c>
       <c r="M46" t="n">
-        <v>132165</v>
+        <v>150310</v>
       </c>
       <c r="N46" t="inlineStr">
         <is>
@@ -13048,7 +13038,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>2026-10-16T09:03:38</t>
+          <t>2026-10-24T09:03:51</t>
         </is>
       </c>
     </row>
@@ -13160,7 +13150,7 @@
         </is>
       </c>
       <c r="J48" t="n">
-        <v>195869</v>
+        <v>227886</v>
       </c>
       <c r="K48" t="inlineStr">
         <is>
@@ -13173,7 +13163,7 @@
         </is>
       </c>
       <c r="M48" t="n">
-        <v>195869</v>
+        <v>227886</v>
       </c>
       <c r="N48" t="inlineStr">
         <is>
@@ -13182,7 +13172,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>2026-10-16T09:03:49</t>
+          <t>2026-10-24T09:04:02</t>
         </is>
       </c>
     </row>
@@ -13490,7 +13480,7 @@
         </is>
       </c>
       <c r="J54" t="n">
-        <v>367327</v>
+        <v>398892</v>
       </c>
       <c r="K54" t="inlineStr">
         <is>
@@ -13503,7 +13493,7 @@
         </is>
       </c>
       <c r="M54" t="n">
-        <v>367327</v>
+        <v>398892</v>
       </c>
       <c r="N54" t="inlineStr">
         <is>
@@ -13512,7 +13502,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>2026-10-16T09:03:58</t>
+          <t>2026-10-24T09:04:19</t>
         </is>
       </c>
     </row>
@@ -13667,19 +13657,29 @@
         </is>
       </c>
       <c r="J57" t="n">
-        <v>9834</v>
+        <v>15779</v>
       </c>
       <c r="K57" t="inlineStr">
         <is>
           <t>Suupeas</t>
         </is>
       </c>
-      <c r="L57" t="inlineStr"/>
-      <c r="M57" t="inlineStr"/>
-      <c r="N57" t="inlineStr"/>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=vEOp-AhraEM</t>
+        </is>
+      </c>
+      <c r="M57" t="n">
+        <v>4844</v>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>博報堂DY ミュージック&amp;ピクチャーズ【Showgate】ch</t>
+        </is>
+      </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>2026-10-16T09:04:30</t>
+          <t>2026-10-24T09:04:47</t>
         </is>
       </c>
     </row>
@@ -14054,7 +14054,7 @@
         </is>
       </c>
       <c r="J64" t="n">
-        <v>119092</v>
+        <v>167392</v>
       </c>
       <c r="K64" t="inlineStr">
         <is>
@@ -14067,7 +14067,7 @@
         </is>
       </c>
       <c r="M64" t="n">
-        <v>119092</v>
+        <v>167392</v>
       </c>
       <c r="N64" t="inlineStr">
         <is>
@@ -14076,7 +14076,7 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>2026-10-16T09:04:43</t>
+          <t>2026-10-24T09:05:03</t>
         </is>
       </c>
     </row>
@@ -14121,7 +14121,7 @@
         </is>
       </c>
       <c r="J65" t="n">
-        <v>1824</v>
+        <v>20205</v>
       </c>
       <c r="K65" t="inlineStr">
         <is>
@@ -14134,7 +14134,7 @@
         </is>
       </c>
       <c r="M65" t="n">
-        <v>1824</v>
+        <v>20205</v>
       </c>
       <c r="N65" t="inlineStr">
         <is>
@@ -14143,7 +14143,7 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>2026-10-16T09:04:53</t>
+          <t>2026-10-24T09:05:13</t>
         </is>
       </c>
     </row>
@@ -14475,7 +14475,7 @@
         </is>
       </c>
       <c r="J71" t="n">
-        <v>13284</v>
+        <v>25758</v>
       </c>
       <c r="K71" t="inlineStr">
         <is>
@@ -14488,7 +14488,7 @@
         </is>
       </c>
       <c r="M71" t="n">
-        <v>13284</v>
+        <v>25758</v>
       </c>
       <c r="N71" t="inlineStr">
         <is>
@@ -14497,7 +14497,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>2026-10-16T09:05:11</t>
+          <t>2026-10-24T09:05:26</t>
         </is>
       </c>
     </row>
@@ -14781,7 +14781,7 @@
         </is>
       </c>
       <c r="J77" t="n">
-        <v>311377</v>
+        <v>352947</v>
       </c>
       <c r="K77" t="inlineStr">
         <is>
@@ -14794,7 +14794,7 @@
         </is>
       </c>
       <c r="M77" t="n">
-        <v>311377</v>
+        <v>352947</v>
       </c>
       <c r="N77" t="inlineStr">
         <is>
@@ -14803,7 +14803,7 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>2026-10-16T09:05:32</t>
+          <t>2026-10-24T09:05:50</t>
         </is>
       </c>
     </row>
@@ -14915,7 +14915,7 @@
         </is>
       </c>
       <c r="J79" t="n">
-        <v>366275</v>
+        <v>419733</v>
       </c>
       <c r="K79" t="inlineStr">
         <is>
@@ -14928,7 +14928,7 @@
         </is>
       </c>
       <c r="M79" t="n">
-        <v>366275</v>
+        <v>419733</v>
       </c>
       <c r="N79" t="inlineStr">
         <is>
@@ -14937,7 +14937,7 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>2026-10-16T09:05:41</t>
+          <t>2026-10-24T09:06:00</t>
         </is>
       </c>
     </row>
@@ -15112,11 +15112,11 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
+          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
         </is>
       </c>
       <c r="J82" t="n">
-        <v>789945</v>
+        <v>452275</v>
       </c>
       <c r="K82" t="inlineStr">
         <is>
@@ -15125,11 +15125,11 @@
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
+          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
         </is>
       </c>
       <c r="M82" t="n">
-        <v>789945</v>
+        <v>452275</v>
       </c>
       <c r="N82" t="inlineStr">
         <is>
@@ -15138,7 +15138,7 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>2026-10-16T09:05:51</t>
+          <t>2026-10-24T09:06:10</t>
         </is>
       </c>
     </row>
@@ -15250,19 +15250,29 @@
         </is>
       </c>
       <c r="J84" t="n">
-        <v>9336</v>
+        <v>27824</v>
       </c>
       <c r="K84" t="inlineStr">
         <is>
           <t>aruma</t>
         </is>
       </c>
-      <c r="L84" t="inlineStr"/>
-      <c r="M84" t="inlineStr"/>
-      <c r="N84" t="inlineStr"/>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=UdXoB5IOFqk</t>
+        </is>
+      </c>
+      <c r="M84" t="n">
+        <v>21972</v>
+      </c>
+      <c r="N84" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>2026-10-16T09:06:06</t>
+          <t>2026-10-24T09:06:21</t>
         </is>
       </c>
     </row>
@@ -15407,7 +15417,7 @@
         </is>
       </c>
       <c r="J87" t="n">
-        <v>58558</v>
+        <v>72177</v>
       </c>
       <c r="K87" t="inlineStr">
         <is>
@@ -15420,7 +15430,7 @@
         </is>
       </c>
       <c r="M87" t="n">
-        <v>58558</v>
+        <v>72177</v>
       </c>
       <c r="N87" t="inlineStr">
         <is>
@@ -15429,7 +15439,7 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>2026-10-16T09:06:34</t>
+          <t>2026-10-24T09:06:41</t>
         </is>
       </c>
     </row>
@@ -15962,7 +15972,7 @@
         </is>
       </c>
       <c r="J96" t="n">
-        <v>203398</v>
+        <v>207084</v>
       </c>
       <c r="K96" t="inlineStr">
         <is>
@@ -15975,7 +15985,7 @@
         </is>
       </c>
       <c r="M96" t="n">
-        <v>203398</v>
+        <v>207084</v>
       </c>
       <c r="N96" t="inlineStr">
         <is>
@@ -15984,7 +15994,7 @@
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t>2026-10-16T09:06:55</t>
+          <t>2026-10-24T09:07:04</t>
         </is>
       </c>
     </row>
@@ -16297,7 +16307,7 @@
         </is>
       </c>
       <c r="J101" t="n">
-        <v>146112</v>
+        <v>178948</v>
       </c>
       <c r="K101" t="inlineStr">
         <is>
@@ -16310,7 +16320,7 @@
         </is>
       </c>
       <c r="M101" t="n">
-        <v>146112</v>
+        <v>178948</v>
       </c>
       <c r="N101" t="inlineStr">
         <is>
@@ -16319,7 +16329,7 @@
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>2026-10-16T09:07:19</t>
+          <t>2026-10-24T09:07:14</t>
         </is>
       </c>
     </row>
@@ -16364,7 +16374,7 @@
         </is>
       </c>
       <c r="J102" t="n">
-        <v>51739</v>
+        <v>64814</v>
       </c>
       <c r="K102" t="inlineStr">
         <is>
@@ -16377,7 +16387,7 @@
         </is>
       </c>
       <c r="M102" t="n">
-        <v>51739</v>
+        <v>64814</v>
       </c>
       <c r="N102" t="inlineStr">
         <is>
@@ -16386,7 +16396,7 @@
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>2026-10-16T09:07:28</t>
+          <t>2026-10-24T09:07:25</t>
         </is>
       </c>
     </row>
@@ -16565,7 +16575,7 @@
         </is>
       </c>
       <c r="J105" t="n">
-        <v>2990757</v>
+        <v>3578937</v>
       </c>
       <c r="K105" t="inlineStr">
         <is>
@@ -16578,7 +16588,7 @@
         </is>
       </c>
       <c r="M105" t="n">
-        <v>2990757</v>
+        <v>3578937</v>
       </c>
       <c r="N105" t="inlineStr">
         <is>
@@ -16587,7 +16597,7 @@
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>2026-10-16T09:07:41</t>
+          <t>2026-10-24T09:07:35</t>
         </is>
       </c>
     </row>
@@ -16632,7 +16642,7 @@
         </is>
       </c>
       <c r="J106" t="n">
-        <v>396249</v>
+        <v>495289</v>
       </c>
       <c r="K106" t="inlineStr">
         <is>
@@ -16645,7 +16655,7 @@
         </is>
       </c>
       <c r="M106" t="n">
-        <v>396249</v>
+        <v>495289</v>
       </c>
       <c r="N106" t="inlineStr">
         <is>
@@ -16654,7 +16664,7 @@
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>2026-10-16T09:07:51</t>
+          <t>2026-10-24T09:07:45</t>
         </is>
       </c>
     </row>
@@ -17128,13 +17138,37 @@
           <t>冨岡愛</t>
         </is>
       </c>
-      <c r="I114" t="inlineStr"/>
-      <c r="J114" t="inlineStr"/>
-      <c r="K114" t="inlineStr"/>
-      <c r="L114" t="inlineStr"/>
-      <c r="M114" t="inlineStr"/>
-      <c r="N114" t="inlineStr"/>
-      <c r="O114" t="inlineStr"/>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JfXkG3WEtx8</t>
+        </is>
+      </c>
+      <c r="J114" t="n">
+        <v>1562</v>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>Amuse Creative Studio【ACS Animation】</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JfXkG3WEtx8</t>
+        </is>
+      </c>
+      <c r="M114" t="n">
+        <v>1562</v>
+      </c>
+      <c r="N114" t="inlineStr">
+        <is>
+          <t>Amuse Creative Studio【ACS Animation】</t>
+        </is>
+      </c>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>2026-10-24T09:08:04</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -17354,7 +17388,7 @@
         </is>
       </c>
       <c r="J118" t="n">
-        <v>113748</v>
+        <v>118772</v>
       </c>
       <c r="K118" t="inlineStr">
         <is>
@@ -17367,7 +17401,7 @@
         </is>
       </c>
       <c r="M118" t="n">
-        <v>62407</v>
+        <v>91599</v>
       </c>
       <c r="N118" t="inlineStr">
         <is>
@@ -17376,7 +17410,7 @@
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>2026-10-16T09:08:26</t>
+          <t>2026-10-24T09:08:27</t>
         </is>
       </c>
     </row>
@@ -17421,7 +17455,7 @@
         </is>
       </c>
       <c r="J119" t="n">
-        <v>113748</v>
+        <v>118729</v>
       </c>
       <c r="K119" t="inlineStr">
         <is>
@@ -17434,7 +17468,7 @@
         </is>
       </c>
       <c r="M119" t="n">
-        <v>20700</v>
+        <v>35621</v>
       </c>
       <c r="N119" t="inlineStr">
         <is>
@@ -17443,7 +17477,7 @@
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>2026-10-16T09:08:35</t>
+          <t>2026-10-24T09:08:38</t>
         </is>
       </c>
     </row>
@@ -18953,7 +18987,7 @@
         </is>
       </c>
       <c r="J143" t="n">
-        <v>346532</v>
+        <v>353489</v>
       </c>
       <c r="K143" t="inlineStr">
         <is>
@@ -18966,7 +19000,7 @@
         </is>
       </c>
       <c r="M143" t="n">
-        <v>346532</v>
+        <v>353489</v>
       </c>
       <c r="N143" t="inlineStr">
         <is>
@@ -18975,7 +19009,7 @@
       </c>
       <c r="O143" t="inlineStr">
         <is>
-          <t>2026-10-16T09:08:53</t>
+          <t>2026-10-24T09:08:58</t>
         </is>
       </c>
     </row>
@@ -19087,7 +19121,7 @@
         </is>
       </c>
       <c r="J145" t="n">
-        <v>346532</v>
+        <v>353489</v>
       </c>
       <c r="K145" t="inlineStr">
         <is>
@@ -19100,7 +19134,7 @@
         </is>
       </c>
       <c r="M145" t="n">
-        <v>346532</v>
+        <v>353489</v>
       </c>
       <c r="N145" t="inlineStr">
         <is>
@@ -19109,7 +19143,7 @@
       </c>
       <c r="O145" t="inlineStr">
         <is>
-          <t>2026-10-16T09:09:03</t>
+          <t>2026-10-24T09:09:09</t>
         </is>
       </c>
     </row>
@@ -19728,7 +19762,7 @@
         </is>
       </c>
       <c r="J156" t="n">
-        <v>2178</v>
+        <v>3054</v>
       </c>
       <c r="K156" t="inlineStr">
         <is>
@@ -19741,7 +19775,7 @@
         </is>
       </c>
       <c r="M156" t="n">
-        <v>2178</v>
+        <v>3054</v>
       </c>
       <c r="N156" t="inlineStr">
         <is>
@@ -19750,7 +19784,7 @@
       </c>
       <c r="O156" t="inlineStr">
         <is>
-          <t>2026-10-16T09:09:17</t>
+          <t>2026-10-24T09:09:27</t>
         </is>
       </c>
     </row>
@@ -20240,7 +20274,7 @@
         </is>
       </c>
       <c r="J164" t="n">
-        <v>537609</v>
+        <v>781220</v>
       </c>
       <c r="K164" t="inlineStr">
         <is>
@@ -20253,7 +20287,7 @@
         </is>
       </c>
       <c r="M164" t="n">
-        <v>223758</v>
+        <v>253501</v>
       </c>
       <c r="N164" t="inlineStr">
         <is>
@@ -20262,7 +20296,7 @@
       </c>
       <c r="O164" t="inlineStr">
         <is>
-          <t>2026-10-16T09:09:35</t>
+          <t>2026-10-24T09:09:41</t>
         </is>
       </c>
     </row>
@@ -20303,11 +20337,11 @@
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=k8G3_ZYNC-I</t>
+          <t>https://www.youtube.com/watch?v=_PIj78IgPmA</t>
         </is>
       </c>
       <c r="J165" t="n">
-        <v>1063766</v>
+        <v>85297</v>
       </c>
       <c r="K165" t="inlineStr">
         <is>
@@ -20320,7 +20354,7 @@
         </is>
       </c>
       <c r="M165" t="n">
-        <v>72084</v>
+        <v>85297</v>
       </c>
       <c r="N165" t="inlineStr">
         <is>
@@ -20329,7 +20363,7 @@
       </c>
       <c r="O165" t="inlineStr">
         <is>
-          <t>2026-10-16T09:09:44</t>
+          <t>2026-10-24T09:09:52</t>
         </is>
       </c>
     </row>
@@ -20374,7 +20408,7 @@
         </is>
       </c>
       <c r="J166" t="n">
-        <v>72084</v>
+        <v>85297</v>
       </c>
       <c r="K166" t="inlineStr">
         <is>
@@ -20387,7 +20421,7 @@
         </is>
       </c>
       <c r="M166" t="n">
-        <v>6134</v>
+        <v>15017</v>
       </c>
       <c r="N166" t="inlineStr">
         <is>
@@ -20396,7 +20430,7 @@
       </c>
       <c r="O166" t="inlineStr">
         <is>
-          <t>2026-10-16T09:09:54</t>
+          <t>2026-10-24T09:10:02</t>
         </is>
       </c>
     </row>
@@ -20751,7 +20785,7 @@
         </is>
       </c>
       <c r="J173" t="n">
-        <v>277688</v>
+        <v>371002</v>
       </c>
       <c r="K173" t="inlineStr">
         <is>
@@ -20763,7 +20797,7 @@
       <c r="N173" t="inlineStr"/>
       <c r="O173" t="inlineStr">
         <is>
-          <t>2026-10-16T09:10:24</t>
+          <t>2026-10-24T09:10:42</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-10-25
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -11078,7 +11078,7 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>10386</v>
+        <v>11596</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -11091,7 +11091,7 @@
         </is>
       </c>
       <c r="M16" t="n">
-        <v>10386</v>
+        <v>11596</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
@@ -11100,7 +11100,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2026-10-17T09:03:54</t>
+          <t>2026-10-25T09:00:24</t>
         </is>
       </c>
     </row>
@@ -11657,7 +11657,7 @@
         </is>
       </c>
       <c r="J25" t="n">
-        <v>301465</v>
+        <v>304779</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
@@ -11670,7 +11670,7 @@
         </is>
       </c>
       <c r="M25" t="n">
-        <v>301465</v>
+        <v>304779</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
@@ -11679,7 +11679,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>2026-10-17T09:04:25</t>
+          <t>2026-10-25T09:00:38</t>
         </is>
       </c>
     </row>
@@ -11925,7 +11925,7 @@
         </is>
       </c>
       <c r="J29" t="n">
-        <v>7690</v>
+        <v>104375</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
@@ -11938,7 +11938,7 @@
         </is>
       </c>
       <c r="M29" t="n">
-        <v>7690</v>
+        <v>104375</v>
       </c>
       <c r="N29" t="inlineStr">
         <is>
@@ -11947,7 +11947,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>2026-10-18T09:00:33</t>
+          <t>2026-10-25T09:00:48</t>
         </is>
       </c>
     </row>
@@ -14408,7 +14408,7 @@
         </is>
       </c>
       <c r="J70" t="n">
-        <v>135144</v>
+        <v>168198</v>
       </c>
       <c r="K70" t="inlineStr">
         <is>
@@ -14421,7 +14421,7 @@
         </is>
       </c>
       <c r="M70" t="n">
-        <v>135144</v>
+        <v>168198</v>
       </c>
       <c r="N70" t="inlineStr">
         <is>
@@ -14430,7 +14430,7 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>2026-10-18T09:01:19</t>
+          <t>2026-10-25T09:01:36</t>
         </is>
       </c>
     </row>
@@ -15527,7 +15527,7 @@
         </is>
       </c>
       <c r="J89" t="n">
-        <v>60606</v>
+        <v>82324</v>
       </c>
       <c r="K89" t="inlineStr">
         <is>
@@ -15540,7 +15540,7 @@
         </is>
       </c>
       <c r="M89" t="n">
-        <v>60606</v>
+        <v>82324</v>
       </c>
       <c r="N89" t="inlineStr">
         <is>
@@ -15549,7 +15549,7 @@
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>2026-10-17T09:07:59</t>
+          <t>2026-10-25T09:02:11</t>
         </is>
       </c>
     </row>
@@ -15588,37 +15588,13 @@
           <t>導凰</t>
         </is>
       </c>
-      <c r="I90" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=obP86ik2Y7A</t>
-        </is>
-      </c>
-      <c r="J90" t="n">
-        <v>6864</v>
-      </c>
-      <c r="K90" t="inlineStr">
-        <is>
-          <t>導凰 - TAO</t>
-        </is>
-      </c>
-      <c r="L90" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=m_w460cA1ko</t>
-        </is>
-      </c>
-      <c r="M90" t="n">
-        <v>53745</v>
-      </c>
-      <c r="N90" t="inlineStr">
-        <is>
-          <t>ぽにきゃん-Anime PONY CANYON</t>
-        </is>
-      </c>
-      <c r="O90" t="inlineStr">
-        <is>
-          <t>2026-10-17T09:08:18</t>
-        </is>
-      </c>
+      <c r="I90" t="inlineStr"/>
+      <c r="J90" t="inlineStr"/>
+      <c r="K90" t="inlineStr"/>
+      <c r="L90" t="inlineStr"/>
+      <c r="M90" t="inlineStr"/>
+      <c r="N90" t="inlineStr"/>
+      <c r="O90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -16240,7 +16216,7 @@
         </is>
       </c>
       <c r="J100" t="n">
-        <v>600663</v>
+        <v>655623</v>
       </c>
       <c r="K100" t="inlineStr">
         <is>
@@ -16253,7 +16229,7 @@
         </is>
       </c>
       <c r="M100" t="n">
-        <v>49709</v>
+        <v>72279</v>
       </c>
       <c r="N100" t="inlineStr">
         <is>
@@ -16262,7 +16238,7 @@
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:13</t>
+          <t>2026-10-25T09:02:44</t>
         </is>
       </c>
     </row>
@@ -18546,7 +18522,7 @@
         </is>
       </c>
       <c r="J136" t="n">
-        <v>127796</v>
+        <v>161295</v>
       </c>
       <c r="K136" t="inlineStr">
         <is>
@@ -18559,7 +18535,7 @@
         </is>
       </c>
       <c r="M136" t="n">
-        <v>127796</v>
+        <v>161295</v>
       </c>
       <c r="N136" t="inlineStr">
         <is>
@@ -18568,7 +18544,7 @@
       </c>
       <c r="O136" t="inlineStr">
         <is>
-          <t>2026-10-17T09:12:47</t>
+          <t>2026-10-25T09:03:19</t>
         </is>
       </c>
     </row>
@@ -18609,33 +18585,33 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/watch?v=VmotQGt_17A</t>
+        </is>
+      </c>
+      <c r="J137" t="n">
+        <v>83279</v>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>ASCA Official YouTube Channel</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
           <t>https://www.youtube.com/watch?v=nxpUVd6LHFg</t>
         </is>
       </c>
-      <c r="J137" t="n">
-        <v>67353</v>
-      </c>
-      <c r="K137" t="inlineStr">
+      <c r="M137" t="n">
+        <v>82895</v>
+      </c>
+      <c r="N137" t="inlineStr">
         <is>
           <t>アニプレックス チャンネル</t>
         </is>
       </c>
-      <c r="L137" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=nxpUVd6LHFg</t>
-        </is>
-      </c>
-      <c r="M137" t="n">
-        <v>67353</v>
-      </c>
-      <c r="N137" t="inlineStr">
-        <is>
-          <t>アニプレックス チャンネル</t>
-        </is>
-      </c>
       <c r="O137" t="inlineStr">
         <is>
-          <t>2026-10-17T09:12:58</t>
+          <t>2026-10-25T09:03:29</t>
         </is>
       </c>
     </row>
@@ -19298,7 +19274,7 @@
         </is>
       </c>
       <c r="J148" t="n">
-        <v>12164</v>
+        <v>14482</v>
       </c>
       <c r="K148" t="inlineStr">
         <is>
@@ -19311,7 +19287,7 @@
         </is>
       </c>
       <c r="M148" t="n">
-        <v>12164</v>
+        <v>14482</v>
       </c>
       <c r="N148" t="inlineStr">
         <is>
@@ -19320,7 +19296,7 @@
       </c>
       <c r="O148" t="inlineStr">
         <is>
-          <t>2026-10-17T09:13:51</t>
+          <t>2026-10-25T09:03:44</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-10-26
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -15588,13 +15588,37 @@
           <t>導凰</t>
         </is>
       </c>
-      <c r="I90" t="inlineStr"/>
-      <c r="J90" t="inlineStr"/>
-      <c r="K90" t="inlineStr"/>
-      <c r="L90" t="inlineStr"/>
-      <c r="M90" t="inlineStr"/>
-      <c r="N90" t="inlineStr"/>
-      <c r="O90" t="inlineStr"/>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=m_w460cA1ko</t>
+        </is>
+      </c>
+      <c r="J90" t="n">
+        <v>65602</v>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>ぽにきゃん-Anime PONY CANYON</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=m_w460cA1ko</t>
+        </is>
+      </c>
+      <c r="M90" t="n">
+        <v>65602</v>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>ぽにきゃん-Anime PONY CANYON</t>
+        </is>
+      </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>2026-10-26T09:01:30</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -20502,13 +20526,37 @@
           <t>伊東歌詞太郎</t>
         </is>
       </c>
-      <c r="I168" t="inlineStr"/>
-      <c r="J168" t="inlineStr"/>
-      <c r="K168" t="inlineStr"/>
-      <c r="L168" t="inlineStr"/>
-      <c r="M168" t="inlineStr"/>
-      <c r="N168" t="inlineStr"/>
-      <c r="O168" t="inlineStr"/>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=F152_iD2IRc</t>
+        </is>
+      </c>
+      <c r="J168" t="n">
+        <v>33977</v>
+      </c>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L168" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=F152_iD2IRc</t>
+        </is>
+      </c>
+      <c r="M168" t="n">
+        <v>33977</v>
+      </c>
+      <c r="N168" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O168" t="inlineStr">
+        <is>
+          <t>2026-10-26T09:02:33</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="n">

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-10-27
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M189"/>
+  <dimension ref="A1:M188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6249,7 +6249,11 @@
           <t>2027年1月～ テレビ朝日系全国24局ネット“IMAnimation”枠・BS朝日ほか</t>
         </is>
       </c>
-      <c r="H105" t="inlineStr"/>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>ゼクシズ（</t>
+        </is>
+      </c>
       <c r="I105" t="inlineStr"/>
       <c r="J105" t="inlineStr"/>
       <c r="K105" t="inlineStr"/>
@@ -7035,10 +7039,26 @@
           <t>STUDIO MASSKET</t>
         </is>
       </c>
-      <c r="I122" t="inlineStr"/>
-      <c r="J122" t="inlineStr"/>
-      <c r="K122" t="inlineStr"/>
-      <c r="L122" t="inlineStr"/>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>Play the Play</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>MindaRyn</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>My Life Story</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>LINKL PLANET</t>
+        </is>
+      </c>
       <c r="M122" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=27910</t>
@@ -8012,7 +8032,7 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>BanG Dream! It's MyGO!!!!!／Ave Mujica（続編）</t>
+          <t>BanG Dream! MyGO!!!!! // Ave Mujica</t>
         </is>
       </c>
       <c r="E144" t="b">
@@ -8025,7 +8045,7 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>2027年1月～ 日本テレビ系全国30局ネットにて</t>
+          <t>2027年1月8日（金）～ 日本テレビ系全国30局ネットにて</t>
         </is>
       </c>
       <c r="H144" t="inlineStr"/>
@@ -9018,7 +9038,7 @@
     </row>
     <row r="166">
       <c r="A166" t="n">
-        <v>-133007</v>
+        <v>-194116</v>
       </c>
       <c r="B166" t="inlineStr">
         <is>
@@ -9030,7 +9050,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>劇場版 魔法少女まどか☆マギカ〈ワルプルギスの廻天〉</t>
+          <t>最終楽章 響け！ユーフォニアム後編</t>
         </is>
       </c>
       <c r="E166" t="b">
@@ -9043,12 +9063,12 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>2026年8月28日</t>
+          <t>2026年9月11日</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>Shaft</t>
+          <t>Kyoto Animation</t>
         </is>
       </c>
       <c r="I166" t="inlineStr"/>
@@ -9057,13 +9077,13 @@
       <c r="L166" t="inlineStr"/>
       <c r="M166" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/133007</t>
+          <t>https://anilist.co/anime/194116</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
-        <v>-194116</v>
+        <v>-198654</v>
       </c>
       <c r="B167" t="inlineStr">
         <is>
@@ -9075,7 +9095,7 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>最終楽章 響け！ユーフォニアム後編</t>
+          <t>名探偵プリキュア！不思議な庭と2人の秘密</t>
         </is>
       </c>
       <c r="E167" t="b">
@@ -9088,12 +9108,12 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>2026年9月11日</t>
+          <t>2026年9月18日</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>Kyoto Animation</t>
+          <t>Toei Animation</t>
         </is>
       </c>
       <c r="I167" t="inlineStr"/>
@@ -9102,13 +9122,13 @@
       <c r="L167" t="inlineStr"/>
       <c r="M167" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/194116</t>
+          <t>https://anilist.co/anime/198654</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
-        <v>-198654</v>
+        <v>-202429</v>
       </c>
       <c r="B168" t="inlineStr">
         <is>
@@ -9120,7 +9140,7 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>名探偵プリキュア！不思議な庭と2人の秘密</t>
+          <t>我々は宇宙人</t>
         </is>
       </c>
       <c r="E168" t="b">
@@ -9133,12 +9153,12 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>2026年9月18日</t>
+          <t>2026年9月25日</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>Toei Animation</t>
+          <t>NOTHING NEW, Miyu Productions</t>
         </is>
       </c>
       <c r="I168" t="inlineStr"/>
@@ -9147,17 +9167,17 @@
       <c r="L168" t="inlineStr"/>
       <c r="M168" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/198654</t>
+          <t>https://anilist.co/anime/202429</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="n">
-        <v>-202429</v>
+        <v>-202390</v>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026夏アニメ</t>
+          <t>2026秋アニメ</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -9165,7 +9185,7 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>我々は宇宙人</t>
+          <t>ガールズ＆パンツァー 最終章 第5話</t>
         </is>
       </c>
       <c r="E169" t="b">
@@ -9178,12 +9198,12 @@
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>2026年9月25日</t>
+          <t>2026年10月9日</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>NOTHING NEW, Miyu Productions</t>
+          <t>Actas</t>
         </is>
       </c>
       <c r="I169" t="inlineStr"/>
@@ -9192,13 +9212,13 @@
       <c r="L169" t="inlineStr"/>
       <c r="M169" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/202429</t>
+          <t>https://anilist.co/anime/202390</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="n">
-        <v>-202390</v>
+        <v>-207327</v>
       </c>
       <c r="B170" t="inlineStr">
         <is>
@@ -9210,7 +9230,7 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>ガールズ＆パンツァー 最終章 第5話</t>
+          <t>どこよりも遠い場所にいる君へ</t>
         </is>
       </c>
       <c r="E170" t="b">
@@ -9228,7 +9248,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>Actas</t>
+          <t>TMS Entertainment</t>
         </is>
       </c>
       <c r="I170" t="inlineStr"/>
@@ -9237,13 +9257,13 @@
       <c r="L170" t="inlineStr"/>
       <c r="M170" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/202390</t>
+          <t>https://anilist.co/anime/207327</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="n">
-        <v>-207327</v>
+        <v>-197543</v>
       </c>
       <c r="B171" t="inlineStr">
         <is>
@@ -9255,7 +9275,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>どこよりも遠い場所にいる君へ</t>
+          <t>BanG Dream! Ave Mujica prima aurora</t>
         </is>
       </c>
       <c r="E171" t="b">
@@ -9268,12 +9288,12 @@
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>2026年10月9日</t>
+          <t>2026年10月16日</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>TMS Entertainment</t>
+          <t>NICHICALINE</t>
         </is>
       </c>
       <c r="I171" t="inlineStr"/>
@@ -9282,13 +9302,13 @@
       <c r="L171" t="inlineStr"/>
       <c r="M171" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/207327</t>
+          <t>https://anilist.co/anime/197543</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="n">
-        <v>-197543</v>
+        <v>-199340</v>
       </c>
       <c r="B172" t="inlineStr">
         <is>
@@ -9300,7 +9320,7 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>BanG Dream! Ave Mujica prima aurora</t>
+          <t>青春ブタ野郎はディアフレンドの夢を見ない</t>
         </is>
       </c>
       <c r="E172" t="b">
@@ -9318,7 +9338,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>NICHICALINE</t>
+          <t>CloverWorks</t>
         </is>
       </c>
       <c r="I172" t="inlineStr"/>
@@ -9327,13 +9347,13 @@
       <c r="L172" t="inlineStr"/>
       <c r="M172" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/197543</t>
+          <t>https://anilist.co/anime/199340</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
-        <v>-199340</v>
+        <v>-160275</v>
       </c>
       <c r="B173" t="inlineStr">
         <is>
@@ -9345,7 +9365,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>青春ブタ野郎はディアフレンドの夢を見ない</t>
+          <t>メイドインアビス 目覚める神秘</t>
         </is>
       </c>
       <c r="E173" t="b">
@@ -9358,12 +9378,12 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>2026年10月16日</t>
+          <t>2026年10月23日</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>CloverWorks</t>
+          <t>Kinema Citrus</t>
         </is>
       </c>
       <c r="I173" t="inlineStr"/>
@@ -9372,13 +9392,13 @@
       <c r="L173" t="inlineStr"/>
       <c r="M173" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/199340</t>
+          <t>https://anilist.co/anime/160275</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="n">
-        <v>-160275</v>
+        <v>-209642</v>
       </c>
       <c r="B174" t="inlineStr">
         <is>
@@ -9390,7 +9410,7 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>メイドインアビス 目覚める神秘</t>
+          <t>劇場版 前橋ウィッチーズ ～魔女見習いのエモエモリーズ～</t>
         </is>
       </c>
       <c r="E174" t="b">
@@ -9408,7 +9428,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>Kinema Citrus</t>
+          <t>Sunrise</t>
         </is>
       </c>
       <c r="I174" t="inlineStr"/>
@@ -9417,13 +9437,13 @@
       <c r="L174" t="inlineStr"/>
       <c r="M174" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/160275</t>
+          <t>https://anilist.co/anime/209642</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="n">
-        <v>-209642</v>
+        <v>-178972</v>
       </c>
       <c r="B175" t="inlineStr">
         <is>
@@ -9435,7 +9455,7 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>劇場版 前橋ウィッチーズ ～魔女見習いのエモエモリーズ～</t>
+          <t>GROTESQQQUE-グロテスク-</t>
         </is>
       </c>
       <c r="E175" t="b">
@@ -9448,12 +9468,12 @@
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>2026年10月23日</t>
+          <t>2026年11月6日</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>Sunrise</t>
+          <t>CloverWorks</t>
         </is>
       </c>
       <c r="I175" t="inlineStr"/>
@@ -9462,13 +9482,13 @@
       <c r="L175" t="inlineStr"/>
       <c r="M175" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/209642</t>
+          <t>https://anilist.co/anime/178972</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="n">
-        <v>-178972</v>
+        <v>-157330</v>
       </c>
       <c r="B176" t="inlineStr">
         <is>
@@ -9480,7 +9500,7 @@
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>GROTESQQQUE-グロテスク-</t>
+          <t>楽園追放 心のレゾナンス</t>
         </is>
       </c>
       <c r="E176" t="b">
@@ -9493,12 +9513,12 @@
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>2026年11月6日</t>
+          <t>2026年11月13日</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>CloverWorks</t>
+          <t>Toei Animation</t>
         </is>
       </c>
       <c r="I176" t="inlineStr"/>
@@ -9507,13 +9527,13 @@
       <c r="L176" t="inlineStr"/>
       <c r="M176" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/178972</t>
+          <t>https://anilist.co/anime/157330</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="n">
-        <v>-157330</v>
+        <v>-143103</v>
       </c>
       <c r="B177" t="inlineStr">
         <is>
@@ -9525,7 +9545,7 @@
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>楽園追放 心のレゾナンス</t>
+          <t>魔法使いの夜</t>
         </is>
       </c>
       <c r="E177" t="b">
@@ -9538,12 +9558,12 @@
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>2026年11月13日</t>
+          <t>2026年11月20日</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>Toei Animation</t>
+          <t>ufotable</t>
         </is>
       </c>
       <c r="I177" t="inlineStr"/>
@@ -9552,13 +9572,13 @@
       <c r="L177" t="inlineStr"/>
       <c r="M177" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/157330</t>
+          <t>https://anilist.co/anime/143103</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
-        <v>-143103</v>
+        <v>-206163</v>
       </c>
       <c r="B178" t="inlineStr">
         <is>
@@ -9570,7 +9590,7 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>魔法使いの夜</t>
+          <t>装甲騎兵ボトムズ 灰色の魔女</t>
         </is>
       </c>
       <c r="E178" t="b">
@@ -9588,7 +9608,7 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>ufotable</t>
+          <t>Production I.G, Sunrise</t>
         </is>
       </c>
       <c r="I178" t="inlineStr"/>
@@ -9597,13 +9617,13 @@
       <c r="L178" t="inlineStr"/>
       <c r="M178" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/143103</t>
+          <t>https://anilist.co/anime/206163</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="n">
-        <v>-206163</v>
+        <v>-212539</v>
       </c>
       <c r="B179" t="inlineStr">
         <is>
@@ -9615,7 +9635,7 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>装甲騎兵ボトムズ 灰色の魔女</t>
+          <t>タコピーの原罪 -ありがとう、また明日-</t>
         </is>
       </c>
       <c r="E179" t="b">
@@ -9628,12 +9648,12 @@
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>2026年11月20日</t>
+          <t>2026年11月27日</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>Production I.G, Sunrise</t>
+          <t>ENISHIYA</t>
         </is>
       </c>
       <c r="I179" t="inlineStr"/>
@@ -9642,13 +9662,13 @@
       <c r="L179" t="inlineStr"/>
       <c r="M179" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/206163</t>
+          <t>https://anilist.co/anime/212539</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="n">
-        <v>-212539</v>
+        <v>-205289</v>
       </c>
       <c r="B180" t="inlineStr">
         <is>
@@ -9660,7 +9680,7 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>タコピーの原罪 -ありがとう、また明日-</t>
+          <t>ノーマン・ザ・スノーマン ~こどもたちのひとつ星~</t>
         </is>
       </c>
       <c r="E180" t="b">
@@ -9673,12 +9693,12 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>2026年11月27日</t>
+          <t>2026年12月</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>ENISHIYA</t>
+          <t>TECARAT</t>
         </is>
       </c>
       <c r="I180" t="inlineStr"/>
@@ -9687,13 +9707,13 @@
       <c r="L180" t="inlineStr"/>
       <c r="M180" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/212539</t>
+          <t>https://anilist.co/anime/205289</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
-        <v>-205289</v>
+        <v>-200929</v>
       </c>
       <c r="B181" t="inlineStr">
         <is>
@@ -9705,7 +9725,7 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>ノーマン・ザ・スノーマン ~こどもたちのひとつ星~</t>
+          <t>薬屋のひとりごと 亡妃の秘宝</t>
         </is>
       </c>
       <c r="E181" t="b">
@@ -9718,12 +9738,12 @@
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>2026年12月</t>
+          <t>2026年12月11日</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>TECARAT</t>
+          <t>TOHO animation STUDIO</t>
         </is>
       </c>
       <c r="I181" t="inlineStr"/>
@@ -9732,17 +9752,17 @@
       <c r="L181" t="inlineStr"/>
       <c r="M181" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/205289</t>
+          <t>https://anilist.co/anime/200929</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
-        <v>-200929</v>
+        <v>-183692</v>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026秋アニメ</t>
+          <t>2027冬アニメ</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -9750,7 +9770,7 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>薬屋のひとりごと 亡妃の秘宝</t>
+          <t>機動戦士ガンダムSEED FREEDOM ZERO</t>
         </is>
       </c>
       <c r="E182" t="b">
@@ -9763,12 +9783,12 @@
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>2026年12月11日</t>
+          <t>2027年1月15日</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>TOHO animation STUDIO</t>
+          <t>Sunrise</t>
         </is>
       </c>
       <c r="I182" t="inlineStr"/>
@@ -9777,13 +9797,13 @@
       <c r="L182" t="inlineStr"/>
       <c r="M182" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/200929</t>
+          <t>https://anilist.co/anime/183692</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
-        <v>-183692</v>
+        <v>-213814</v>
       </c>
       <c r="B183" t="inlineStr">
         <is>
@@ -9795,7 +9815,7 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>機動戦士ガンダムSEED FREEDOM ZERO</t>
+          <t>アイカツスターズ！ ～星々のProgress～</t>
         </is>
       </c>
       <c r="E183" t="b">
@@ -9808,12 +9828,12 @@
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>2027年1月15日</t>
+          <t>2027年1月22日</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>Sunrise</t>
+          <t>Bandai Namco Pictures</t>
         </is>
       </c>
       <c r="I183" t="inlineStr"/>
@@ -9822,13 +9842,13 @@
       <c r="L183" t="inlineStr"/>
       <c r="M183" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/183692</t>
+          <t>https://anilist.co/anime/213814</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
-        <v>-213814</v>
+        <v>-186603</v>
       </c>
       <c r="B184" t="inlineStr">
         <is>
@@ -9840,7 +9860,7 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>アイカツスターズ！ ～星々のProgress～</t>
+          <t>ラブライブ！虹ヶ咲学園スクールアイドル同好会 完結編 最終章</t>
         </is>
       </c>
       <c r="E184" t="b">
@@ -9853,12 +9873,12 @@
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>2027年1月22日</t>
+          <t>2027年2月5日</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>Bandai Namco Pictures</t>
+          <t>Sunrise</t>
         </is>
       </c>
       <c r="I184" t="inlineStr"/>
@@ -9867,13 +9887,13 @@
       <c r="L184" t="inlineStr"/>
       <c r="M184" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/213814</t>
+          <t>https://anilist.co/anime/186603</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
-        <v>-186603</v>
+        <v>-194213</v>
       </c>
       <c r="B185" t="inlineStr">
         <is>
@@ -9885,7 +9905,7 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>ラブライブ！虹ヶ咲学園スクールアイドル同好会 完結編 最終章</t>
+          <t>ghost／夜の果て</t>
         </is>
       </c>
       <c r="E185" t="b">
@@ -9898,12 +9918,12 @@
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>2027年2月5日</t>
+          <t>2027年2月11日</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>Sunrise</t>
+          <t>MADHOUSE</t>
         </is>
       </c>
       <c r="I185" t="inlineStr"/>
@@ -9912,13 +9932,13 @@
       <c r="L185" t="inlineStr"/>
       <c r="M185" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/186603</t>
+          <t>https://anilist.co/anime/194213</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="n">
-        <v>-194213</v>
+        <v>-206298</v>
       </c>
       <c r="B186" t="inlineStr">
         <is>
@@ -9930,7 +9950,7 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>ghost／夜の果て</t>
+          <t>劇場版 メダリスト</t>
         </is>
       </c>
       <c r="E186" t="b">
@@ -9943,12 +9963,12 @@
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>2027年2月11日</t>
+          <t>2027年2月19日</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>MADHOUSE</t>
+          <t>ENGI</t>
         </is>
       </c>
       <c r="I186" t="inlineStr"/>
@@ -9957,13 +9977,13 @@
       <c r="L186" t="inlineStr"/>
       <c r="M186" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/194213</t>
+          <t>https://anilist.co/anime/206298</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
-        <v>-206298</v>
+        <v>-216623</v>
       </c>
       <c r="B187" t="inlineStr">
         <is>
@@ -9975,7 +9995,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>劇場版 メダリスト</t>
+          <t>ドラえもん のび太の蒸気時間車</t>
         </is>
       </c>
       <c r="E187" t="b">
@@ -9988,12 +10008,12 @@
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>2027年2月19日</t>
+          <t>2027年3月5日</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>ENGI</t>
+          <t>Shin-Ei Animation</t>
         </is>
       </c>
       <c r="I187" t="inlineStr"/>
@@ -10002,13 +10022,13 @@
       <c r="L187" t="inlineStr"/>
       <c r="M187" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/206298</t>
+          <t>https://anilist.co/anime/216623</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="n">
-        <v>-216623</v>
+        <v>-190244</v>
       </c>
       <c r="B188" t="inlineStr">
         <is>
@@ -10020,7 +10040,7 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>ドラえもん のび太の蒸気時間車</t>
+          <t>デート・ア・ライブF Last Date</t>
         </is>
       </c>
       <c r="E188" t="b">
@@ -10033,12 +10053,12 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>2027年3月5日</t>
+          <t>2027年3月26日</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>Shin-Ei Animation</t>
+          <t>Fugaku</t>
         </is>
       </c>
       <c r="I188" t="inlineStr"/>
@@ -10046,51 +10066,6 @@
       <c r="K188" t="inlineStr"/>
       <c r="L188" t="inlineStr"/>
       <c r="M188" t="inlineStr">
-        <is>
-          <t>https://anilist.co/anime/216623</t>
-        </is>
-      </c>
-    </row>
-    <row r="189">
-      <c r="A189" t="n">
-        <v>-190244</v>
-      </c>
-      <c r="B189" t="inlineStr">
-        <is>
-          <t>2027冬アニメ</t>
-        </is>
-      </c>
-      <c r="C189" t="n">
-        <v>0</v>
-      </c>
-      <c r="D189" t="inlineStr">
-        <is>
-          <t>デート・ア・ライブF Last Date</t>
-        </is>
-      </c>
-      <c r="E189" t="b">
-        <v>0</v>
-      </c>
-      <c r="F189" t="inlineStr">
-        <is>
-          <t>劇場版</t>
-        </is>
-      </c>
-      <c r="G189" t="inlineStr">
-        <is>
-          <t>2027年3月26日</t>
-        </is>
-      </c>
-      <c r="H189" t="inlineStr">
-        <is>
-          <t>Fugaku</t>
-        </is>
-      </c>
-      <c r="I189" t="inlineStr"/>
-      <c r="J189" t="inlineStr"/>
-      <c r="K189" t="inlineStr"/>
-      <c r="L189" t="inlineStr"/>
-      <c r="M189" t="inlineStr">
         <is>
           <t>https://anilist.co/anime/190244</t>
         </is>
@@ -10107,7 +10082,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O183"/>
+  <dimension ref="A1:O185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19713,13 +19688,37 @@
           <t>環琴葉とはーちゃん（ACS Anime records）</t>
         </is>
       </c>
-      <c r="I155" t="inlineStr"/>
-      <c r="J155" t="inlineStr"/>
-      <c r="K155" t="inlineStr"/>
-      <c r="L155" t="inlineStr"/>
-      <c r="M155" t="inlineStr"/>
-      <c r="N155" t="inlineStr"/>
-      <c r="O155" t="inlineStr"/>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=CIHY9MfocTY</t>
+        </is>
+      </c>
+      <c r="J155" t="n">
+        <v>12191</v>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>【フジテレビ】アニメ公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=CIHY9MfocTY</t>
+        </is>
+      </c>
+      <c r="M155" t="n">
+        <v>12191</v>
+      </c>
+      <c r="N155" t="inlineStr">
+        <is>
+          <t>【フジテレビ】アニメ公式チャンネル</t>
+        </is>
+      </c>
+      <c r="O155" t="inlineStr">
+        <is>
+          <t>2026-10-27T09:02:31</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -20779,7 +20778,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>雑用付与術師が自分の最強に気付くまで</t>
+          <t>ゲーム世界転生〈ダン活〉～ゲーマーは【ダンジョン就活のススメ】を〈はじめから〉プレイする～</t>
         </is>
       </c>
       <c r="D173" t="b">
@@ -20795,35 +20794,21 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>Ecstatic Buffer</t>
+          <t>Play the Play</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>LiSA</t>
-        </is>
-      </c>
-      <c r="I173" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=yqvAv5li9Pw</t>
-        </is>
-      </c>
-      <c r="J173" t="n">
-        <v>371002</v>
-      </c>
-      <c r="K173" t="inlineStr">
-        <is>
-          <t>StarryCube 公式チャンネル</t>
-        </is>
-      </c>
+          <t>MindaRyn</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr"/>
+      <c r="J173" t="inlineStr"/>
+      <c r="K173" t="inlineStr"/>
       <c r="L173" t="inlineStr"/>
       <c r="M173" t="inlineStr"/>
       <c r="N173" t="inlineStr"/>
-      <c r="O173" t="inlineStr">
-        <is>
-          <t>2026-10-24T09:10:42</t>
-        </is>
-      </c>
+      <c r="O173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -20836,7 +20821,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>ゾンビのあふれた世界で俺だけが襲われない</t>
+          <t>ゲーム世界転生〈ダン活〉～ゲーマーは【ダンジョン就活のススメ】を〈はじめから〉プレイする～</t>
         </is>
       </c>
       <c r="D174" t="b">
@@ -20844,7 +20829,7 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F174" t="n">
@@ -20852,12 +20837,12 @@
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>ノーリアクション</t>
+          <t>My Life Story</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>レトベア（unknown Vo：0in）</t>
+          <t>LINKL PLANET</t>
         </is>
       </c>
       <c r="I174" t="inlineStr"/>
@@ -20879,7 +20864,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>ゾンビのあふれた世界で俺だけが襲われない</t>
+          <t>雑用付与術師が自分の最強に気付くまで</t>
         </is>
       </c>
       <c r="D175" t="b">
@@ -20887,7 +20872,7 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F175" t="n">
@@ -20895,21 +20880,35 @@
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>ツキカゲ</t>
+          <t>Ecstatic Buffer</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>イツカ▶</t>
-        </is>
-      </c>
-      <c r="I175" t="inlineStr"/>
-      <c r="J175" t="inlineStr"/>
-      <c r="K175" t="inlineStr"/>
+          <t>LiSA</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=yqvAv5li9Pw</t>
+        </is>
+      </c>
+      <c r="J175" t="n">
+        <v>371002</v>
+      </c>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>StarryCube 公式チャンネル</t>
+        </is>
+      </c>
       <c r="L175" t="inlineStr"/>
       <c r="M175" t="inlineStr"/>
       <c r="N175" t="inlineStr"/>
-      <c r="O175" t="inlineStr"/>
+      <c r="O175" t="inlineStr">
+        <is>
+          <t>2026-10-24T09:10:42</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -20922,7 +20921,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>姫騎士様のヒモ</t>
+          <t>ゾンビのあふれた世界で俺だけが襲われない</t>
         </is>
       </c>
       <c r="D176" t="b">
@@ -20938,12 +20937,12 @@
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>TRUE-TABOO</t>
+          <t>ノーリアクション</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>MYTH &amp; ROID</t>
+          <t>レトベア（unknown Vo：0in）</t>
         </is>
       </c>
       <c r="I176" t="inlineStr"/>
@@ -20965,7 +20964,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>姫騎士様のヒモ</t>
+          <t>ゾンビのあふれた世界で俺だけが襲われない</t>
         </is>
       </c>
       <c r="D177" t="b">
@@ -20981,12 +20980,12 @@
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>偽花</t>
+          <t>ツキカゲ</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>sajou no hana</t>
+          <t>イツカ▶</t>
         </is>
       </c>
       <c r="I177" t="inlineStr"/>
@@ -21008,7 +21007,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>ふつつかな悪女ではございますが～雛宮蝶鼠とりかえ伝～ 第2クール</t>
+          <t>姫騎士様のヒモ</t>
         </is>
       </c>
       <c r="D178" t="b">
@@ -21024,35 +21023,21 @@
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>Sunny</t>
+          <t>TRUE-TABOO</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>milet</t>
-        </is>
-      </c>
-      <c r="I178" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=nR_vqhD2rGM</t>
-        </is>
-      </c>
-      <c r="J178" t="n">
-        <v>816684</v>
-      </c>
-      <c r="K178" t="inlineStr">
-        <is>
-          <t>TOHO animation</t>
-        </is>
-      </c>
+          <t>MYTH &amp; ROID</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr"/>
+      <c r="J178" t="inlineStr"/>
+      <c r="K178" t="inlineStr"/>
       <c r="L178" t="inlineStr"/>
       <c r="M178" t="inlineStr"/>
       <c r="N178" t="inlineStr"/>
-      <c r="O178" t="inlineStr">
-        <is>
-          <t>2026-10-21T09:17:22</t>
-        </is>
-      </c>
+      <c r="O178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -21065,7 +21050,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>ふつつかな悪女ではございますが～雛宮蝶鼠とりかえ伝～ 第2クール</t>
+          <t>姫騎士様のヒモ</t>
         </is>
       </c>
       <c r="D179" t="b">
@@ -21081,12 +21066,12 @@
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>ホウキボシ</t>
+          <t>偽花</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>ロクデナシ</t>
+          <t>sajou no hana</t>
         </is>
       </c>
       <c r="I179" t="inlineStr"/>
@@ -21108,7 +21093,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>茉莉花官吏伝</t>
+          <t>ふつつかな悪女ではございますが～雛宮蝶鼠とりかえ伝～ 第2クール</t>
         </is>
       </c>
       <c r="D180" t="b">
@@ -21124,43 +21109,33 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>花噺</t>
+          <t>Sunny</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>KANA-BOON</t>
+          <t>milet</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=7ja8PqzctBg</t>
+          <t>https://www.youtube.com/watch?v=nR_vqhD2rGM</t>
         </is>
       </c>
       <c r="J180" t="n">
-        <v>220388</v>
+        <v>816684</v>
       </c>
       <c r="K180" t="inlineStr">
         <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="L180" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=7ja8PqzctBg</t>
-        </is>
-      </c>
-      <c r="M180" t="n">
-        <v>220388</v>
-      </c>
-      <c r="N180" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
+          <t>TOHO animation</t>
+        </is>
+      </c>
+      <c r="L180" t="inlineStr"/>
+      <c r="M180" t="inlineStr"/>
+      <c r="N180" t="inlineStr"/>
       <c r="O180" t="inlineStr">
         <is>
-          <t>2026-10-21T09:17:39</t>
+          <t>2026-10-21T09:17:22</t>
         </is>
       </c>
     </row>
@@ -21175,7 +21150,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>ワンパンマン 第3期 第2クール</t>
+          <t>ふつつかな悪女ではございますが～雛宮蝶鼠とりかえ伝～ 第2クール</t>
         </is>
       </c>
       <c r="D181" t="b">
@@ -21183,7 +21158,7 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F181" t="n">
@@ -21191,45 +21166,21 @@
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>Get No Satisfied !</t>
+          <t>ホウキボシ</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>JAM Project feat.BABYMETAL</t>
-        </is>
-      </c>
-      <c r="I181" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=lpGSwTUSynM</t>
-        </is>
-      </c>
-      <c r="J181" t="n">
-        <v>2078765</v>
-      </c>
-      <c r="K181" t="inlineStr">
-        <is>
-          <t>Lantis Channel</t>
-        </is>
-      </c>
-      <c r="L181" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=lpGSwTUSynM</t>
-        </is>
-      </c>
-      <c r="M181" t="n">
-        <v>2078765</v>
-      </c>
-      <c r="N181" t="inlineStr">
-        <is>
-          <t>Lantis Channel</t>
-        </is>
-      </c>
-      <c r="O181" t="inlineStr">
-        <is>
-          <t>2026-10-21T09:17:48</t>
-        </is>
-      </c>
+          <t>ロクデナシ</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr"/>
+      <c r="J181" t="inlineStr"/>
+      <c r="K181" t="inlineStr"/>
+      <c r="L181" t="inlineStr"/>
+      <c r="M181" t="inlineStr"/>
+      <c r="N181" t="inlineStr"/>
+      <c r="O181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -21242,7 +21193,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>ワンパンマン 第3期 第2クール</t>
+          <t>茉莉花官吏伝</t>
         </is>
       </c>
       <c r="D182" t="b">
@@ -21254,25 +21205,49 @@
         </is>
       </c>
       <c r="F182" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>Never Done～最強VS最恐～</t>
+          <t>花噺</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>JAM Project</t>
-        </is>
-      </c>
-      <c r="I182" t="inlineStr"/>
-      <c r="J182" t="inlineStr"/>
-      <c r="K182" t="inlineStr"/>
-      <c r="L182" t="inlineStr"/>
-      <c r="M182" t="inlineStr"/>
-      <c r="N182" t="inlineStr"/>
-      <c r="O182" t="inlineStr"/>
+          <t>KANA-BOON</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=7ja8PqzctBg</t>
+        </is>
+      </c>
+      <c r="J182" t="n">
+        <v>220388</v>
+      </c>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=7ja8PqzctBg</t>
+        </is>
+      </c>
+      <c r="M182" t="n">
+        <v>220388</v>
+      </c>
+      <c r="N182" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O182" t="inlineStr">
+        <is>
+          <t>2026-10-21T09:17:39</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -21293,7 +21268,7 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F183" t="n">
@@ -21301,21 +21276,131 @@
       </c>
       <c r="G183" t="inlineStr">
         <is>
+          <t>Get No Satisfied !</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>JAM Project feat.BABYMETAL</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=lpGSwTUSynM</t>
+        </is>
+      </c>
+      <c r="J183" t="n">
+        <v>2078765</v>
+      </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>Lantis Channel</t>
+        </is>
+      </c>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=lpGSwTUSynM</t>
+        </is>
+      </c>
+      <c r="M183" t="n">
+        <v>2078765</v>
+      </c>
+      <c r="N183" t="inlineStr">
+        <is>
+          <t>Lantis Channel</t>
+        </is>
+      </c>
+      <c r="O183" t="inlineStr">
+        <is>
+          <t>2026-10-21T09:17:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="n">
+        <v>6212</v>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>2027冬アニメ</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>ワンパンマン 第3期 第2クール</t>
+        </is>
+      </c>
+      <c r="D184" t="b">
+        <v>0</v>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F184" t="n">
+        <v>2</v>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>Never Done～最強VS最恐～</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>JAM Project</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr"/>
+      <c r="J184" t="inlineStr"/>
+      <c r="K184" t="inlineStr"/>
+      <c r="L184" t="inlineStr"/>
+      <c r="M184" t="inlineStr"/>
+      <c r="N184" t="inlineStr"/>
+      <c r="O184" t="inlineStr"/>
+    </row>
+    <row r="185">
+      <c r="A185" t="n">
+        <v>6212</v>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>2027冬アニメ</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>ワンパンマン 第3期 第2クール</t>
+        </is>
+      </c>
+      <c r="D185" t="b">
+        <v>0</v>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
+      <c r="F185" t="n">
+        <v>1</v>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
           <t>そこに有る灯り</t>
         </is>
       </c>
-      <c r="H183" t="inlineStr">
+      <c r="H185" t="inlineStr">
         <is>
           <t>古川慎</t>
         </is>
       </c>
-      <c r="I183" t="inlineStr"/>
-      <c r="J183" t="inlineStr"/>
-      <c r="K183" t="inlineStr"/>
-      <c r="L183" t="inlineStr"/>
-      <c r="M183" t="inlineStr"/>
-      <c r="N183" t="inlineStr"/>
-      <c r="O183" t="inlineStr"/>
+      <c r="I185" t="inlineStr"/>
+      <c r="J185" t="inlineStr"/>
+      <c r="K185" t="inlineStr"/>
+      <c r="L185" t="inlineStr"/>
+      <c r="M185" t="inlineStr"/>
+      <c r="N185" t="inlineStr"/>
+      <c r="O185" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-10-29
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -8466,10 +8466,14 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>2027年1月～ NHK総合にて</t>
-        </is>
-      </c>
-      <c r="H153" t="inlineStr"/>
+          <t>2027年1月4日（月）〜 NHK総合にて</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>タツノコプロ</t>
+        </is>
+      </c>
       <c r="I153" t="inlineStr"/>
       <c r="J153" t="inlineStr"/>
       <c r="K153" t="inlineStr"/>
@@ -10742,7 +10746,7 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>166587</v>
+        <v>183416</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -10755,7 +10759,7 @@
         </is>
       </c>
       <c r="M11" t="n">
-        <v>166587</v>
+        <v>183416</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
@@ -10764,7 +10768,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2026-10-21T09:00:32</t>
+          <t>2026-10-29T09:00:28</t>
         </is>
       </c>
     </row>
@@ -10986,7 +10990,7 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>1286808</v>
+        <v>1460772</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -10999,7 +11003,7 @@
         </is>
       </c>
       <c r="M15" t="n">
-        <v>1286808</v>
+        <v>1460772</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
@@ -11008,7 +11012,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026-10-21T09:00:45</t>
+          <t>2026-10-29T09:00:41</t>
         </is>
       </c>
     </row>
@@ -11053,7 +11057,7 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>445384</v>
+        <v>1362669</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -11066,7 +11070,7 @@
         </is>
       </c>
       <c r="M16" t="n">
-        <v>20500</v>
+        <v>24060</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
@@ -11075,7 +11079,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2026-10-21T09:00:54</t>
+          <t>2026-10-29T09:00:51</t>
         </is>
       </c>
     </row>
@@ -11187,7 +11191,7 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>7402111</v>
+        <v>7462052</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -11200,7 +11204,7 @@
         </is>
       </c>
       <c r="M18" t="n">
-        <v>637574</v>
+        <v>639215</v>
       </c>
       <c r="N18" t="inlineStr">
         <is>
@@ -11209,7 +11213,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>2026-10-21T09:01:13</t>
+          <t>2026-10-29T09:01:10</t>
         </is>
       </c>
     </row>
@@ -11254,7 +11258,7 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>52468</v>
+        <v>63662</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
@@ -11267,7 +11271,7 @@
         </is>
       </c>
       <c r="M19" t="n">
-        <v>52468</v>
+        <v>63662</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
@@ -11276,7 +11280,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>2026-10-21T09:01:22</t>
+          <t>2026-10-29T09:01:20</t>
         </is>
       </c>
     </row>
@@ -11321,7 +11325,7 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>22982</v>
+        <v>27860</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -11334,7 +11338,7 @@
         </is>
       </c>
       <c r="M20" t="n">
-        <v>22982</v>
+        <v>27860</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
@@ -11343,7 +11347,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026-10-21T09:01:32</t>
+          <t>2026-10-29T09:01:31</t>
         </is>
       </c>
     </row>
@@ -11455,7 +11459,7 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>106640</v>
+        <v>112306</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
@@ -11468,7 +11472,7 @@
         </is>
       </c>
       <c r="M22" t="n">
-        <v>106640</v>
+        <v>112306</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
@@ -11477,7 +11481,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>2026-10-21T09:01:42</t>
+          <t>2026-10-29T09:01:41</t>
         </is>
       </c>
     </row>
@@ -11565,7 +11569,7 @@
         </is>
       </c>
       <c r="J24" t="n">
-        <v>17471</v>
+        <v>19229</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
@@ -11578,7 +11582,7 @@
         </is>
       </c>
       <c r="M24" t="n">
-        <v>17471</v>
+        <v>19229</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
@@ -11587,7 +11591,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>2026-10-21T09:01:50</t>
+          <t>2026-10-29T09:01:51</t>
         </is>
       </c>
     </row>
@@ -11833,7 +11837,7 @@
         </is>
       </c>
       <c r="J28" t="n">
-        <v>225762</v>
+        <v>250202</v>
       </c>
       <c r="K28" t="inlineStr">
         <is>
@@ -11846,7 +11850,7 @@
         </is>
       </c>
       <c r="M28" t="n">
-        <v>225762</v>
+        <v>250202</v>
       </c>
       <c r="N28" t="inlineStr">
         <is>
@@ -11855,7 +11859,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>2026-10-21T09:02:01</t>
+          <t>2026-10-29T09:02:00</t>
         </is>
       </c>
     </row>
@@ -11896,33 +11900,33 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/watch?v=KSgf2t0wjGw</t>
+        </is>
+      </c>
+      <c r="J29" t="n">
+        <v>9150</v>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>月追う彼方</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
           <t>https://www.youtube.com/watch?v=HwJXu_CirFQ</t>
         </is>
       </c>
-      <c r="J29" t="n">
-        <v>2728</v>
-      </c>
-      <c r="K29" t="inlineStr">
+      <c r="M29" t="n">
+        <v>3992</v>
+      </c>
+      <c r="N29" t="inlineStr">
         <is>
           <t xml:space="preserve">AnimationID </t>
         </is>
       </c>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=HwJXu_CirFQ</t>
-        </is>
-      </c>
-      <c r="M29" t="n">
-        <v>2728</v>
-      </c>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">AnimationID </t>
-        </is>
-      </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>2026-10-21T09:02:07</t>
+          <t>2026-10-29T09:02:09</t>
         </is>
       </c>
     </row>
@@ -12030,33 +12034,33 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/watch?v=MuX1HliRC2c</t>
+        </is>
+      </c>
+      <c r="J31" t="n">
+        <v>26845</v>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>スガ シカオ</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
           <t>https://www.youtube.com/watch?v=tG7X7oUnbZc</t>
         </is>
       </c>
-      <c r="J31" t="n">
-        <v>74694</v>
-      </c>
-      <c r="K31" t="inlineStr">
+      <c r="M31" t="n">
+        <v>120488</v>
+      </c>
+      <c r="N31" t="inlineStr">
         <is>
           <t>NHK ENTERPRISES Animation</t>
         </is>
       </c>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=tG7X7oUnbZc</t>
-        </is>
-      </c>
-      <c r="M31" t="n">
-        <v>74694</v>
-      </c>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>NHK ENTERPRISES Animation</t>
-        </is>
-      </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>2026-10-21T09:02:14</t>
+          <t>2026-10-29T09:02:18</t>
         </is>
       </c>
     </row>
@@ -12168,7 +12172,7 @@
         </is>
       </c>
       <c r="J33" t="n">
-        <v>654985</v>
+        <v>929773</v>
       </c>
       <c r="K33" t="inlineStr">
         <is>
@@ -12181,7 +12185,7 @@
         </is>
       </c>
       <c r="M33" t="n">
-        <v>654985</v>
+        <v>929773</v>
       </c>
       <c r="N33" t="inlineStr">
         <is>
@@ -12190,7 +12194,7 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>2026-10-21T09:02:19</t>
+          <t>2026-10-29T09:02:24</t>
         </is>
       </c>
     </row>
@@ -12231,33 +12235,33 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/watch?v=J5-NUv2fNtk</t>
+        </is>
+      </c>
+      <c r="J34" t="n">
+        <v>3756094</v>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>ヨルシカ / n-buna Official</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
           <t>https://www.youtube.com/watch?v=lBsQCQDbgOE</t>
         </is>
       </c>
-      <c r="J34" t="n">
-        <v>3404615</v>
-      </c>
-      <c r="K34" t="inlineStr">
+      <c r="M34" t="n">
+        <v>3620733</v>
+      </c>
+      <c r="N34" t="inlineStr">
         <is>
           <t>TOHO animation</t>
         </is>
       </c>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=lBsQCQDbgOE</t>
-        </is>
-      </c>
-      <c r="M34" t="n">
-        <v>3404615</v>
-      </c>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>TOHO animation</t>
-        </is>
-      </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>2026-10-21T09:02:29</t>
+          <t>2026-10-29T09:02:33</t>
         </is>
       </c>
     </row>
@@ -12522,7 +12526,7 @@
         </is>
       </c>
       <c r="J39" t="n">
-        <v>89979</v>
+        <v>98493</v>
       </c>
       <c r="K39" t="inlineStr">
         <is>
@@ -12535,7 +12539,7 @@
         </is>
       </c>
       <c r="M39" t="n">
-        <v>89979</v>
+        <v>98493</v>
       </c>
       <c r="N39" t="inlineStr">
         <is>
@@ -12544,7 +12548,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>2026-10-21T09:02:45</t>
+          <t>2026-10-29T09:02:49</t>
         </is>
       </c>
     </row>
@@ -12589,7 +12593,7 @@
         </is>
       </c>
       <c r="J40" t="n">
-        <v>217684</v>
+        <v>279845</v>
       </c>
       <c r="K40" t="inlineStr">
         <is>
@@ -12602,7 +12606,7 @@
         </is>
       </c>
       <c r="M40" t="n">
-        <v>166556</v>
+        <v>178981</v>
       </c>
       <c r="N40" t="inlineStr">
         <is>
@@ -12611,7 +12615,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>2026-10-21T09:02:55</t>
+          <t>2026-10-29T09:02:59</t>
         </is>
       </c>
     </row>
@@ -12656,7 +12660,7 @@
         </is>
       </c>
       <c r="J41" t="n">
-        <v>40370</v>
+        <v>44465</v>
       </c>
       <c r="K41" t="inlineStr">
         <is>
@@ -12669,7 +12673,7 @@
         </is>
       </c>
       <c r="M41" t="n">
-        <v>40370</v>
+        <v>44465</v>
       </c>
       <c r="N41" t="inlineStr">
         <is>
@@ -12678,7 +12682,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>2026-10-21T09:03:05</t>
+          <t>2026-10-29T09:03:09</t>
         </is>
       </c>
     </row>
@@ -12924,7 +12928,7 @@
         </is>
       </c>
       <c r="J45" t="n">
-        <v>421</v>
+        <v>614</v>
       </c>
       <c r="K45" t="inlineStr">
         <is>
@@ -12937,7 +12941,7 @@
         </is>
       </c>
       <c r="M45" t="n">
-        <v>421</v>
+        <v>614</v>
       </c>
       <c r="N45" t="inlineStr">
         <is>
@@ -12946,7 +12950,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>2026-10-21T09:03:14</t>
+          <t>2026-10-29T09:03:18</t>
         </is>
       </c>
     </row>
@@ -13125,7 +13129,7 @@
         </is>
       </c>
       <c r="J48" t="n">
-        <v>2495396</v>
+        <v>2618505</v>
       </c>
       <c r="K48" t="inlineStr">
         <is>
@@ -13138,7 +13142,7 @@
         </is>
       </c>
       <c r="M48" t="n">
-        <v>35222</v>
+        <v>41294</v>
       </c>
       <c r="N48" t="inlineStr">
         <is>
@@ -13147,7 +13151,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>2026-10-21T09:03:24</t>
+          <t>2026-10-29T09:03:27</t>
         </is>
       </c>
     </row>
@@ -13388,7 +13392,7 @@
         </is>
       </c>
       <c r="J53" t="n">
-        <v>93112</v>
+        <v>109977</v>
       </c>
       <c r="K53" t="inlineStr">
         <is>
@@ -13401,7 +13405,7 @@
         </is>
       </c>
       <c r="M53" t="n">
-        <v>93112</v>
+        <v>109977</v>
       </c>
       <c r="N53" t="inlineStr">
         <is>
@@ -13410,7 +13414,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>2026-10-21T09:03:41</t>
+          <t>2026-10-29T09:03:45</t>
         </is>
       </c>
     </row>
@@ -13455,7 +13459,7 @@
         </is>
       </c>
       <c r="J54" t="n">
-        <v>29459</v>
+        <v>99828</v>
       </c>
       <c r="K54" t="inlineStr">
         <is>
@@ -13468,7 +13472,7 @@
         </is>
       </c>
       <c r="M54" t="n">
-        <v>19976</v>
+        <v>23776</v>
       </c>
       <c r="N54" t="inlineStr">
         <is>
@@ -13477,7 +13481,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>2026-10-21T09:03:50</t>
+          <t>2026-10-29T09:03:54</t>
         </is>
       </c>
     </row>
@@ -13632,7 +13636,7 @@
         </is>
       </c>
       <c r="J57" t="n">
-        <v>32173</v>
+        <v>58424</v>
       </c>
       <c r="K57" t="inlineStr">
         <is>
@@ -13645,7 +13649,7 @@
         </is>
       </c>
       <c r="M57" t="n">
-        <v>32173</v>
+        <v>58424</v>
       </c>
       <c r="N57" t="inlineStr">
         <is>
@@ -13654,7 +13658,7 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>2026-10-21T09:04:10</t>
+          <t>2026-10-29T09:04:14</t>
         </is>
       </c>
     </row>
@@ -13809,7 +13813,7 @@
         </is>
       </c>
       <c r="J60" t="n">
-        <v>832772</v>
+        <v>833396</v>
       </c>
       <c r="K60" t="inlineStr">
         <is>
@@ -13822,7 +13826,7 @@
         </is>
       </c>
       <c r="M60" t="n">
-        <v>118021</v>
+        <v>127353</v>
       </c>
       <c r="N60" t="inlineStr">
         <is>
@@ -13831,7 +13835,7 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>2026-10-21T09:04:23</t>
+          <t>2026-10-29T09:04:27</t>
         </is>
       </c>
     </row>
@@ -13876,7 +13880,7 @@
         </is>
       </c>
       <c r="J61" t="n">
-        <v>18072328</v>
+        <v>19823197</v>
       </c>
       <c r="K61" t="inlineStr">
         <is>
@@ -13889,7 +13893,7 @@
         </is>
       </c>
       <c r="M61" t="n">
-        <v>18072328</v>
+        <v>19823197</v>
       </c>
       <c r="N61" t="inlineStr">
         <is>
@@ -13898,7 +13902,7 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>2026-10-21T09:04:33</t>
+          <t>2026-10-29T09:04:37</t>
         </is>
       </c>
     </row>
@@ -13943,7 +13947,7 @@
         </is>
       </c>
       <c r="J62" t="n">
-        <v>6208323</v>
+        <v>6620419</v>
       </c>
       <c r="K62" t="inlineStr">
         <is>
@@ -13956,7 +13960,7 @@
         </is>
       </c>
       <c r="M62" t="n">
-        <v>6208323</v>
+        <v>6620419</v>
       </c>
       <c r="N62" t="inlineStr">
         <is>
@@ -13965,7 +13969,7 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>2026-10-21T09:04:42</t>
+          <t>2026-10-29T09:04:48</t>
         </is>
       </c>
     </row>
@@ -14230,7 +14234,7 @@
         </is>
       </c>
       <c r="J67" t="n">
-        <v>55973</v>
+        <v>401908</v>
       </c>
       <c r="K67" t="inlineStr">
         <is>
@@ -14243,7 +14247,7 @@
         </is>
       </c>
       <c r="M67" t="n">
-        <v>50668</v>
+        <v>56212</v>
       </c>
       <c r="N67" t="inlineStr">
         <is>
@@ -14252,7 +14256,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>2026-10-21T09:04:59</t>
+          <t>2026-10-29T09:05:04</t>
         </is>
       </c>
     </row>
@@ -14297,7 +14301,7 @@
         </is>
       </c>
       <c r="J68" t="n">
-        <v>35062</v>
+        <v>52796</v>
       </c>
       <c r="K68" t="inlineStr">
         <is>
@@ -14310,7 +14314,7 @@
         </is>
       </c>
       <c r="M68" t="n">
-        <v>25126</v>
+        <v>27669</v>
       </c>
       <c r="N68" t="inlineStr">
         <is>
@@ -14319,7 +14323,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>2026-10-21T09:05:09</t>
+          <t>2026-10-29T09:05:13</t>
         </is>
       </c>
     </row>
@@ -14756,7 +14760,7 @@
         </is>
       </c>
       <c r="J77" t="n">
-        <v>1023034</v>
+        <v>1042361</v>
       </c>
       <c r="K77" t="inlineStr">
         <is>
@@ -14769,7 +14773,7 @@
         </is>
       </c>
       <c r="M77" t="n">
-        <v>166225</v>
+        <v>168640</v>
       </c>
       <c r="N77" t="inlineStr">
         <is>
@@ -14778,7 +14782,7 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>2026-10-21T09:05:37</t>
+          <t>2026-10-29T09:05:40</t>
         </is>
       </c>
     </row>
@@ -14886,33 +14890,33 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/watch?v=_BTD65fVrOo</t>
+        </is>
+      </c>
+      <c r="J79" t="n">
+        <v>41776</v>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>Daoko</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
           <t>https://www.youtube.com/watch?v=AQ8euxxP7JQ</t>
         </is>
       </c>
-      <c r="J79" t="n">
-        <v>35146</v>
-      </c>
-      <c r="K79" t="inlineStr">
+      <c r="M79" t="n">
+        <v>38824</v>
+      </c>
+      <c r="N79" t="inlineStr">
         <is>
           <t>Bandai Namco Filmworks Channel</t>
         </is>
       </c>
-      <c r="L79" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=AQ8euxxP7JQ</t>
-        </is>
-      </c>
-      <c r="M79" t="n">
-        <v>35146</v>
-      </c>
-      <c r="N79" t="inlineStr">
-        <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>2026-10-21T09:05:47</t>
+          <t>2026-10-29T09:05:50</t>
         </is>
       </c>
     </row>
@@ -15024,7 +15028,7 @@
         </is>
       </c>
       <c r="J81" t="n">
-        <v>2609201</v>
+        <v>2617792</v>
       </c>
       <c r="K81" t="inlineStr">
         <is>
@@ -15037,7 +15041,7 @@
         </is>
       </c>
       <c r="M81" t="n">
-        <v>57723</v>
+        <v>70090</v>
       </c>
       <c r="N81" t="inlineStr">
         <is>
@@ -15046,7 +15050,7 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>2026-10-21T09:05:57</t>
+          <t>2026-10-29T09:06:00</t>
         </is>
       </c>
     </row>
@@ -15091,7 +15095,7 @@
         </is>
       </c>
       <c r="J82" t="n">
-        <v>798675</v>
+        <v>811705</v>
       </c>
       <c r="K82" t="inlineStr">
         <is>
@@ -15104,7 +15108,7 @@
         </is>
       </c>
       <c r="M82" t="n">
-        <v>798675</v>
+        <v>811705</v>
       </c>
       <c r="N82" t="inlineStr">
         <is>
@@ -15113,7 +15117,7 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>2026-10-21T09:06:07</t>
+          <t>2026-10-29T09:06:10</t>
         </is>
       </c>
     </row>
@@ -15225,7 +15229,7 @@
         </is>
       </c>
       <c r="J84" t="n">
-        <v>449129</v>
+        <v>456949</v>
       </c>
       <c r="K84" t="inlineStr">
         <is>
@@ -15238,7 +15242,7 @@
         </is>
       </c>
       <c r="M84" t="n">
-        <v>449129</v>
+        <v>456949</v>
       </c>
       <c r="N84" t="inlineStr">
         <is>
@@ -15247,7 +15251,7 @@
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>2026-10-21T09:06:17</t>
+          <t>2026-10-29T09:06:20</t>
         </is>
       </c>
     </row>
@@ -15520,13 +15524,37 @@
           <t>てつりょー会（橘めい・庄子真央・福嶋晴菜・月城日花）</t>
         </is>
       </c>
-      <c r="I89" t="inlineStr"/>
-      <c r="J89" t="inlineStr"/>
-      <c r="K89" t="inlineStr"/>
-      <c r="L89" t="inlineStr"/>
-      <c r="M89" t="inlineStr"/>
-      <c r="N89" t="inlineStr"/>
-      <c r="O89" t="inlineStr"/>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Nbc7I6y97FI</t>
+        </is>
+      </c>
+      <c r="J89" t="n">
+        <v>37116</v>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>ぽにきゃん-Anime PONY CANYON</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Nbc7I6y97FI</t>
+        </is>
+      </c>
+      <c r="M89" t="n">
+        <v>37116</v>
+      </c>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>ぽにきゃん-Anime PONY CANYON</t>
+        </is>
+      </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>2026-10-29T09:06:41</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -15746,7 +15774,7 @@
         </is>
       </c>
       <c r="J93" t="n">
-        <v>7067</v>
+        <v>7698</v>
       </c>
       <c r="K93" t="inlineStr">
         <is>
@@ -15759,7 +15787,7 @@
         </is>
       </c>
       <c r="M93" t="n">
-        <v>7067</v>
+        <v>7698</v>
       </c>
       <c r="N93" t="inlineStr">
         <is>
@@ -15768,7 +15796,7 @@
       </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t>2026-10-21T09:07:00</t>
+          <t>2026-10-29T09:07:00</t>
         </is>
       </c>
     </row>
@@ -15809,11 +15837,11 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=dYHTC2QyGTs</t>
+          <t>https://www.youtube.com/watch?v=-UqbEqhoheE</t>
         </is>
       </c>
       <c r="J94" t="n">
-        <v>53087</v>
+        <v>53795</v>
       </c>
       <c r="K94" t="inlineStr">
         <is>
@@ -15826,7 +15854,7 @@
         </is>
       </c>
       <c r="M94" t="n">
-        <v>52832</v>
+        <v>53795</v>
       </c>
       <c r="N94" t="inlineStr">
         <is>
@@ -15835,7 +15863,7 @@
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>2026-10-21T09:07:09</t>
+          <t>2026-10-29T09:07:10</t>
         </is>
       </c>
     </row>
@@ -15880,7 +15908,7 @@
         </is>
       </c>
       <c r="J95" t="n">
-        <v>225573</v>
+        <v>227970</v>
       </c>
       <c r="K95" t="inlineStr">
         <is>
@@ -15893,7 +15921,7 @@
         </is>
       </c>
       <c r="M95" t="n">
-        <v>225573</v>
+        <v>227970</v>
       </c>
       <c r="N95" t="inlineStr">
         <is>
@@ -15902,7 +15930,7 @@
       </c>
       <c r="O95" t="inlineStr">
         <is>
-          <t>2026-10-21T09:07:19</t>
+          <t>2026-10-29T09:07:20</t>
         </is>
       </c>
     </row>
@@ -15947,7 +15975,7 @@
         </is>
       </c>
       <c r="J96" t="n">
-        <v>201975</v>
+        <v>210785</v>
       </c>
       <c r="K96" t="inlineStr">
         <is>
@@ -15960,7 +15988,7 @@
         </is>
       </c>
       <c r="M96" t="n">
-        <v>201975</v>
+        <v>210785</v>
       </c>
       <c r="N96" t="inlineStr">
         <is>
@@ -15969,7 +15997,7 @@
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t>2026-10-21T09:07:31</t>
+          <t>2026-10-29T09:07:30</t>
         </is>
       </c>
     </row>
@@ -16081,7 +16109,7 @@
         </is>
       </c>
       <c r="J98" t="n">
-        <v>35107</v>
+        <v>43301</v>
       </c>
       <c r="K98" t="inlineStr">
         <is>
@@ -16094,7 +16122,7 @@
         </is>
       </c>
       <c r="M98" t="n">
-        <v>3576</v>
+        <v>8802</v>
       </c>
       <c r="N98" t="inlineStr">
         <is>
@@ -16103,7 +16131,7 @@
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>2026-10-22T09:02:19</t>
+          <t>2026-10-29T09:07:40</t>
         </is>
       </c>
     </row>
@@ -16144,33 +16172,33 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/watch?v=fpcF8ONqzAI</t>
+        </is>
+      </c>
+      <c r="J99" t="n">
+        <v>30396</v>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>エイハブ / AHUB</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
           <t>https://www.youtube.com/watch?v=fCGf1VojfIY</t>
         </is>
       </c>
-      <c r="J99" t="n">
-        <v>1524</v>
-      </c>
-      <c r="K99" t="inlineStr">
+      <c r="M99" t="n">
+        <v>4707</v>
+      </c>
+      <c r="N99" t="inlineStr">
         <is>
           <t>博報堂DY ミュージック&amp;ピクチャーズ【Showgate】ch</t>
         </is>
       </c>
-      <c r="L99" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=fCGf1VojfIY</t>
-        </is>
-      </c>
-      <c r="M99" t="n">
-        <v>1524</v>
-      </c>
-      <c r="N99" t="inlineStr">
-        <is>
-          <t>博報堂DY ミュージック&amp;ピクチャーズ【Showgate】ch</t>
-        </is>
-      </c>
       <c r="O99" t="inlineStr">
         <is>
-          <t>2026-10-22T09:02:26</t>
+          <t>2026-10-29T09:07:49</t>
         </is>
       </c>
     </row>
@@ -16215,7 +16243,7 @@
         </is>
       </c>
       <c r="J100" t="n">
-        <v>49048</v>
+        <v>71740</v>
       </c>
       <c r="K100" t="inlineStr">
         <is>
@@ -16228,7 +16256,7 @@
         </is>
       </c>
       <c r="M100" t="n">
-        <v>58486</v>
+        <v>79870</v>
       </c>
       <c r="N100" t="inlineStr">
         <is>
@@ -16237,7 +16265,7 @@
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>2026-10-21T09:07:56</t>
+          <t>2026-10-29T09:07:59</t>
         </is>
       </c>
     </row>
@@ -16479,15 +16507,15 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=gROJDME4FTU</t>
+          <t>https://www.youtube.com/watch?v=D3D5UpQNwJo</t>
         </is>
       </c>
       <c r="J104" t="n">
-        <v>81755</v>
+        <v>388872</v>
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>East Of Eden</t>
+          <t>とあるプロジェクト公式toaru.project</t>
         </is>
       </c>
       <c r="L104" t="inlineStr">
@@ -16496,7 +16524,7 @@
         </is>
       </c>
       <c r="M104" t="n">
-        <v>249933</v>
+        <v>388872</v>
       </c>
       <c r="N104" t="inlineStr">
         <is>
@@ -16505,7 +16533,7 @@
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>2026-10-21T09:08:13</t>
+          <t>2026-10-29T09:08:09</t>
         </is>
       </c>
     </row>
@@ -16544,37 +16572,13 @@
           <t>岸田教団&amp;THE明星ロケッツ</t>
         </is>
       </c>
-      <c r="I105" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=f5kBk9DgLqk</t>
-        </is>
-      </c>
-      <c r="J105" t="n">
-        <v>219491</v>
-      </c>
-      <c r="K105" t="inlineStr">
-        <is>
-          <t>とあるプロジェクト公式toaru.project</t>
-        </is>
-      </c>
-      <c r="L105" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=f5kBk9DgLqk</t>
-        </is>
-      </c>
-      <c r="M105" t="n">
-        <v>219491</v>
-      </c>
-      <c r="N105" t="inlineStr">
-        <is>
-          <t>とあるプロジェクト公式toaru.project</t>
-        </is>
-      </c>
-      <c r="O105" t="inlineStr">
-        <is>
-          <t>2026-10-21T09:08:23</t>
-        </is>
-      </c>
+      <c r="I105" t="inlineStr"/>
+      <c r="J105" t="inlineStr"/>
+      <c r="K105" t="inlineStr"/>
+      <c r="L105" t="inlineStr"/>
+      <c r="M105" t="inlineStr"/>
+      <c r="N105" t="inlineStr"/>
+      <c r="O105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -16751,7 +16755,7 @@
         </is>
       </c>
       <c r="J108" t="n">
-        <v>1525271</v>
+        <v>1580446</v>
       </c>
       <c r="K108" t="inlineStr">
         <is>
@@ -16764,7 +16768,7 @@
         </is>
       </c>
       <c r="M108" t="n">
-        <v>419535</v>
+        <v>496989</v>
       </c>
       <c r="N108" t="inlineStr">
         <is>
@@ -16773,7 +16777,7 @@
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t>2026-10-21T09:08:33</t>
+          <t>2026-10-29T09:08:22</t>
         </is>
       </c>
     </row>
@@ -16818,7 +16822,7 @@
         </is>
       </c>
       <c r="J109" t="n">
-        <v>535938</v>
+        <v>548217</v>
       </c>
       <c r="K109" t="inlineStr">
         <is>
@@ -16831,7 +16835,7 @@
         </is>
       </c>
       <c r="M109" t="n">
-        <v>81661</v>
+        <v>88544</v>
       </c>
       <c r="N109" t="inlineStr">
         <is>
@@ -16840,7 +16844,7 @@
       </c>
       <c r="O109" t="inlineStr">
         <is>
-          <t>2026-10-21T09:08:43</t>
+          <t>2026-10-29T09:08:33</t>
         </is>
       </c>
     </row>
@@ -16885,7 +16889,7 @@
         </is>
       </c>
       <c r="J110" t="n">
-        <v>404259</v>
+        <v>461031</v>
       </c>
       <c r="K110" t="inlineStr">
         <is>
@@ -16898,7 +16902,7 @@
         </is>
       </c>
       <c r="M110" t="n">
-        <v>404259</v>
+        <v>461031</v>
       </c>
       <c r="N110" t="inlineStr">
         <is>
@@ -16907,7 +16911,7 @@
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>2026-10-21T09:08:52</t>
+          <t>2026-10-29T09:08:43</t>
         </is>
       </c>
     </row>
@@ -16952,7 +16956,7 @@
         </is>
       </c>
       <c r="J111" t="n">
-        <v>69822</v>
+        <v>84379</v>
       </c>
       <c r="K111" t="inlineStr">
         <is>
@@ -16965,7 +16969,7 @@
         </is>
       </c>
       <c r="M111" t="n">
-        <v>69822</v>
+        <v>84379</v>
       </c>
       <c r="N111" t="inlineStr">
         <is>
@@ -16974,7 +16978,7 @@
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>2026-10-21T09:09:02</t>
+          <t>2026-10-29T09:08:53</t>
         </is>
       </c>
     </row>
@@ -17019,7 +17023,7 @@
         </is>
       </c>
       <c r="J112" t="n">
-        <v>1165514</v>
+        <v>1516629</v>
       </c>
       <c r="K112" t="inlineStr">
         <is>
@@ -17031,7 +17035,7 @@
       <c r="N112" t="inlineStr"/>
       <c r="O112" t="inlineStr">
         <is>
-          <t>2026-10-21T09:09:32</t>
+          <t>2026-10-29T09:09:23</t>
         </is>
       </c>
     </row>
@@ -17115,11 +17119,11 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=UXrdCCIr58I</t>
+          <t>https://www.youtube.com/watch?v=y0htrB1JdDA</t>
         </is>
       </c>
       <c r="J114" t="n">
-        <v>42990</v>
+        <v>50806</v>
       </c>
       <c r="K114" t="inlineStr">
         <is>
@@ -17132,7 +17136,7 @@
         </is>
       </c>
       <c r="M114" t="n">
-        <v>17669</v>
+        <v>29827</v>
       </c>
       <c r="N114" t="inlineStr">
         <is>
@@ -17141,7 +17145,7 @@
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>2026-10-21T09:09:49</t>
+          <t>2026-10-29T09:09:43</t>
         </is>
       </c>
     </row>
@@ -17292,33 +17296,33 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/watch?v=j4qxC7WSd4c</t>
+        </is>
+      </c>
+      <c r="J117" t="n">
+        <v>528134</v>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>ClariS Official YouTube Channel</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
           <t>https://www.youtube.com/watch?v=pGD0RhKZk4I</t>
         </is>
       </c>
-      <c r="J117" t="n">
-        <v>351936</v>
-      </c>
-      <c r="K117" t="inlineStr">
+      <c r="M117" t="n">
+        <v>366572</v>
+      </c>
+      <c r="N117" t="inlineStr">
         <is>
           <t>アニプレックス チャンネル</t>
         </is>
       </c>
-      <c r="L117" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=pGD0RhKZk4I</t>
-        </is>
-      </c>
-      <c r="M117" t="n">
-        <v>351936</v>
-      </c>
-      <c r="N117" t="inlineStr">
-        <is>
-          <t>アニプレックス チャンネル</t>
-        </is>
-      </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>2026-10-21T09:10:11</t>
+          <t>2026-10-29T09:10:00</t>
         </is>
       </c>
     </row>
@@ -17363,7 +17367,7 @@
         </is>
       </c>
       <c r="J118" t="n">
-        <v>44354</v>
+        <v>49255</v>
       </c>
       <c r="K118" t="inlineStr">
         <is>
@@ -17376,7 +17380,7 @@
         </is>
       </c>
       <c r="M118" t="n">
-        <v>44354</v>
+        <v>49255</v>
       </c>
       <c r="N118" t="inlineStr">
         <is>
@@ -17385,7 +17389,7 @@
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>2026-10-21T09:10:21</t>
+          <t>2026-10-29T09:10:10</t>
         </is>
       </c>
     </row>
@@ -17564,7 +17568,7 @@
         </is>
       </c>
       <c r="J121" t="n">
-        <v>552489</v>
+        <v>847284</v>
       </c>
       <c r="K121" t="inlineStr">
         <is>
@@ -17577,7 +17581,7 @@
         </is>
       </c>
       <c r="M121" t="n">
-        <v>319203</v>
+        <v>436987</v>
       </c>
       <c r="N121" t="inlineStr">
         <is>
@@ -17586,7 +17590,7 @@
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>2026-10-21T09:10:30</t>
+          <t>2026-10-29T09:10:19</t>
         </is>
       </c>
     </row>
@@ -17631,7 +17635,7 @@
         </is>
       </c>
       <c r="J122" t="n">
-        <v>552489</v>
+        <v>847284</v>
       </c>
       <c r="K122" t="inlineStr">
         <is>
@@ -17644,7 +17648,7 @@
         </is>
       </c>
       <c r="M122" t="n">
-        <v>552489</v>
+        <v>847284</v>
       </c>
       <c r="N122" t="inlineStr">
         <is>
@@ -17653,7 +17657,7 @@
       </c>
       <c r="O122" t="inlineStr">
         <is>
-          <t>2026-10-21T09:10:39</t>
+          <t>2026-10-29T09:10:29</t>
         </is>
       </c>
     </row>
@@ -17741,7 +17745,7 @@
         </is>
       </c>
       <c r="J124" t="n">
-        <v>5313011</v>
+        <v>5329638</v>
       </c>
       <c r="K124" t="inlineStr">
         <is>
@@ -17754,7 +17758,7 @@
         </is>
       </c>
       <c r="M124" t="n">
-        <v>48623</v>
+        <v>57967</v>
       </c>
       <c r="N124" t="inlineStr">
         <is>
@@ -17763,7 +17767,7 @@
       </c>
       <c r="O124" t="inlineStr">
         <is>
-          <t>2026-10-21T09:10:51</t>
+          <t>2026-10-29T09:10:41</t>
         </is>
       </c>
     </row>
@@ -17808,7 +17812,7 @@
         </is>
       </c>
       <c r="J125" t="n">
-        <v>1006082</v>
+        <v>1009851</v>
       </c>
       <c r="K125" t="inlineStr">
         <is>
@@ -17821,7 +17825,7 @@
         </is>
       </c>
       <c r="M125" t="n">
-        <v>33156</v>
+        <v>37223</v>
       </c>
       <c r="N125" t="inlineStr">
         <is>
@@ -17830,7 +17834,7 @@
       </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>2026-10-21T09:11:02</t>
+          <t>2026-10-29T09:10:59</t>
         </is>
       </c>
     </row>
@@ -17875,7 +17879,7 @@
         </is>
       </c>
       <c r="J126" t="n">
-        <v>2568819</v>
+        <v>2977770</v>
       </c>
       <c r="K126" t="inlineStr">
         <is>
@@ -17888,7 +17892,7 @@
         </is>
       </c>
       <c r="M126" t="n">
-        <v>2568819</v>
+        <v>2977770</v>
       </c>
       <c r="N126" t="inlineStr">
         <is>
@@ -17897,7 +17901,7 @@
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>2026-10-21T09:11:11</t>
+          <t>2026-10-29T09:11:09</t>
         </is>
       </c>
     </row>
@@ -17942,7 +17946,7 @@
         </is>
       </c>
       <c r="J127" t="n">
-        <v>659004</v>
+        <v>2895117</v>
       </c>
       <c r="K127" t="inlineStr">
         <is>
@@ -17955,7 +17959,7 @@
         </is>
       </c>
       <c r="M127" t="n">
-        <v>566601</v>
+        <v>646598</v>
       </c>
       <c r="N127" t="inlineStr">
         <is>
@@ -17964,7 +17968,7 @@
       </c>
       <c r="O127" t="inlineStr">
         <is>
-          <t>2026-10-21T09:11:23</t>
+          <t>2026-10-29T09:11:21</t>
         </is>
       </c>
     </row>
@@ -18009,7 +18013,7 @@
         </is>
       </c>
       <c r="J128" t="n">
-        <v>613922</v>
+        <v>826552</v>
       </c>
       <c r="K128" t="inlineStr">
         <is>
@@ -18022,7 +18026,7 @@
         </is>
       </c>
       <c r="M128" t="n">
-        <v>613922</v>
+        <v>826552</v>
       </c>
       <c r="N128" t="inlineStr">
         <is>
@@ -18031,7 +18035,7 @@
       </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t>2026-10-21T09:11:33</t>
+          <t>2026-10-29T09:11:31</t>
         </is>
       </c>
     </row>
@@ -18076,7 +18080,7 @@
         </is>
       </c>
       <c r="J129" t="n">
-        <v>613922</v>
+        <v>826827</v>
       </c>
       <c r="K129" t="inlineStr">
         <is>
@@ -18089,7 +18093,7 @@
         </is>
       </c>
       <c r="M129" t="n">
-        <v>210119</v>
+        <v>234831</v>
       </c>
       <c r="N129" t="inlineStr">
         <is>
@@ -18098,7 +18102,7 @@
       </c>
       <c r="O129" t="inlineStr">
         <is>
-          <t>2026-10-21T09:11:43</t>
+          <t>2026-10-29T09:11:40</t>
         </is>
       </c>
     </row>
@@ -18143,7 +18147,7 @@
         </is>
       </c>
       <c r="J130" t="n">
-        <v>549396</v>
+        <v>572574</v>
       </c>
       <c r="K130" t="inlineStr">
         <is>
@@ -18156,7 +18160,7 @@
         </is>
       </c>
       <c r="M130" t="n">
-        <v>549396</v>
+        <v>572574</v>
       </c>
       <c r="N130" t="inlineStr">
         <is>
@@ -18165,7 +18169,7 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>2026-10-21T09:11:50</t>
+          <t>2026-10-29T09:11:47</t>
         </is>
       </c>
     </row>
@@ -18210,7 +18214,7 @@
         </is>
       </c>
       <c r="J131" t="n">
-        <v>549396</v>
+        <v>572574</v>
       </c>
       <c r="K131" t="inlineStr">
         <is>
@@ -18223,7 +18227,7 @@
         </is>
       </c>
       <c r="M131" t="n">
-        <v>549396</v>
+        <v>572574</v>
       </c>
       <c r="N131" t="inlineStr">
         <is>
@@ -18232,7 +18236,7 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>2026-10-21T09:11:56</t>
+          <t>2026-10-29T09:11:54</t>
         </is>
       </c>
     </row>
@@ -18277,7 +18281,7 @@
         </is>
       </c>
       <c r="J132" t="n">
-        <v>571020</v>
+        <v>691698</v>
       </c>
       <c r="K132" t="inlineStr">
         <is>
@@ -18290,7 +18294,7 @@
         </is>
       </c>
       <c r="M132" t="n">
-        <v>571020</v>
+        <v>691698</v>
       </c>
       <c r="N132" t="inlineStr">
         <is>
@@ -18299,7 +18303,7 @@
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t>2026-10-22T09:03:04</t>
+          <t>2026-10-29T09:12:03</t>
         </is>
       </c>
     </row>
@@ -18344,7 +18348,7 @@
         </is>
       </c>
       <c r="J133" t="n">
-        <v>166617</v>
+        <v>199771</v>
       </c>
       <c r="K133" t="inlineStr">
         <is>
@@ -18357,7 +18361,7 @@
         </is>
       </c>
       <c r="M133" t="n">
-        <v>166617</v>
+        <v>199771</v>
       </c>
       <c r="N133" t="inlineStr">
         <is>
@@ -18366,7 +18370,7 @@
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t>2026-10-21T09:12:06</t>
+          <t>2026-10-29T09:12:13</t>
         </is>
       </c>
     </row>
@@ -18411,7 +18415,7 @@
         </is>
       </c>
       <c r="J134" t="n">
-        <v>17605</v>
+        <v>19696</v>
       </c>
       <c r="K134" t="inlineStr">
         <is>
@@ -18424,7 +18428,7 @@
         </is>
       </c>
       <c r="M134" t="n">
-        <v>17605</v>
+        <v>19696</v>
       </c>
       <c r="N134" t="inlineStr">
         <is>
@@ -18433,7 +18437,7 @@
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>2026-10-21T09:12:15</t>
+          <t>2026-10-29T09:12:22</t>
         </is>
       </c>
     </row>
@@ -18478,7 +18482,7 @@
         </is>
       </c>
       <c r="J135" t="n">
-        <v>41732</v>
+        <v>45974</v>
       </c>
       <c r="K135" t="inlineStr">
         <is>
@@ -18491,7 +18495,7 @@
         </is>
       </c>
       <c r="M135" t="n">
-        <v>41732</v>
+        <v>45974</v>
       </c>
       <c r="N135" t="inlineStr">
         <is>
@@ -18500,7 +18504,7 @@
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>2026-10-21T09:12:24</t>
+          <t>2026-10-29T09:12:32</t>
         </is>
       </c>
     </row>
@@ -18722,7 +18726,7 @@
         </is>
       </c>
       <c r="J139" t="n">
-        <v>733028</v>
+        <v>790828</v>
       </c>
       <c r="K139" t="inlineStr">
         <is>
@@ -18735,7 +18739,7 @@
         </is>
       </c>
       <c r="M139" t="n">
-        <v>733028</v>
+        <v>790828</v>
       </c>
       <c r="N139" t="inlineStr">
         <is>
@@ -18744,7 +18748,7 @@
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>2026-10-21T09:12:36</t>
+          <t>2026-10-29T09:12:44</t>
         </is>
       </c>
     </row>
@@ -18828,7 +18832,7 @@
         </is>
       </c>
       <c r="J141" t="n">
-        <v>5315</v>
+        <v>5869</v>
       </c>
       <c r="K141" t="inlineStr">
         <is>
@@ -18841,7 +18845,7 @@
         </is>
       </c>
       <c r="M141" t="n">
-        <v>5315</v>
+        <v>5869</v>
       </c>
       <c r="N141" t="inlineStr">
         <is>
@@ -18850,7 +18854,7 @@
       </c>
       <c r="O141" t="inlineStr">
         <is>
-          <t>2026-10-22T09:03:19</t>
+          <t>2026-10-29T09:12:56</t>
         </is>
       </c>
     </row>
@@ -18895,7 +18899,7 @@
         </is>
       </c>
       <c r="J142" t="n">
-        <v>143386</v>
+        <v>148048</v>
       </c>
       <c r="K142" t="inlineStr">
         <is>
@@ -18908,7 +18912,7 @@
         </is>
       </c>
       <c r="M142" t="n">
-        <v>42915</v>
+        <v>62744</v>
       </c>
       <c r="N142" t="inlineStr">
         <is>
@@ -18917,7 +18921,7 @@
       </c>
       <c r="O142" t="inlineStr">
         <is>
-          <t>2026-10-21T09:12:48</t>
+          <t>2026-10-29T09:13:06</t>
         </is>
       </c>
     </row>
@@ -18962,7 +18966,7 @@
         </is>
       </c>
       <c r="J143" t="n">
-        <v>143386</v>
+        <v>147999</v>
       </c>
       <c r="K143" t="inlineStr">
         <is>
@@ -18975,7 +18979,7 @@
         </is>
       </c>
       <c r="M143" t="n">
-        <v>42503</v>
+        <v>70149</v>
       </c>
       <c r="N143" t="inlineStr">
         <is>
@@ -18984,7 +18988,7 @@
       </c>
       <c r="O143" t="inlineStr">
         <is>
-          <t>2026-10-21T09:12:57</t>
+          <t>2026-10-29T09:13:16</t>
         </is>
       </c>
     </row>
@@ -19096,7 +19100,7 @@
         </is>
       </c>
       <c r="J145" t="n">
-        <v>350896</v>
+        <v>357682</v>
       </c>
       <c r="K145" t="inlineStr">
         <is>
@@ -19109,7 +19113,7 @@
         </is>
       </c>
       <c r="M145" t="n">
-        <v>350896</v>
+        <v>357682</v>
       </c>
       <c r="N145" t="inlineStr">
         <is>
@@ -19118,7 +19122,7 @@
       </c>
       <c r="O145" t="inlineStr">
         <is>
-          <t>2026-10-21T09:13:07</t>
+          <t>2026-10-29T09:13:27</t>
         </is>
       </c>
     </row>
@@ -19273,7 +19277,7 @@
         </is>
       </c>
       <c r="J148" t="n">
-        <v>218630</v>
+        <v>329401</v>
       </c>
       <c r="K148" t="inlineStr">
         <is>
@@ -19286,7 +19290,7 @@
         </is>
       </c>
       <c r="M148" t="n">
-        <v>52695</v>
+        <v>57978</v>
       </c>
       <c r="N148" t="inlineStr">
         <is>
@@ -19295,7 +19299,7 @@
       </c>
       <c r="O148" t="inlineStr">
         <is>
-          <t>2026-10-21T09:13:19</t>
+          <t>2026-10-29T09:13:40</t>
         </is>
       </c>
     </row>
@@ -19407,7 +19411,7 @@
         </is>
       </c>
       <c r="J150" t="n">
-        <v>125799</v>
+        <v>143382</v>
       </c>
       <c r="K150" t="inlineStr">
         <is>
@@ -19420,7 +19424,7 @@
         </is>
       </c>
       <c r="M150" t="n">
-        <v>125799</v>
+        <v>143382</v>
       </c>
       <c r="N150" t="inlineStr">
         <is>
@@ -19429,7 +19433,7 @@
       </c>
       <c r="O150" t="inlineStr">
         <is>
-          <t>2026-10-21T09:13:29</t>
+          <t>2026-10-29T09:13:50</t>
         </is>
       </c>
     </row>
@@ -19474,7 +19478,7 @@
         </is>
       </c>
       <c r="J151" t="n">
-        <v>46508</v>
+        <v>52283</v>
       </c>
       <c r="K151" t="inlineStr">
         <is>
@@ -19487,7 +19491,7 @@
         </is>
       </c>
       <c r="M151" t="n">
-        <v>46508</v>
+        <v>52283</v>
       </c>
       <c r="N151" t="inlineStr">
         <is>
@@ -19496,7 +19500,7 @@
       </c>
       <c r="O151" t="inlineStr">
         <is>
-          <t>2026-10-21T09:13:38</t>
+          <t>2026-10-29T09:14:00</t>
         </is>
       </c>
     </row>
@@ -19627,7 +19631,7 @@
         </is>
       </c>
       <c r="J154" t="n">
-        <v>121795</v>
+        <v>144443</v>
       </c>
       <c r="K154" t="inlineStr">
         <is>
@@ -19640,7 +19644,7 @@
         </is>
       </c>
       <c r="M154" t="n">
-        <v>121795</v>
+        <v>144443</v>
       </c>
       <c r="N154" t="inlineStr">
         <is>
@@ -19649,7 +19653,7 @@
       </c>
       <c r="O154" t="inlineStr">
         <is>
-          <t>2026-10-21T09:13:47</t>
+          <t>2026-10-29T09:14:10</t>
         </is>
       </c>
     </row>
@@ -19694,7 +19698,7 @@
         </is>
       </c>
       <c r="J155" t="n">
-        <v>35166</v>
+        <v>50400</v>
       </c>
       <c r="K155" t="inlineStr">
         <is>
@@ -19707,7 +19711,7 @@
         </is>
       </c>
       <c r="M155" t="n">
-        <v>35166</v>
+        <v>50400</v>
       </c>
       <c r="N155" t="inlineStr">
         <is>
@@ -19716,7 +19720,7 @@
       </c>
       <c r="O155" t="inlineStr">
         <is>
-          <t>2026-10-21T09:13:57</t>
+          <t>2026-10-29T09:14:20</t>
         </is>
       </c>
     </row>
@@ -19895,7 +19899,7 @@
         </is>
       </c>
       <c r="J158" t="n">
-        <v>1285938</v>
+        <v>1308108</v>
       </c>
       <c r="K158" t="inlineStr">
         <is>
@@ -19908,7 +19912,7 @@
         </is>
       </c>
       <c r="M158" t="n">
-        <v>471606</v>
+        <v>480333</v>
       </c>
       <c r="N158" t="inlineStr">
         <is>
@@ -19917,7 +19921,7 @@
       </c>
       <c r="O158" t="inlineStr">
         <is>
-          <t>2026-10-21T09:14:17</t>
+          <t>2026-10-29T09:14:30</t>
         </is>
       </c>
     </row>
@@ -19958,11 +19962,11 @@
       </c>
       <c r="I159" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=fb_iz-tfUdg</t>
+          <t>https://www.youtube.com/watch?v=f7QJtQL-LFU</t>
         </is>
       </c>
       <c r="J159" t="n">
-        <v>198739</v>
+        <v>1979605</v>
       </c>
       <c r="K159" t="inlineStr">
         <is>
@@ -19971,11 +19975,11 @@
       </c>
       <c r="L159" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=fb_iz-tfUdg</t>
+          <t>https://www.youtube.com/watch?v=f7QJtQL-LFU</t>
         </is>
       </c>
       <c r="M159" t="n">
-        <v>198739</v>
+        <v>1979605</v>
       </c>
       <c r="N159" t="inlineStr">
         <is>
@@ -19984,7 +19988,7 @@
       </c>
       <c r="O159" t="inlineStr">
         <is>
-          <t>2026-10-21T09:14:27</t>
+          <t>2026-10-29T09:14:40</t>
         </is>
       </c>
     </row>
@@ -20029,7 +20033,7 @@
         </is>
       </c>
       <c r="J160" t="n">
-        <v>551370</v>
+        <v>562825</v>
       </c>
       <c r="K160" t="inlineStr">
         <is>
@@ -20042,7 +20046,7 @@
         </is>
       </c>
       <c r="M160" t="n">
-        <v>463007</v>
+        <v>469764</v>
       </c>
       <c r="N160" t="inlineStr">
         <is>
@@ -20051,7 +20055,7 @@
       </c>
       <c r="O160" t="inlineStr">
         <is>
-          <t>2026-10-21T09:14:36</t>
+          <t>2026-10-29T09:14:50</t>
         </is>
       </c>
     </row>
@@ -20092,33 +20096,33 @@
       </c>
       <c r="I161" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/watch?v=p0R_VblbHsc</t>
+        </is>
+      </c>
+      <c r="J161" t="n">
+        <v>1242898</v>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>KID PHENOMENON</t>
+        </is>
+      </c>
+      <c r="L161" t="inlineStr">
+        <is>
           <t>https://www.youtube.com/watch?v=EwFd3PnUqso</t>
         </is>
       </c>
-      <c r="J161" t="n">
-        <v>55156</v>
-      </c>
-      <c r="K161" t="inlineStr">
+      <c r="M161" t="n">
+        <v>83164</v>
+      </c>
+      <c r="N161" t="inlineStr">
         <is>
           <t>NBCUniversal Anime/Music</t>
         </is>
       </c>
-      <c r="L161" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=EwFd3PnUqso</t>
-        </is>
-      </c>
-      <c r="M161" t="n">
-        <v>55156</v>
-      </c>
-      <c r="N161" t="inlineStr">
-        <is>
-          <t>NBCUniversal Anime/Music</t>
-        </is>
-      </c>
       <c r="O161" t="inlineStr">
         <is>
-          <t>2026-10-21T09:14:46</t>
+          <t>2026-10-29T09:15:01</t>
         </is>
       </c>
     </row>
@@ -20206,7 +20210,7 @@
         </is>
       </c>
       <c r="J163" t="n">
-        <v>284997</v>
+        <v>286116</v>
       </c>
       <c r="K163" t="inlineStr">
         <is>
@@ -20219,7 +20223,7 @@
         </is>
       </c>
       <c r="M163" t="n">
-        <v>284997</v>
+        <v>286116</v>
       </c>
       <c r="N163" t="inlineStr">
         <is>
@@ -20228,7 +20232,7 @@
       </c>
       <c r="O163" t="inlineStr">
         <is>
-          <t>2026-10-21T09:14:59</t>
+          <t>2026-10-29T09:15:14</t>
         </is>
       </c>
     </row>
@@ -20273,7 +20277,7 @@
         </is>
       </c>
       <c r="J164" t="n">
-        <v>368620</v>
+        <v>417543</v>
       </c>
       <c r="K164" t="inlineStr">
         <is>
@@ -20286,7 +20290,7 @@
         </is>
       </c>
       <c r="M164" t="n">
-        <v>368620</v>
+        <v>417543</v>
       </c>
       <c r="N164" t="inlineStr">
         <is>
@@ -20295,7 +20299,7 @@
       </c>
       <c r="O164" t="inlineStr">
         <is>
-          <t>2026-10-21T09:15:08</t>
+          <t>2026-10-29T09:15:24</t>
         </is>
       </c>
     </row>
@@ -20541,19 +20545,29 @@
         </is>
       </c>
       <c r="J168" t="n">
-        <v>3300190</v>
+        <v>3325293</v>
       </c>
       <c r="K168" t="inlineStr">
         <is>
           <t>りりあ。</t>
         </is>
       </c>
-      <c r="L168" t="inlineStr"/>
-      <c r="M168" t="inlineStr"/>
-      <c r="N168" t="inlineStr"/>
+      <c r="L168" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=wv6mh_cVIdQ</t>
+        </is>
+      </c>
+      <c r="M168" t="n">
+        <v>120682</v>
+      </c>
+      <c r="N168" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
       <c r="O168" t="inlineStr">
         <is>
-          <t>2026-10-21T09:15:38</t>
+          <t>2026-10-29T09:15:34</t>
         </is>
       </c>
     </row>
@@ -20708,7 +20722,7 @@
         </is>
       </c>
       <c r="J171" t="n">
-        <v>245681</v>
+        <v>250589</v>
       </c>
       <c r="K171" t="inlineStr">
         <is>
@@ -20721,7 +20735,7 @@
         </is>
       </c>
       <c r="M171" t="n">
-        <v>245681</v>
+        <v>250589</v>
       </c>
       <c r="N171" t="inlineStr">
         <is>
@@ -20730,7 +20744,7 @@
       </c>
       <c r="O171" t="inlineStr">
         <is>
-          <t>2026-10-21T09:15:59</t>
+          <t>2026-10-29T09:15:50</t>
         </is>
       </c>
     </row>
@@ -20818,7 +20832,7 @@
         </is>
       </c>
       <c r="J173" t="n">
-        <v>9260465</v>
+        <v>9333743</v>
       </c>
       <c r="K173" t="inlineStr">
         <is>
@@ -20830,7 +20844,7 @@
       <c r="N173" t="inlineStr"/>
       <c r="O173" t="inlineStr">
         <is>
-          <t>2026-10-21T09:16:45</t>
+          <t>2026-10-29T09:16:29</t>
         </is>
       </c>
     </row>
@@ -21190,7 +21204,7 @@
         </is>
       </c>
       <c r="J181" t="n">
-        <v>816684</v>
+        <v>821833</v>
       </c>
       <c r="K181" t="inlineStr">
         <is>
@@ -21202,7 +21216,7 @@
       <c r="N181" t="inlineStr"/>
       <c r="O181" t="inlineStr">
         <is>
-          <t>2026-10-21T09:17:22</t>
+          <t>2026-10-29T09:17:13</t>
         </is>
       </c>
     </row>
@@ -21290,7 +21304,7 @@
         </is>
       </c>
       <c r="J183" t="n">
-        <v>220388</v>
+        <v>233269</v>
       </c>
       <c r="K183" t="inlineStr">
         <is>
@@ -21303,7 +21317,7 @@
         </is>
       </c>
       <c r="M183" t="n">
-        <v>220388</v>
+        <v>233269</v>
       </c>
       <c r="N183" t="inlineStr">
         <is>
@@ -21312,7 +21326,7 @@
       </c>
       <c r="O183" t="inlineStr">
         <is>
-          <t>2026-10-21T09:17:39</t>
+          <t>2026-10-29T09:17:28</t>
         </is>
       </c>
     </row>
@@ -21357,7 +21371,7 @@
         </is>
       </c>
       <c r="J184" t="n">
-        <v>2078765</v>
+        <v>2082452</v>
       </c>
       <c r="K184" t="inlineStr">
         <is>
@@ -21370,7 +21384,7 @@
         </is>
       </c>
       <c r="M184" t="n">
-        <v>2078765</v>
+        <v>2082452</v>
       </c>
       <c r="N184" t="inlineStr">
         <is>
@@ -21379,7 +21393,7 @@
       </c>
       <c r="O184" t="inlineStr">
         <is>
-          <t>2026-10-21T09:17:48</t>
+          <t>2026-10-29T09:17:38</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-10-31
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M188"/>
+  <dimension ref="A1:M189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5487,7 +5487,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>メカザムライ</t>
         </is>
       </c>
       <c r="E91" t="b">
@@ -5495,42 +5495,26 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>2026年10月4日（日）〜 TOKYO MX・読売テレビ・中京テレビほか</t>
+          <t>2026年11月2日（月）～ YouTube・Xほか</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>studio A-CAT</t>
-        </is>
-      </c>
-      <c r="I91" t="inlineStr">
-        <is>
-          <t>UNSTOPPABLE</t>
-        </is>
-      </c>
-      <c r="J91" t="inlineStr">
-        <is>
-          <t>FLOW</t>
-        </is>
-      </c>
-      <c r="K91" t="inlineStr">
-        <is>
-          <t>MY WAY</t>
-        </is>
-      </c>
-      <c r="L91" t="inlineStr">
-        <is>
-          <t>ASTERISM</t>
-        </is>
-      </c>
+          <t>Plott</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr"/>
+      <c r="J91" t="inlineStr"/>
+      <c r="K91" t="inlineStr"/>
+      <c r="L91" t="inlineStr"/>
       <c r="M91" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25525</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=29288</t>
         </is>
       </c>
     </row>
@@ -5548,11 +5532,11 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>メダリスト</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="E92" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
@@ -5561,37 +5545,37 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>2025年1月4日（土）～2025年3月29日（土） テレビ朝日系にて 【再放送】 2026年10月1日（木）〜 TOKYO MXにて</t>
+          <t>2026年10月4日（日）〜 TOKYO MX・読売テレビ・中京テレビほか</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>ENGI</t>
+          <t>studio A-CAT</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>BOW AND ARROW</t>
+          <t>UNSTOPPABLE</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>米津玄師</t>
+          <t>FLOW</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>アタシのドレス</t>
+          <t>MY WAY</t>
         </is>
       </c>
       <c r="L92" t="inlineStr">
         <is>
-          <t>ねぐせ。</t>
+          <t>ASTERISM</t>
         </is>
       </c>
       <c r="M92" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=21115</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25525</t>
         </is>
       </c>
     </row>
@@ -5609,11 +5593,11 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>野生のラスボスが現れた！ 第2期</t>
+          <t>メダリスト</t>
         </is>
       </c>
       <c r="E93" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F93" t="inlineStr">
         <is>
@@ -5622,37 +5606,37 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>2026年10月3日（土）～ TOKYO MXほか</t>
+          <t>2025年1月4日（土）～2025年3月29日（土） テレビ朝日系にて 【再放送】 2026年10月1日（木）〜 TOKYO MXにて</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>ワオワールド</t>
+          <t>ENGI</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>Melodic Impact</t>
+          <t>BOW AND ARROW</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>Suspended 4th</t>
+          <t>米津玄師</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>揺れてスカート</t>
+          <t>アタシのドレス</t>
         </is>
       </c>
       <c r="L93" t="inlineStr">
         <is>
-          <t>ちゃくら</t>
+          <t>ねぐせ。</t>
         </is>
       </c>
       <c r="M93" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27288</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=21115</t>
         </is>
       </c>
     </row>
@@ -5670,7 +5654,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>ゆうさんち！from 遊ハち</t>
+          <t>野生のラスボスが現れた！ 第2期</t>
         </is>
       </c>
       <c r="E94" t="b">
@@ -5683,21 +5667,37 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>2026年10月5日（月）～ フジテレビ・カンテレにて</t>
+          <t>2026年10月3日（土）～ TOKYO MXほか</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>ファンワークス</t>
-        </is>
-      </c>
-      <c r="I94" t="inlineStr"/>
-      <c r="J94" t="inlineStr"/>
-      <c r="K94" t="inlineStr"/>
-      <c r="L94" t="inlineStr"/>
+          <t>ワオワールド</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Melodic Impact</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>Suspended 4th</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>揺れてスカート</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>ちゃくら</t>
+        </is>
+      </c>
       <c r="M94" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28884</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27288</t>
         </is>
       </c>
     </row>
@@ -5715,7 +5715,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>ゆるゆる図鑑</t>
+          <t>ゆうさんち！from 遊ハち</t>
         </is>
       </c>
       <c r="E95" t="b">
@@ -5728,12 +5728,12 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>2026年10月4日（日）～ テレ東系列6局ネット「アニもり！」内にて</t>
+          <t>2026年10月5日（月）～ フジテレビ・カンテレにて</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>Imagica Infos</t>
+          <t>ファンワークス</t>
         </is>
       </c>
       <c r="I95" t="inlineStr"/>
@@ -5742,7 +5742,7 @@
       <c r="L95" t="inlineStr"/>
       <c r="M95" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28579</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28884</t>
         </is>
       </c>
     </row>
@@ -5760,7 +5760,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>ゆるゆる図鑑</t>
         </is>
       </c>
       <c r="E96" t="b">
@@ -5773,37 +5773,21 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>第1クール：2026年4月12日（日）～2026年6月28日（日） 第2クール：2026年10月11日（日）～ MBS／TBS系全国28局ネットにて</t>
+          <t>2026年10月4日（日）～ テレ東系列6局ネット「アニもり！」内にて</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>SILVER LINK.</t>
-        </is>
-      </c>
-      <c r="I96" t="inlineStr">
-        <is>
-          <t>What's "KAZOKU"</t>
-        </is>
-      </c>
-      <c r="J96" t="inlineStr">
-        <is>
-          <t>櫻坂46</t>
-        </is>
-      </c>
-      <c r="K96" t="inlineStr">
-        <is>
-          <t>Shalala</t>
-        </is>
-      </c>
-      <c r="L96" t="inlineStr">
-        <is>
-          <t>ピラフ星人</t>
-        </is>
-      </c>
+          <t>Imagica Infos</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr"/>
+      <c r="J96" t="inlineStr"/>
+      <c r="K96" t="inlineStr"/>
+      <c r="L96" t="inlineStr"/>
       <c r="M96" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25032</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28579</t>
         </is>
       </c>
     </row>
@@ -5821,7 +5805,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>弱気MAX令嬢なのに、辣腕婚約者様の賭けに乗ってしまった</t>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
         </is>
       </c>
       <c r="E97" t="b">
@@ -5834,37 +5818,37 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>2026年10月4日（日）～ TOKYO MXほか</t>
+          <t>第1クール：2026年4月12日（日）～2026年6月28日（日） 第2クール：2026年10月11日（日）～ MBS／TBS系全国28局ネットにて</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>寿門堂</t>
+          <t>SILVER LINK.</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>強気MAX宣言</t>
+          <t>What's "KAZOKU"</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>鈴木このみ</t>
+          <t>櫻坂46</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>夜明けまでに</t>
+          <t>Shalala</t>
         </is>
       </c>
       <c r="L97" t="inlineStr">
         <is>
-          <t>伊藤美来</t>
+          <t>ピラフ星人</t>
         </is>
       </c>
       <c r="M97" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26947</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25032</t>
         </is>
       </c>
     </row>
@@ -5882,7 +5866,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>楽楽飯店</t>
+          <t>弱気MAX令嬢なのに、辣腕婚約者様の賭けに乗ってしまった</t>
         </is>
       </c>
       <c r="E98" t="b">
@@ -5890,22 +5874,42 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>2026年9月18日（金）～ 公式YouTubeチャンネルにて</t>
-        </is>
-      </c>
-      <c r="H98" t="inlineStr"/>
-      <c r="I98" t="inlineStr"/>
-      <c r="J98" t="inlineStr"/>
-      <c r="K98" t="inlineStr"/>
-      <c r="L98" t="inlineStr"/>
+          <t>2026年10月4日（日）～ TOKYO MXほか</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>寿門堂</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>強気MAX宣言</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>鈴木このみ</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>夜明けまでに</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>伊藤美来</t>
+        </is>
+      </c>
       <c r="M98" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28945</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26947</t>
         </is>
       </c>
     </row>
@@ -5923,34 +5927,30 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>ラブライブ！虹ヶ咲学園スクールアイドル同好会 第2期</t>
+          <t>楽楽飯店</t>
         </is>
       </c>
       <c r="E99" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>2022年4月2日（土）～2022年6月25日（土） TOKYO MXほか 【再放送】 2026年9月30日（水）〜 BS日テレにて</t>
-        </is>
-      </c>
-      <c r="H99" t="inlineStr">
-        <is>
-          <t>サンライズ</t>
-        </is>
-      </c>
+          <t>2026年9月18日（金）～ 公式YouTubeチャンネルにて</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr"/>
       <c r="I99" t="inlineStr"/>
       <c r="J99" t="inlineStr"/>
       <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr"/>
       <c r="M99" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=14120</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28945</t>
         </is>
       </c>
     </row>
@@ -5968,11 +5968,11 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>らんま1/2 第3期</t>
+          <t>ラブライブ！虹ヶ咲学園スクールアイドル同好会 第2期</t>
         </is>
       </c>
       <c r="E100" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F100" t="inlineStr">
         <is>
@@ -5981,33 +5981,21 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>2026年10月3日（土）～ 日本テレビにて</t>
-        </is>
-      </c>
-      <c r="H100" t="inlineStr"/>
-      <c r="I100" t="inlineStr">
-        <is>
-          <t>素直未満</t>
-        </is>
-      </c>
-      <c r="J100" t="inlineStr">
-        <is>
-          <t>ふみの</t>
-        </is>
-      </c>
-      <c r="K100" t="inlineStr">
-        <is>
-          <t>かわいくない</t>
-        </is>
-      </c>
-      <c r="L100" t="inlineStr">
-        <is>
-          <t>『ユイカ』</t>
-        </is>
-      </c>
+          <t>2022年4月2日（土）～2022年6月25日（土） TOKYO MXほか 【再放送】 2026年9月30日（水）〜 BS日テレにて</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>サンライズ</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr"/>
+      <c r="J100" t="inlineStr"/>
+      <c r="K100" t="inlineStr"/>
+      <c r="L100" t="inlineStr"/>
       <c r="M100" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28013</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=14120</t>
         </is>
       </c>
     </row>
@@ -6025,7 +6013,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>LEGO® ONE PIECE</t>
+          <t>らんま1/2 第3期</t>
         </is>
       </c>
       <c r="E101" t="b">
@@ -6033,22 +6021,38 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>2026年9月29日（火） Netflixにて</t>
+          <t>2026年10月3日（土）～ 日本テレビにて</t>
         </is>
       </c>
       <c r="H101" t="inlineStr"/>
-      <c r="I101" t="inlineStr"/>
-      <c r="J101" t="inlineStr"/>
-      <c r="K101" t="inlineStr"/>
-      <c r="L101" t="inlineStr"/>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>素直未満</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>ふみの</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>かわいくない</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>『ユイカ』</t>
+        </is>
+      </c>
       <c r="M101" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28168</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28013</t>
         </is>
       </c>
     </row>
@@ -6066,7 +6070,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>ロメリア戦記</t>
+          <t>LEGO® ONE PIECE</t>
         </is>
       </c>
       <c r="E102" t="b">
@@ -6074,42 +6078,22 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>2026年10月5日（月）～ TOKYO MXほか</t>
-        </is>
-      </c>
-      <c r="H102" t="inlineStr">
-        <is>
-          <t>Atra</t>
-        </is>
-      </c>
-      <c r="I102" t="inlineStr">
-        <is>
-          <t>暁に鳴る</t>
-        </is>
-      </c>
-      <c r="J102" t="inlineStr">
-        <is>
-          <t>超学生</t>
-        </is>
-      </c>
-      <c r="K102" t="inlineStr">
-        <is>
-          <t>Nightfall feat. Maika Loubté</t>
-        </is>
-      </c>
-      <c r="L102" t="inlineStr">
-        <is>
-          <t>KOHTA YAMAMOTO</t>
-        </is>
-      </c>
+          <t>2026年9月29日（火） Netflixにて</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr"/>
+      <c r="I102" t="inlineStr"/>
+      <c r="J102" t="inlineStr"/>
+      <c r="K102" t="inlineStr"/>
+      <c r="L102" t="inlineStr"/>
       <c r="M102" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27077</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28168</t>
         </is>
       </c>
     </row>
@@ -6127,7 +6111,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>わたしの幸せな結婚 特別篇</t>
+          <t>ロメリア戦記</t>
         </is>
       </c>
       <c r="E103" t="b">
@@ -6140,55 +6124,55 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>2026年10月25日（日）～ TOKYO MXほかにて</t>
+          <t>2026年10月5日（月）～ TOKYO MXほか</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>キネマシトラス</t>
+          <t>Atra</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>幸せで涙が出るのは。</t>
+          <t>暁に鳴る</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>りりあ。</t>
+          <t>超学生</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>プレリュードの手前に ～for me&amp;you～</t>
+          <t>Nightfall feat. Maika Loubté</t>
         </is>
       </c>
       <c r="L103" t="inlineStr">
         <is>
-          <t>伊東歌詞太郎</t>
+          <t>KOHTA YAMAMOTO</t>
         </is>
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25803</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27077</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>6212</v>
+        <v>5947</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2027冬アニメ</t>
+          <t>2026秋アニメ</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>1</v>
+        <v>103</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>赤ずきん、旅の途中で死体と出会う。</t>
+          <t>わたしの幸せな結婚 特別篇</t>
         </is>
       </c>
       <c r="E104" t="b">
@@ -6201,21 +6185,37 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>2027年1月～ TOKYO MX・BS日テレほか</t>
+          <t>2026年10月25日（日）～ TOKYO MXほかにて</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>BENTEN Film</t>
-        </is>
-      </c>
-      <c r="I104" t="inlineStr"/>
-      <c r="J104" t="inlineStr"/>
-      <c r="K104" t="inlineStr"/>
-      <c r="L104" t="inlineStr"/>
+          <t>キネマシトラス</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>幸せで涙が出るのは。</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>りりあ。</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>プレリュードの手前に ～for me&amp;you～</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>伊東歌詞太郎</t>
+        </is>
+      </c>
       <c r="M104" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28922</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25803</t>
         </is>
       </c>
     </row>
@@ -6229,11 +6229,11 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>あかね噺 第2期</t>
+          <t>赤ずきん、旅の途中で死体と出会う。</t>
         </is>
       </c>
       <c r="E105" t="b">
@@ -6246,12 +6246,12 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>2027年1月～ テレビ朝日系全国24局ネット“IMAnimation”枠・BS朝日ほか</t>
+          <t>2027年1月～ TOKYO MX・BS日テレほか</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>ゼクシズ（</t>
+          <t>BENTEN Film</t>
         </is>
       </c>
       <c r="I105" t="inlineStr"/>
@@ -6260,7 +6260,7 @@
       <c r="L105" t="inlineStr"/>
       <c r="M105" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28590</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28922</t>
         </is>
       </c>
     </row>
@@ -6274,11 +6274,11 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>アラフォー賢者の異世界生活日記</t>
+          <t>あかね噺 第2期</t>
         </is>
       </c>
       <c r="E106" t="b">
@@ -6291,12 +6291,12 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>2027年1月～</t>
+          <t>2027年1月～ テレビ朝日系全国24局ネット“IMAnimation”枠・BS朝日ほか</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>YANCHESTER</t>
+          <t>ゼクシズ（</t>
         </is>
       </c>
       <c r="I106" t="inlineStr"/>
@@ -6305,7 +6305,7 @@
       <c r="L106" t="inlineStr"/>
       <c r="M106" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28265</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28590</t>
         </is>
       </c>
     </row>
@@ -6319,11 +6319,11 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>アルカナディア</t>
+          <t>アラフォー賢者の異世界生活日記</t>
         </is>
       </c>
       <c r="E107" t="b">
@@ -6336,12 +6336,12 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>2027年1月〜 テレビ朝日系ほか</t>
+          <t>2027年1月～</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>横浜アニメーションラボ</t>
+          <t>YANCHESTER</t>
         </is>
       </c>
       <c r="I107" t="inlineStr"/>
@@ -6350,7 +6350,7 @@
       <c r="L107" t="inlineStr"/>
       <c r="M107" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25380</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28265</t>
         </is>
       </c>
     </row>
@@ -6364,11 +6364,11 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>異世界でチート能力を手にした俺は、現実世界をも無双する～レベルアップは人生を変えた～ 2nd Season</t>
+          <t>アルカナディア</t>
         </is>
       </c>
       <c r="E108" t="b">
@@ -6381,12 +6381,12 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>2027年1月～</t>
+          <t>2027年1月〜 テレビ朝日系ほか</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>ミルパンセ</t>
+          <t>横浜アニメーションラボ</t>
         </is>
       </c>
       <c r="I108" t="inlineStr"/>
@@ -6395,7 +6395,7 @@
       <c r="L108" t="inlineStr"/>
       <c r="M108" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28025</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25380</t>
         </is>
       </c>
     </row>
@@ -6409,11 +6409,11 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>異世界転生騒動記</t>
+          <t>異世界でチート能力を手にした俺は、現実世界をも無双する～レベルアップは人生を変えた～ 2nd Season</t>
         </is>
       </c>
       <c r="E109" t="b">
@@ -6426,17 +6426,21 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>2027年1月〜</t>
-        </is>
-      </c>
-      <c r="H109" t="inlineStr"/>
+          <t>2027年1月～</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>ミルパンセ</t>
+        </is>
+      </c>
       <c r="I109" t="inlineStr"/>
       <c r="J109" t="inlineStr"/>
       <c r="K109" t="inlineStr"/>
       <c r="L109" t="inlineStr"/>
       <c r="M109" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27924</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28025</t>
         </is>
       </c>
     </row>
@@ -6450,11 +6454,11 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>一式さんは恋を知りたい。</t>
+          <t>異世界転生騒動記</t>
         </is>
       </c>
       <c r="E110" t="b">
@@ -6467,21 +6471,17 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>2027年1月～</t>
-        </is>
-      </c>
-      <c r="H110" t="inlineStr">
-        <is>
-          <t>作楽クリエイト</t>
-        </is>
-      </c>
+          <t>2027年1月〜</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr"/>
       <c r="I110" t="inlineStr"/>
       <c r="J110" t="inlineStr"/>
       <c r="K110" t="inlineStr"/>
       <c r="L110" t="inlineStr"/>
       <c r="M110" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26981</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27924</t>
         </is>
       </c>
     </row>
@@ -6495,11 +6495,11 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>えぶりでいホスト 続編</t>
+          <t>一式さんは恋を知りたい。</t>
         </is>
       </c>
       <c r="E111" t="b">
@@ -6512,17 +6512,21 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>2027年1月〜</t>
-        </is>
-      </c>
-      <c r="H111" t="inlineStr"/>
+          <t>2027年1月～</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>作楽クリエイト</t>
+        </is>
+      </c>
       <c r="I111" t="inlineStr"/>
       <c r="J111" t="inlineStr"/>
       <c r="K111" t="inlineStr"/>
       <c r="L111" t="inlineStr"/>
       <c r="M111" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27178</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26981</t>
         </is>
       </c>
     </row>
@@ -6536,11 +6540,11 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>おデブ悪女に転生したら、なぜかラスボス王子様に執着されています</t>
+          <t>えぶりでいホスト 続編</t>
         </is>
       </c>
       <c r="E112" t="b">
@@ -6553,21 +6557,17 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>2027年1月～ TOKYO MX・ＢＳ日テレほか</t>
-        </is>
-      </c>
-      <c r="H112" t="inlineStr">
-        <is>
-          <t>スタジオリングス</t>
-        </is>
-      </c>
+          <t>2027年1月〜</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr"/>
       <c r="I112" t="inlineStr"/>
       <c r="J112" t="inlineStr"/>
       <c r="K112" t="inlineStr"/>
       <c r="L112" t="inlineStr"/>
       <c r="M112" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27688</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27178</t>
         </is>
       </c>
     </row>
@@ -6581,11 +6581,11 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>俺と悠兄！</t>
+          <t>おデブ悪女に転生したら、なぜかラスボス王子様に執着されています</t>
         </is>
       </c>
       <c r="E113" t="b">
@@ -6598,12 +6598,12 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>2027年1月～</t>
+          <t>2027年1月～ TOKYO MX・ＢＳ日テレほか</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>スタジオ雲雀</t>
+          <t>スタジオリングス</t>
         </is>
       </c>
       <c r="I113" t="inlineStr"/>
@@ -6612,7 +6612,7 @@
       <c r="L113" t="inlineStr"/>
       <c r="M113" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27281</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27688</t>
         </is>
       </c>
     </row>
@@ -6626,11 +6626,11 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>描くなるうえは</t>
+          <t>俺と悠兄！</t>
         </is>
       </c>
       <c r="E114" t="b">
@@ -6648,24 +6648,16 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>ROLL2</t>
-        </is>
-      </c>
-      <c r="I114" t="inlineStr">
-        <is>
-          <t>キミイロヒラリ</t>
-        </is>
-      </c>
-      <c r="J114" t="inlineStr">
-        <is>
-          <t>shallm</t>
-        </is>
-      </c>
+          <t>スタジオ雲雀</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr"/>
+      <c r="J114" t="inlineStr"/>
       <c r="K114" t="inlineStr"/>
       <c r="L114" t="inlineStr"/>
       <c r="M114" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27140</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27281</t>
         </is>
       </c>
     </row>
@@ -6679,11 +6671,11 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>欠けた月のメルセデス～吸血鬼の貴族に転生したけど捨てられそうなのでダンジョンを制覇する～</t>
+          <t>描くなるうえは</t>
         </is>
       </c>
       <c r="E115" t="b">
@@ -6701,16 +6693,24 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>テディ―</t>
-        </is>
-      </c>
-      <c r="I115" t="inlineStr"/>
-      <c r="J115" t="inlineStr"/>
+          <t>ROLL2</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>キミイロヒラリ</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>shallm</t>
+        </is>
+      </c>
       <c r="K115" t="inlineStr"/>
       <c r="L115" t="inlineStr"/>
       <c r="M115" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28808</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27140</t>
         </is>
       </c>
     </row>
@@ -6724,11 +6724,11 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>風を継ぐもの</t>
+          <t>欠けた月のメルセデス～吸血鬼の貴族に転生したけど捨てられそうなのでダンジョンを制覇する～</t>
         </is>
       </c>
       <c r="E116" t="b">
@@ -6741,37 +6741,21 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>2027年1月～ CBC/TBS系全国28局ネットにて 【劇場先行上映】 2026年11月13日（金）</t>
+          <t>2027年1月～</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>Live2D Creative Studio×</t>
-        </is>
-      </c>
-      <c r="I116" t="inlineStr">
-        <is>
-          <t>風を継ぐもの</t>
-        </is>
-      </c>
-      <c r="J116" t="inlineStr">
-        <is>
-          <t>くるり＋羊文学</t>
-        </is>
-      </c>
-      <c r="K116" t="inlineStr">
-        <is>
-          <t>涙の河</t>
-        </is>
-      </c>
-      <c r="L116" t="inlineStr">
-        <is>
-          <t>羊文学＋くるり</t>
-        </is>
-      </c>
+          <t>テディ―</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr"/>
+      <c r="J116" t="inlineStr"/>
+      <c r="K116" t="inlineStr"/>
+      <c r="L116" t="inlineStr"/>
       <c r="M116" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26790</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28808</t>
         </is>
       </c>
     </row>
@@ -6785,11 +6769,11 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>ガチャを回して仲間を増やす 最強の美少女軍団を作り上げろ</t>
+          <t>風を継ぐもの</t>
         </is>
       </c>
       <c r="E117" t="b">
@@ -6802,21 +6786,37 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>2027年1月～</t>
+          <t>2027年1月～ CBC/TBS系全国28局ネットにて 【劇場先行上映】 2026年11月13日（金）</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>ゼロジー</t>
-        </is>
-      </c>
-      <c r="I117" t="inlineStr"/>
-      <c r="J117" t="inlineStr"/>
-      <c r="K117" t="inlineStr"/>
-      <c r="L117" t="inlineStr"/>
+          <t>Live2D Creative Studio×</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>風を継ぐもの</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>くるり＋羊文学</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>涙の河</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>羊文学＋くるり</t>
+        </is>
+      </c>
       <c r="M117" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28643</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26790</t>
         </is>
       </c>
     </row>
@@ -6830,11 +6830,11 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>カリスマ</t>
+          <t>ガチャを回して仲間を増やす 最強の美少女軍団を作り上げろ</t>
         </is>
       </c>
       <c r="E118" t="b">
@@ -6847,12 +6847,12 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>2027年1月～ TBS系にて</t>
+          <t>2027年1月～</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>PIERROT FILMS（</t>
+          <t>ゼロジー</t>
         </is>
       </c>
       <c r="I118" t="inlineStr"/>
@@ -6861,7 +6861,7 @@
       <c r="L118" t="inlineStr"/>
       <c r="M118" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27177</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28643</t>
         </is>
       </c>
     </row>
@@ -6875,11 +6875,11 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>傷口と包帯</t>
+          <t>カリスマ</t>
         </is>
       </c>
       <c r="E119" t="b">
@@ -6892,12 +6892,12 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>2027年1月9日（土）～ ABCテレビ・テレビ朝日系全国ネットANiMAZiNG!!!ほか</t>
+          <t>2027年1月～ TBS系にて</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>J.C.STAFF</t>
+          <t>PIERROT FILMS（</t>
         </is>
       </c>
       <c r="I119" t="inlineStr"/>
@@ -6906,7 +6906,7 @@
       <c r="L119" t="inlineStr"/>
       <c r="M119" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28777</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27177</t>
         </is>
       </c>
     </row>
@@ -6920,11 +6920,11 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>気になってる人が男じゃなかった</t>
+          <t>傷口と包帯</t>
         </is>
       </c>
       <c r="E120" t="b">
@@ -6937,25 +6937,21 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>2027年1月8日（金）～ 日本テレビ系「フラアニ」枠にて</t>
-        </is>
-      </c>
-      <c r="H120" t="inlineStr"/>
-      <c r="I120" t="inlineStr">
-        <is>
-          <t>Breed</t>
-        </is>
-      </c>
-      <c r="J120" t="inlineStr">
-        <is>
-          <t>Nirvana</t>
-        </is>
-      </c>
+          <t>2027年1月9日（土）～ ABCテレビ・テレビ朝日系全国ネットANiMAZiNG!!!ほか</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>J.C.STAFF</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr"/>
+      <c r="J120" t="inlineStr"/>
       <c r="K120" t="inlineStr"/>
       <c r="L120" t="inlineStr"/>
       <c r="M120" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25569</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28777</t>
         </is>
       </c>
     </row>
@@ -6969,11 +6965,11 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>黒岩メダカに私の可愛いが通じない Season2</t>
+          <t>気になってる人が男じゃなかった</t>
         </is>
       </c>
       <c r="E121" t="b">
@@ -6986,21 +6982,25 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>2027年1月～</t>
-        </is>
-      </c>
-      <c r="H121" t="inlineStr">
-        <is>
-          <t>SynergySP</t>
-        </is>
-      </c>
-      <c r="I121" t="inlineStr"/>
-      <c r="J121" t="inlineStr"/>
+          <t>2027年1月8日（金）～ 日本テレビ系「フラアニ」枠にて</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr"/>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>Breed</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>Nirvana</t>
+        </is>
+      </c>
       <c r="K121" t="inlineStr"/>
       <c r="L121" t="inlineStr"/>
       <c r="M121" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28331</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25569</t>
         </is>
       </c>
     </row>
@@ -7014,11 +7014,11 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>ゲーム世界転生〈ダン活〉～ゲーマーは【ダンジョン就活のススメ】を〈はじめから〉プレイする～</t>
+          <t>黒岩メダカに私の可愛いが通じない Season2</t>
         </is>
       </c>
       <c r="E122" t="b">
@@ -7036,32 +7036,16 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>STUDIO MASSKET</t>
-        </is>
-      </c>
-      <c r="I122" t="inlineStr">
-        <is>
-          <t>Play the Play</t>
-        </is>
-      </c>
-      <c r="J122" t="inlineStr">
-        <is>
-          <t>MindaRyn</t>
-        </is>
-      </c>
-      <c r="K122" t="inlineStr">
-        <is>
-          <t>My Life Story</t>
-        </is>
-      </c>
-      <c r="L122" t="inlineStr">
-        <is>
-          <t>LINKL PLANET</t>
-        </is>
-      </c>
+          <t>SynergySP</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr"/>
+      <c r="J122" t="inlineStr"/>
+      <c r="K122" t="inlineStr"/>
+      <c r="L122" t="inlineStr"/>
       <c r="M122" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27910</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28331</t>
         </is>
       </c>
     </row>
@@ -7075,11 +7059,11 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>結界師の一輪華</t>
+          <t>ゲーム世界転生〈ダン活〉～ゲーマーは【ダンジョン就活のススメ】を〈はじめから〉プレイする～</t>
         </is>
       </c>
       <c r="E123" t="b">
@@ -7097,16 +7081,32 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>TROYCA</t>
-        </is>
-      </c>
-      <c r="I123" t="inlineStr"/>
-      <c r="J123" t="inlineStr"/>
-      <c r="K123" t="inlineStr"/>
-      <c r="L123" t="inlineStr"/>
+          <t>STUDIO MASSKET</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>Play the Play</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>MindaRyn</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>My Life Story</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>LINKL PLANET</t>
+        </is>
+      </c>
       <c r="M123" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26630</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27910</t>
         </is>
       </c>
     </row>
@@ -7120,11 +7120,11 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>ゴールデンカムイ 最終章「暴走列車編」</t>
+          <t>結界師の一輪華</t>
         </is>
       </c>
       <c r="E124" t="b">
@@ -7137,17 +7137,21 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>2027年冬</t>
-        </is>
-      </c>
-      <c r="H124" t="inlineStr"/>
+          <t>2027年1月～</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>TROYCA</t>
+        </is>
+      </c>
       <c r="I124" t="inlineStr"/>
       <c r="J124" t="inlineStr"/>
       <c r="K124" t="inlineStr"/>
       <c r="L124" t="inlineStr"/>
       <c r="M124" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=21895</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26630</t>
         </is>
       </c>
     </row>
@@ -7161,34 +7165,34 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>こまどり モフモフパレード</t>
+          <t>ゴールデンカムイ 最終章「暴走列車編」</t>
         </is>
       </c>
       <c r="E125" t="b">
         <v>0</v>
       </c>
-      <c r="F125" t="inlineStr"/>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>TVアニメ</t>
+        </is>
+      </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>2027年1月～ テレ東系列6局ネットにて</t>
-        </is>
-      </c>
-      <c r="H125" t="inlineStr">
-        <is>
-          <t>ドワーフスタジオ</t>
-        </is>
-      </c>
+          <t>2027年冬</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr"/>
       <c r="I125" t="inlineStr"/>
       <c r="J125" t="inlineStr"/>
       <c r="K125" t="inlineStr"/>
       <c r="L125" t="inlineStr"/>
       <c r="M125" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27414</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=21895</t>
         </is>
       </c>
     </row>
@@ -7202,29 +7206,25 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>SAKAMOTO DAYS 第2期</t>
+          <t>こまどり モフモフパレード</t>
         </is>
       </c>
       <c r="E126" t="b">
         <v>0</v>
       </c>
-      <c r="F126" t="inlineStr">
-        <is>
-          <t>TVアニメ</t>
-        </is>
-      </c>
+      <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr">
         <is>
-          <t>2027年1月～</t>
+          <t>2027年1月～ テレ東系列6局ネットにて</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>トムス・エンタテインメント</t>
+          <t>ドワーフスタジオ</t>
         </is>
       </c>
       <c r="I126" t="inlineStr"/>
@@ -7233,7 +7233,7 @@
       <c r="L126" t="inlineStr"/>
       <c r="M126" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27287</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27414</t>
         </is>
       </c>
     </row>
@@ -7247,11 +7247,11 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>雑用付与術師が自分の最強に気付くまで</t>
+          <t>SAKAMOTO DAYS 第2期</t>
         </is>
       </c>
       <c r="E127" t="b">
@@ -7264,29 +7264,21 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>2027年1月4日（月）〜 TOKYO MX・MBSほか</t>
+          <t>2027年1月～</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>J.C.STAFF</t>
-        </is>
-      </c>
-      <c r="I127" t="inlineStr">
-        <is>
-          <t>Ecstatic Buffer</t>
-        </is>
-      </c>
-      <c r="J127" t="inlineStr">
-        <is>
-          <t>LiSA</t>
-        </is>
-      </c>
+          <t>トムス・エンタテインメント</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr"/>
+      <c r="J127" t="inlineStr"/>
       <c r="K127" t="inlineStr"/>
       <c r="L127" t="inlineStr"/>
       <c r="M127" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27970</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27287</t>
         </is>
       </c>
     </row>
@@ -7300,11 +7292,11 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>ザ・ファブル 第2期</t>
+          <t>雑用付与術師が自分の最強に気付くまで</t>
         </is>
       </c>
       <c r="E128" t="b">
@@ -7317,21 +7309,29 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>2027年1月～ 日本テレビ系にて</t>
+          <t>2027年1月4日（月）〜 TOKYO MX・MBSほか</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>手塚プロダクション</t>
-        </is>
-      </c>
-      <c r="I128" t="inlineStr"/>
-      <c r="J128" t="inlineStr"/>
+          <t>J.C.STAFF</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>Ecstatic Buffer</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>LiSA</t>
+        </is>
+      </c>
       <c r="K128" t="inlineStr"/>
       <c r="L128" t="inlineStr"/>
       <c r="M128" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28092</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27970</t>
         </is>
       </c>
     </row>
@@ -7345,11 +7345,11 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>THE ONE PIECE</t>
+          <t>ザ・ファブル 第2期</t>
         </is>
       </c>
       <c r="E129" t="b">
@@ -7357,17 +7357,17 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>2027年2月～ Netflixにて</t>
+          <t>2027年1月～ 日本テレビ系にて</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>WIT STUDIO</t>
+          <t>手塚プロダクション</t>
         </is>
       </c>
       <c r="I129" t="inlineStr"/>
@@ -7376,7 +7376,7 @@
       <c r="L129" t="inlineStr"/>
       <c r="M129" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=23247</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28092</t>
         </is>
       </c>
     </row>
@@ -7390,11 +7390,11 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>死して生きるSSS級ハンター</t>
+          <t>THE ONE PIECE</t>
         </is>
       </c>
       <c r="E130" t="b">
@@ -7402,17 +7402,17 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>2027年1月～ フジテレビ「+Ultra」ほか</t>
+          <t>2027年2月～ Netflixにて</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>スタジオ fu</t>
+          <t>WIT STUDIO</t>
         </is>
       </c>
       <c r="I130" t="inlineStr"/>
@@ -7421,7 +7421,7 @@
       <c r="L130" t="inlineStr"/>
       <c r="M130" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=29082</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=23247</t>
         </is>
       </c>
     </row>
@@ -7435,11 +7435,11 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>ジャイアントお嬢様</t>
+          <t>死して生きるSSS級ハンター</t>
         </is>
       </c>
       <c r="E131" t="b">
@@ -7452,12 +7452,12 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>2027年1月～</t>
+          <t>2027年1月～ フジテレビ「+Ultra」ほか</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>タツノコプロ</t>
+          <t>スタジオ fu</t>
         </is>
       </c>
       <c r="I131" t="inlineStr"/>
@@ -7466,7 +7466,7 @@
       <c r="L131" t="inlineStr"/>
       <c r="M131" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25610</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=29082</t>
         </is>
       </c>
     </row>
@@ -7480,11 +7480,11 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>シャングリラ・フロンティア 3rd season</t>
+          <t>ジャイアントお嬢様</t>
         </is>
       </c>
       <c r="E132" t="b">
@@ -7497,12 +7497,12 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>2027年1月10日（日）～ MBS／TBS系全国28局ネットほか</t>
+          <t>2027年1月～</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>C2C</t>
+          <t>タツノコプロ</t>
         </is>
       </c>
       <c r="I132" t="inlineStr"/>
@@ -7511,7 +7511,7 @@
       <c r="L132" t="inlineStr"/>
       <c r="M132" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25755</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25610</t>
         </is>
       </c>
     </row>
@@ -7525,11 +7525,11 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>じょせまる</t>
+          <t>シャングリラ・フロンティア 3rd season</t>
         </is>
       </c>
       <c r="E133" t="b">
@@ -7542,12 +7542,12 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>2027年1月～ テレビ朝日「PicoAniTime」枠にて</t>
+          <t>2027年1月10日（日）～ MBS／TBS系全国28局ネットほか</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>株式会社フローエンタテイメント</t>
+          <t>C2C</t>
         </is>
       </c>
       <c r="I133" t="inlineStr"/>
@@ -7556,7 +7556,7 @@
       <c r="L133" t="inlineStr"/>
       <c r="M133" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28562</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25755</t>
         </is>
       </c>
     </row>
@@ -7570,11 +7570,11 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>地雷なんですか？地原さん</t>
+          <t>じょせまる</t>
         </is>
       </c>
       <c r="E134" t="b">
@@ -7587,12 +7587,12 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>2027年1月～ MBS・TBSほか</t>
+          <t>2027年1月～ テレビ朝日「PicoAniTime」枠にて</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>SynergySP</t>
+          <t>株式会社フローエンタテイメント</t>
         </is>
       </c>
       <c r="I134" t="inlineStr"/>
@@ -7601,7 +7601,7 @@
       <c r="L134" t="inlineStr"/>
       <c r="M134" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27363</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28562</t>
         </is>
       </c>
     </row>
@@ -7615,11 +7615,11 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>真･侍伝 YAIBA 第2期 かぐや編</t>
+          <t>地雷なんですか？地原さん</t>
         </is>
       </c>
       <c r="E135" t="b">
@@ -7632,12 +7632,12 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>2027年1月9日（土）～ 読売テレビ・日本テレビ系全国ネットにて</t>
+          <t>2027年1月～ MBS・TBSほか</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>WIT STUDIO</t>
+          <t>SynergySP</t>
         </is>
       </c>
       <c r="I135" t="inlineStr"/>
@@ -7646,7 +7646,7 @@
       <c r="L135" t="inlineStr"/>
       <c r="M135" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26849</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27363</t>
         </is>
       </c>
     </row>
@@ -7660,11 +7660,11 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>真の聖女である私は追放されました。だからこの国はもう終わりです</t>
+          <t>真･侍伝 YAIBA 第2期 かぐや編</t>
         </is>
       </c>
       <c r="E136" t="b">
@@ -7677,12 +7677,12 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>2027年1月～</t>
+          <t>2027年1月9日（土）～ 読売テレビ・日本テレビ系全国ネットにて</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>つむぎ秋田アニメLab</t>
+          <t>WIT STUDIO</t>
         </is>
       </c>
       <c r="I136" t="inlineStr"/>
@@ -7691,7 +7691,7 @@
       <c r="L136" t="inlineStr"/>
       <c r="M136" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28845</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26849</t>
         </is>
       </c>
     </row>
@@ -7705,11 +7705,11 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>すだちの魔王城</t>
+          <t>真の聖女である私は追放されました。だからこの国はもう終わりです</t>
         </is>
       </c>
       <c r="E137" t="b">
@@ -7727,7 +7727,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>project No.9</t>
+          <t>つむぎ秋田アニメLab</t>
         </is>
       </c>
       <c r="I137" t="inlineStr"/>
@@ -7736,7 +7736,7 @@
       <c r="L137" t="inlineStr"/>
       <c r="M137" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28645</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28845</t>
         </is>
       </c>
     </row>
@@ -7750,11 +7750,11 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>アニコミ「青春のやり直しは異世界で」</t>
+          <t>すだちの魔王城</t>
         </is>
       </c>
       <c r="E138" t="b">
@@ -7767,12 +7767,12 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>2027年1月～ TOKYO MXにて</t>
+          <t>2027年1月～</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>動楽</t>
+          <t>project No.9</t>
         </is>
       </c>
       <c r="I138" t="inlineStr"/>
@@ -7781,7 +7781,7 @@
       <c r="L138" t="inlineStr"/>
       <c r="M138" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=29083</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28645</t>
         </is>
       </c>
     </row>
@@ -7795,11 +7795,11 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>SEKIRO: NO DEFEAT TV放送</t>
+          <t>アニコミ「青春のやり直しは異世界で」</t>
         </is>
       </c>
       <c r="E139" t="b">
@@ -7807,17 +7807,17 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>劇場版アニメ</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>2026年9月4日（金） 【TVアニメ版】 2027年1月～</t>
+          <t>2027年1月～ TOKYO MXにて</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>Qzil.la</t>
+          <t>動楽</t>
         </is>
       </c>
       <c r="I139" t="inlineStr"/>
@@ -7826,7 +7826,7 @@
       <c r="L139" t="inlineStr"/>
       <c r="M139" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26641</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=29083</t>
         </is>
       </c>
     </row>
@@ -7840,11 +7840,11 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>ゾンビのあふれた世界で俺だけが襲われない</t>
+          <t>SEKIRO: NO DEFEAT TV放送</t>
         </is>
       </c>
       <c r="E140" t="b">
@@ -7852,42 +7852,26 @@
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>劇場版アニメ</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>2027年1月～ AT-Xにて</t>
+          <t>2026年9月4日（金） 【TVアニメ版】 2027年1月～</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>Acca effe</t>
-        </is>
-      </c>
-      <c r="I140" t="inlineStr">
-        <is>
-          <t>ノーリアクション</t>
-        </is>
-      </c>
-      <c r="J140" t="inlineStr">
-        <is>
-          <t>レトベア（unknown Vo：0in）</t>
-        </is>
-      </c>
-      <c r="K140" t="inlineStr">
-        <is>
-          <t>ツキカゲ</t>
-        </is>
-      </c>
-      <c r="L140" t="inlineStr">
-        <is>
-          <t>イツカ▶</t>
-        </is>
-      </c>
+          <t>Qzil.la</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr"/>
+      <c r="J140" t="inlineStr"/>
+      <c r="K140" t="inlineStr"/>
+      <c r="L140" t="inlineStr"/>
       <c r="M140" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=23537</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26641</t>
         </is>
       </c>
     </row>
@@ -7901,11 +7885,11 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>ディズニー ツイステッドワンダーランド ザ アニメーション ～エピソード オブ サバナクロー～</t>
+          <t>ゾンビのあふれた世界で俺だけが襲われない</t>
         </is>
       </c>
       <c r="E141" t="b">
@@ -7913,22 +7897,42 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>2026年12月～</t>
-        </is>
-      </c>
-      <c r="H141" t="inlineStr"/>
-      <c r="I141" t="inlineStr"/>
-      <c r="J141" t="inlineStr"/>
-      <c r="K141" t="inlineStr"/>
-      <c r="L141" t="inlineStr"/>
+          <t>2027年1月～ AT-Xにて</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>Acca effe</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>ノーリアクション</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>レトベア（unknown Vo：0in）</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>ツキカゲ</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>イツカ▶</t>
+        </is>
+      </c>
       <c r="M141" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25212</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=23537</t>
         </is>
       </c>
     </row>
@@ -7942,11 +7946,11 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>電撃デイジー</t>
+          <t>ディズニー ツイステッドワンダーランド ザ アニメーション ～エピソード オブ サバナクロー～</t>
         </is>
       </c>
       <c r="E142" t="b">
@@ -7954,12 +7958,12 @@
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>2027年1月～</t>
+          <t>2026年12月23日（水）～ Disney+にて</t>
         </is>
       </c>
       <c r="H142" t="inlineStr"/>
@@ -7969,7 +7973,7 @@
       <c r="L142" t="inlineStr"/>
       <c r="M142" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28519</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25212</t>
         </is>
       </c>
     </row>
@@ -7983,11 +7987,11 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>ハルとゲン ～70歳、はじめての子育て～</t>
+          <t>電撃デイジー</t>
         </is>
       </c>
       <c r="E143" t="b">
@@ -8000,21 +8004,17 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>2027年1月4日（月）～ tvkにて</t>
-        </is>
-      </c>
-      <c r="H143" t="inlineStr">
-        <is>
-          <t>Imagica Infos</t>
-        </is>
-      </c>
+          <t>2027年1月～</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr"/>
       <c r="I143" t="inlineStr"/>
       <c r="J143" t="inlineStr"/>
       <c r="K143" t="inlineStr"/>
       <c r="L143" t="inlineStr"/>
       <c r="M143" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=29089</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28519</t>
         </is>
       </c>
     </row>
@@ -8028,11 +8028,11 @@
         </is>
       </c>
       <c r="C144" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>BanG Dream! MyGO!!!!! // Ave Mujica</t>
+          <t>ハルとゲン ～70歳、はじめての子育て～</t>
         </is>
       </c>
       <c r="E144" t="b">
@@ -8045,17 +8045,21 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>2027年1月8日（金）～ 日本テレビ系全国30局ネットにて</t>
-        </is>
-      </c>
-      <c r="H144" t="inlineStr"/>
+          <t>2027年1月4日（月）～ tvkにて</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>Imagica Infos</t>
+        </is>
+      </c>
       <c r="I144" t="inlineStr"/>
       <c r="J144" t="inlineStr"/>
       <c r="K144" t="inlineStr"/>
       <c r="L144" t="inlineStr"/>
       <c r="M144" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25765</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=29089</t>
         </is>
       </c>
     </row>
@@ -8069,11 +8073,11 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>ヒストリエ</t>
+          <t>BanG Dream! MyGO!!!!! // Ave Mujica</t>
         </is>
       </c>
       <c r="E145" t="b">
@@ -8086,21 +8090,17 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>2027年1月～</t>
-        </is>
-      </c>
-      <c r="H145" t="inlineStr">
-        <is>
-          <t>ライデンフィルム</t>
-        </is>
-      </c>
+          <t>2027年1月8日（金）～ 日本テレビ系全国30局ネットにて</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr"/>
       <c r="I145" t="inlineStr"/>
       <c r="J145" t="inlineStr"/>
       <c r="K145" t="inlineStr"/>
       <c r="L145" t="inlineStr"/>
       <c r="M145" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27368</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25765</t>
         </is>
       </c>
     </row>
@@ -8114,11 +8114,11 @@
         </is>
       </c>
       <c r="C146" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>姫騎士様のヒモ</t>
+          <t>ヒストリエ</t>
         </is>
       </c>
       <c r="E146" t="b">
@@ -8136,32 +8136,16 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>BLADE</t>
-        </is>
-      </c>
-      <c r="I146" t="inlineStr">
-        <is>
-          <t>TRUE-TABOO</t>
-        </is>
-      </c>
-      <c r="J146" t="inlineStr">
-        <is>
-          <t>MYTH &amp; ROID</t>
-        </is>
-      </c>
-      <c r="K146" t="inlineStr">
-        <is>
-          <t>偽花</t>
-        </is>
-      </c>
-      <c r="L146" t="inlineStr">
-        <is>
-          <t>sajou no hana</t>
-        </is>
-      </c>
+          <t>ライデンフィルム</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr"/>
+      <c r="J146" t="inlineStr"/>
+      <c r="K146" t="inlineStr"/>
+      <c r="L146" t="inlineStr"/>
       <c r="M146" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25551</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27368</t>
         </is>
       </c>
     </row>
@@ -8175,11 +8159,11 @@
         </is>
       </c>
       <c r="C147" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>ひらやすみ</t>
+          <t>姫騎士様のヒモ</t>
         </is>
       </c>
       <c r="E147" t="b">
@@ -8192,21 +8176,37 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>2027年1月～ NHK総合テレビにて</t>
+          <t>2027年1月～</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>Production +h.</t>
-        </is>
-      </c>
-      <c r="I147" t="inlineStr"/>
-      <c r="J147" t="inlineStr"/>
-      <c r="K147" t="inlineStr"/>
-      <c r="L147" t="inlineStr"/>
+          <t>BLADE</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>TRUE-TABOO</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>MYTH &amp; ROID</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>偽花</t>
+        </is>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>sajou no hana</t>
+        </is>
+      </c>
       <c r="M147" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26471</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25551</t>
         </is>
       </c>
     </row>
@@ -8220,11 +8220,11 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>ふつつかな悪女ではございますが～雛宮蝶鼠とりかえ伝～ 第2クール</t>
+          <t>ひらやすみ</t>
         </is>
       </c>
       <c r="E148" t="b">
@@ -8237,37 +8237,21 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>第1クール：2026年7月12日（日）〜2026年9月20日（日） 第2クール：2027年1月～ テレビ東京系列にて</t>
+          <t>2027年1月～ NHK総合テレビにて</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>動画工房</t>
-        </is>
-      </c>
-      <c r="I148" t="inlineStr">
-        <is>
-          <t>Sunny</t>
-        </is>
-      </c>
-      <c r="J148" t="inlineStr">
-        <is>
-          <t>milet</t>
-        </is>
-      </c>
-      <c r="K148" t="inlineStr">
-        <is>
-          <t>ホウキボシ</t>
-        </is>
-      </c>
-      <c r="L148" t="inlineStr">
-        <is>
-          <t>ロクデナシ</t>
-        </is>
-      </c>
+          <t>Production +h.</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr"/>
+      <c r="J148" t="inlineStr"/>
+      <c r="K148" t="inlineStr"/>
+      <c r="L148" t="inlineStr"/>
       <c r="M148" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25702</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26471</t>
         </is>
       </c>
     </row>
@@ -8281,11 +8265,11 @@
         </is>
       </c>
       <c r="C149" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>BLUE EYE SAMURAI/ブルーアイ・サムライ</t>
+          <t>ふつつかな悪女ではございますが～雛宮蝶鼠とりかえ伝～ 第2クール</t>
         </is>
       </c>
       <c r="E149" t="b">
@@ -8293,22 +8277,42 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>シーズン1：2023年11月3日（金）～ シーズン2：2027年1月～ シーズン3：未発表 Netflixにて</t>
-        </is>
-      </c>
-      <c r="H149" t="inlineStr"/>
-      <c r="I149" t="inlineStr"/>
-      <c r="J149" t="inlineStr"/>
-      <c r="K149" t="inlineStr"/>
-      <c r="L149" t="inlineStr"/>
+          <t>第1クール：2026年7月12日（日）〜2026年9月20日（日） 第2クール：2027年1月～ テレビ東京系列にて</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>動画工房</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>Sunny</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>milet</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>ホウキボシ</t>
+        </is>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>ロクデナシ</t>
+        </is>
+      </c>
       <c r="M149" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28984</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25702</t>
         </is>
       </c>
     </row>
@@ -8322,11 +8326,11 @@
         </is>
       </c>
       <c r="C150" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>ブレス</t>
+          <t>BLUE EYE SAMURAI/ブルーアイ・サムライ</t>
         </is>
       </c>
       <c r="E150" t="b">
@@ -8334,12 +8338,12 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>2027年1月〜 フジテレビ系“ ノイタミナ ”にて</t>
+          <t>シーズン1：2023年11月3日（金）～ シーズン2：2027年1月～ シーズン3：未発表 Netflixにて</t>
         </is>
       </c>
       <c r="H150" t="inlineStr"/>
@@ -8349,7 +8353,7 @@
       <c r="L150" t="inlineStr"/>
       <c r="M150" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27878</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28984</t>
         </is>
       </c>
     </row>
@@ -8363,11 +8367,11 @@
         </is>
       </c>
       <c r="C151" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>ペンと手錠と事実婚</t>
+          <t>ブレス</t>
         </is>
       </c>
       <c r="E151" t="b">
@@ -8380,21 +8384,17 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>2027年1月〜</t>
-        </is>
-      </c>
-      <c r="H151" t="inlineStr">
-        <is>
-          <t>EMTスクエアード</t>
-        </is>
-      </c>
+          <t>2027年1月〜 フジテレビ系“ ノイタミナ ”にて</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr"/>
       <c r="I151" t="inlineStr"/>
       <c r="J151" t="inlineStr"/>
       <c r="K151" t="inlineStr"/>
       <c r="L151" t="inlineStr"/>
       <c r="M151" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28250</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27878</t>
         </is>
       </c>
     </row>
@@ -8408,11 +8408,11 @@
         </is>
       </c>
       <c r="C152" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>冒険者ライセンスを剥奪されたおっさんだけど、愛娘ができたのでのんびり人生を謳歌する</t>
+          <t>ペンと手錠と事実婚</t>
         </is>
       </c>
       <c r="E152" t="b">
@@ -8425,17 +8425,21 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>2027年1月～</t>
-        </is>
-      </c>
-      <c r="H152" t="inlineStr"/>
+          <t>2027年1月〜</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>EMTスクエアード</t>
+        </is>
+      </c>
       <c r="I152" t="inlineStr"/>
       <c r="J152" t="inlineStr"/>
       <c r="K152" t="inlineStr"/>
       <c r="L152" t="inlineStr"/>
       <c r="M152" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27372</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28250</t>
         </is>
       </c>
     </row>
@@ -8449,11 +8453,11 @@
         </is>
       </c>
       <c r="C153" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>魔入りました！入間くん if Episode of 魔フィア</t>
+          <t>冒険者ライセンスを剥奪されたおっさんだけど、愛娘ができたのでのんびり人生を謳歌する</t>
         </is>
       </c>
       <c r="E153" t="b">
@@ -8466,21 +8470,17 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>2027年1月4日（月）〜 NHK総合にて</t>
-        </is>
-      </c>
-      <c r="H153" t="inlineStr">
-        <is>
-          <t>タツノコプロ</t>
-        </is>
-      </c>
+          <t>2027年1月～</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr"/>
       <c r="I153" t="inlineStr"/>
       <c r="J153" t="inlineStr"/>
       <c r="K153" t="inlineStr"/>
       <c r="L153" t="inlineStr"/>
       <c r="M153" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27609</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27372</t>
         </is>
       </c>
     </row>
@@ -8494,11 +8494,11 @@
         </is>
       </c>
       <c r="C154" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>魔術を極めて旅に出た転生エルフ、持て余した寿命で生ける伝説となる</t>
+          <t>魔入りました！入間くん if Episode of 魔フィア</t>
         </is>
       </c>
       <c r="E154" t="b">
@@ -8511,12 +8511,12 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>2027年1月～</t>
+          <t>2027年1月4日（月）〜 NHK総合にて</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>studioぱれっと</t>
+          <t>タツノコプロ</t>
         </is>
       </c>
       <c r="I154" t="inlineStr"/>
@@ -8525,7 +8525,7 @@
       <c r="L154" t="inlineStr"/>
       <c r="M154" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28581</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27609</t>
         </is>
       </c>
     </row>
@@ -8539,11 +8539,11 @@
         </is>
       </c>
       <c r="C155" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>マッシュル-MASHLE- 三魔対争神覚者最終試験編</t>
+          <t>魔術を極めて旅に出た転生エルフ、持て余した寿命で生ける伝説となる</t>
         </is>
       </c>
       <c r="E155" t="b">
@@ -8559,14 +8559,18 @@
           <t>2027年1月～</t>
         </is>
       </c>
-      <c r="H155" t="inlineStr"/>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>studioぱれっと</t>
+        </is>
+      </c>
       <c r="I155" t="inlineStr"/>
       <c r="J155" t="inlineStr"/>
       <c r="K155" t="inlineStr"/>
       <c r="L155" t="inlineStr"/>
       <c r="M155" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24109</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28581</t>
         </is>
       </c>
     </row>
@@ -8580,11 +8584,11 @@
         </is>
       </c>
       <c r="C156" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>茉莉花官吏伝</t>
+          <t>マッシュル-MASHLE- 三魔対争神覚者最終試験編</t>
         </is>
       </c>
       <c r="E156" t="b">
@@ -8597,29 +8601,17 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>2027年1月〜 TOKYO MXほか</t>
-        </is>
-      </c>
-      <c r="H156" t="inlineStr">
-        <is>
-          <t>MAHO FILM</t>
-        </is>
-      </c>
-      <c r="I156" t="inlineStr">
-        <is>
-          <t>花噺</t>
-        </is>
-      </c>
-      <c r="J156" t="inlineStr">
-        <is>
-          <t>KANA-BOON</t>
-        </is>
-      </c>
+          <t>2027年1月～</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr"/>
+      <c r="I156" t="inlineStr"/>
+      <c r="J156" t="inlineStr"/>
       <c r="K156" t="inlineStr"/>
       <c r="L156" t="inlineStr"/>
       <c r="M156" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26896</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24109</t>
         </is>
       </c>
     </row>
@@ -8633,11 +8625,11 @@
         </is>
       </c>
       <c r="C157" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>マリッジトキシン 第2期</t>
+          <t>茉莉花官吏伝</t>
         </is>
       </c>
       <c r="E157" t="b">
@@ -8650,21 +8642,29 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>2027年1月～</t>
+          <t>2027年1月〜 TOKYO MXほか</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>ボンズ</t>
-        </is>
-      </c>
-      <c r="I157" t="inlineStr"/>
-      <c r="J157" t="inlineStr"/>
+          <t>MAHO FILM</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>花噺</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>KANA-BOON</t>
+        </is>
+      </c>
       <c r="K157" t="inlineStr"/>
       <c r="L157" t="inlineStr"/>
       <c r="M157" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28681</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26896</t>
         </is>
       </c>
     </row>
@@ -8678,11 +8678,11 @@
         </is>
       </c>
       <c r="C158" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>MURCIÉLAGO-ムルシエラゴ-</t>
+          <t>マリッジトキシン 第2期</t>
         </is>
       </c>
       <c r="E158" t="b">
@@ -8695,12 +8695,12 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>2027年1月〜 TOKYO MX・関西テレビ・BS11にて</t>
+          <t>2027年1月～</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>サテライト</t>
+          <t>ボンズ</t>
         </is>
       </c>
       <c r="I158" t="inlineStr"/>
@@ -8709,7 +8709,7 @@
       <c r="L158" t="inlineStr"/>
       <c r="M158" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28714</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28681</t>
         </is>
       </c>
     </row>
@@ -8723,11 +8723,11 @@
         </is>
       </c>
       <c r="C159" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>メラ×デス 死神と僕の異常な恋</t>
+          <t>MURCIÉLAGO-ムルシエラゴ-</t>
         </is>
       </c>
       <c r="E159" t="b">
@@ -8740,12 +8740,12 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>2027年1月5日（火）～ TOKYO MXほか</t>
+          <t>2027年1月〜 TOKYO MX・関西テレビ・BS11にて</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>Qzil.la</t>
+          <t>サテライト</t>
         </is>
       </c>
       <c r="I159" t="inlineStr"/>
@@ -8754,7 +8754,7 @@
       <c r="L159" t="inlineStr"/>
       <c r="M159" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=29115</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28714</t>
         </is>
       </c>
     </row>
@@ -8768,11 +8768,11 @@
         </is>
       </c>
       <c r="C160" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>モモモ！ニニモ</t>
+          <t>メラ×デス 死神と僕の異常な恋</t>
         </is>
       </c>
       <c r="E160" t="b">
@@ -8785,17 +8785,21 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>2027年1月～ テレビ朝日「PicoAniTime」枠にて</t>
-        </is>
-      </c>
-      <c r="H160" t="inlineStr"/>
+          <t>2027年1月5日（火）～ TOKYO MXほか</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>Qzil.la</t>
+        </is>
+      </c>
       <c r="I160" t="inlineStr"/>
       <c r="J160" t="inlineStr"/>
       <c r="K160" t="inlineStr"/>
       <c r="L160" t="inlineStr"/>
       <c r="M160" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28563</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=29115</t>
         </is>
       </c>
     </row>
@@ -8809,11 +8813,11 @@
         </is>
       </c>
       <c r="C161" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>悠久の愚者アズリーの、賢者のすゝめ</t>
+          <t>モモモ！ニニモ</t>
         </is>
       </c>
       <c r="E161" t="b">
@@ -8826,21 +8830,17 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>2027年1月～</t>
-        </is>
-      </c>
-      <c r="H161" t="inlineStr">
-        <is>
-          <t>スタジオエル</t>
-        </is>
-      </c>
+          <t>2027年1月～ テレビ朝日「PicoAniTime」枠にて</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr"/>
       <c r="I161" t="inlineStr"/>
       <c r="J161" t="inlineStr"/>
       <c r="K161" t="inlineStr"/>
       <c r="L161" t="inlineStr"/>
       <c r="M161" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27618</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28563</t>
         </is>
       </c>
     </row>
@@ -8854,11 +8854,11 @@
         </is>
       </c>
       <c r="C162" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>ラーメン赤猫 其の二</t>
+          <t>悠久の愚者アズリーの、賢者のすゝめ</t>
         </is>
       </c>
       <c r="E162" t="b">
@@ -8876,7 +8876,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>E&amp;H production</t>
+          <t>スタジオエル</t>
         </is>
       </c>
       <c r="I162" t="inlineStr"/>
@@ -8885,7 +8885,7 @@
       <c r="L162" t="inlineStr"/>
       <c r="M162" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25390</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27618</t>
         </is>
       </c>
     </row>
@@ -8899,11 +8899,11 @@
         </is>
       </c>
       <c r="C163" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>ラブライブ！蓮ノ空女学院スクールアイドルクラブ</t>
+          <t>ラーメン赤猫 其の二</t>
         </is>
       </c>
       <c r="E163" t="b">
@@ -8916,12 +8916,12 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>2027年1月～ TOKYO MXほか</t>
+          <t>2027年1月～</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>サブリメイション</t>
+          <t>E&amp;H production</t>
         </is>
       </c>
       <c r="I163" t="inlineStr"/>
@@ -8930,7 +8930,7 @@
       <c r="L163" t="inlineStr"/>
       <c r="M163" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=29222</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25390</t>
         </is>
       </c>
     </row>
@@ -8944,11 +8944,11 @@
         </is>
       </c>
       <c r="C164" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>業物語 かれんオウガ</t>
+          <t>ラブライブ！蓮ノ空女学院スクールアイドルクラブ</t>
         </is>
       </c>
       <c r="E164" t="b">
@@ -8961,12 +8961,12 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>2026年冬</t>
+          <t>2027年1月～ TOKYO MXほか</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>シャフト</t>
+          <t>サブリメイション</t>
         </is>
       </c>
       <c r="I164" t="inlineStr"/>
@@ -8975,7 +8975,7 @@
       <c r="L164" t="inlineStr"/>
       <c r="M164" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26354</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=29222</t>
         </is>
       </c>
     </row>
@@ -8989,11 +8989,11 @@
         </is>
       </c>
       <c r="C165" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>ワンパンマン 第3期 第2クール</t>
+          <t>業物語 かれんオウガ</t>
         </is>
       </c>
       <c r="E165" t="b">
@@ -9006,55 +9006,39 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>第1クール：2025年10月5日（日）〜2025年12月28日（日） テレ東系列にて 第2クール：2027年1月～</t>
+          <t>2026年冬</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>J.C.STAFF</t>
-        </is>
-      </c>
-      <c r="I165" t="inlineStr">
-        <is>
-          <t>Get No Satisfied !</t>
-        </is>
-      </c>
-      <c r="J165" t="inlineStr">
-        <is>
-          <t>JAM Project feat.BABYMETAL</t>
-        </is>
-      </c>
-      <c r="K165" t="inlineStr">
-        <is>
-          <t>そこに有る灯り</t>
-        </is>
-      </c>
-      <c r="L165" t="inlineStr">
-        <is>
-          <t>古川慎</t>
-        </is>
-      </c>
+          <t>シャフト</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr"/>
+      <c r="J165" t="inlineStr"/>
+      <c r="K165" t="inlineStr"/>
+      <c r="L165" t="inlineStr"/>
       <c r="M165" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=16772</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26354</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="n">
-        <v>-194116</v>
+        <v>6212</v>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026夏アニメ</t>
+          <t>2027冬アニメ</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>0</v>
+        <v>62</v>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>最終楽章 響け！ユーフォニアム後編</t>
+          <t>ワンパンマン 第3期 第2クール</t>
         </is>
       </c>
       <c r="E166" t="b">
@@ -9062,32 +9046,48 @@
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>劇場版</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>2026年9月11日</t>
+          <t>第1クール：2025年10月5日（日）〜2025年12月28日（日） テレ東系列にて 第2クール：2027年1月～</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>Kyoto Animation</t>
-        </is>
-      </c>
-      <c r="I166" t="inlineStr"/>
-      <c r="J166" t="inlineStr"/>
-      <c r="K166" t="inlineStr"/>
-      <c r="L166" t="inlineStr"/>
+          <t>J.C.STAFF</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>Get No Satisfied !</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>JAM Project feat.BABYMETAL</t>
+        </is>
+      </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>そこに有る灯り</t>
+        </is>
+      </c>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>古川慎</t>
+        </is>
+      </c>
       <c r="M166" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/194116</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=16772</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
-        <v>-198654</v>
+        <v>-194116</v>
       </c>
       <c r="B167" t="inlineStr">
         <is>
@@ -9099,7 +9099,7 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>名探偵プリキュア！不思議な庭と2人の秘密</t>
+          <t>最終楽章 響け！ユーフォニアム後編</t>
         </is>
       </c>
       <c r="E167" t="b">
@@ -9112,12 +9112,12 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>2026年9月18日</t>
+          <t>2026年9月11日</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>Toei Animation</t>
+          <t>Kyoto Animation</t>
         </is>
       </c>
       <c r="I167" t="inlineStr"/>
@@ -9126,13 +9126,13 @@
       <c r="L167" t="inlineStr"/>
       <c r="M167" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/198654</t>
+          <t>https://anilist.co/anime/194116</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
-        <v>-202429</v>
+        <v>-198654</v>
       </c>
       <c r="B168" t="inlineStr">
         <is>
@@ -9144,7 +9144,7 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>我々は宇宙人</t>
+          <t>名探偵プリキュア！不思議な庭と2人の秘密</t>
         </is>
       </c>
       <c r="E168" t="b">
@@ -9157,12 +9157,12 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>2026年9月25日</t>
+          <t>2026年9月18日</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>NOTHING NEW, Miyu Productions</t>
+          <t>Toei Animation</t>
         </is>
       </c>
       <c r="I168" t="inlineStr"/>
@@ -9171,17 +9171,17 @@
       <c r="L168" t="inlineStr"/>
       <c r="M168" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/202429</t>
+          <t>https://anilist.co/anime/198654</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="n">
-        <v>-202390</v>
+        <v>-202429</v>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026秋アニメ</t>
+          <t>2026夏アニメ</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -9189,7 +9189,7 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>ガールズ＆パンツァー 最終章 第5話</t>
+          <t>我々は宇宙人</t>
         </is>
       </c>
       <c r="E169" t="b">
@@ -9202,12 +9202,12 @@
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>2026年10月9日</t>
+          <t>2026年9月25日</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>Actas</t>
+          <t>NOTHING NEW, Miyu Productions</t>
         </is>
       </c>
       <c r="I169" t="inlineStr"/>
@@ -9216,13 +9216,13 @@
       <c r="L169" t="inlineStr"/>
       <c r="M169" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/202390</t>
+          <t>https://anilist.co/anime/202429</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="n">
-        <v>-207327</v>
+        <v>-202390</v>
       </c>
       <c r="B170" t="inlineStr">
         <is>
@@ -9234,7 +9234,7 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>どこよりも遠い場所にいる君へ</t>
+          <t>ガールズ＆パンツァー 最終章 第5話</t>
         </is>
       </c>
       <c r="E170" t="b">
@@ -9252,7 +9252,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>TMS Entertainment</t>
+          <t>Actas</t>
         </is>
       </c>
       <c r="I170" t="inlineStr"/>
@@ -9261,13 +9261,13 @@
       <c r="L170" t="inlineStr"/>
       <c r="M170" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/207327</t>
+          <t>https://anilist.co/anime/202390</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="n">
-        <v>-197543</v>
+        <v>-207327</v>
       </c>
       <c r="B171" t="inlineStr">
         <is>
@@ -9279,7 +9279,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>BanG Dream! Ave Mujica prima aurora</t>
+          <t>どこよりも遠い場所にいる君へ</t>
         </is>
       </c>
       <c r="E171" t="b">
@@ -9292,12 +9292,12 @@
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>2026年10月16日</t>
+          <t>2026年10月9日</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>NICHICALINE</t>
+          <t>TMS Entertainment</t>
         </is>
       </c>
       <c r="I171" t="inlineStr"/>
@@ -9306,13 +9306,13 @@
       <c r="L171" t="inlineStr"/>
       <c r="M171" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/197543</t>
+          <t>https://anilist.co/anime/207327</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="n">
-        <v>-199340</v>
+        <v>-197543</v>
       </c>
       <c r="B172" t="inlineStr">
         <is>
@@ -9324,7 +9324,7 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>青春ブタ野郎はディアフレンドの夢を見ない</t>
+          <t>BanG Dream! Ave Mujica prima aurora</t>
         </is>
       </c>
       <c r="E172" t="b">
@@ -9342,7 +9342,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>CloverWorks</t>
+          <t>NICHICALINE</t>
         </is>
       </c>
       <c r="I172" t="inlineStr"/>
@@ -9351,13 +9351,13 @@
       <c r="L172" t="inlineStr"/>
       <c r="M172" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/199340</t>
+          <t>https://anilist.co/anime/197543</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
-        <v>-160275</v>
+        <v>-199340</v>
       </c>
       <c r="B173" t="inlineStr">
         <is>
@@ -9369,7 +9369,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>メイドインアビス 目覚める神秘</t>
+          <t>青春ブタ野郎はディアフレンドの夢を見ない</t>
         </is>
       </c>
       <c r="E173" t="b">
@@ -9382,12 +9382,12 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>2026年10月23日</t>
+          <t>2026年10月16日</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>Kinema Citrus</t>
+          <t>CloverWorks</t>
         </is>
       </c>
       <c r="I173" t="inlineStr"/>
@@ -9396,13 +9396,13 @@
       <c r="L173" t="inlineStr"/>
       <c r="M173" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/160275</t>
+          <t>https://anilist.co/anime/199340</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="n">
-        <v>-209642</v>
+        <v>-160275</v>
       </c>
       <c r="B174" t="inlineStr">
         <is>
@@ -9414,7 +9414,7 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>劇場版 前橋ウィッチーズ ～魔女見習いのエモエモリーズ～</t>
+          <t>メイドインアビス 目覚める神秘</t>
         </is>
       </c>
       <c r="E174" t="b">
@@ -9432,7 +9432,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>Sunrise</t>
+          <t>Kinema Citrus</t>
         </is>
       </c>
       <c r="I174" t="inlineStr"/>
@@ -9441,13 +9441,13 @@
       <c r="L174" t="inlineStr"/>
       <c r="M174" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/209642</t>
+          <t>https://anilist.co/anime/160275</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="n">
-        <v>-178972</v>
+        <v>-209642</v>
       </c>
       <c r="B175" t="inlineStr">
         <is>
@@ -9459,7 +9459,7 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>GROTESQQQUE-グロテスク-</t>
+          <t>劇場版 前橋ウィッチーズ ～魔女見習いのエモエモリーズ～</t>
         </is>
       </c>
       <c r="E175" t="b">
@@ -9472,12 +9472,12 @@
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>2026年11月6日</t>
+          <t>2026年10月23日</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>CloverWorks</t>
+          <t>Sunrise</t>
         </is>
       </c>
       <c r="I175" t="inlineStr"/>
@@ -9486,13 +9486,13 @@
       <c r="L175" t="inlineStr"/>
       <c r="M175" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/178972</t>
+          <t>https://anilist.co/anime/209642</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="n">
-        <v>-157330</v>
+        <v>-178972</v>
       </c>
       <c r="B176" t="inlineStr">
         <is>
@@ -9504,7 +9504,7 @@
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>楽園追放 心のレゾナンス</t>
+          <t>GROTESQQQUE-グロテスク-</t>
         </is>
       </c>
       <c r="E176" t="b">
@@ -9517,12 +9517,12 @@
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>2026年11月13日</t>
+          <t>2026年11月6日</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>Toei Animation</t>
+          <t>CloverWorks</t>
         </is>
       </c>
       <c r="I176" t="inlineStr"/>
@@ -9531,13 +9531,13 @@
       <c r="L176" t="inlineStr"/>
       <c r="M176" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/157330</t>
+          <t>https://anilist.co/anime/178972</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="n">
-        <v>-143103</v>
+        <v>-157330</v>
       </c>
       <c r="B177" t="inlineStr">
         <is>
@@ -9549,7 +9549,7 @@
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>魔法使いの夜</t>
+          <t>楽園追放 心のレゾナンス</t>
         </is>
       </c>
       <c r="E177" t="b">
@@ -9562,12 +9562,12 @@
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>2026年11月20日</t>
+          <t>2026年11月13日</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>ufotable</t>
+          <t>Toei Animation</t>
         </is>
       </c>
       <c r="I177" t="inlineStr"/>
@@ -9576,13 +9576,13 @@
       <c r="L177" t="inlineStr"/>
       <c r="M177" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/143103</t>
+          <t>https://anilist.co/anime/157330</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
-        <v>-206163</v>
+        <v>-143103</v>
       </c>
       <c r="B178" t="inlineStr">
         <is>
@@ -9594,7 +9594,7 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>装甲騎兵ボトムズ 灰色の魔女</t>
+          <t>魔法使いの夜</t>
         </is>
       </c>
       <c r="E178" t="b">
@@ -9612,7 +9612,7 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>Production I.G, Sunrise</t>
+          <t>ufotable</t>
         </is>
       </c>
       <c r="I178" t="inlineStr"/>
@@ -9621,13 +9621,13 @@
       <c r="L178" t="inlineStr"/>
       <c r="M178" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/206163</t>
+          <t>https://anilist.co/anime/143103</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="n">
-        <v>-212539</v>
+        <v>-206163</v>
       </c>
       <c r="B179" t="inlineStr">
         <is>
@@ -9639,7 +9639,7 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>タコピーの原罪 -ありがとう、また明日-</t>
+          <t>装甲騎兵ボトムズ 灰色の魔女</t>
         </is>
       </c>
       <c r="E179" t="b">
@@ -9652,12 +9652,12 @@
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>2026年11月27日</t>
+          <t>2026年11月20日</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>ENISHIYA</t>
+          <t>Production I.G, Sunrise</t>
         </is>
       </c>
       <c r="I179" t="inlineStr"/>
@@ -9666,13 +9666,13 @@
       <c r="L179" t="inlineStr"/>
       <c r="M179" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/212539</t>
+          <t>https://anilist.co/anime/206163</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="n">
-        <v>-205289</v>
+        <v>-212539</v>
       </c>
       <c r="B180" t="inlineStr">
         <is>
@@ -9684,7 +9684,7 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>ノーマン・ザ・スノーマン ~こどもたちのひとつ星~</t>
+          <t>タコピーの原罪 -ありがとう、また明日-</t>
         </is>
       </c>
       <c r="E180" t="b">
@@ -9697,12 +9697,12 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>2026年12月</t>
+          <t>2026年11月27日</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>TECARAT</t>
+          <t>ENISHIYA</t>
         </is>
       </c>
       <c r="I180" t="inlineStr"/>
@@ -9711,13 +9711,13 @@
       <c r="L180" t="inlineStr"/>
       <c r="M180" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/205289</t>
+          <t>https://anilist.co/anime/212539</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
-        <v>-200929</v>
+        <v>-205289</v>
       </c>
       <c r="B181" t="inlineStr">
         <is>
@@ -9729,7 +9729,7 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>薬屋のひとりごと 亡妃の秘宝</t>
+          <t>ノーマン・ザ・スノーマン ~こどもたちのひとつ星~</t>
         </is>
       </c>
       <c r="E181" t="b">
@@ -9742,12 +9742,12 @@
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>2026年12月11日</t>
+          <t>2026年12月</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>TOHO animation STUDIO</t>
+          <t>TECARAT</t>
         </is>
       </c>
       <c r="I181" t="inlineStr"/>
@@ -9756,17 +9756,17 @@
       <c r="L181" t="inlineStr"/>
       <c r="M181" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/200929</t>
+          <t>https://anilist.co/anime/205289</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
-        <v>-183692</v>
+        <v>-200929</v>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2027冬アニメ</t>
+          <t>2026秋アニメ</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -9774,7 +9774,7 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>機動戦士ガンダムSEED FREEDOM ZERO</t>
+          <t>薬屋のひとりごと 亡妃の秘宝</t>
         </is>
       </c>
       <c r="E182" t="b">
@@ -9787,12 +9787,12 @@
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>2027年1月15日</t>
+          <t>2026年12月11日</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>Sunrise</t>
+          <t>TOHO animation STUDIO</t>
         </is>
       </c>
       <c r="I182" t="inlineStr"/>
@@ -9801,13 +9801,13 @@
       <c r="L182" t="inlineStr"/>
       <c r="M182" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/183692</t>
+          <t>https://anilist.co/anime/200929</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
-        <v>-213814</v>
+        <v>-183692</v>
       </c>
       <c r="B183" t="inlineStr">
         <is>
@@ -9819,7 +9819,7 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>アイカツスターズ！ ～星々のProgress～</t>
+          <t>機動戦士ガンダムSEED FREEDOM ZERO</t>
         </is>
       </c>
       <c r="E183" t="b">
@@ -9832,12 +9832,12 @@
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>2027年1月22日</t>
+          <t>2027年1月15日</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>Bandai Namco Pictures</t>
+          <t>Sunrise</t>
         </is>
       </c>
       <c r="I183" t="inlineStr"/>
@@ -9846,13 +9846,13 @@
       <c r="L183" t="inlineStr"/>
       <c r="M183" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/213814</t>
+          <t>https://anilist.co/anime/183692</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
-        <v>-186603</v>
+        <v>-213814</v>
       </c>
       <c r="B184" t="inlineStr">
         <is>
@@ -9864,7 +9864,7 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>ラブライブ！虹ヶ咲学園スクールアイドル同好会 完結編 最終章</t>
+          <t>アイカツスターズ！ ～星々のProgress～</t>
         </is>
       </c>
       <c r="E184" t="b">
@@ -9877,12 +9877,12 @@
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>2027年2月5日</t>
+          <t>2027年1月22日</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>Sunrise</t>
+          <t>Bandai Namco Pictures</t>
         </is>
       </c>
       <c r="I184" t="inlineStr"/>
@@ -9891,13 +9891,13 @@
       <c r="L184" t="inlineStr"/>
       <c r="M184" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/186603</t>
+          <t>https://anilist.co/anime/213814</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
-        <v>-194213</v>
+        <v>-186603</v>
       </c>
       <c r="B185" t="inlineStr">
         <is>
@@ -9909,7 +9909,7 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>ghost／夜の果て</t>
+          <t>ラブライブ！虹ヶ咲学園スクールアイドル同好会 完結編 最終章</t>
         </is>
       </c>
       <c r="E185" t="b">
@@ -9922,12 +9922,12 @@
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>2027年2月11日</t>
+          <t>2027年2月5日</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>MADHOUSE</t>
+          <t>Sunrise</t>
         </is>
       </c>
       <c r="I185" t="inlineStr"/>
@@ -9936,13 +9936,13 @@
       <c r="L185" t="inlineStr"/>
       <c r="M185" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/194213</t>
+          <t>https://anilist.co/anime/186603</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="n">
-        <v>-206298</v>
+        <v>-194213</v>
       </c>
       <c r="B186" t="inlineStr">
         <is>
@@ -9954,7 +9954,7 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>劇場版 メダリスト</t>
+          <t>ghost／夜の果て</t>
         </is>
       </c>
       <c r="E186" t="b">
@@ -9967,12 +9967,12 @@
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>2027年2月19日</t>
+          <t>2027年2月11日</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>ENGI</t>
+          <t>MADHOUSE</t>
         </is>
       </c>
       <c r="I186" t="inlineStr"/>
@@ -9981,13 +9981,13 @@
       <c r="L186" t="inlineStr"/>
       <c r="M186" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/206298</t>
+          <t>https://anilist.co/anime/194213</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
-        <v>-216623</v>
+        <v>-206298</v>
       </c>
       <c r="B187" t="inlineStr">
         <is>
@@ -9999,7 +9999,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>ドラえもん のび太の蒸気時間車</t>
+          <t>劇場版 メダリスト</t>
         </is>
       </c>
       <c r="E187" t="b">
@@ -10012,12 +10012,12 @@
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>2027年3月5日</t>
+          <t>2027年2月19日</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>Shin-Ei Animation</t>
+          <t>ENGI</t>
         </is>
       </c>
       <c r="I187" t="inlineStr"/>
@@ -10026,13 +10026,13 @@
       <c r="L187" t="inlineStr"/>
       <c r="M187" t="inlineStr">
         <is>
-          <t>https://anilist.co/anime/216623</t>
+          <t>https://anilist.co/anime/206298</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="n">
-        <v>-190244</v>
+        <v>-216623</v>
       </c>
       <c r="B188" t="inlineStr">
         <is>
@@ -10044,7 +10044,7 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>デート・ア・ライブF Last Date</t>
+          <t>ドラえもん のび太の蒸気時間車</t>
         </is>
       </c>
       <c r="E188" t="b">
@@ -10057,12 +10057,12 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>2027年3月26日</t>
+          <t>2027年3月5日</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>Fugaku</t>
+          <t>Shin-Ei Animation</t>
         </is>
       </c>
       <c r="I188" t="inlineStr"/>
@@ -10070,6 +10070,51 @@
       <c r="K188" t="inlineStr"/>
       <c r="L188" t="inlineStr"/>
       <c r="M188" t="inlineStr">
+        <is>
+          <t>https://anilist.co/anime/216623</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="n">
+        <v>-190244</v>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>2027冬アニメ</t>
+        </is>
+      </c>
+      <c r="C189" t="n">
+        <v>0</v>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>デート・ア・ライブF Last Date</t>
+        </is>
+      </c>
+      <c r="E189" t="b">
+        <v>0</v>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>劇場版</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>2027年3月26日</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>Fugaku</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr"/>
+      <c r="J189" t="inlineStr"/>
+      <c r="K189" t="inlineStr"/>
+      <c r="L189" t="inlineStr"/>
+      <c r="M189" t="inlineStr">
         <is>
           <t>https://anilist.co/anime/190244</t>
         </is>
@@ -10455,7 +10500,7 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>410931</v>
+        <v>463076</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -10468,7 +10513,7 @@
         </is>
       </c>
       <c r="M6" t="n">
-        <v>410931</v>
+        <v>463076</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
@@ -10477,7 +10522,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>2026-10-22T09:00:25</t>
+          <t>2026-10-31T09:00:20</t>
         </is>
       </c>
     </row>
@@ -10522,7 +10567,7 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>87258</v>
+        <v>102146</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -10535,7 +10580,7 @@
         </is>
       </c>
       <c r="M7" t="n">
-        <v>87258</v>
+        <v>102146</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
@@ -10544,7 +10589,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026-10-22T09:00:35</t>
+          <t>2026-10-31T09:00:30</t>
         </is>
       </c>
     </row>
@@ -13587,13 +13632,27 @@
           <t>DayRe:</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=wNax51a6bAw</t>
+        </is>
+      </c>
+      <c r="J56" t="n">
+        <v>22315</v>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>DayRe:</t>
+        </is>
+      </c>
       <c r="L56" t="inlineStr"/>
       <c r="M56" t="inlineStr"/>
       <c r="N56" t="inlineStr"/>
-      <c r="O56" t="inlineStr"/>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>2026-10-31T09:01:21</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -15357,13 +15416,27 @@
           <t>sumika</t>
         </is>
       </c>
-      <c r="I86" t="inlineStr"/>
-      <c r="J86" t="inlineStr"/>
-      <c r="K86" t="inlineStr"/>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=OnbOB91hVwk</t>
+        </is>
+      </c>
+      <c r="J86" t="n">
+        <v>718126</v>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>sumika official</t>
+        </is>
+      </c>
       <c r="L86" t="inlineStr"/>
       <c r="M86" t="inlineStr"/>
       <c r="N86" t="inlineStr"/>
-      <c r="O86" t="inlineStr"/>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>2026-10-31T09:02:27</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -15406,7 +15479,7 @@
         </is>
       </c>
       <c r="J87" t="n">
-        <v>24102</v>
+        <v>113036</v>
       </c>
       <c r="K87" t="inlineStr">
         <is>
@@ -15418,7 +15491,7 @@
       <c r="N87" t="inlineStr"/>
       <c r="O87" t="inlineStr">
         <is>
-          <t>2026-10-23T09:01:58</t>
+          <t>2026-10-31T09:02:58</t>
         </is>
       </c>
     </row>

</xml_diff>